<commit_message>
Fix sentiment colours for puts (long put = bearish, short put = bullish)
Puts now invert the long/short/net colouring relative to futures and calls:
Added Put Longs and net-bought puts show red (bearish); Added Put Shorts and
net-sold puts show green (bullish). Futures and calls are unchanged.
Also commit a baseline report_data.hash so nightly commit-on-change is seeded.
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -784,7 +784,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -794,7 +794,7 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q4" s="11" t="n">
+      <c r="Q4" s="14" t="n">
         <v>66456</v>
       </c>
     </row>
@@ -955,7 +955,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="O7" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -965,7 +965,7 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q7" s="11" t="n">
+      <c r="Q7" s="14" t="n">
         <v>983</v>
       </c>
     </row>
@@ -1140,7 +1140,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O10" s="9" t="inlineStr">
+      <c r="O10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,7 +1150,7 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q10" s="11" t="n">
+      <c r="Q10" s="14" t="n">
         <v>5880</v>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1321,7 +1321,7 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q13" s="14" t="n">
+      <c r="Q13" s="11" t="n">
         <v>-3901</v>
       </c>
     </row>
@@ -1390,28 +1390,28 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C15" s="14" t="n">
         <v>488059</v>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="11" t="n">
         <v>421603</v>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="14" t="n">
         <v>66456</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
@@ -1453,28 +1453,28 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
+      <c r="C16" s="14" t="n">
         <v>5920</v>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="11" t="n">
         <v>40</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="14" t="n">
         <v>5880</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
@@ -1496,7 +1496,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O16" s="13" t="inlineStr">
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1506,7 +1506,7 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q16" s="14" t="n">
+      <c r="Q16" s="11" t="n">
         <v>-11350</v>
       </c>
     </row>
@@ -1516,28 +1516,28 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C17" s="14" t="n">
         <v>87926</v>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="11" t="n">
         <v>99276</v>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
+      <c r="G17" s="11" t="n">
         <v>-11350</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
@@ -1579,28 +1579,28 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
+      <c r="C18" s="14" t="n">
         <v>99106</v>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="11" t="n">
         <v>160093</v>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
+      <c r="G18" s="11" t="n">
         <v>-60987</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
@@ -1667,7 +1667,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O19" s="9" t="inlineStr">
+      <c r="O19" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1677,7 +1677,7 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q19" s="11" t="n">
+      <c r="Q19" s="14" t="n">
         <v>12049</v>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O22" s="13" t="inlineStr">
+      <c r="O22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1862,7 +1862,7 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q22" s="14" t="n">
+      <c r="Q22" s="11" t="n">
         <v>-60987</v>
       </c>
     </row>
@@ -2023,7 +2023,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O25" s="13" t="inlineStr">
+      <c r="O25" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2033,7 +2033,7 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q25" s="14" t="n">
+      <c r="Q25" s="11" t="n">
         <v>-9131</v>
       </c>
     </row>
@@ -2396,28 +2396,28 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
+      <c r="C33" s="11" t="n">
         <v>-39656</v>
       </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
+      <c r="E33" s="14" t="n">
         <v>-40639</v>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
+      <c r="G33" s="14" t="n">
         <v>983</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
@@ -2457,28 +2457,28 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
+      <c r="C34" s="11" t="n">
         <v>-3311</v>
       </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
+      <c r="E34" s="11" t="n">
         <v>590</v>
       </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
+      <c r="G34" s="11" t="n">
         <v>-3901</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
@@ -2518,28 +2518,28 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
+      <c r="C35" s="14" t="n">
         <v>292</v>
       </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
+      <c r="E35" s="14" t="n">
         <v>-11757</v>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n">
+      <c r="G35" s="14" t="n">
         <v>12049</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
@@ -2573,28 +2573,28 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
+      <c r="C36" s="11" t="n">
         <v>-31030</v>
       </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
+      <c r="E36" s="14" t="n">
         <v>-21899</v>
       </c>
-      <c r="F36" s="13" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="14" t="n">
+      <c r="G36" s="11" t="n">
         <v>-9131</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
@@ -2886,7 +2886,7 @@
     <row r="54">
       <c r="A54" s="32" t="inlineStr">
         <is>
-          <t>TODAY = 24-Jul-2026    1 DAY AGO = 23-Jul-2026    2 DAYS AGO = 22-Jul-2026    (generated 26-Jul-2026 00:46 IST)</t>
+          <t>TODAY = 24-Jul-2026    1 DAY AGO = 23-Jul-2026    2 DAYS AGO = 22-Jul-2026    (generated 26-Jul-2026 01:13 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-07-27
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -137,13 +137,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -180,6 +180,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -191,9 +194,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -660,7 +660,7 @@
       </c>
       <c r="O2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P2" s="10" t="inlineStr">
@@ -669,7 +669,7 @@
         </is>
       </c>
       <c r="Q2" s="11" t="n">
-        <v>9011</v>
+        <v>-7305</v>
       </c>
     </row>
     <row r="3">
@@ -680,59 +680,59 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>6852</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+        <v>-8837</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>-2159</v>
+      <c r="E3" s="13" t="n">
+        <v>-1532</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>-7305</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>169193</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>176498</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>167487</v>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="O3" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>9011</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>176498</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>167487</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>164583</v>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="O3" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q3" s="14" t="n">
-        <v>-122286</v>
+      <c r="Q3" s="13" t="n">
+        <v>21857</v>
       </c>
     </row>
     <row r="4">
@@ -741,50 +741,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>-2260</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C4" s="11" t="n">
+        <v>-76</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>-82</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E4" s="13" t="n">
+        <v>-33</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-2178</v>
+      <c r="G4" s="11" t="n">
+        <v>-43</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>65085</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>65128</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>67306</v>
       </c>
-      <c r="L4" s="12" t="n">
-        <v>73822</v>
-      </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O4" s="13" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -794,8 +794,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q4" s="14" t="n">
-        <v>66456</v>
+      <c r="Q4" s="11" t="n">
+        <v>48533</v>
       </c>
     </row>
     <row r="5">
@@ -804,61 +804,61 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>3963</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>11728</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="C5" s="13" t="n">
+        <v>192</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>-3730</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>3922</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>-266925</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>-270847</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>-263082</v>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-7765</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-270847</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-263082</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-251704</v>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="O5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="Q5" s="11" t="n">
-        <v>34754</v>
+        <v>-15599</v>
       </c>
     </row>
     <row r="6">
@@ -867,50 +867,50 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>4082</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>3150</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="C6" s="13" t="n">
+        <v>1247</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>-2179</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>932</v>
+      <c r="G6" s="13" t="n">
+        <v>3426</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>32647</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>29221</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>28289</v>
       </c>
-      <c r="L6" s="12" t="n">
-        <v>13299</v>
-      </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O6" s="13" t="inlineStr">
+      <c r="O6" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -920,8 +920,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q6" s="14" t="n">
-        <v>-42168</v>
+      <c r="Q6" s="11" t="n">
+        <v>-123469</v>
       </c>
     </row>
     <row r="7">
@@ -932,11 +932,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>12637</v>
+        <v>-7474</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>12637</v>
+        <v>-7474</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -955,7 +955,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q7" s="14" t="n">
-        <v>983</v>
+      <c r="Q7" s="11" t="n">
+        <v>56997</v>
       </c>
     </row>
     <row r="8">
@@ -1014,7 +1014,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="O8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1024,8 +1024,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q8" s="14" t="n">
-        <v>-2178</v>
+      <c r="Q8" s="11" t="n">
+        <v>-43</v>
       </c>
     </row>
     <row r="9">
@@ -1036,59 +1036,59 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>61199</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>183485</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+        <v>-59831</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>-81688</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>21857</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>66623</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>44766</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>167052</v>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-122286</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>44766</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>167052</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>172273</v>
-      </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="O9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="P9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q9" s="14" t="n">
-        <v>-50</v>
+      <c r="Q9" s="11" t="n">
+        <v>-5</v>
       </c>
     </row>
     <row r="10">
@@ -1099,48 +1099,48 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+        <v>-45</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>-40</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-50</v>
+      <c r="G10" s="11" t="n">
+        <v>-5</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>7535</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>7540</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>7590</v>
       </c>
-      <c r="L10" s="12" t="n">
-        <v>7695</v>
-      </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O10" s="13" t="inlineStr">
+      <c r="O10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q10" s="14" t="n">
-        <v>5880</v>
+      <c r="Q10" s="11" t="n">
+        <v>9472</v>
       </c>
     </row>
     <row r="11">
@@ -1160,50 +1160,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>63166</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>7489</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="C11" s="13" t="n">
+        <v>12002</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>-21270</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>55677</v>
+      <c r="G11" s="13" t="n">
+        <v>33272</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-225538</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-258810</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-314487</v>
       </c>
-      <c r="L11" s="12" t="n">
-        <v>-248973</v>
-      </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1213,8 +1213,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q11" s="14" t="n">
-        <v>-80818</v>
+      <c r="Q11" s="11" t="n">
+        <v>-25294</v>
       </c>
     </row>
     <row r="12">
@@ -1225,59 +1225,59 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>92223</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>25565</v>
+        <v>-92323</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>-37199</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>-55124</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>151379</v>
+      </c>
+      <c r="K12" s="14" t="n">
+        <v>206503</v>
+      </c>
+      <c r="L12" s="14" t="n">
+        <v>139845</v>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="O12" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>66658</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>206503</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>139845</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>69005</v>
-      </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="O12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="P12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q12" s="11" t="n">
-        <v>2657</v>
+      <c r="Q12" s="13" t="n">
+        <v>12172</v>
       </c>
     </row>
     <row r="13">
@@ -1288,15 +1288,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>216588</v>
+        <v>-140197</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>216589</v>
+        <v>-140197</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1313,7 +1313,7 @@
       </c>
       <c r="O13" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="P13" s="10" t="inlineStr">
@@ -1322,7 +1322,7 @@
         </is>
       </c>
       <c r="Q13" s="11" t="n">
-        <v>-3901</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="14">
@@ -1370,9 +1370,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="O14" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="P14" s="10" t="inlineStr">
@@ -1380,8 +1380,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q14" s="14" t="n">
-        <v>-7765</v>
+      <c r="Q14" s="13" t="n">
+        <v>3922</v>
       </c>
     </row>
     <row r="15">
@@ -1390,50 +1390,50 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>488059</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>558888</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>421603</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="E15" s="13" t="n">
+        <v>510355</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>66456</v>
+      <c r="G15" s="11" t="n">
+        <v>48533</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-654358</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-702891</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-769347</v>
       </c>
-      <c r="L15" s="12" t="n">
-        <v>-691782</v>
-      </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
+      <c r="O15" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1443,8 +1443,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q15" s="11" t="n">
-        <v>55677</v>
+      <c r="Q15" s="13" t="n">
+        <v>33272</v>
       </c>
     </row>
     <row r="16">
@@ -1453,50 +1453,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>5920</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>9472</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="E16" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>5880</v>
+      <c r="G16" s="11" t="n">
+        <v>9472</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>50521</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>41049</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>35169</v>
       </c>
-      <c r="L16" s="12" t="n">
-        <v>34102</v>
-      </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O16" s="9" t="inlineStr">
+      <c r="O16" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1506,8 +1506,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q16" s="11" t="n">
-        <v>-11350</v>
+      <c r="Q16" s="13" t="n">
+        <v>-53129</v>
       </c>
     </row>
     <row r="17">
@@ -1516,50 +1516,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>87926</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>-670</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>99276</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="13" t="n">
+        <v>52459</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-11350</v>
+      <c r="G17" s="13" t="n">
+        <v>-53129</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>482049</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>535178</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>546528</v>
       </c>
-      <c r="L17" s="12" t="n">
-        <v>544408</v>
-      </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O17" s="9" t="inlineStr">
+      <c r="O17" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1569,8 +1569,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q17" s="11" t="n">
-        <v>27563</v>
+      <c r="Q17" s="13" t="n">
+        <v>76479</v>
       </c>
     </row>
     <row r="18">
@@ -1579,52 +1579,52 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>99106</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>213492</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>160093</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="E18" s="13" t="n">
+        <v>218369</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-60987</v>
+      <c r="G18" s="13" t="n">
+        <v>-4877</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>121788</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>126665</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>187652</v>
       </c>
-      <c r="L18" s="12" t="n">
-        <v>113272</v>
-      </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="O18" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="P18" s="10" t="inlineStr">
@@ -1632,8 +1632,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q18" s="14" t="n">
-        <v>-35067</v>
+      <c r="Q18" s="13" t="n">
+        <v>3826</v>
       </c>
     </row>
     <row r="19">
@@ -1644,11 +1644,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>681011</v>
+        <v>781182</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>681012</v>
+        <v>781183</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1667,9 +1667,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O19" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="O19" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P19" s="10" t="inlineStr">
@@ -1677,8 +1677,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q19" s="14" t="n">
-        <v>12049</v>
+      <c r="Q19" s="13" t="n">
+        <v>-16885</v>
       </c>
     </row>
     <row r="20">
@@ -1726,7 +1726,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O20" s="9" t="inlineStr">
+      <c r="O20" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1736,8 +1736,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q20" s="11" t="n">
-        <v>932</v>
+      <c r="Q20" s="13" t="n">
+        <v>3426</v>
       </c>
     </row>
     <row r="21">
@@ -1746,44 +1746,44 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>-3872</v>
+      <c r="C21" s="11" t="n">
+        <v>-5437</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-38626</v>
+        <v>10162</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>34754</v>
+        <v>-15599</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>2898480</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>2914079</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>2879325</v>
       </c>
-      <c r="L21" s="12" t="n">
-        <v>2891344</v>
-      </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O21" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P21" s="10" t="inlineStr">
@@ -1800,7 +1800,7 @@
         </is>
       </c>
       <c r="Q21" s="11" t="n">
-        <v>66658</v>
+        <v>-55124</v>
       </c>
     </row>
     <row r="22">
@@ -1809,50 +1809,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>2776</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="13" t="n">
+        <v>13548</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>83594</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>38842</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-80818</v>
+      <c r="G22" s="11" t="n">
+        <v>-25294</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-3930238</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-3904944</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-3824126</v>
       </c>
-      <c r="L22" s="12" t="n">
-        <v>-3820778</v>
-      </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="O22" s="9" t="inlineStr">
+      <c r="O22" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1862,8 +1862,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q22" s="11" t="n">
-        <v>-60987</v>
+      <c r="Q22" s="13" t="n">
+        <v>-4877</v>
       </c>
     </row>
     <row r="23">
@@ -1874,42 +1874,42 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>1321</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+        <v>-8892</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>-26242</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="13" t="n">
+        <v>-85371</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>27563</v>
+      <c r="G23" s="13" t="n">
+        <v>76479</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>651191</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>574712</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>547149</v>
       </c>
-      <c r="L23" s="12" t="n">
-        <v>510676</v>
-      </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1917,7 +1917,7 @@
       </c>
       <c r="O23" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P23" s="10" t="inlineStr">
@@ -1926,7 +1926,7 @@
         </is>
       </c>
       <c r="Q23" s="11" t="n">
-        <v>18501</v>
+        <v>-35586</v>
       </c>
     </row>
     <row r="24">
@@ -1935,61 +1935,61 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>-73175</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>-53049</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>-91676</v>
+      <c r="E24" s="13" t="n">
+        <v>-17463</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>-35586</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>380567</v>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>416153</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>397652</v>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="O24" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>18501</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>416153</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>397652</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>418758</v>
-      </c>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="O24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="P24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q24" s="11" t="n">
-        <v>74578</v>
+      <c r="Q24" s="13" t="n">
+        <v>107471</v>
       </c>
     </row>
     <row r="25">
@@ -2000,11 +2000,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-72950</v>
+        <v>-53830</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-72950</v>
+        <v>-53830</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2023,7 +2023,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
+      <c r="O25" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2033,8 +2033,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q25" s="11" t="n">
-        <v>-9131</v>
+      <c r="Q25" s="13" t="n">
+        <v>-42390</v>
       </c>
     </row>
     <row r="26">
@@ -2084,43 +2084,43 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>-94225</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>-197385</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>-52057</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="13" t="n">
+        <v>-73916</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>-42168</v>
+      <c r="G27" s="11" t="n">
+        <v>-123469</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>991712</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>1115181</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>1157349</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>1200637</v>
       </c>
     </row>
     <row r="28">
@@ -2131,41 +2131,41 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>631</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>-1362</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>-2026</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>-13534</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>2657</v>
+      <c r="G28" s="13" t="n">
+        <v>12172</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-421370</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-433542</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-436199</v>
-      </c>
-      <c r="L28" s="12" t="n">
-        <v>-432078</v>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
@@ -2182,47 +2182,47 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>-23502</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>11565</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>-35067</v>
+      <c r="C29" s="11" t="n">
+        <v>-30157</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>-33983</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>3826</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-212909</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-216735</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-181668</v>
       </c>
-      <c r="L29" s="12" t="n">
-        <v>-188237</v>
-      </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 24-Jul-2026 OHLC</t>
+          <t>Next session  -  based on 27-Jul-2026 OHLC</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
@@ -2235,51 +2235,51 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>-16557</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>-14721</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>-91135</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="13" t="n">
+        <v>-122192</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>74578</v>
+      <c r="G30" s="13" t="n">
+        <v>107471</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-357433</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-464904</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-539482</v>
       </c>
-      <c r="L30" s="12" t="n">
-        <v>-580322</v>
-      </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="O30" s="18" t="n">
-        <v>23666.35</v>
+        <v>23928.4</v>
       </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23823.6</v>
+        <v>24011.6</v>
       </c>
     </row>
     <row r="31">
@@ -2298,11 +2298,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-133653</v>
+        <v>-243625</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-133653</v>
+        <v>-243625</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="O31" s="18" t="n">
-        <v>23606.3</v>
+        <v>23891.55</v>
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
@@ -2330,7 +2330,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23767.45</v>
+        <v>23995.95</v>
       </c>
     </row>
     <row r="32">
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="O32" s="20" t="n">
-        <v>24075.89999999999</v>
+        <v>24161.23333333333</v>
       </c>
       <c r="P32" s="8" t="inlineStr">
         <is>
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="Q32" s="21" t="n">
-        <v>23749.95</v>
+        <v>23981.15833333333</v>
       </c>
     </row>
     <row r="33">
@@ -2398,49 +2398,49 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-39656</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+        <v>2025</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>-40639</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="E33" s="11" t="n">
+        <v>-54972</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>983</v>
+      <c r="G33" s="11" t="n">
+        <v>56997</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-344565</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-401562</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-402545</v>
       </c>
-      <c r="L33" s="12" t="n">
-        <v>-405137</v>
-      </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="O33" s="20" t="n">
-        <v>23949.75</v>
+        <v>24086.41666666666</v>
       </c>
       <c r="P33" s="8" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
         </is>
       </c>
       <c r="Q33" s="21" t="n">
-        <v>23732.45</v>
+        <v>23966.36666666666</v>
       </c>
     </row>
     <row r="34">
@@ -2459,49 +2459,49 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>-3311</v>
+        <v>1707</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>590</v>
+        <v>-571</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-3901</v>
+        <v>2278</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>23915</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>21637</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>25538</v>
       </c>
-      <c r="L34" s="12" t="n">
-        <v>26070</v>
-      </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="O34" s="20" t="n">
-        <v>23858.59999999999</v>
+        <v>24041.18333333333</v>
       </c>
       <c r="P34" s="8" t="inlineStr">
         <is>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q34" s="21" t="n">
-        <v>23714.95</v>
+        <v>23951.575</v>
       </c>
     </row>
     <row r="35">
@@ -2518,51 +2518,51 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="n">
-        <v>292</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>-52769</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>-11757</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>12049</v>
+      <c r="E35" s="11" t="n">
+        <v>-35884</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="n">
+        <v>-16885</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>176868</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>193753</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>181704</v>
       </c>
-      <c r="L35" s="12" t="n">
-        <v>169545</v>
-      </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="O35" s="21" t="n">
-        <v>23732.45</v>
+        <v>23966.36666666666</v>
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
@@ -2573,51 +2573,51 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>-31030</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="13" t="n">
+        <v>-56286</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>-21899</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="E36" s="11" t="n">
+        <v>-13896</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n">
-        <v>-9131</v>
+      <c r="G36" s="13" t="n">
+        <v>-42390</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>143782</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>186172</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>195303</v>
       </c>
-      <c r="L36" s="12" t="n">
-        <v>209522</v>
-      </c>
       <c r="N36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="O36" s="23" t="n">
-        <v>23641.3</v>
+        <v>23921.13333333333</v>
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
@@ -2630,11 +2630,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-73705</v>
+        <v>-105323</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-73705</v>
+        <v>-105323</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2654,7 +2654,7 @@
         </is>
       </c>
       <c r="O37" s="23" t="n">
-        <v>23515.15</v>
+        <v>23846.31666666667</v>
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="O38" s="23" t="n">
-        <v>23424</v>
+        <v>23801.08333333333</v>
       </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
@@ -2685,7 +2685,7 @@
     <row r="42">
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,767    PCR(OI) 0.83    Max Pain 23,900</t>
+          <t>Spot 23,996    PCR(OI) 1.12    Max Pain 24,000</t>
         </is>
       </c>
       <c r="O42" s="6" t="n"/>
@@ -2735,18 +2735,18 @@
       <c r="N45" s="26" t="n">
         <v>24000</v>
       </c>
-      <c r="O45" s="12" t="n">
-        <v>207372</v>
+      <c r="O45" s="14" t="n">
+        <v>191831</v>
       </c>
       <c r="P45" s="11" t="n">
-        <v>8169</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>3682197</v>
+        <v>-15541</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>10162515</v>
       </c>
       <c r="R45" s="27" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -2754,18 +2754,18 @@
       <c r="N46" s="26" t="n">
         <v>24200</v>
       </c>
-      <c r="O46" s="12" t="n">
-        <v>203857</v>
-      </c>
-      <c r="P46" s="11" t="n">
-        <v>5766</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>1843347</v>
+      <c r="O46" s="14" t="n">
+        <v>226746</v>
+      </c>
+      <c r="P46" s="13" t="n">
+        <v>22889</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>3967068</v>
       </c>
       <c r="R46" s="28" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -2773,23 +2773,23 @@
       <c r="N47" s="26" t="n">
         <v>25000</v>
       </c>
-      <c r="O47" s="12" t="n">
-        <v>231527</v>
-      </c>
-      <c r="P47" s="14" t="n">
-        <v>-15414</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>945928</v>
-      </c>
-      <c r="R47" s="28" t="inlineStr">
+      <c r="O47" s="14" t="n">
+        <v>182389</v>
+      </c>
+      <c r="P47" s="11" t="n">
+        <v>-49138</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>758461</v>
+      </c>
+      <c r="R47" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="N48" s="29" t="inlineStr">
+      <c r="N48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -2827,57 +2827,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="N50" s="30" t="n">
-        <v>23700</v>
-      </c>
-      <c r="O50" s="12" t="n">
-        <v>127850</v>
-      </c>
-      <c r="P50" s="11" t="n">
-        <v>49654</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>5657061</v>
-      </c>
-      <c r="R50" s="31" t="inlineStr">
+      <c r="N50" s="31" t="n">
+        <v>24000</v>
+      </c>
+      <c r="O50" s="14" t="n">
+        <v>208738</v>
+      </c>
+      <c r="P50" s="13" t="n">
+        <v>136619</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>7020028</v>
+      </c>
+      <c r="R50" s="27" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="N51" s="30" t="n">
-        <v>23500</v>
-      </c>
-      <c r="O51" s="12" t="n">
-        <v>159245</v>
-      </c>
-      <c r="P51" s="11" t="n">
-        <v>21692</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>3560576</v>
+      <c r="N51" s="31" t="n">
+        <v>23900</v>
+      </c>
+      <c r="O51" s="14" t="n">
+        <v>190077</v>
+      </c>
+      <c r="P51" s="13" t="n">
+        <v>141236</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>8312324</v>
       </c>
       <c r="R51" s="27" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="N52" s="30" t="n">
+      <c r="N52" s="31" t="n">
         <v>23000</v>
       </c>
-      <c r="O52" s="12" t="n">
-        <v>203409</v>
-      </c>
-      <c r="P52" s="11" t="n">
-        <v>39094</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>1544770</v>
-      </c>
-      <c r="R52" s="28" t="inlineStr">
+      <c r="O52" s="14" t="n">
+        <v>216353</v>
+      </c>
+      <c r="P52" s="13" t="n">
+        <v>12944</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>1386067</v>
+      </c>
+      <c r="R52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2886,7 +2886,7 @@
     <row r="54">
       <c r="A54" s="32" t="inlineStr">
         <is>
-          <t>TODAY = 24-Jul-2026    1 DAY AGO = 23-Jul-2026    2 DAYS AGO = 22-Jul-2026    (generated 26-Jul-2026 01:13 IST)</t>
+          <t>TODAY = 27-Jul-2026    1 DAY AGO = 24-Jul-2026    2 DAYS AGO = 23-Jul-2026    (generated 27-Jul-2026 22:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-07-28
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -184,9 +184,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -669,7 +666,7 @@
         </is>
       </c>
       <c r="Q2" s="11" t="n">
-        <v>-7305</v>
+        <v>-15940</v>
       </c>
     </row>
     <row r="3">
@@ -684,7 +681,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-8837</v>
+        <v>-25089</v>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
@@ -692,7 +689,7 @@
         </is>
       </c>
       <c r="E3" s="13" t="n">
-        <v>-1532</v>
+        <v>-9149</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -700,7 +697,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-7305</v>
+        <v>-15940</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -708,14 +705,14 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>153253</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>169193</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>176498</v>
       </c>
-      <c r="L3" s="14" t="n">
-        <v>167487</v>
-      </c>
       <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -732,7 +729,7 @@
         </is>
       </c>
       <c r="Q3" s="13" t="n">
-        <v>21857</v>
+        <v>122423</v>
       </c>
     </row>
     <row r="4">
@@ -747,7 +744,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-76</v>
+        <v>-10618</v>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
@@ -755,7 +752,7 @@
         </is>
       </c>
       <c r="E4" s="13" t="n">
-        <v>-33</v>
+        <v>-4</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -763,7 +760,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>-43</v>
+        <v>-10614</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -771,14 +768,14 @@
         </is>
       </c>
       <c r="J4" s="14" t="n">
+        <v>54471</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>65085</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="14" t="n">
         <v>65128</v>
       </c>
-      <c r="L4" s="14" t="n">
-        <v>67306</v>
-      </c>
       <c r="N4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -795,7 +792,7 @@
         </is>
       </c>
       <c r="Q4" s="11" t="n">
-        <v>48533</v>
+        <v>31031</v>
       </c>
     </row>
     <row r="5">
@@ -804,13 +801,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>192</v>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>-6567</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
@@ -818,7 +815,7 @@
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>-3730</v>
+        <v>-67891</v>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
@@ -826,7 +823,7 @@
         </is>
       </c>
       <c r="G5" s="13" t="n">
-        <v>3922</v>
+        <v>61324</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -834,14 +831,14 @@
         </is>
       </c>
       <c r="J5" s="14" t="n">
+        <v>-205601</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-266925</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="14" t="n">
         <v>-270847</v>
       </c>
-      <c r="L5" s="14" t="n">
-        <v>-263082</v>
-      </c>
       <c r="N5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -858,7 +855,7 @@
         </is>
       </c>
       <c r="Q5" s="11" t="n">
-        <v>-15599</v>
+        <v>-20076</v>
       </c>
     </row>
     <row r="6">
@@ -867,13 +864,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>1247</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>-45411</v>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
@@ -881,15 +878,15 @@
         </is>
       </c>
       <c r="E6" s="13" t="n">
-        <v>-2179</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>3426</v>
+        <v>-10641</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-34770</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -897,14 +894,14 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>-2123</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>32647</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>29221</v>
       </c>
-      <c r="L6" s="14" t="n">
-        <v>28289</v>
-      </c>
       <c r="N6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -921,7 +918,7 @@
         </is>
       </c>
       <c r="Q6" s="11" t="n">
-        <v>-123469</v>
+        <v>-579099</v>
       </c>
     </row>
     <row r="7">
@@ -932,11 +929,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-7474</v>
+        <v>-87685</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-7474</v>
+        <v>-87685</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -966,7 +963,7 @@
         </is>
       </c>
       <c r="Q7" s="11" t="n">
-        <v>56997</v>
+        <v>92551</v>
       </c>
     </row>
     <row r="8">
@@ -1025,7 +1022,7 @@
         </is>
       </c>
       <c r="Q8" s="11" t="n">
-        <v>-43</v>
+        <v>-10614</v>
       </c>
     </row>
     <row r="9">
@@ -1040,7 +1037,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-59831</v>
+        <v>-1689253</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1048,7 +1045,7 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>-81688</v>
+        <v>-1811676</v>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
@@ -1056,7 +1053,7 @@
         </is>
       </c>
       <c r="G9" s="13" t="n">
-        <v>21857</v>
+        <v>122423</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1064,14 +1061,14 @@
         </is>
       </c>
       <c r="J9" s="14" t="n">
+        <v>189046</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>66623</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="14" t="n">
         <v>44766</v>
       </c>
-      <c r="L9" s="14" t="n">
-        <v>167052</v>
-      </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1088,7 +1085,7 @@
         </is>
       </c>
       <c r="Q9" s="11" t="n">
-        <v>-5</v>
+        <v>-4255</v>
       </c>
     </row>
     <row r="10">
@@ -1103,7 +1100,7 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>-45</v>
+        <v>-4410</v>
       </c>
       <c r="D10" s="12" t="inlineStr">
         <is>
@@ -1111,7 +1108,7 @@
         </is>
       </c>
       <c r="E10" s="13" t="n">
-        <v>-40</v>
+        <v>-155</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1119,7 +1116,7 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>-5</v>
+        <v>-4255</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1127,22 +1124,22 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
+        <v>3280</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>7535</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="14" t="n">
         <v>7540</v>
       </c>
-      <c r="L10" s="14" t="n">
-        <v>7590</v>
-      </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="O10" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P10" s="10" t="inlineStr">
@@ -1150,8 +1147,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q10" s="11" t="n">
-        <v>9472</v>
+      <c r="Q10" s="13" t="n">
+        <v>-12444</v>
       </c>
     </row>
     <row r="11">
@@ -1160,13 +1157,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="n">
-        <v>12002</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>-388990</v>
       </c>
       <c r="D11" s="12" t="inlineStr">
         <is>
@@ -1174,15 +1171,15 @@
         </is>
       </c>
       <c r="E11" s="13" t="n">
-        <v>-21270</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="n">
-        <v>33272</v>
+        <v>-366981</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>-22009</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1190,14 +1187,14 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-247547</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-225538</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-258810</v>
       </c>
-      <c r="L11" s="14" t="n">
-        <v>-314487</v>
-      </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1214,7 +1211,7 @@
         </is>
       </c>
       <c r="Q11" s="11" t="n">
-        <v>-25294</v>
+        <v>-10741</v>
       </c>
     </row>
     <row r="12">
@@ -1229,7 +1226,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-92323</v>
+        <v>-701443</v>
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
@@ -1237,7 +1234,7 @@
         </is>
       </c>
       <c r="E12" s="13" t="n">
-        <v>-37199</v>
+        <v>-605285</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1245,7 +1242,7 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>-55124</v>
+        <v>-96158</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1253,14 +1250,14 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
+        <v>55221</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>151379</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="14" t="n">
         <v>206503</v>
       </c>
-      <c r="L12" s="14" t="n">
-        <v>139845</v>
-      </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1277,7 +1274,7 @@
         </is>
       </c>
       <c r="Q12" s="13" t="n">
-        <v>12172</v>
+        <v>345566</v>
       </c>
     </row>
     <row r="13">
@@ -1288,15 +1285,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-140197</v>
+        <v>-2784096</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-140197</v>
+        <v>-2784097</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1322,7 +1319,7 @@
         </is>
       </c>
       <c r="Q13" s="11" t="n">
-        <v>2278</v>
+        <v>3740</v>
       </c>
     </row>
     <row r="14">
@@ -1381,7 +1378,7 @@
         </is>
       </c>
       <c r="Q14" s="13" t="n">
-        <v>3922</v>
+        <v>61324</v>
       </c>
     </row>
     <row r="15">
@@ -1390,21 +1387,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>558888</v>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="n">
-        <v>510355</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>-1816714</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>-1847745</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1412,7 +1409,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>48533</v>
+        <v>31031</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1420,22 +1417,22 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-623327</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-654358</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-702891</v>
       </c>
-      <c r="L15" s="14" t="n">
-        <v>-769347</v>
-      </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O15" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="O15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P15" s="10" t="inlineStr">
@@ -1443,8 +1440,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="n">
-        <v>33272</v>
+      <c r="Q15" s="11" t="n">
+        <v>-22009</v>
       </c>
     </row>
     <row r="16">
@@ -1453,61 +1450,61 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>9472</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>-12544</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>-100</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>-12444</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>38077</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <v>50521</v>
+      </c>
+      <c r="L16" s="14" t="n">
+        <v>41049</v>
+      </c>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="O16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>9472</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>50521</v>
-      </c>
-      <c r="K16" s="14" t="n">
-        <v>41049</v>
-      </c>
-      <c r="L16" s="14" t="n">
-        <v>35169</v>
-      </c>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="O16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="P16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="n">
-        <v>-53129</v>
+      <c r="Q16" s="11" t="n">
+        <v>39851</v>
       </c>
     </row>
     <row r="17">
@@ -1522,55 +1519,55 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>-670</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>52459</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+        <v>-391322</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>-431173</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>39851</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>521900</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>482049</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>535178</v>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>-53129</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>482049</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>535178</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>546528</v>
-      </c>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="O17" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="P17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="n">
-        <v>76479</v>
+      <c r="Q17" s="11" t="n">
+        <v>-86982</v>
       </c>
     </row>
     <row r="18">
@@ -1579,21 +1576,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>213492</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="n">
-        <v>218369</v>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>-716833</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>-658395</v>
       </c>
       <c r="F18" s="12" t="inlineStr">
         <is>
@@ -1601,7 +1598,7 @@
         </is>
       </c>
       <c r="G18" s="13" t="n">
-        <v>-4877</v>
+        <v>-58438</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1609,14 +1606,14 @@
         </is>
       </c>
       <c r="J18" s="14" t="n">
+        <v>63350</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>121788</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="14" t="n">
         <v>126665</v>
       </c>
-      <c r="L18" s="14" t="n">
-        <v>187652</v>
-      </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1633,7 +1630,7 @@
         </is>
       </c>
       <c r="Q18" s="13" t="n">
-        <v>3826</v>
+        <v>165045</v>
       </c>
     </row>
     <row r="19">
@@ -1644,15 +1641,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>781182</v>
+        <v>-2937413</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>781183</v>
+        <v>-2937413</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1678,7 +1675,7 @@
         </is>
       </c>
       <c r="Q19" s="13" t="n">
-        <v>-16885</v>
+        <v>-113861</v>
       </c>
     </row>
     <row r="20">
@@ -1726,9 +1723,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O20" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="O20" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="P20" s="10" t="inlineStr">
@@ -1736,8 +1733,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="n">
-        <v>3426</v>
+      <c r="Q20" s="11" t="n">
+        <v>-34770</v>
       </c>
     </row>
     <row r="21">
@@ -1752,15 +1749,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-5437</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>10162</v>
+        <v>-114039</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>-93963</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1768,7 +1765,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>-15599</v>
+        <v>-20076</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1776,14 +1773,14 @@
         </is>
       </c>
       <c r="J21" s="14" t="n">
+        <v>2878404</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>2898480</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="14" t="n">
         <v>2914079</v>
       </c>
-      <c r="L21" s="14" t="n">
-        <v>2879325</v>
-      </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1800,7 +1797,7 @@
         </is>
       </c>
       <c r="Q21" s="11" t="n">
-        <v>-55124</v>
+        <v>-96158</v>
       </c>
     </row>
     <row r="22">
@@ -1809,21 +1806,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="13" t="n">
-        <v>13548</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>38842</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>-161696</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>-150955</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1831,7 +1828,7 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-25294</v>
+        <v>-10741</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1839,14 +1836,14 @@
         </is>
       </c>
       <c r="J22" s="14" t="n">
+        <v>-3940979</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-3930238</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="14" t="n">
         <v>-3904944</v>
       </c>
-      <c r="L22" s="14" t="n">
-        <v>-3824126</v>
-      </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1863,7 +1860,7 @@
         </is>
       </c>
       <c r="Q22" s="13" t="n">
-        <v>-4877</v>
+        <v>-58438</v>
       </c>
     </row>
     <row r="23">
@@ -1878,7 +1875,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>-8892</v>
+        <v>-230667</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -1886,47 +1883,47 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>-85371</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+        <v>-143685</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-86982</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="14" t="n">
+        <v>564209</v>
+      </c>
+      <c r="K23" s="14" t="n">
+        <v>651191</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>574712</v>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="O23" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>76479</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>651191</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>574712</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>547149</v>
-      </c>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="O23" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="P23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q23" s="11" t="n">
-        <v>-35586</v>
+      <c r="Q23" s="13" t="n">
+        <v>117799</v>
       </c>
     </row>
     <row r="24">
@@ -1941,7 +1938,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-53049</v>
+        <v>-105728</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -1949,15 +1946,15 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>-17463</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>-35586</v>
+        <v>-223527</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>117799</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -1965,14 +1962,14 @@
         </is>
       </c>
       <c r="J24" s="14" t="n">
+        <v>498366</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>380567</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="14" t="n">
         <v>416153</v>
       </c>
-      <c r="L24" s="14" t="n">
-        <v>397652</v>
-      </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1989,7 +1986,7 @@
         </is>
       </c>
       <c r="Q24" s="13" t="n">
-        <v>107471</v>
+        <v>68488</v>
       </c>
     </row>
     <row r="25">
@@ -2000,11 +1997,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-53830</v>
+        <v>-612130</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-53830</v>
+        <v>-612130</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2023,9 +2020,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="O25" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="O25" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="P25" s="10" t="inlineStr">
@@ -2033,8 +2030,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="n">
-        <v>-42390</v>
+      <c r="Q25" s="11" t="n">
+        <v>17570</v>
       </c>
     </row>
     <row r="26">
@@ -2090,7 +2087,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-197385</v>
+        <v>-1232410</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -2098,7 +2095,7 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>-73916</v>
+        <v>-653311</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2106,7 +2103,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-123469</v>
+        <v>-579099</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2114,13 +2111,13 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>412613</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>991712</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>1115181</v>
-      </c>
-      <c r="L27" s="14" t="n">
-        <v>1157349</v>
       </c>
     </row>
     <row r="28">
@@ -2135,7 +2132,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-1362</v>
+        <v>-2246</v>
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
@@ -2143,7 +2140,7 @@
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>-13534</v>
+        <v>-347812</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
@@ -2151,7 +2148,7 @@
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>12172</v>
+        <v>345566</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2159,13 +2156,13 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-75804</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-421370</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-433542</v>
-      </c>
-      <c r="L28" s="14" t="n">
-        <v>-436199</v>
       </c>
       <c r="N28" s="3" t="inlineStr">
         <is>
@@ -2188,7 +2185,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>-30157</v>
+        <v>-171405</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -2196,7 +2193,7 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>-33983</v>
+        <v>-336450</v>
       </c>
       <c r="F29" s="12" t="inlineStr">
         <is>
@@ -2204,7 +2201,7 @@
         </is>
       </c>
       <c r="G29" s="13" t="n">
-        <v>3826</v>
+        <v>165045</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2212,17 +2209,17 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-47864</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-212909</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-216735</v>
       </c>
-      <c r="L29" s="14" t="n">
-        <v>-181668</v>
-      </c>
       <c r="N29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 27-Jul-2026 OHLC</t>
+          <t>Next session  -  based on 28-Jul-2026 OHLC</t>
         </is>
       </c>
       <c r="O29" s="6" t="inlineStr"/>
@@ -2241,7 +2238,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>-14721</v>
+        <v>-778878</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -2249,7 +2246,7 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>-122192</v>
+        <v>-847366</v>
       </c>
       <c r="F30" s="12" t="inlineStr">
         <is>
@@ -2257,7 +2254,7 @@
         </is>
       </c>
       <c r="G30" s="13" t="n">
-        <v>107471</v>
+        <v>68488</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2265,21 +2262,21 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-288945</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-357433</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-464904</v>
       </c>
-      <c r="L30" s="14" t="n">
-        <v>-539482</v>
-      </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="O30" s="18" t="n">
-        <v>23928.4</v>
+        <v>23971.25</v>
       </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
@@ -2287,7 +2284,7 @@
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24011.6</v>
+        <v>24041.15</v>
       </c>
     </row>
     <row r="31">
@@ -2298,11 +2295,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-243625</v>
+        <v>-2184939</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-243625</v>
+        <v>-2184939</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2322,7 +2319,7 @@
         </is>
       </c>
       <c r="O31" s="18" t="n">
-        <v>23891.55</v>
+        <v>23954.6</v>
       </c>
       <c r="P31" s="8" t="inlineStr">
         <is>
@@ -2330,7 +2327,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23995.95</v>
+        <v>23985.35</v>
       </c>
     </row>
     <row r="32">
@@ -2379,7 +2376,7 @@
         </is>
       </c>
       <c r="O32" s="20" t="n">
-        <v>24161.23333333333</v>
+        <v>24119.35000000001</v>
       </c>
       <c r="P32" s="8" t="inlineStr">
         <is>
@@ -2387,7 +2384,7 @@
         </is>
       </c>
       <c r="Q32" s="21" t="n">
-        <v>23981.15833333333</v>
+        <v>23989.525</v>
       </c>
     </row>
     <row r="33">
@@ -2396,13 +2393,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>2025</v>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>-386911</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2410,7 +2407,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-54972</v>
+        <v>-479462</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2418,7 +2415,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>56997</v>
+        <v>92551</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2426,21 +2423,21 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-252014</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-344565</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-401562</v>
       </c>
-      <c r="L33" s="14" t="n">
-        <v>-402545</v>
-      </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="O33" s="20" t="n">
-        <v>24086.41666666666</v>
+        <v>24080.25</v>
       </c>
       <c r="P33" s="8" t="inlineStr">
         <is>
@@ -2448,7 +2445,7 @@
         </is>
       </c>
       <c r="Q33" s="21" t="n">
-        <v>23966.36666666666</v>
+        <v>23993.7</v>
       </c>
     </row>
     <row r="34">
@@ -2457,13 +2454,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="n">
-        <v>1707</v>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>-6780</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2471,7 +2468,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>-571</v>
+        <v>-10520</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2479,7 +2476,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>2278</v>
+        <v>3740</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2487,21 +2484,21 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>27655</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>23915</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>21637</v>
       </c>
-      <c r="L34" s="14" t="n">
-        <v>25538</v>
-      </c>
       <c r="N34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="O34" s="20" t="n">
-        <v>24041.18333333333</v>
+        <v>24032.8</v>
       </c>
       <c r="P34" s="8" t="inlineStr">
         <is>
@@ -2509,7 +2506,7 @@
         </is>
       </c>
       <c r="Q34" s="21" t="n">
-        <v>23951.575</v>
+        <v>23997.875</v>
       </c>
     </row>
     <row r="35">
@@ -2524,7 +2521,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>-52769</v>
+        <v>-297205</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2532,7 +2529,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>-35884</v>
+        <v>-183344</v>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
@@ -2540,7 +2537,7 @@
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>-16885</v>
+        <v>-113861</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2548,21 +2545,21 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>63007</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>176868</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>193753</v>
       </c>
-      <c r="L35" s="14" t="n">
-        <v>181704</v>
-      </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="O35" s="21" t="n">
-        <v>23966.36666666666</v>
+        <v>23993.7</v>
       </c>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
@@ -2579,7 +2576,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="n">
-        <v>-56286</v>
+        <v>-604692</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2587,15 +2584,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>-13896</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="n">
-        <v>-42390</v>
+        <v>-622262</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>17570</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2603,21 +2600,21 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>161352</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>143782</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>186172</v>
       </c>
-      <c r="L36" s="14" t="n">
-        <v>195303</v>
-      </c>
       <c r="N36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="O36" s="23" t="n">
-        <v>23921.13333333333</v>
+        <v>23946.25</v>
       </c>
       <c r="P36" t="inlineStr"/>
       <c r="Q36" t="inlineStr"/>
@@ -2630,11 +2627,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-105323</v>
+        <v>-1295588</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-105323</v>
+        <v>-1295588</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2654,7 +2651,7 @@
         </is>
       </c>
       <c r="O37" s="23" t="n">
-        <v>23846.31666666667</v>
+        <v>23907.15</v>
       </c>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
@@ -2666,7 +2663,7 @@
         </is>
       </c>
       <c r="O38" s="23" t="n">
-        <v>23801.08333333333</v>
+        <v>23859.7</v>
       </c>
       <c r="P38" t="inlineStr"/>
       <c r="Q38" t="inlineStr"/>
@@ -2685,7 +2682,7 @@
     <row r="42">
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,996    PCR(OI) 1.12    Max Pain 24,000</t>
+          <t>Spot 23,985    PCR(OI) 0.94    Max Pain 24,000</t>
         </is>
       </c>
       <c r="O42" s="6" t="n"/>
@@ -2736,13 +2733,13 @@
         <v>24000</v>
       </c>
       <c r="O45" s="14" t="n">
-        <v>191831</v>
-      </c>
-      <c r="P45" s="11" t="n">
-        <v>-15541</v>
+        <v>479480</v>
+      </c>
+      <c r="P45" s="13" t="n">
+        <v>287649</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>10162515</v>
+        <v>40300828</v>
       </c>
       <c r="R45" s="27" t="inlineStr">
         <is>
@@ -2752,16 +2749,16 @@
     </row>
     <row r="46">
       <c r="N46" s="26" t="n">
-        <v>24200</v>
+        <v>24050</v>
       </c>
       <c r="O46" s="14" t="n">
-        <v>226746</v>
+        <v>201655</v>
       </c>
       <c r="P46" s="13" t="n">
-        <v>22889</v>
+        <v>105631</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>3967068</v>
+        <v>25118624</v>
       </c>
       <c r="R46" s="28" t="inlineStr">
         <is>
@@ -2771,25 +2768,25 @@
     </row>
     <row r="47">
       <c r="N47" s="26" t="n">
-        <v>25000</v>
+        <v>24100</v>
       </c>
       <c r="O47" s="14" t="n">
-        <v>182389</v>
-      </c>
-      <c r="P47" s="11" t="n">
-        <v>-49138</v>
+        <v>167825</v>
+      </c>
+      <c r="P47" s="13" t="n">
+        <v>7477</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>758461</v>
-      </c>
-      <c r="R47" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>15245129</v>
+      </c>
+      <c r="R47" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="N48" s="30" t="inlineStr">
+      <c r="N48" s="29" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -2827,17 +2824,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="N50" s="31" t="n">
+      <c r="N50" s="30" t="n">
         <v>24000</v>
       </c>
       <c r="O50" s="14" t="n">
-        <v>208738</v>
+        <v>246462</v>
       </c>
       <c r="P50" s="13" t="n">
-        <v>136619</v>
+        <v>37724</v>
       </c>
       <c r="Q50" s="14" t="n">
-        <v>7020028</v>
+        <v>37388862</v>
       </c>
       <c r="R50" s="27" t="inlineStr">
         <is>
@@ -2846,47 +2843,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="N51" s="31" t="n">
+      <c r="N51" s="30" t="n">
+        <v>23950</v>
+      </c>
+      <c r="O51" s="14" t="n">
+        <v>347399</v>
+      </c>
+      <c r="P51" s="13" t="n">
+        <v>193814</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>35295089</v>
+      </c>
+      <c r="R51" s="27" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="N52" s="30" t="n">
         <v>23900</v>
       </c>
-      <c r="O51" s="14" t="n">
-        <v>190077</v>
-      </c>
-      <c r="P51" s="13" t="n">
-        <v>141236</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>8312324</v>
-      </c>
-      <c r="R51" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="N52" s="31" t="n">
-        <v>23000</v>
-      </c>
       <c r="O52" s="14" t="n">
-        <v>216353</v>
+        <v>207991</v>
       </c>
       <c r="P52" s="13" t="n">
-        <v>12944</v>
+        <v>17914</v>
       </c>
       <c r="Q52" s="14" t="n">
-        <v>1386067</v>
-      </c>
-      <c r="R52" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>18346898</v>
+      </c>
+      <c r="R52" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="32" t="inlineStr">
-        <is>
-          <t>TODAY = 27-Jul-2026    1 DAY AGO = 24-Jul-2026    2 DAYS AGO = 23-Jul-2026    (generated 27-Jul-2026 22:30 IST)</t>
+      <c r="A54" s="31" t="inlineStr">
+        <is>
+          <t>TODAY = 28-Jul-2026    1 DAY AGO = 27-Jul-2026    2 DAYS AGO = 24-Jul-2026    (generated 28-Jul-2026 22:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-07-29
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -137,13 +137,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -171,6 +171,9 @@
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -180,7 +183,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -191,6 +194,9 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -558,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:T54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -573,12 +579,14 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="2" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="15" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="2" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -601,14 +609,16 @@
       <c r="J1" s="2" t="n"/>
       <c r="K1" s="2" t="n"/>
       <c r="L1" s="2" t="n"/>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>Positions Bought / Sold Today</t>
         </is>
       </c>
-      <c r="O1" s="2" t="n"/>
-      <c r="P1" s="2" t="n"/>
       <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+      <c r="S1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr"/>
@@ -650,23 +660,33 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
-      <c r="N2" s="8" t="inlineStr">
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N2" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="P2" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="Q2" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="P2" s="10" t="inlineStr">
+      <c r="R2" s="10" t="inlineStr">
         <is>
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q2" s="11" t="n">
-        <v>-15940</v>
+      <c r="S2" s="11" t="n">
+        <v>-17863</v>
       </c>
     </row>
     <row r="3">
@@ -681,15 +701,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-25089</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>-9149</v>
+        <v>-13703</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>4160</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -697,39 +717,45 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-15940</v>
+        <v>-17863</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>135390</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>153253</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>169193</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>176498</v>
       </c>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="N3" s="12" t="n">
+        <v>167487</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O3" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P3" s="10" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="n">
-        <v>122423</v>
+      <c r="S3" s="11" t="n">
+        <v>-180398</v>
       </c>
     </row>
     <row r="4">
@@ -744,15 +770,15 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-10618</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="n">
-        <v>-4</v>
+        <v>-279</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -760,39 +786,45 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>-10614</v>
+        <v>-279</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>54192</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>54471</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>65085</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>65128</v>
       </c>
-      <c r="N4" s="8" t="inlineStr">
+      <c r="N4" s="12" t="n">
+        <v>67306</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
+      <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q4" s="11" t="n">
-        <v>31031</v>
+      <c r="S4" s="11" t="n">
+        <v>137134</v>
       </c>
     </row>
     <row r="5">
@@ -801,61 +833,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>-6567</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>1342</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>-67891</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>-9441</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>61324</v>
+      <c r="G5" s="14" t="n">
+        <v>10783</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-194818</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-205601</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-266925</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-270847</v>
       </c>
-      <c r="N5" s="8" t="inlineStr">
+      <c r="N5" s="12" t="n">
+        <v>-263082</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="P5" s="10" t="inlineStr">
+      <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q5" s="11" t="n">
-        <v>-20076</v>
+      <c r="S5" s="11" t="n">
+        <v>-34142</v>
       </c>
     </row>
     <row r="6">
@@ -864,61 +902,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>-45411</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="n">
-        <v>-10641</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>-34770</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>7706</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>347</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>7359</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>5236</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-2123</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>32647</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>29221</v>
       </c>
-      <c r="N6" s="8" t="inlineStr">
+      <c r="N6" s="12" t="n">
+        <v>28289</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P6" s="10" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q6" s="11" t="n">
-        <v>-579099</v>
+      <c r="S6" s="14" t="n">
+        <v>44673</v>
       </c>
     </row>
     <row r="7">
@@ -929,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-87685</v>
+        <v>-4934</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-87685</v>
+        <v>-4934</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -947,23 +991,25 @@
       <c r="J7" s="15" t="inlineStr"/>
       <c r="K7" s="15" t="inlineStr"/>
       <c r="L7" s="15" t="inlineStr"/>
-      <c r="N7" s="8" t="inlineStr">
+      <c r="M7" s="15" t="inlineStr"/>
+      <c r="N7" s="15" t="inlineStr"/>
+      <c r="P7" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="P7" s="10" t="inlineStr">
+      <c r="R7" s="10" t="inlineStr">
         <is>
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q7" s="11" t="n">
-        <v>92551</v>
+      <c r="S7" s="11" t="n">
+        <v>13715</v>
       </c>
     </row>
     <row r="8">
@@ -1006,23 +1052,33 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
-      <c r="N8" s="8" t="inlineStr">
+      <c r="M8" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="P8" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="P8" s="10" t="inlineStr">
+      <c r="R8" s="10" t="inlineStr">
         <is>
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q8" s="11" t="n">
-        <v>-10614</v>
+      <c r="S8" s="11" t="n">
+        <v>-279</v>
       </c>
     </row>
     <row r="9">
@@ -1031,61 +1087,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>-1689253</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>-1811676</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>266498</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>446896</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-180398</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>8648</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>189046</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>66623</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>44766</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>167052</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
-        <v>122423</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>189046</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>66623</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>44766</v>
-      </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="O9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P9" s="10" t="inlineStr">
+      <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q9" s="11" t="n">
-        <v>-4255</v>
+      <c r="S9" s="14" t="n">
+        <v>1050</v>
       </c>
     </row>
     <row r="10">
@@ -1094,61 +1156,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>-4410</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>-155</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>-4255</v>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>1050</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>1050</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>4330</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3280</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>7535</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>7540</v>
       </c>
-      <c r="N10" s="8" t="inlineStr">
+      <c r="N10" s="12" t="n">
+        <v>7590</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P10" s="10" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="n">
-        <v>-12444</v>
+      <c r="S10" s="11" t="n">
+        <v>7837</v>
       </c>
     </row>
     <row r="11">
@@ -1157,61 +1225,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>-388990</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>-366981</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>97478</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>8144</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>89334</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-158213</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-247547</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-225538</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-258810</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-314487</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>-22009</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-247547</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-225538</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-258810</v>
-      </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="O11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P11" s="10" t="inlineStr">
+      <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q11" s="11" t="n">
-        <v>-10741</v>
+      <c r="S11" s="11" t="n">
+        <v>-7199</v>
       </c>
     </row>
     <row r="12">
@@ -1220,61 +1294,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>-701443</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>-605285</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>183106</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>93092</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>90014</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>145235</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>55221</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>151379</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>206503</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>139845</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>-96158</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>55221</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>151379</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>206503</v>
-      </c>
-      <c r="N12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="O12" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P12" s="10" t="inlineStr">
+      <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="n">
-        <v>345566</v>
+      <c r="S12" s="11" t="n">
+        <v>-52122</v>
       </c>
     </row>
     <row r="13">
@@ -1285,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-2784096</v>
+        <v>548132</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-2784097</v>
+        <v>548132</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1303,23 +1383,25 @@
       <c r="J13" s="15" t="inlineStr"/>
       <c r="K13" s="15" t="inlineStr"/>
       <c r="L13" s="15" t="inlineStr"/>
-      <c r="N13" s="8" t="inlineStr">
+      <c r="M13" s="15" t="inlineStr"/>
+      <c r="N13" s="15" t="inlineStr"/>
+      <c r="P13" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="O13" s="9" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="P13" s="10" t="inlineStr">
+      <c r="R13" s="10" t="inlineStr">
         <is>
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q13" s="11" t="n">
-        <v>3740</v>
+      <c r="S13" s="11" t="n">
+        <v>439</v>
       </c>
     </row>
     <row r="14">
@@ -1362,23 +1444,33 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
-      <c r="N14" s="8" t="inlineStr">
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="P14" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="P14" s="10" t="inlineStr">
+      <c r="R14" s="10" t="inlineStr">
         <is>
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="n">
-        <v>61324</v>
+      <c r="S14" s="14" t="n">
+        <v>10783</v>
       </c>
     </row>
     <row r="15">
@@ -1387,21 +1479,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>-1816714</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>-1847745</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>701899</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>564765</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1409,39 +1501,45 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>31031</v>
+        <v>137134</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-486193</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-623327</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-654358</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-702891</v>
       </c>
-      <c r="N15" s="8" t="inlineStr">
+      <c r="N15" s="12" t="n">
+        <v>-769347</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P15" s="10" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q15" s="11" t="n">
-        <v>-22009</v>
+      <c r="S15" s="14" t="n">
+        <v>89334</v>
       </c>
     </row>
     <row r="16">
@@ -1450,61 +1548,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>-12544</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>-100</v>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>7837</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>7837</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>45914</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>38077</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>50521</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>41049</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>35169</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>-12444</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="14" t="n">
-        <v>38077</v>
-      </c>
-      <c r="K16" s="14" t="n">
-        <v>50521</v>
-      </c>
-      <c r="L16" s="14" t="n">
-        <v>41049</v>
-      </c>
-      <c r="N16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="O16" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P16" s="10" t="inlineStr">
+      <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q16" s="11" t="n">
-        <v>39851</v>
+      <c r="S16" s="14" t="n">
+        <v>-44724</v>
       </c>
     </row>
     <row r="17">
@@ -1513,61 +1617,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>-391322</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>-431173</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>44502</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>89226</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-44724</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>477176</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>521900</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>482049</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>535178</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>546528</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>39851</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>521900</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>482049</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>535178</v>
-      </c>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="O17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P17" s="10" t="inlineStr">
+      <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q17" s="11" t="n">
-        <v>-86982</v>
+      <c r="S17" s="14" t="n">
+        <v>62169</v>
       </c>
     </row>
     <row r="18">
@@ -1576,61 +1686,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>-716833</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>-658395</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>185242</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>285489</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>-58438</v>
+      <c r="G18" s="14" t="n">
+        <v>-100247</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>-36897</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>63350</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>121788</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>126665</v>
       </c>
-      <c r="N18" s="8" t="inlineStr">
+      <c r="N18" s="12" t="n">
+        <v>187652</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O18" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P18" s="10" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="n">
-        <v>165045</v>
+      <c r="S18" s="11" t="n">
+        <v>-4977</v>
       </c>
     </row>
     <row r="19">
@@ -1641,11 +1757,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2937413</v>
+        <v>939480</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2937413</v>
+        <v>939480</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1659,23 +1775,25 @@
       <c r="J19" s="15" t="inlineStr"/>
       <c r="K19" s="15" t="inlineStr"/>
       <c r="L19" s="15" t="inlineStr"/>
-      <c r="N19" s="8" t="inlineStr">
+      <c r="M19" s="15" t="inlineStr"/>
+      <c r="N19" s="15" t="inlineStr"/>
+      <c r="P19" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="O19" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P19" s="10" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R19" s="10" t="inlineStr">
         <is>
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="n">
-        <v>-113861</v>
+      <c r="S19" s="11" t="n">
+        <v>12416</v>
       </c>
     </row>
     <row r="20">
@@ -1718,23 +1836,33 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
-      <c r="N20" s="8" t="inlineStr">
+      <c r="M20" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="P20" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="O20" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P20" s="10" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R20" s="10" t="inlineStr">
         <is>
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="Q20" s="11" t="n">
-        <v>-34770</v>
+      <c r="S20" s="14" t="n">
+        <v>7359</v>
       </c>
     </row>
     <row r="21">
@@ -1749,15 +1877,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-114039</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>-93963</v>
+        <v>-17580</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>16562</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1765,39 +1893,45 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>-20076</v>
+        <v>-34142</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>2844262</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2878404</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>2898480</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>2914079</v>
       </c>
-      <c r="N21" s="8" t="inlineStr">
+      <c r="N21" s="12" t="n">
+        <v>2879325</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="O21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="P21" s="10" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="Q21" s="11" t="n">
-        <v>-96158</v>
+      <c r="S21" s="14" t="n">
+        <v>90014</v>
       </c>
     </row>
     <row r="22">
@@ -1806,21 +1940,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>-161696</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>-150955</v>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>10731</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>17930</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1828,39 +1962,45 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-10741</v>
+        <v>-7199</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-3948178</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3940979</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3930238</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3904944</v>
       </c>
-      <c r="N22" s="8" t="inlineStr">
+      <c r="N22" s="12" t="n">
+        <v>-3824126</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="O22" s="12" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="P22" s="10" t="inlineStr">
+      <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="n">
-        <v>-58438</v>
+      <c r="S22" s="14" t="n">
+        <v>-100247</v>
       </c>
     </row>
     <row r="23">
@@ -1875,55 +2015,61 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>-230667</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+        <v>-4929</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>-143685</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>-67098</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>62169</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>626378</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>564209</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>651191</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>574712</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>547149</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-86982</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>564209</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>651191</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>574712</v>
-      </c>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="O23" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P23" s="10" t="inlineStr">
+      <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="n">
-        <v>117799</v>
+      <c r="S23" s="11" t="n">
+        <v>-20828</v>
       </c>
     </row>
     <row r="24">
@@ -1938,55 +2084,61 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-105728</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="n">
-        <v>-223527</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+        <v>-6857</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>13971</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>-20828</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>477538</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>498366</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>380567</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>416153</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>397652</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>117799</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="n">
-        <v>498366</v>
-      </c>
-      <c r="K24" s="14" t="n">
-        <v>380567</v>
-      </c>
-      <c r="L24" s="14" t="n">
-        <v>416153</v>
-      </c>
-      <c r="N24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="O24" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P24" s="10" t="inlineStr">
+      <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="n">
-        <v>68488</v>
+      <c r="S24" s="14" t="n">
+        <v>12426</v>
       </c>
     </row>
     <row r="25">
@@ -1997,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-612130</v>
+        <v>-18635</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-612130</v>
+        <v>-18635</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2015,23 +2167,25 @@
       <c r="J25" s="15" t="inlineStr"/>
       <c r="K25" s="15" t="inlineStr"/>
       <c r="L25" s="15" t="inlineStr"/>
-      <c r="N25" s="8" t="inlineStr">
+      <c r="M25" s="15" t="inlineStr"/>
+      <c r="N25" s="15" t="inlineStr"/>
+      <c r="P25" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="O25" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="P25" s="10" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="R25" s="10" t="inlineStr">
         <is>
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="Q25" s="11" t="n">
-        <v>17570</v>
+      <c r="S25" s="14" t="n">
+        <v>-26570</v>
       </c>
     </row>
     <row r="26">
@@ -2074,6 +2228,16 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
+      <c r="M26" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -2081,43 +2245,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="n">
-        <v>-1232410</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="n">
-        <v>-653311</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="n">
-        <v>-579099</v>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>195546</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>150873</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>44673</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>457286</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>412613</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>991712</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>1115181</v>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>1157349</v>
       </c>
     </row>
     <row r="28">
@@ -2126,52 +2296,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>-2246</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="13" t="n">
-        <v>-347812</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="n">
-        <v>345566</v>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>52122</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>-52122</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-127926</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-75804</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-421370</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-433542</v>
       </c>
-      <c r="N28" s="3" t="inlineStr">
+      <c r="N28" s="12" t="n">
+        <v>-436199</v>
+      </c>
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>Nifty 50  -  Support &amp; Resistance</t>
         </is>
       </c>
-      <c r="O28" s="2" t="n"/>
-      <c r="P28" s="2" t="n"/>
       <c r="Q28" s="2" t="n"/>
+      <c r="R28" s="2" t="n"/>
+      <c r="S28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -2179,52 +2355,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>-171405</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="13" t="n">
-        <v>-336450</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="13" t="n">
-        <v>165045</v>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>22324</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="n">
+        <v>27301</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>-4977</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-52841</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-47864</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-212909</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-216735</v>
       </c>
-      <c r="N29" s="5" t="inlineStr">
-        <is>
-          <t>Next session  -  based on 28-Jul-2026 OHLC</t>
-        </is>
-      </c>
-      <c r="O29" s="6" t="inlineStr"/>
-      <c r="P29" s="6" t="inlineStr"/>
+      <c r="N29" s="12" t="n">
+        <v>-181668</v>
+      </c>
+      <c r="P29" s="5" t="inlineStr">
+        <is>
+          <t>Next session  -  based on 29-Jul-2026 OHLC</t>
+        </is>
+      </c>
       <c r="Q29" s="6" t="inlineStr"/>
+      <c r="R29" s="6" t="inlineStr"/>
+      <c r="S29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -2232,59 +2414,65 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="n">
-        <v>-778878</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="13" t="n">
-        <v>-847366</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="n">
+        <v>156173</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>143747</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n">
-        <v>68488</v>
+      <c r="G30" s="14" t="n">
+        <v>12426</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-276519</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-288945</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-357433</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-464904</v>
       </c>
-      <c r="N30" s="8" t="inlineStr">
+      <c r="N30" s="12" t="n">
+        <v>-539482</v>
+      </c>
+      <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="O30" s="18" t="n">
-        <v>23971.25</v>
-      </c>
-      <c r="P30" s="8" t="inlineStr">
+      <c r="Q30" s="18" t="n">
+        <v>24176.65</v>
+      </c>
+      <c r="R30" s="8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q30" s="18" t="n">
-        <v>24041.15</v>
+      <c r="S30" s="18" t="n">
+        <v>24283.55</v>
       </c>
     </row>
     <row r="31">
@@ -2295,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-2184939</v>
+        <v>374043</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-2184939</v>
+        <v>374043</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2313,21 +2501,23 @@
       <c r="J31" s="15" t="inlineStr"/>
       <c r="K31" s="15" t="inlineStr"/>
       <c r="L31" s="15" t="inlineStr"/>
-      <c r="N31" s="8" t="inlineStr">
+      <c r="M31" s="15" t="inlineStr"/>
+      <c r="N31" s="15" t="inlineStr"/>
+      <c r="P31" s="8" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="O31" s="18" t="n">
-        <v>23954.6</v>
-      </c>
-      <c r="P31" s="8" t="inlineStr">
+      <c r="Q31" s="18" t="n">
+        <v>24136.75</v>
+      </c>
+      <c r="R31" s="8" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="Q31" s="18" t="n">
-        <v>23985.35</v>
+      <c r="S31" s="18" t="n">
+        <v>24250.2</v>
       </c>
     </row>
     <row r="32">
@@ -2370,21 +2560,31 @@
           <t>2 DAYS AGO</t>
         </is>
       </c>
-      <c r="N32" s="19" t="inlineStr">
+      <c r="M32" s="5" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="P32" s="19" t="inlineStr">
         <is>
           <t>R3</t>
         </is>
       </c>
-      <c r="O32" s="20" t="n">
-        <v>24119.35000000001</v>
-      </c>
-      <c r="P32" s="8" t="inlineStr">
+      <c r="Q32" s="20" t="n">
+        <v>24457.05</v>
+      </c>
+      <c r="R32" s="8" t="inlineStr">
         <is>
           <t>CPR Top</t>
         </is>
       </c>
-      <c r="Q32" s="21" t="n">
-        <v>23989.525</v>
+      <c r="S32" s="21" t="n">
+        <v>24236.85</v>
       </c>
     </row>
     <row r="33">
@@ -2393,21 +2593,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>-386911</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="n">
-        <v>-479462</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>108818</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>95103</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2415,37 +2615,43 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>92551</v>
+        <v>13715</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-238299</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-252014</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-344565</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-401562</v>
       </c>
-      <c r="N33" s="19" t="inlineStr">
+      <c r="N33" s="12" t="n">
+        <v>-402545</v>
+      </c>
+      <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="O33" s="20" t="n">
-        <v>24080.25</v>
-      </c>
-      <c r="P33" s="8" t="inlineStr">
+      <c r="Q33" s="20" t="n">
+        <v>24370.3</v>
+      </c>
+      <c r="R33" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
-      <c r="Q33" s="21" t="n">
-        <v>23993.7</v>
+      <c r="S33" s="21" t="n">
+        <v>24223.5</v>
       </c>
     </row>
     <row r="34">
@@ -2454,21 +2660,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>-6780</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E34" s="11" t="n">
-        <v>-10520</v>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="n">
+        <v>2513</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>2074</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2476,37 +2682,43 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>3740</v>
+        <v>439</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>28094</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>27655</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>23915</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>21637</v>
       </c>
-      <c r="N34" s="19" t="inlineStr">
+      <c r="N34" s="12" t="n">
+        <v>25538</v>
+      </c>
+      <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="O34" s="20" t="n">
-        <v>24032.8</v>
-      </c>
-      <c r="P34" s="8" t="inlineStr">
+      <c r="Q34" s="20" t="n">
+        <v>24310.25</v>
+      </c>
+      <c r="R34" s="8" t="inlineStr">
         <is>
           <t>CPR Bottom</t>
         </is>
       </c>
-      <c r="Q34" s="21" t="n">
-        <v>23997.875</v>
+      <c r="S34" s="21" t="n">
+        <v>24210.15</v>
       </c>
     </row>
     <row r="35">
@@ -2515,54 +2727,60 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="13" t="n">
-        <v>-297205</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>-183344</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="13" t="n">
-        <v>-113861</v>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>27583</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>15167</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>12416</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>75423</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>63007</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>176868</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>193753</v>
       </c>
-      <c r="N35" s="8" t="inlineStr">
+      <c r="N35" s="12" t="n">
+        <v>181704</v>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
-      <c r="O35" s="21" t="n">
-        <v>23993.7</v>
-      </c>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
+      <c r="Q35" s="21" t="n">
+        <v>24223.5</v>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -2570,54 +2788,60 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C36" s="13" t="n">
-        <v>-604692</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>-622262</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>17570</v>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="n">
+        <v>91395</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>117965</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>-26570</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>134782</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>161352</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>143782</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>186172</v>
       </c>
-      <c r="N36" s="22" t="inlineStr">
+      <c r="N36" s="12" t="n">
+        <v>195303</v>
+      </c>
+      <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="O36" s="23" t="n">
-        <v>23946.25</v>
-      </c>
-      <c r="P36" t="inlineStr"/>
-      <c r="Q36" t="inlineStr"/>
+      <c r="Q36" s="23" t="n">
+        <v>24163.45</v>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
@@ -2627,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-1295588</v>
+        <v>230309</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-1295588</v>
+        <v>230309</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2645,254 +2869,310 @@
       <c r="J37" s="15" t="inlineStr"/>
       <c r="K37" s="15" t="inlineStr"/>
       <c r="L37" s="15" t="inlineStr"/>
-      <c r="N37" s="22" t="inlineStr">
+      <c r="M37" s="15" t="inlineStr"/>
+      <c r="N37" s="15" t="inlineStr"/>
+      <c r="P37" s="22" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="O37" s="23" t="n">
-        <v>23907.15</v>
-      </c>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
+      <c r="Q37" s="23" t="n">
+        <v>24076.7</v>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="N38" s="22" t="inlineStr">
+      <c r="P38" s="22" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="O38" s="23" t="n">
-        <v>23859.7</v>
-      </c>
-      <c r="P38" t="inlineStr"/>
-      <c r="Q38" t="inlineStr"/>
+      <c r="Q38" s="23" t="n">
+        <v>24016.65</v>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>India VIX</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>1 DAY AGO</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>2 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="I40" s="7" t="inlineStr">
+        <is>
+          <t>Close</t>
+        </is>
+      </c>
+      <c r="J40" s="24" t="n">
+        <v>12.01</v>
+      </c>
+      <c r="K40" s="24" t="n">
+        <v>12.56</v>
+      </c>
+      <c r="L40" s="24" t="n">
+        <v>12.66</v>
+      </c>
+      <c r="M40" s="24" t="n">
+        <v>14.03</v>
+      </c>
+      <c r="N40" s="24" t="n">
+        <v>13.48</v>
+      </c>
     </row>
     <row r="41">
-      <c r="N41" s="3" t="inlineStr">
-        <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 28-Jul-2026</t>
-        </is>
-      </c>
-      <c r="O41" s="2" t="n"/>
-      <c r="P41" s="2" t="n"/>
+      <c r="P41" s="3" t="inlineStr">
+        <is>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 04-Aug-2026</t>
+        </is>
+      </c>
       <c r="Q41" s="2" t="n"/>
       <c r="R41" s="2" t="n"/>
+      <c r="S41" s="2" t="n"/>
+      <c r="T41" s="2" t="n"/>
     </row>
     <row r="42">
-      <c r="N42" s="5" t="inlineStr">
-        <is>
-          <t>Spot 23,985    PCR(OI) 0.94    Max Pain 24,000</t>
-        </is>
-      </c>
-      <c r="O42" s="6" t="n"/>
-      <c r="P42" s="6" t="n"/>
+      <c r="P42" s="5" t="inlineStr">
+        <is>
+          <t>Spot 24,250    PCR(OI) 1.17    Max Pain 24,200</t>
+        </is>
+      </c>
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
+      <c r="S42" s="6" t="n"/>
+      <c r="T42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="N43" s="24" t="inlineStr">
+      <c r="P43" s="25" t="inlineStr">
         <is>
           <t>RESISTANCE   -   Call OI walls (higher = stronger cap)</t>
         </is>
       </c>
-      <c r="O43" s="6" t="n"/>
-      <c r="P43" s="6" t="n"/>
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
+      <c r="S43" s="6" t="n"/>
+      <c r="T43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="N44" s="25" t="inlineStr">
+      <c r="P44" s="26" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="O44" s="25" t="inlineStr">
+      <c r="Q44" s="26" t="inlineStr">
         <is>
           <t>Call OI</t>
         </is>
       </c>
-      <c r="P44" s="25" t="inlineStr">
+      <c r="R44" s="26" t="inlineStr">
         <is>
           <t>Chg OI</t>
         </is>
       </c>
-      <c r="Q44" s="25" t="inlineStr">
+      <c r="S44" s="26" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="R44" s="25" t="inlineStr">
+      <c r="T44" s="26" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="N45" s="26" t="n">
-        <v>24000</v>
-      </c>
-      <c r="O45" s="14" t="n">
-        <v>479480</v>
-      </c>
-      <c r="P45" s="13" t="n">
-        <v>287649</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>40300828</v>
-      </c>
-      <c r="R45" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="P45" s="27" t="n">
+        <v>24600</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>111160</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>56516</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>844976</v>
+      </c>
+      <c r="T45" s="28" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="N46" s="26" t="n">
-        <v>24050</v>
-      </c>
-      <c r="O46" s="14" t="n">
-        <v>201655</v>
-      </c>
-      <c r="P46" s="13" t="n">
-        <v>105631</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>25118624</v>
-      </c>
-      <c r="R46" s="28" t="inlineStr">
+      <c r="P46" s="27" t="n">
+        <v>24700</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>114210</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>41983</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>733722</v>
+      </c>
+      <c r="T46" s="28" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="P47" s="27" t="n">
+        <v>25000</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>136897</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>49314</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>863880</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="N47" s="26" t="n">
-        <v>24100</v>
-      </c>
-      <c r="O47" s="14" t="n">
-        <v>167825</v>
-      </c>
-      <c r="P47" s="13" t="n">
-        <v>7477</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>15245129</v>
-      </c>
-      <c r="R47" s="28" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
     <row r="48">
-      <c r="N48" s="29" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
       </c>
-      <c r="O48" s="6" t="n"/>
-      <c r="P48" s="6" t="n"/>
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
+      <c r="S48" s="6" t="n"/>
+      <c r="T48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="N49" s="25" t="inlineStr">
+      <c r="P49" s="26" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="O49" s="25" t="inlineStr">
+      <c r="Q49" s="26" t="inlineStr">
         <is>
           <t>Put OI</t>
         </is>
       </c>
-      <c r="P49" s="25" t="inlineStr">
+      <c r="R49" s="26" t="inlineStr">
         <is>
           <t>Chg OI</t>
         </is>
       </c>
-      <c r="Q49" s="25" t="inlineStr">
+      <c r="S49" s="26" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="R49" s="25" t="inlineStr">
+      <c r="T49" s="26" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="N50" s="30" t="n">
+      <c r="P50" s="31" t="n">
+        <v>24200</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>136116</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>121288</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>2580607</v>
+      </c>
+      <c r="T50" s="32" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="O50" s="14" t="n">
-        <v>246462</v>
-      </c>
-      <c r="P50" s="13" t="n">
-        <v>37724</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>37388862</v>
-      </c>
-      <c r="R50" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="N51" s="30" t="n">
-        <v>23950</v>
-      </c>
-      <c r="O51" s="14" t="n">
-        <v>347399</v>
-      </c>
-      <c r="P51" s="13" t="n">
-        <v>193814</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>35295089</v>
-      </c>
-      <c r="R51" s="27" t="inlineStr">
-        <is>
-          <t>High</t>
+      <c r="Q51" s="12" t="n">
+        <v>139785</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>48834</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>1148097</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="N52" s="30" t="n">
-        <v>23900</v>
-      </c>
-      <c r="O52" s="14" t="n">
-        <v>207991</v>
-      </c>
-      <c r="P52" s="13" t="n">
-        <v>17914</v>
-      </c>
-      <c r="Q52" s="14" t="n">
-        <v>18346898</v>
-      </c>
-      <c r="R52" s="28" t="inlineStr">
-        <is>
-          <t>Medium</t>
+      <c r="P52" s="31" t="n">
+        <v>23000</v>
+      </c>
+      <c r="Q52" s="12" t="n">
+        <v>97824</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>13446</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>439209</v>
+      </c>
+      <c r="T52" s="28" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="31" t="inlineStr">
-        <is>
-          <t>TODAY = 28-Jul-2026    1 DAY AGO = 27-Jul-2026    2 DAYS AGO = 24-Jul-2026    (generated 28-Jul-2026 22:30 IST)</t>
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>TODAY = 29-Jul-2026    1 DAY AGO = 28-Jul-2026    2 DAYS AGO = 27-Jul-2026    3 DAYS AGO = 24-Jul-2026    4 DAYS AGO = 23-Jul-2026    (generated 29-Jul-2026 22:30 IST)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="N41:R41"/>
-    <mergeCell ref="N48:R48"/>
-    <mergeCell ref="N43:R43"/>
-    <mergeCell ref="N42:R42"/>
+    <mergeCell ref="P43:T43"/>
+    <mergeCell ref="P41:T41"/>
+    <mergeCell ref="P42:T42"/>
+    <mergeCell ref="P48:T48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update participant OI report - 2026-07-30
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -128,22 +128,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,7 +183,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -195,7 +195,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-17863</v>
+        <v>-1902</v>
       </c>
     </row>
     <row r="3">
@@ -695,13 +695,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="11" t="n">
-        <v>-13703</v>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="n">
+        <v>94</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>4160</v>
+        <v>1996</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,36 +717,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-17863</v>
+        <v>-1902</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>133488</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>135390</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>153253</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>169193</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>176498</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>167487</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>-180398</v>
+      <c r="S3" s="13" t="n">
+        <v>31226</v>
       </c>
     </row>
     <row r="4">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-279</v>
+        <v>-254</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>0</v>
+        <v>4380</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -786,28 +786,28 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>-279</v>
+        <v>-4634</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>49558</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>54192</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>54471</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>65085</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>65128</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>67306</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>137134</v>
+        <v>15984</v>
       </c>
     </row>
     <row r="5">
@@ -833,58 +833,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>1342</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="13" t="n">
+        <v>1231</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>-9441</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="13" t="n">
+        <v>-6975</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>10783</v>
+      <c r="G5" s="13" t="n">
+        <v>8206</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-186612</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-194818</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-205601</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-266925</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-270847</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-263082</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -892,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>-34142</v>
+      <c r="S5" s="13" t="n">
+        <v>11332</v>
       </c>
     </row>
     <row r="6">
@@ -902,13 +902,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>7706</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>-779</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -916,53 +916,53 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>347</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+        <v>891</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-1670</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="14" t="n">
+        <v>3566</v>
+      </c>
+      <c r="K6" s="14" t="n">
+        <v>5236</v>
+      </c>
+      <c r="L6" s="14" t="n">
+        <v>-2123</v>
+      </c>
+      <c r="M6" s="14" t="n">
+        <v>32647</v>
+      </c>
+      <c r="N6" s="14" t="n">
+        <v>29221</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>7359</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>5236</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>-2123</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>32647</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>29221</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>28289</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>44673</v>
+      <c r="S6" s="13" t="n">
+        <v>71242</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-4934</v>
+        <v>292</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-4934</v>
+        <v>292</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -998,9 +998,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1008,8 +1008,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>13715</v>
+      <c r="S7" s="13" t="n">
+        <v>-24117</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-279</v>
+        <v>-4634</v>
       </c>
     </row>
     <row r="9">
@@ -1087,13 +1087,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
-        <v>266498</v>
+      <c r="C9" s="13" t="n">
+        <v>251857</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -1101,42 +1101,42 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>446896</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>-180398</v>
+        <v>220631</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>31226</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>39874</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>8648</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>189046</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>66623</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>44766</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>167052</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>1050</v>
+      <c r="S9" s="13" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="10">
@@ -1156,13 +1156,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>1050</v>
+      <c r="C10" s="13" t="n">
+        <v>15</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1172,34 +1172,34 @@
       <c r="E10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>1050</v>
+      <c r="G10" s="13" t="n">
+        <v>15</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>4345</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>4330</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>3280</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>7535</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>7540</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7590</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>7837</v>
+        <v>6491</v>
       </c>
     </row>
     <row r="11">
@@ -1225,13 +1225,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>97478</v>
+      <c r="C11" s="13" t="n">
+        <v>22253</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
@@ -1239,53 +1239,53 @@
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>8144</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>40325</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>-18072</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>-176285</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>-158213</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>-247547</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>-225538</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>-258810</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>89334</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-158213</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-247547</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-225538</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-258810</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-314487</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-7199</v>
+      <c r="S11" s="13" t="n">
+        <v>16740</v>
       </c>
     </row>
     <row r="12">
@@ -1294,13 +1294,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
-        <v>183106</v>
+      <c r="C12" s="13" t="n">
+        <v>61395</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -1308,36 +1308,36 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>93092</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>90014</v>
+        <v>74563</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>-13168</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>132067</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>145235</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>55221</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>151379</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>206503</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>139845</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="S12" s="11" t="n">
-        <v>-52122</v>
+        <v>-36472</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>548132</v>
+        <v>335520</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>548132</v>
+        <v>335519</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>439</v>
+        <v>2532</v>
       </c>
     </row>
     <row r="14">
@@ -1459,7 +1459,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1469,8 +1469,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>10783</v>
+      <c r="S14" s="13" t="n">
+        <v>8206</v>
       </c>
     </row>
     <row r="15">
@@ -1485,15 +1485,15 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>701899</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+        <v>449272</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>564765</v>
+      <c r="E15" s="13" t="n">
+        <v>433288</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1501,36 +1501,36 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>137134</v>
+        <v>15984</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-470209</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-486193</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-623327</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-654358</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-702891</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-769347</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1538,8 +1538,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>89334</v>
+      <c r="S15" s="11" t="n">
+        <v>-18072</v>
       </c>
     </row>
     <row r="16">
@@ -1554,15 +1554,15 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>7837</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>0</v>
+        <v>6431</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>-60</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -1570,34 +1570,34 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>7837</v>
+        <v>6491</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>52405</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>45914</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>38077</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>50521</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>41049</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>35169</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
+      <c r="Q16" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1607,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>-44724</v>
+      <c r="S16" s="13" t="n">
+        <v>-36451</v>
       </c>
     </row>
     <row r="17">
@@ -1623,52 +1623,52 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>44502</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+        <v>19985</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>89226</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="E17" s="13" t="n">
+        <v>56436</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-44724</v>
+      <c r="G17" s="13" t="n">
+        <v>-36451</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>440725</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>477176</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>521900</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>482049</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>535178</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>546528</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>62169</v>
+      <c r="S17" s="11" t="n">
+        <v>-4089</v>
       </c>
     </row>
     <row r="18">
@@ -1692,61 +1692,61 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>185242</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+        <v>129834</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>285489</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="E18" s="13" t="n">
+        <v>115858</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>13976</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>-22921</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>-36897</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>63350</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>121788</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>126665</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-100247</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-36897</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>63350</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>121788</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>126665</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>187652</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="11" t="n">
-        <v>-4977</v>
+        <v>-12397</v>
       </c>
     </row>
     <row r="19">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>939480</v>
+        <v>605522</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>939480</v>
+        <v>605522</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="11" t="n">
-        <v>12416</v>
+        <v>10559</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>7359</v>
+      <c r="S20" s="11" t="n">
+        <v>-1670</v>
       </c>
     </row>
     <row r="21">
@@ -1871,13 +1871,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>-17580</v>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="n">
+        <v>18556</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1885,53 +1885,53 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>16562</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>7224</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="13" t="n">
+        <v>11332</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>2855594</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>2844262</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>2878404</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>2898480</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>2914079</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-34142</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>2844262</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>2878404</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>2898480</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>2914079</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>2879325</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>90014</v>
+      <c r="S21" s="11" t="n">
+        <v>-13168</v>
       </c>
     </row>
     <row r="22">
@@ -1940,58 +1940,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>10731</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>17930</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="n">
-        <v>-7199</v>
+      <c r="C22" s="13" t="n">
+        <v>894</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>-15846</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>16740</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-3931438</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-3948178</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-3940979</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-3930238</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-3904944</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3824126</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -1999,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>-100247</v>
+      <c r="S22" s="11" t="n">
+        <v>13976</v>
       </c>
     </row>
     <row r="23">
@@ -2015,44 +2015,44 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>-4929</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+        <v>-12635</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>-67098</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>62169</v>
+      <c r="E23" s="13" t="n">
+        <v>-8546</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-4089</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>622289</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>626378</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>564209</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>651191</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>574712</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>547149</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-20828</v>
+        <v>-23983</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-6857</v>
+        <v>-3612</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>13971</v>
+        <v>20371</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,36 +2100,36 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-20828</v>
+        <v>-23983</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>453555</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>477538</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>498366</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>380567</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>416153</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>397652</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>12426</v>
+      <c r="S24" s="11" t="n">
+        <v>-22373</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-18635</v>
+        <v>3203</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-18635</v>
+        <v>3203</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,9 +2174,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2184,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>-26570</v>
+      <c r="S25" s="11" t="n">
+        <v>11026</v>
       </c>
     </row>
     <row r="26">
@@ -2245,13 +2245,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>195546</v>
+      <c r="C27" s="13" t="n">
+        <v>170446</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2259,35 +2259,35 @@
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>150873</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+        <v>99204</v>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>44673</v>
+      <c r="G27" s="13" t="n">
+        <v>71242</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>528528</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>457286</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>412613</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>991712</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1115181</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1157349</v>
       </c>
     </row>
     <row r="28">
@@ -2296,12 +2296,12 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
+      <c r="C28" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>52122</v>
+        <v>36472</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -2318,27 +2318,27 @@
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>-52122</v>
+        <v>-36472</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-164398</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-127926</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-75804</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-421370</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-433542</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-436199</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,13 +2355,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>22324</v>
+      <c r="C29" s="13" t="n">
+        <v>11826</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="11" t="n">
-        <v>27301</v>
+        <v>24223</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -2377,31 +2377,31 @@
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>-4977</v>
+        <v>-12397</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-65238</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-52841</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-47864</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-212909</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-216735</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-181668</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 29-Jul-2026 OHLC</t>
+          <t>Next session  -  based on 30-Jul-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,13 +2414,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>156173</v>
+      <c r="C30" s="13" t="n">
+        <v>77670</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -2428,43 +2428,43 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>143747</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>12426</v>
+        <v>100043</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>-22373</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-298892</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-276519</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-288945</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-357433</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-464904</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-539482</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24176.65</v>
+        <v>24249.55</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24283.55</v>
+        <v>24342.95</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>374043</v>
+        <v>259942</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>374043</v>
+        <v>259942</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24136.75</v>
+        <v>24187.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24250.2</v>
+        <v>24317.15</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24457.05</v>
+        <v>24533.55000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24236.85</v>
+        <v>24299.77500000001</v>
       </c>
     </row>
     <row r="33">
@@ -2599,51 +2599,51 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>108818</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+        <v>68247</v>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>95103</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>13715</v>
+      <c r="E33" s="13" t="n">
+        <v>92364</v>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>-24117</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-262416</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-238299</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-252014</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-344565</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-401562</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-402545</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24370.3</v>
+        <v>24438.25000000001</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24223.5</v>
+        <v>24282.40000000001</v>
       </c>
     </row>
     <row r="34">
@@ -2666,15 +2666,15 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>2513</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+        <v>3304</v>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>2074</v>
+      <c r="E34" s="13" t="n">
+        <v>772</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,35 +2682,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>439</v>
+        <v>2532</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>30626</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>28094</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>27655</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>23915</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>21637</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>25538</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24310.25</v>
+        <v>24377.70000000001</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24210.15</v>
+        <v>24265.025</v>
       </c>
     </row>
     <row r="35">
@@ -2733,15 +2733,15 @@
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>27583</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+        <v>24403</v>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>15167</v>
+      <c r="E35" s="13" t="n">
+        <v>13844</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
@@ -2749,35 +2749,35 @@
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>12416</v>
+        <v>10559</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>85982</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>75423</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>63007</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>176868</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>193753</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>181704</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24223.5</v>
+        <v>24282.40000000001</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,51 +2794,51 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>91395</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+        <v>75806</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>117965</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>-26570</v>
+      <c r="E36" s="13" t="n">
+        <v>64780</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>11026</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>145808</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>134782</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>161352</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>143782</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>186172</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>195303</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24163.45</v>
+        <v>24221.85000000001</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>230309</v>
+        <v>171760</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>230309</v>
+        <v>171760</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24076.7</v>
+        <v>24126.55</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24016.65</v>
+        <v>24066.00000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.01</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.56</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.66</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>14.03</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>13.48</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,250    PCR(OI) 1.17    Max Pain 24,200</t>
+          <t>Spot 24,317    PCR(OI) 1.29    Max Pain 24,250</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,39 +3010,39 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24600</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>111160</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>56516</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>844976</v>
+        <v>24500</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>153600</v>
+      </c>
+      <c r="R45" s="13" t="n">
+        <v>47982</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>1773049</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24700</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>114210</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>41983</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>733722</v>
-      </c>
-      <c r="T46" s="28" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>24600</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>156591</v>
+      </c>
+      <c r="R46" s="13" t="n">
+        <v>45431</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1283227</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3050,14 +3050,14 @@
       <c r="P47" s="27" t="n">
         <v>25000</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>136897</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>49314</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>863880</v>
+      <c r="Q47" s="14" t="n">
+        <v>133100</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>-3797</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>985908</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
@@ -3107,16 +3107,16 @@
       <c r="P50" s="31" t="n">
         <v>24200</v>
       </c>
-      <c r="Q50" s="12" t="n">
-        <v>136116</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>121288</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>2580607</v>
-      </c>
-      <c r="T50" s="32" t="inlineStr">
+      <c r="Q50" s="14" t="n">
+        <v>165654</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>29538</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>2565821</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3126,14 +3126,14 @@
       <c r="P51" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>139785</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>48834</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1148097</v>
+      <c r="Q51" s="14" t="n">
+        <v>168158</v>
+      </c>
+      <c r="R51" s="13" t="n">
+        <v>28373</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1328136</v>
       </c>
       <c r="T51" s="29" t="inlineStr">
         <is>
@@ -3145,16 +3145,16 @@
       <c r="P52" s="31" t="n">
         <v>23000</v>
       </c>
-      <c r="Q52" s="12" t="n">
-        <v>97824</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>13446</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>439209</v>
-      </c>
-      <c r="T52" s="28" t="inlineStr">
+      <c r="Q52" s="14" t="n">
+        <v>117548</v>
+      </c>
+      <c r="R52" s="13" t="n">
+        <v>19724</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>445627</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 29-Jul-2026    1 DAY AGO = 28-Jul-2026    2 DAYS AGO = 27-Jul-2026    3 DAYS AGO = 24-Jul-2026    4 DAYS AGO = 23-Jul-2026    (generated 29-Jul-2026 22:30 IST)</t>
+          <t>TODAY = 30-Jul-2026    1 DAY AGO = 29-Jul-2026    2 DAYS AGO = 28-Jul-2026    3 DAYS AGO = 27-Jul-2026    4 DAYS AGO = 24-Jul-2026    (generated 30-Jul-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-07-31
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -128,22 +128,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-1902</v>
+        <v>-5564</v>
       </c>
     </row>
     <row r="3">
@@ -695,13 +695,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C3" s="13" t="n">
-        <v>94</v>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="n">
+        <v>-2403</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1996</v>
+        <v>3161</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,36 +717,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-1902</v>
+        <v>-5564</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>127924</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>133488</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>135390</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>153253</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>169193</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>176498</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>31226</v>
+      <c r="S3" s="11" t="n">
+        <v>-15758</v>
       </c>
     </row>
     <row r="4">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-254</v>
+        <v>-4351</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>4380</v>
+        <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -786,36 +786,36 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>-4634</v>
+        <v>-4351</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>45207</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>49558</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>54192</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>54471</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>65085</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>65128</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -823,8 +823,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>15984</v>
+      <c r="S4" s="14" t="n">
+        <v>-217411</v>
       </c>
     </row>
     <row r="5">
@@ -833,58 +833,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n">
-        <v>1231</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="C5" s="14" t="n">
+        <v>326</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>-6975</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>-13173</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>8206</v>
+      <c r="G5" s="14" t="n">
+        <v>13499</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-173113</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-186612</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-194818</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-205601</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-266925</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-270847</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -892,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>11332</v>
+      <c r="S5" s="11" t="n">
+        <v>-8073</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-779</v>
+        <v>-1488</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>891</v>
+        <v>2096</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -924,34 +924,34 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>-1670</v>
+        <v>-3584</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>-18</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>3566</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>5236</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>-2123</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>32647</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>29221</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -961,8 +961,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="13" t="n">
-        <v>71242</v>
+      <c r="S6" s="14" t="n">
+        <v>35083</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>292</v>
+        <v>-7916</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>292</v>
+        <v>-7916</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -998,9 +998,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1008,8 +1008,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="13" t="n">
-        <v>-24117</v>
+      <c r="S7" s="11" t="n">
+        <v>17013</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-4634</v>
+        <v>-4351</v>
       </c>
     </row>
     <row r="9">
@@ -1087,13 +1087,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>251857</v>
+      <c r="C9" s="14" t="n">
+        <v>282432</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -1101,53 +1101,53 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>220631</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+        <v>298190</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>-15758</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>24116</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>39874</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>8648</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>189046</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>66623</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
-        <v>31226</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>39874</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>8648</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>189046</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>66623</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>44766</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>15</v>
+      <c r="S9" s="14" t="n">
+        <v>150</v>
       </c>
     </row>
     <row r="10">
@@ -1156,13 +1156,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="13" t="n">
-        <v>15</v>
+      <c r="C10" s="14" t="n">
+        <v>150</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1172,34 +1172,34 @@
       <c r="E10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>15</v>
+      <c r="G10" s="14" t="n">
+        <v>150</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>4495</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4345</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>4330</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>3280</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>7535</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>7540</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>6491</v>
+        <v>295</v>
       </c>
     </row>
     <row r="11">
@@ -1225,13 +1225,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="13" t="n">
-        <v>22253</v>
+      <c r="C11" s="14" t="n">
+        <v>27717</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>40325</v>
+        <v>35957</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1247,36 +1247,36 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>-18072</v>
+        <v>-8240</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-184525</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-176285</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-158213</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-247547</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-225538</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-258810</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1284,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>16740</v>
+      <c r="S11" s="11" t="n">
+        <v>-8270</v>
       </c>
     </row>
     <row r="12">
@@ -1294,13 +1294,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="13" t="n">
-        <v>61395</v>
+      <c r="C12" s="14" t="n">
+        <v>115520</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -1308,53 +1308,53 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>74563</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>91673</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>23847</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>155914</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>132067</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>145235</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>55221</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>151379</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>-13168</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="n">
-        <v>132067</v>
-      </c>
-      <c r="K12" s="14" t="n">
-        <v>145235</v>
-      </c>
-      <c r="L12" s="14" t="n">
-        <v>55221</v>
-      </c>
-      <c r="M12" s="14" t="n">
-        <v>151379</v>
-      </c>
-      <c r="N12" s="14" t="n">
-        <v>206503</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="11" t="n">
-        <v>-36472</v>
+        <v>-16585</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>335520</v>
+        <v>425819</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>335519</v>
+        <v>425820</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>2532</v>
+        <v>720</v>
       </c>
     </row>
     <row r="14">
@@ -1459,7 +1459,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1469,8 +1469,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>8206</v>
+      <c r="S14" s="14" t="n">
+        <v>13499</v>
       </c>
     </row>
     <row r="15">
@@ -1485,44 +1485,44 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>449272</v>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
+        <v>438295</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="13" t="n">
-        <v>433288</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>15984</v>
+      <c r="E15" s="14" t="n">
+        <v>655706</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>-217411</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-687620</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-470209</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-486193</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-623327</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-654358</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-702891</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>-18072</v>
+        <v>-8240</v>
       </c>
     </row>
     <row r="16">
@@ -1554,15 +1554,15 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>6431</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>-60</v>
+        <v>320</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>25</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -1570,36 +1570,36 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>6491</v>
+        <v>295</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>52700</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>52405</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>45914</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>38077</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>50521</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>41049</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1607,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>-36451</v>
+      <c r="S16" s="11" t="n">
+        <v>13045</v>
       </c>
     </row>
     <row r="17">
@@ -1623,52 +1623,52 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>19985</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
+        <v>109958</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="13" t="n">
-        <v>56436</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G17" s="13" t="n">
-        <v>-36451</v>
+      <c r="E17" s="14" t="n">
+        <v>96913</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>13045</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>453770</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>440725</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>477176</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>521900</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>482049</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>535178</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>-4089</v>
+      <c r="S17" s="14" t="n">
+        <v>22174</v>
       </c>
     </row>
     <row r="18">
@@ -1692,15 +1692,15 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>129834</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
+        <v>418219</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="13" t="n">
-        <v>115858</v>
+      <c r="E18" s="14" t="n">
+        <v>214148</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1708,28 +1708,28 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>13976</v>
+        <v>204071</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>181150</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>-22921</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>-36897</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>63350</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>121788</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>126665</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="11" t="n">
-        <v>-12397</v>
+        <v>-8703</v>
       </c>
     </row>
     <row r="19">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>605522</v>
+        <v>966792</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>605522</v>
+        <v>966792</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="11" t="n">
-        <v>10559</v>
+        <v>7366</v>
       </c>
     </row>
     <row r="20">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>-1670</v>
+        <v>-3584</v>
       </c>
     </row>
     <row r="21">
@@ -1871,13 +1871,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>18556</v>
+      <c r="C21" s="14" t="n">
+        <v>896</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1885,53 +1885,53 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>7224</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+        <v>8969</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-8073</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>2847521</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>2855594</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>2844262</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>2878404</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>2898480</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>11332</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="14" t="n">
-        <v>2855594</v>
-      </c>
-      <c r="K21" s="14" t="n">
-        <v>2844262</v>
-      </c>
-      <c r="L21" s="14" t="n">
-        <v>2878404</v>
-      </c>
-      <c r="M21" s="14" t="n">
-        <v>2898480</v>
-      </c>
-      <c r="N21" s="14" t="n">
-        <v>2914079</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>-13168</v>
+      <c r="S21" s="14" t="n">
+        <v>23847</v>
       </c>
     </row>
     <row r="22">
@@ -1940,67 +1940,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n">
-        <v>894</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>-15846</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>5094</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>13364</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>-8270</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-3939708</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-3931438</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-3948178</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-3940979</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-3930238</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>16740</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="n">
-        <v>-3931438</v>
-      </c>
-      <c r="K22" s="14" t="n">
-        <v>-3948178</v>
-      </c>
-      <c r="L22" s="14" t="n">
-        <v>-3940979</v>
-      </c>
-      <c r="M22" s="14" t="n">
-        <v>-3930238</v>
-      </c>
-      <c r="N22" s="14" t="n">
-        <v>-3904944</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>13976</v>
+        <v>204071</v>
       </c>
     </row>
     <row r="23">
@@ -2009,67 +2009,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>-12635</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>6491</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>-8546</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>-15683</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>22174</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>644463</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>622289</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>626378</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>564209</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>651191</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-4089</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="14" t="n">
-        <v>622289</v>
-      </c>
-      <c r="K23" s="14" t="n">
-        <v>626378</v>
-      </c>
-      <c r="L23" s="14" t="n">
-        <v>564209</v>
-      </c>
-      <c r="M23" s="14" t="n">
-        <v>651191</v>
-      </c>
-      <c r="N23" s="14" t="n">
-        <v>574712</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-23983</v>
+        <v>-5831</v>
       </c>
     </row>
     <row r="24">
@@ -2078,13 +2078,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>-3612</v>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>5063</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>20371</v>
+        <v>10894</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,28 +2100,28 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-23983</v>
+        <v>-5831</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>447724</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>453555</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>477538</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>498366</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>380567</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>416153</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="11" t="n">
-        <v>-22373</v>
+        <v>-9795</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>3203</v>
+        <v>17544</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>3203</v>
+        <v>17544</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,9 +2174,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2184,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>11026</v>
+      <c r="S25" s="14" t="n">
+        <v>-25099</v>
       </c>
     </row>
     <row r="26">
@@ -2245,13 +2245,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="13" t="n">
-        <v>170446</v>
+      <c r="C27" s="14" t="n">
+        <v>128687</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2259,35 +2259,35 @@
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>99204</v>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
+        <v>93604</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="13" t="n">
-        <v>71242</v>
+      <c r="G27" s="14" t="n">
+        <v>35083</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>563611</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>528528</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>457286</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>412613</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>991712</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1115181</v>
       </c>
     </row>
     <row r="28">
@@ -2296,13 +2296,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="13" t="n">
-        <v>0</v>
+      <c r="C28" s="14" t="n">
+        <v>40</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>36472</v>
+        <v>16625</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -2318,27 +2318,27 @@
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>-36472</v>
+        <v>-16585</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-180983</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-164398</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-127926</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-75804</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-421370</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-433542</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,13 +2355,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>11826</v>
+      <c r="C29" s="14" t="n">
+        <v>14599</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="11" t="n">
-        <v>24223</v>
+        <v>23302</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -2377,31 +2377,31 @@
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>-12397</v>
+        <v>-8703</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-73941</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-65238</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-52841</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-47864</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-212909</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-216735</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 30-Jul-2026 OHLC</t>
+          <t>Next session  -  based on 31-Jul-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,13 +2414,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="13" t="n">
-        <v>77670</v>
+      <c r="C30" s="14" t="n">
+        <v>70193</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>100043</v>
+        <v>79988</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -2436,35 +2436,35 @@
         </is>
       </c>
       <c r="G30" s="11" t="n">
-        <v>-22373</v>
+        <v>-9795</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-308687</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-298892</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-276519</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-288945</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-357433</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-464904</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24249.55</v>
+        <v>24361.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24342.95</v>
+        <v>24429.4</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>259942</v>
+        <v>213519</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>259942</v>
+        <v>213519</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24187.1</v>
+        <v>24299.7</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24317.15</v>
+        <v>24383.6</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24533.55000000001</v>
+        <v>24571.80000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24299.77500000001</v>
+        <v>24377.25000000001</v>
       </c>
     </row>
     <row r="33">
@@ -2599,51 +2599,51 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>68247</v>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
+        <v>80006</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="13" t="n">
-        <v>92364</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>-24117</v>
+      <c r="E33" s="14" t="n">
+        <v>62993</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>17013</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-245403</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-262416</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-238299</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-252014</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-344565</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-401562</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24438.25000000001</v>
+        <v>24500.60000000001</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24282.40000000001</v>
+        <v>24370.90000000001</v>
       </c>
     </row>
     <row r="34">
@@ -2666,15 +2666,15 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>3304</v>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
+        <v>1342</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="13" t="n">
-        <v>772</v>
+      <c r="E34" s="14" t="n">
+        <v>622</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,35 +2682,35 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>2532</v>
+        <v>720</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>31346</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>30626</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>28094</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>27655</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>23915</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>21637</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24377.70000000001</v>
+        <v>24442.10000000001</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24265.025</v>
+        <v>24364.55</v>
       </c>
     </row>
     <row r="35">
@@ -2733,15 +2733,15 @@
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>24403</v>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
+        <v>24007</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="13" t="n">
-        <v>13844</v>
+      <c r="E35" s="14" t="n">
+        <v>16641</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
@@ -2749,35 +2749,35 @@
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>10559</v>
+        <v>7366</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>93348</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>85982</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>75423</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>63007</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>176868</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>193753</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24282.40000000001</v>
+        <v>24370.90000000001</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,51 +2794,51 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>75806</v>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
+        <v>43482</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="13" t="n">
-        <v>64780</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>11026</v>
+      <c r="E36" s="14" t="n">
+        <v>68581</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>-25099</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>120709</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>145808</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>134782</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>161352</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>143782</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>186172</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24221.85000000001</v>
+        <v>24312.40000000001</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>171760</v>
+        <v>148837</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>171760</v>
+        <v>148837</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24126.55</v>
+        <v>24241.2</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24066.00000000001</v>
+        <v>24182.70000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.01</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.56</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.66</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>14.03</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,317    PCR(OI) 1.29    Max Pain 24,250</t>
+          <t>Spot 24,384    PCR(OI) 1.49    Max Pain 24,350</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,16 +3010,16 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>153600</v>
-      </c>
-      <c r="R45" s="13" t="n">
-        <v>47982</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>1773049</v>
+        <v>24600</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>185155</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>28564</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>2814363</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,16 +3029,16 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24600</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>156591</v>
-      </c>
-      <c r="R46" s="13" t="n">
-        <v>45431</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>1283227</v>
+        <v>24700</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>141486</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>22311</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>1617484</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3050,14 +3050,14 @@
       <c r="P47" s="27" t="n">
         <v>25000</v>
       </c>
-      <c r="Q47" s="14" t="n">
-        <v>133100</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>-3797</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>985908</v>
+      <c r="Q47" s="12" t="n">
+        <v>167690</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>34590</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>1001992</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
@@ -3107,14 +3107,14 @@
       <c r="P50" s="31" t="n">
         <v>24200</v>
       </c>
-      <c r="Q50" s="14" t="n">
-        <v>165654</v>
-      </c>
-      <c r="R50" s="13" t="n">
-        <v>29538</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>2565821</v>
+      <c r="Q50" s="12" t="n">
+        <v>181766</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>16112</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>2638271</v>
       </c>
       <c r="T50" s="28" t="inlineStr">
         <is>
@@ -3126,14 +3126,14 @@
       <c r="P51" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>168158</v>
-      </c>
-      <c r="R51" s="13" t="n">
-        <v>28373</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>1328136</v>
+      <c r="Q51" s="12" t="n">
+        <v>225941</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>57783</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>1756313</v>
       </c>
       <c r="T51" s="29" t="inlineStr">
         <is>
@@ -3145,14 +3145,14 @@
       <c r="P52" s="31" t="n">
         <v>23000</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>117548</v>
-      </c>
-      <c r="R52" s="13" t="n">
-        <v>19724</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>445627</v>
+      <c r="Q52" s="12" t="n">
+        <v>166355</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>48807</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>821482</v>
       </c>
       <c r="T52" s="32" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 30-Jul-2026    1 DAY AGO = 29-Jul-2026    2 DAYS AGO = 28-Jul-2026    3 DAYS AGO = 27-Jul-2026    4 DAYS AGO = 24-Jul-2026    (generated 30-Jul-2026 20:30 IST)</t>
+          <t>TODAY = 31-Jul-2026    1 DAY AGO = 30-Jul-2026    2 DAYS AGO = 29-Jul-2026    3 DAYS AGO = 28-Jul-2026    4 DAYS AGO = 27-Jul-2026    (generated 31-Jul-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-03
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -183,10 +183,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -195,7 +195,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-5564</v>
+        <v>-11642</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-2403</v>
+        <v>-9486</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>3161</v>
+        <v>2156</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-5564</v>
+        <v>-11642</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,20 +725,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>116282</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>127924</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>133488</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>135390</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>153253</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>169193</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-15758</v>
+        <v>-81790</v>
       </c>
     </row>
     <row r="4">
@@ -764,29 +764,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>-4351</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>-4351</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>323</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>-125</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>448</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,28 +794,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>45655</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>45207</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>49558</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>54192</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>54471</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>65085</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -823,8 +823,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>-217411</v>
+      <c r="S4" s="11" t="n">
+        <v>126588</v>
       </c>
     </row>
     <row r="5">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>326</v>
+        <v>1784</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-13173</v>
+        <v>-20513</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>13499</v>
+        <v>22297</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,28 +863,28 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-150816</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-173113</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-186612</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-194818</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-205601</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-266925</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -892,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>-8073</v>
+      <c r="S5" s="14" t="n">
+        <v>2877</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-1488</v>
+        <v>-2424</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>2096</v>
+        <v>8679</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>-3584</v>
+        <v>-11103</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-11121</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-18</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>3566</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>5236</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-2123</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>32647</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="14" t="n">
-        <v>35083</v>
+        <v>73430</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-7916</v>
+        <v>-9803</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-7916</v>
+        <v>-9803</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>17013</v>
+        <v>25964</v>
       </c>
     </row>
     <row r="8">
@@ -1067,9 +1067,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-4351</v>
+      <c r="S8" s="14" t="n">
+        <v>448</v>
       </c>
     </row>
     <row r="9">
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>282432</v>
+        <v>254667</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>298190</v>
+        <v>336457</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-15758</v>
+        <v>-81790</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,28 +1117,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>-57674</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>24116</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>39874</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>8648</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>189046</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>66623</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>150</v>
+      <c r="S9" s="11" t="n">
+        <v>-255</v>
       </c>
     </row>
     <row r="10">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>150</v>
+        <v>565</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1170,15 +1170,15 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>150</v>
+        <v>820</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>-255</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,28 +1186,28 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>4240</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4495</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4345</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4330</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>3280</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7535</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1215,8 +1215,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>295</v>
+      <c r="S10" s="14" t="n">
+        <v>-795</v>
       </c>
     </row>
     <row r="11">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>27717</v>
+        <v>60397</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
@@ -1239,15 +1239,15 @@
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>35957</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>-8240</v>
+        <v>4402</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>55995</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,28 +1255,28 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-128530</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-184525</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-176285</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-158213</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-247547</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-225538</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1284,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-8270</v>
+      <c r="S11" s="14" t="n">
+        <v>16785</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>115520</v>
+        <v>83607</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>91673</v>
+        <v>57558</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>23847</v>
+        <v>26049</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,20 +1324,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>181963</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>155914</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>132067</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>145235</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>55221</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>151379</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="S12" s="11" t="n">
-        <v>-16585</v>
+        <v>-37018</v>
       </c>
     </row>
     <row r="13">
@@ -1365,11 +1365,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>425819</v>
+        <v>399236</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>425820</v>
+        <v>399237</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1390,9 +1390,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1400,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>720</v>
+      <c r="S13" s="14" t="n">
+        <v>-1250</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>13499</v>
+        <v>22297</v>
       </c>
     </row>
     <row r="15">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>438295</v>
+        <v>520402</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1493,15 +1493,15 @@
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>655706</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>-217411</v>
+        <v>393814</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>126588</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,28 +1509,28 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-561032</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-687620</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-470209</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-486193</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-623327</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-654358</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1538,8 +1538,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>-8240</v>
+      <c r="S15" s="14" t="n">
+        <v>55995</v>
       </c>
     </row>
     <row r="16">
@@ -1548,13 +1548,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>320</v>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>-40</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -1562,15 +1562,15 @@
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>295</v>
+        <v>755</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>-795</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,28 +1578,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>51905</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>52700</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>52405</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>45914</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>38077</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50521</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1607,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>13045</v>
+      <c r="S16" s="14" t="n">
+        <v>-20375</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>109958</v>
+        <v>80956</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1631,15 +1631,15 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>96913</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>13045</v>
+        <v>101331</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>-20375</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,28 +1647,28 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>433395</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>453770</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>440725</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>477176</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>521900</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>482049</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>22174</v>
+      <c r="S17" s="11" t="n">
+        <v>-1237</v>
       </c>
     </row>
     <row r="18">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>418219</v>
+        <v>4890</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1700,15 +1700,15 @@
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>214148</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="n">
-        <v>204071</v>
+        <v>110308</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-105418</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1716,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>75732</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>181150</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-22921</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>-36897</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>63350</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>121788</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="11" t="n">
-        <v>-8703</v>
+        <v>-6882</v>
       </c>
     </row>
     <row r="19">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>966792</v>
+        <v>606208</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>966792</v>
+        <v>606208</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="11" t="n">
-        <v>7366</v>
+        <v>4569</v>
       </c>
     </row>
     <row r="20">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>-3584</v>
+        <v>-11103</v>
       </c>
     </row>
     <row r="21">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="C21" s="14" t="n">
-        <v>896</v>
+        <v>10018</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1885,15 +1885,15 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>8969</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>-8073</v>
+        <v>7141</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>2877</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1901,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2850398</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2847521</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2855594</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2844262</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2878404</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2898480</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>23847</v>
+        <v>26049</v>
       </c>
     </row>
     <row r="22">
@@ -1946,61 +1946,61 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>5094</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>13364</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>8947</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>-7838</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>16785</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-3922923</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-3939708</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-3931438</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-3948178</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-3940979</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-8270</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-3939708</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-3931438</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-3948178</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-3940979</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-3930238</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>204071</v>
+      <c r="S22" s="14" t="n">
+        <v>-105418</v>
       </c>
     </row>
     <row r="23">
@@ -2009,13 +2009,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>6491</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>-8261</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-15683</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>22174</v>
+        <v>-7024</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-1237</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,20 +2039,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>643226</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>644463</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>622289</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>626378</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>564209</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>651191</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-5831</v>
+        <v>-18425</v>
       </c>
     </row>
     <row r="24">
@@ -2078,13 +2078,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>5063</v>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>-4920</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>10894</v>
+        <v>13505</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-5831</v>
+        <v>-18425</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,20 +2108,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>429299</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>447724</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>453555</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>477538</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>498366</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>380567</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="11" t="n">
-        <v>-9795</v>
+        <v>-29530</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>17544</v>
+        <v>5784</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>17544</v>
+        <v>5784</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-25099</v>
+        <v>-29283</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="14" t="n">
-        <v>128687</v>
+        <v>124976</v>
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="11" t="n">
-        <v>93604</v>
+        <v>51546</v>
       </c>
       <c r="F27" s="13" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="14" t="n">
-        <v>35083</v>
+        <v>73430</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>637041</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>563611</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>528528</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>457286</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>412613</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>991712</v>
       </c>
     </row>
     <row r="28">
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="11" t="n">
-        <v>16625</v>
+        <v>37018</v>
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="G28" s="11" t="n">
-        <v>-16585</v>
+        <v>-37018</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-218001</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-180983</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-164398</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-127926</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-75804</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-421370</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="14" t="n">
-        <v>14599</v>
+        <v>15279</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="11" t="n">
-        <v>23302</v>
+        <v>22161</v>
       </c>
       <c r="F29" s="9" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="11" t="n">
-        <v>-8703</v>
+        <v>-6882</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-80823</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-73941</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-65238</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-52841</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-47864</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-212909</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 31-Jul-2026 OHLC</t>
+          <t>Next session  -  based on 03-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="14" t="n">
-        <v>70193</v>
+        <v>64137</v>
       </c>
       <c r="D30" s="9" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="11" t="n">
-        <v>79988</v>
+        <v>93667</v>
       </c>
       <c r="F30" s="9" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="11" t="n">
-        <v>-9795</v>
+        <v>-29530</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-338217</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-308687</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-298892</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-276519</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-288945</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-357433</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24361.45</v>
+        <v>24572.7</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24429.4</v>
+        <v>24774.3</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>213519</v>
+        <v>204392</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>213519</v>
+        <v>204392</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24299.7</v>
+        <v>24515.15</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24383.6</v>
+        <v>24774.3</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24571.80000000001</v>
+        <v>25119.83333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24377.25000000001</v>
+        <v>24731.10833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>80006</v>
+        <v>57394</v>
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="14" t="n">
-        <v>62993</v>
+        <v>31430</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>17013</v>
+        <v>25964</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-219439</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-245403</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-262416</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-238299</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-252014</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-344565</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24500.60000000001</v>
+        <v>24947.06666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24370.90000000001</v>
+        <v>24687.91666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>1342</v>
+        <v>148</v>
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
@@ -2674,15 +2674,15 @@
         </is>
       </c>
       <c r="E34" s="14" t="n">
-        <v>622</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="11" t="n">
-        <v>720</v>
+        <v>1398</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>-1250</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>30096</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>31346</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>30626</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>28094</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>27655</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>23915</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24442.10000000001</v>
+        <v>24860.68333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24364.55</v>
+        <v>24644.725</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="11" t="n">
-        <v>24007</v>
+        <v>20930</v>
       </c>
       <c r="D35" s="13" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="14" t="n">
-        <v>16641</v>
+        <v>16361</v>
       </c>
       <c r="F35" s="9" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="11" t="n">
-        <v>7366</v>
+        <v>4569</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>97917</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>93348</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>85982</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>75423</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>63007</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>176868</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24370.90000000001</v>
+        <v>24687.91666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C36" s="11" t="n">
-        <v>43482</v>
+        <v>31916</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>68581</v>
+        <v>61199</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-25099</v>
+        <v>-29283</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>91426</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>120709</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>145808</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>134782</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>161352</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>143782</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24312.40000000001</v>
+        <v>24601.53333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>148837</v>
+        <v>110388</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>148837</v>
+        <v>110388</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24241.2</v>
+        <v>24428.76666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24182.70000000001</v>
+        <v>24342.38333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.76</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.01</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.56</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.66</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,384    PCR(OI) 1.49    Max Pain 24,350</t>
+          <t>Spot 24,774    PCR(OI) 1.57    Max Pain 24,550</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,37 +3010,37 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24600</v>
+        <v>24750</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>185155</v>
+        <v>94987</v>
       </c>
       <c r="R45" s="14" t="n">
-        <v>28564</v>
+        <v>35014</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2814363</v>
+        <v>3490451</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24700</v>
+        <v>24800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>141486</v>
+        <v>179659</v>
       </c>
       <c r="R46" s="14" t="n">
-        <v>22311</v>
+        <v>74585</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1617484</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
+        <v>3888481</v>
+      </c>
+      <c r="T46" s="28" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3051,17 +3051,17 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>167690</v>
+        <v>182879</v>
       </c>
       <c r="R47" s="14" t="n">
-        <v>34590</v>
+        <v>15189</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>1001992</v>
+        <v>1922012</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3105,18 +3105,18 @@
     </row>
     <row r="50">
       <c r="P50" s="31" t="n">
-        <v>24200</v>
+        <v>24500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>181766</v>
+        <v>191111</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>16112</v>
+        <v>159592</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>2638271</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+        <v>6831963</v>
+      </c>
+      <c r="T50" s="32" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3124,37 +3124,37 @@
     </row>
     <row r="51">
       <c r="P51" s="31" t="n">
-        <v>24000</v>
+        <v>24200</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>225941</v>
+        <v>225769</v>
       </c>
       <c r="R51" s="14" t="n">
-        <v>57783</v>
+        <v>44003</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1756313</v>
+        <v>1851528</v>
       </c>
       <c r="T51" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="31" t="n">
-        <v>23000</v>
+        <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>166355</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>48807</v>
+        <v>218938</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>-7003</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>821482</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
+        <v>1600851</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 31-Jul-2026    1 DAY AGO = 30-Jul-2026    2 DAYS AGO = 29-Jul-2026    3 DAYS AGO = 28-Jul-2026    4 DAYS AGO = 27-Jul-2026    (generated 31-Jul-2026 20:30 IST)</t>
+          <t>TODAY = 03-Aug-2026    1 DAY AGO = 31-Jul-2026    2 DAYS AGO = 30-Jul-2026    3 DAYS AGO = 29-Jul-2026    4 DAYS AGO = 28-Jul-2026    (generated 03-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-04
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -183,6 +183,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -194,9 +197,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -677,7 +677,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-11642</v>
+        <v>18015</v>
       </c>
     </row>
     <row r="3">
@@ -697,27 +697,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-9486</v>
+        <v>13441</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>2156</v>
+        <v>-4574</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-11642</v>
+        <v>18015</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,20 +725,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>134297</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>116282</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>127924</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>133488</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>135390</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>153253</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -746,7 +746,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-81790</v>
+        <v>235479</v>
       </c>
     </row>
     <row r="4">
@@ -766,65 +766,65 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>323</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>-12156</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>-125</v>
+      <c r="E4" s="11" t="n">
+        <v>-4340</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-7816</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>37839</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>45655</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>45207</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>49558</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>54192</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>448</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>45655</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>45207</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>49558</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>54192</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>54471</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>126588</v>
+      <c r="S4" s="14" t="n">
+        <v>61030</v>
       </c>
     </row>
     <row r="5">
@@ -835,65 +835,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>1784</v>
+        <v>-844</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-20513</v>
+        <v>2113</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-2957</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-153773</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-150816</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-173113</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-186612</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-194818</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>22297</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-150816</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-173113</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-186612</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-194818</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-205601</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>2877</v>
+      <c r="S5" s="11" t="n">
+        <v>30291</v>
       </c>
     </row>
     <row r="6">
@@ -904,27 +904,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-2424</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+        <v>1236</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>8679</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>8478</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>-11103</v>
+      <c r="G6" s="14" t="n">
+        <v>-7242</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,26 +932,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-18363</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-11121</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-18</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>3566</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>5236</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-2123</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -961,8 +961,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>73430</v>
+      <c r="S6" s="11" t="n">
+        <v>113185</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-9803</v>
+        <v>1677</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-9803</v>
+        <v>1677</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>25964</v>
+        <v>-41736</v>
       </c>
     </row>
     <row r="8">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>448</v>
+        <v>-7816</v>
       </c>
     </row>
     <row r="9">
@@ -1089,27 +1089,27 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="14" t="n">
-        <v>254667</v>
+        <v>-776152</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>336457</v>
+        <v>-1011631</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-81790</v>
+        <v>235479</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,20 +1117,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>177805</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>-57674</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>24116</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>39874</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>8648</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>189046</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="Q9" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>-255</v>
+        <v>1030</v>
       </c>
     </row>
     <row r="10">
@@ -1156,67 +1156,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>565</v>
+      <c r="C10" s="11" t="n">
+        <v>230</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>820</v>
+        <v>-800</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>1030</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>5270</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>4240</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>4495</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>4345</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>4330</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-255</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>4240</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>4495</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>4345</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>4330</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>3280</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>-795</v>
+      <c r="S10" s="11" t="n">
+        <v>-3380</v>
       </c>
     </row>
     <row r="11">
@@ -1227,65 +1227,65 @@
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>60397</v>
+        <v>-93462</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
-        <v>4402</v>
+        <v>-56995</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-36467</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-164997</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-128530</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-184525</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-176285</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-158213</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>55995</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-128530</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-184525</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-176285</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-158213</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-247547</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>16785</v>
+      <c r="S11" s="11" t="n">
+        <v>3331</v>
       </c>
     </row>
     <row r="12">
@@ -1296,27 +1296,27 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="14" t="n">
-        <v>83607</v>
+        <v>-324922</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>57558</v>
+        <v>-124881</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>26049</v>
+        <v>-200041</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,26 +1324,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-18078</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>181963</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>155914</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>132067</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>145235</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>55221</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1353,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-37018</v>
+      <c r="S12" s="14" t="n">
+        <v>-5202</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>399236</v>
+        <v>-1194306</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>399237</v>
+        <v>-1194307</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1400,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-1250</v>
+      <c r="S13" s="11" t="n">
+        <v>-477</v>
       </c>
     </row>
     <row r="14">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>22297</v>
+        <v>-2957</v>
       </c>
     </row>
     <row r="15">
@@ -1481,27 +1481,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>520402</v>
+        <v>-1809939</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>393814</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>-1870969</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>126588</v>
+      <c r="G15" s="14" t="n">
+        <v>61030</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-500002</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-561032</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-687620</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-470209</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-486193</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-623327</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>55995</v>
+        <v>-36467</v>
       </c>
     </row>
     <row r="16">
@@ -1548,29 +1548,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>-40</v>
+      <c r="C16" s="11" t="n">
+        <v>-4225</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
-        <v>755</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
+        <v>-845</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>-795</v>
+      <c r="G16" s="11" t="n">
+        <v>-3380</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,20 +1578,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>48525</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>51905</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>52700</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>52405</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>45914</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>38077</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-20375</v>
+        <v>52333</v>
       </c>
     </row>
     <row r="17">
@@ -1619,65 +1619,65 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>80956</v>
+        <v>-230462</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>101331</v>
+        <v>-282795</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>52333</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>485728</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>433395</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>453770</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>440725</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>477176</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-20375</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>433395</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>453770</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>440725</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>477176</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>521900</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>-1237</v>
+      <c r="S17" s="14" t="n">
+        <v>-15688</v>
       </c>
     </row>
     <row r="18">
@@ -1688,27 +1688,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>4890</v>
+        <v>-723717</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>110308</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>-613733</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-105418</v>
+      <c r="G18" s="11" t="n">
+        <v>-109984</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,26 +1716,26 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>-34252</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>75732</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>181150</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>-22921</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>-36897</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>63350</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="9" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1745,8 +1745,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-6882</v>
+      <c r="S18" s="14" t="n">
+        <v>-7139</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>606208</v>
+        <v>-2768343</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>606208</v>
+        <v>-2768342</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1792,8 +1792,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>4569</v>
+      <c r="S19" s="14" t="n">
+        <v>9377</v>
       </c>
     </row>
     <row r="20">
@@ -1851,7 +1851,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>-11103</v>
+      <c r="S20" s="14" t="n">
+        <v>-7242</v>
       </c>
     </row>
     <row r="21">
@@ -1871,29 +1871,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>10018</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C21" s="11" t="n">
+        <v>53414</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>7141</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="E21" s="14" t="n">
+        <v>23123</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>2877</v>
+      <c r="G21" s="11" t="n">
+        <v>30291</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1901,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2880689</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2850398</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2847521</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2855594</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2844262</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2878404</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1922,7 +1922,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>26049</v>
+        <v>-200041</v>
       </c>
     </row>
     <row r="22">
@@ -1940,29 +1940,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>8947</v>
+      <c r="C22" s="11" t="n">
+        <v>4367</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>-7838</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+        <v>1036</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>16785</v>
+      <c r="G22" s="11" t="n">
+        <v>3331</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,26 +1970,26 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-3919592</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3922923</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3939708</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3931438</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3948178</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3940979</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1999,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>-105418</v>
+      <c r="S22" s="11" t="n">
+        <v>-109984</v>
       </c>
     </row>
     <row r="23">
@@ -2009,29 +2009,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>-8261</v>
+      <c r="C23" s="14" t="n">
+        <v>-3218</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>-7024</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+        <v>12470</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-1237</v>
+      <c r="G23" s="14" t="n">
+        <v>-15688</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,26 +2039,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>627538</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>643226</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>644463</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>622289</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>626378</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>564209</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-18425</v>
+      <c r="S23" s="14" t="n">
+        <v>-17934</v>
       </c>
     </row>
     <row r="24">
@@ -2080,27 +2080,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-4920</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+        <v>1383</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>13505</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>19317</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-18425</v>
+      <c r="G24" s="14" t="n">
+        <v>-17934</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,26 +2108,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>411365</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>429299</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>447724</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>453555</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>477538</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>498366</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>-29530</v>
+      <c r="S24" s="14" t="n">
+        <v>-100844</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>5784</v>
+        <v>55946</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>5784</v>
+        <v>55946</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-29283</v>
+        <v>32836</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2245,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>124976</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>164212</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>51546</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>51027</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>73430</v>
+      <c r="G27" s="11" t="n">
+        <v>113185</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>750226</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>637041</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>563611</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>528528</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>457286</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>412613</v>
       </c>
     </row>
     <row r="28">
@@ -2298,27 +2298,27 @@
       </c>
       <c r="B28" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>-954</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>37018</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>4248</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-37018</v>
+      <c r="G28" s="14" t="n">
+        <v>-5202</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-223203</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-218001</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-180983</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-164398</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-127926</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-75804</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,29 +2355,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>15279</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>10444</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>22161</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>17583</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>-6882</v>
+      <c r="G29" s="14" t="n">
+        <v>-7139</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-87962</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-80823</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-73941</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-65238</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-52841</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-47864</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 03-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 04-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,29 +2414,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>64137</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>2101</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>93667</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>102945</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>-29530</v>
+      <c r="G30" s="14" t="n">
+        <v>-100844</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-439061</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-338217</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-308687</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-298892</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-276519</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-288945</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24572.7</v>
+        <v>24703.9</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24774.3</v>
+        <v>24703.9</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>204392</v>
+        <v>175803</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>204392</v>
+        <v>175803</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24515.15</v>
+        <v>24427.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24774.3</v>
+        <v>24614.9</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>25119.83333333333</v>
+        <v>25012.5</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24731.10833333334</v>
+        <v>24598.575</v>
       </c>
     </row>
     <row r="33">
@@ -2593,29 +2593,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>57394</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>16621</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>31430</v>
+      <c r="E33" s="11" t="n">
+        <v>58357</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>25964</v>
+        <v>-41736</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-261175</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-219439</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-245403</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-262416</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-238299</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-252014</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24947.06666666667</v>
+        <v>24858.2</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24687.91666666667</v>
+        <v>24582.25</v>
       </c>
     </row>
     <row r="34">
@@ -2660,29 +2660,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>148</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>1398</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>552</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-1250</v>
+      <c r="G34" s="11" t="n">
+        <v>-477</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>29619</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>30096</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>31346</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>30626</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>28094</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>27655</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24860.68333333333</v>
+        <v>24736.55</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24644.725</v>
+        <v>24565.925</v>
       </c>
     </row>
     <row r="35">
@@ -2727,29 +2727,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>20930</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>18783</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>16361</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="E35" s="11" t="n">
+        <v>9406</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n">
-        <v>4569</v>
+      <c r="G35" s="14" t="n">
+        <v>9377</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>107294</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>97917</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>93348</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>85982</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>75423</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>63007</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24687.91666666667</v>
+        <v>24582.25</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2788,29 +2788,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>31916</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>51687</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>61199</v>
+      <c r="E36" s="11" t="n">
+        <v>18851</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-29283</v>
+        <v>32836</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>124262</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>91426</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>120709</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>145808</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>134782</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>161352</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24601.53333333334</v>
+        <v>24460.6</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>110388</v>
+        <v>87166</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>110388</v>
+        <v>87166</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24428.76666666667</v>
+        <v>24306.3</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24342.38333333334</v>
+        <v>24184.65</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.19</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.93</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.76</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.16</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.01</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.56</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,774    PCR(OI) 1.57    Max Pain 24,550</t>
+          <t>Spot 24,615    PCR(OI) 1.01    Max Pain 24,550</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,37 +3010,37 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24750</v>
+        <v>24600</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>94987</v>
+        <v>159349</v>
       </c>
       <c r="R45" s="14" t="n">
-        <v>35014</v>
+        <v>-72389</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>3490451</v>
+        <v>25976250</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24800</v>
+        <v>24650</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>179659</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>74585</v>
+        <v>164073</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>49257</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>3888481</v>
-      </c>
-      <c r="T46" s="28" t="inlineStr">
+        <v>17035749</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3051,22 +3051,22 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>182879</v>
+        <v>137289</v>
       </c>
       <c r="R47" s="14" t="n">
-        <v>15189</v>
+        <v>-45590</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>1922012</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
+        <v>3048686</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,57 +3104,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="31" t="n">
-        <v>24500</v>
+      <c r="P50" s="32" t="n">
+        <v>24600</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>191111</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>159592</v>
+        <v>223307</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>45437</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>6831963</v>
-      </c>
-      <c r="T50" s="32" t="inlineStr">
+        <v>17466099</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="31" t="n">
-        <v>24200</v>
+      <c r="P51" s="32" t="n">
+        <v>24450</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>225769</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>44003</v>
+        <v>180784</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>93643</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1851528</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>23597300</v>
+      </c>
+      <c r="T51" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="31" t="n">
+      <c r="P52" s="32" t="n">
         <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>218938</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>-7003</v>
+        <v>121629</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-97309</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1600851</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>2551524</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 03-Aug-2026    1 DAY AGO = 31-Jul-2026    2 DAYS AGO = 30-Jul-2026    3 DAYS AGO = 29-Jul-2026    4 DAYS AGO = 28-Jul-2026    (generated 03-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 04-Aug-2026    1 DAY AGO = 03-Aug-2026    2 DAYS AGO = 31-Jul-2026    3 DAYS AGO = 30-Jul-2026    4 DAYS AGO = 29-Jul-2026    (generated 04-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-05
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>18015</v>
+        <v>1854</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>13441</v>
+        <v>1181</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-4574</v>
+        <v>-673</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>18015</v>
+        <v>1854</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,28 +725,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>136151</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>134297</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>116282</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>127924</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>133488</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>135390</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>235479</v>
+      <c r="S3" s="14" t="n">
+        <v>-101689</v>
       </c>
     </row>
     <row r="4">
@@ -764,21 +764,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-12156</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-4340</v>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>1373</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>4220</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>-7816</v>
+        <v>-2847</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,28 +794,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>34992</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>37839</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>45655</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>45207</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>49558</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>54192</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -823,8 +823,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>61030</v>
+      <c r="S4" s="11" t="n">
+        <v>-57618</v>
       </c>
     </row>
     <row r="5">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-844</v>
+        <v>-264</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>2113</v>
+        <v>4866</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-2957</v>
+        <v>-5130</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-158903</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-153773</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-150816</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-173113</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-186612</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-194818</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>30291</v>
+        <v>21234</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1236</v>
+        <v>8361</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -916,15 +916,15 @@
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>8478</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-7242</v>
+        <v>2238</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>6123</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-12240</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-18363</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-11121</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-18</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>3566</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>5236</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>113185</v>
+        <v>62825</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1677</v>
+        <v>10651</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1677</v>
+        <v>10651</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-41736</v>
+        <v>-10504</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>-7816</v>
+        <v>-2847</v>
       </c>
     </row>
     <row r="9">
@@ -1087,29 +1087,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-776152</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-1011631</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>235479</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>518457</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>620146</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-101689</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,28 +1117,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>76116</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>177805</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>-57674</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>24116</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>39874</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>8648</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>1030</v>
+      <c r="S9" s="14" t="n">
+        <v>-10</v>
       </c>
     </row>
     <row r="10">
@@ -1156,13 +1156,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>230</v>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-30</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1170,53 +1170,53 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-800</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+        <v>-20</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-10</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>5260</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>5270</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>4240</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>4495</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>4345</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>1030</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>5270</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>4240</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>4495</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>4345</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>4330</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-3380</v>
+      <c r="S10" s="14" t="n">
+        <v>1254</v>
       </c>
     </row>
     <row r="11">
@@ -1225,21 +1225,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-93462</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-56995</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>27039</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>90633</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-36467</v>
+        <v>-63594</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,28 +1255,28 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-228591</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-164997</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-128530</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-184525</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-176285</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-158213</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1284,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>3331</v>
+      <c r="S11" s="14" t="n">
+        <v>-42059</v>
       </c>
     </row>
     <row r="12">
@@ -1294,67 +1294,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-324922</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-124881</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>268920</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>103628</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>165292</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>147214</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-18078</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>181963</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>155914</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>132067</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-200041</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-18078</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>181963</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>155914</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>132067</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>145235</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-5202</v>
+        <v>-8318</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1194306</v>
+        <v>814386</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1194307</v>
+        <v>814387</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-477</v>
+        <v>-2873</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-2957</v>
+        <v>-5130</v>
       </c>
     </row>
     <row r="15">
@@ -1479,29 +1479,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>-1809939</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1870969</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>61030</v>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>314918</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>372536</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-57618</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-557620</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-500002</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-561032</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-687620</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-470209</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-486193</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-36467</v>
+        <v>-63594</v>
       </c>
     </row>
     <row r="16">
@@ -1548,67 +1548,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>-4225</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="14" t="n">
-        <v>-845</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>1254</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>1254</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>49779</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>48525</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>51905</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>52700</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>52405</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-3380</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>48525</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>51905</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>52700</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>52405</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>45914</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>52333</v>
+      <c r="S16" s="11" t="n">
+        <v>-24556</v>
       </c>
     </row>
     <row r="17">
@@ -1617,67 +1617,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>-230462</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-282795</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>32510</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>57066</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-24556</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>461172</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>485728</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>433395</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>453770</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>440725</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>52333</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>485728</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>433395</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>453770</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>440725</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>477176</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-15688</v>
+      <c r="S17" s="11" t="n">
+        <v>8537</v>
       </c>
     </row>
     <row r="18">
@@ -1686,67 +1686,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>-723717</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-613733</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>156640</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>75719</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>80921</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>46669</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-34252</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>75732</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>181150</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-22921</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-109984</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-34252</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>75732</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>181150</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>-22921</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>-36897</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-7139</v>
+        <v>-22267</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2768343</v>
+        <v>505322</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2768342</v>
+        <v>505321</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>9377</v>
+        <v>21282</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-7242</v>
+      <c r="S20" s="11" t="n">
+        <v>6123</v>
       </c>
     </row>
     <row r="21">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>53414</v>
+        <v>25105</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>23123</v>
+        <v>3871</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>30291</v>
+        <v>21234</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2901923</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2880689</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2850398</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2847521</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2855594</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2844262</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-200041</v>
+      <c r="S21" s="11" t="n">
+        <v>165292</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>4367</v>
+        <v>2866</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,53 +1954,53 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>1036</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>44925</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>-42059</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-3961651</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-3919592</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-3922923</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-3939708</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-3931438</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>3331</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-3919592</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-3922923</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-3939708</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-3931438</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-3948178</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-109984</v>
+      <c r="S22" s="14" t="n">
+        <v>80921</v>
       </c>
     </row>
     <row r="23">
@@ -2009,13 +2009,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>-3218</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>16435</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>12470</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-15688</v>
+        <v>7898</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>8537</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,28 +2039,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>636075</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>627538</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>643226</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>644463</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>622289</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>626378</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-17934</v>
+      <c r="S23" s="11" t="n">
+        <v>12288</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>1383</v>
+        <v>22490</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,53 +2092,53 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>19317</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+        <v>10202</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>12288</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>423653</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>411365</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>429299</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>447724</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>453555</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-17934</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>411365</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>429299</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>447724</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>453555</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>477538</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-100844</v>
+        <v>-32240</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>55946</v>
+        <v>66896</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>55946</v>
+        <v>66896</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,9 +2174,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2184,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>32836</v>
+      <c r="S25" s="11" t="n">
+        <v>-7905</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>164212</v>
+        <v>135343</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>51027</v>
+        <v>72518</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>113185</v>
+        <v>62825</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>813051</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>750226</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>637041</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>563611</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>528528</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>457286</v>
       </c>
     </row>
     <row r="28">
@@ -2296,13 +2296,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>-954</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>4248</v>
+        <v>8318</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-5202</v>
+        <v>-8318</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-231521</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-223203</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-218001</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-180983</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-164398</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-127926</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>10444</v>
+        <v>18605</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>17583</v>
+        <v>40872</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-7139</v>
+        <v>-22267</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-110229</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-87962</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-80823</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-73941</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-65238</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-52841</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 04-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 05-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>2101</v>
+        <v>56720</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>102945</v>
+        <v>88960</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-100844</v>
+        <v>-32240</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-471301</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-439061</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-338217</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-308687</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-298892</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-276519</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24703.9</v>
+        <v>24669.2</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24703.9</v>
+        <v>24677.6</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>175803</v>
+        <v>210668</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>175803</v>
+        <v>210668</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24427.95</v>
+        <v>24497.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24614.9</v>
+        <v>24624.65</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>25012.5</v>
+        <v>24881.83333333334</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24598.575</v>
+        <v>24612.35833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>16621</v>
+        <v>40004</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>58357</v>
+        <v>50508</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-41736</v>
+        <v>-10504</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-271679</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-261175</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-219439</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-245403</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-262416</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-238299</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24858.2</v>
+        <v>24779.71666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24582.25</v>
+        <v>24600.06666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>552</v>
+        <v>2893</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-477</v>
+        <v>-2873</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>26746</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>29619</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>30096</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>31346</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>30626</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>28094</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24736.55</v>
+        <v>24702.18333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24565.925</v>
+        <v>24587.775</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>18783</v>
+        <v>36721</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>9406</v>
+        <v>15439</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>9377</v>
+        <v>21282</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>128576</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>107294</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>97917</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>93348</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>85982</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>75423</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24582.25</v>
+        <v>24600.06666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>51687</v>
+        <v>40663</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2802,15 +2802,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>18851</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>32836</v>
+        <v>48568</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-7905</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>116357</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>124262</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>91426</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>120709</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>145808</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>134782</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24460.6</v>
+        <v>24522.53333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>87166</v>
+        <v>117408</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>87166</v>
+        <v>117408</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24306.3</v>
+        <v>24420.41666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24184.65</v>
+        <v>24342.88333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,25 +2933,25 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.06</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.19</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.93</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.76</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.16</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.01</v>
       </c>
     </row>
     <row r="41">
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 04-Aug-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 11-Aug-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,615    PCR(OI) 1.01    Max Pain 24,550</t>
+          <t>Spot 24,625    PCR(OI) 0.72    Max Pain 24,550</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3013,13 +3013,13 @@
         <v>24600</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>159349</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>-72389</v>
+        <v>121838</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>23183</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>25976250</v>
+        <v>3169999</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,16 +3029,16 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24650</v>
+        <v>25000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>164073</v>
+        <v>135553</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>49257</v>
+        <v>39890</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>17035749</v>
+        <v>1460738</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3048,16 +3048,16 @@
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>25000</v>
+        <v>26000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>137289</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>-45590</v>
+        <v>132731</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>49532</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>3048686</v>
+        <v>423346</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3105,54 +3105,54 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>24600</v>
+        <v>24200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>223307</v>
+        <v>81815</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>45437</v>
+        <v>34061</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>17466099</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1156619</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>24450</v>
+        <v>24000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>180784</v>
+        <v>113539</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>93643</v>
+        <v>31977</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>23597300</v>
-      </c>
-      <c r="T51" s="28" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1370223</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>24000</v>
+        <v>23500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>121629</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-97309</v>
+        <v>87860</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>19410</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>2551524</v>
+        <v>503851</v>
       </c>
       <c r="T52" s="30" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 04-Aug-2026    1 DAY AGO = 03-Aug-2026    2 DAYS AGO = 31-Jul-2026    3 DAYS AGO = 30-Jul-2026    4 DAYS AGO = 29-Jul-2026    (generated 04-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 05-Aug-2026    1 DAY AGO = 04-Aug-2026    2 DAYS AGO = 03-Aug-2026    3 DAYS AGO = 31-Jul-2026    4 DAYS AGO = 30-Jul-2026    (generated 05-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-06
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -677,7 +677,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>1854</v>
+        <v>-12284</v>
       </c>
     </row>
     <row r="3">
@@ -697,27 +697,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>1181</v>
+        <v>-11192</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-673</v>
+        <v>1092</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>1854</v>
+        <v>-12284</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,26 +725,26 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>123867</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>136151</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>134297</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>116282</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>127924</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>133488</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-101689</v>
+      <c r="S3" s="11" t="n">
+        <v>-109549</v>
       </c>
     </row>
     <row r="4">
@@ -766,27 +766,27 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>1373</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>-516</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>4220</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+      <c r="E4" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-2847</v>
+      <c r="G4" s="11" t="n">
+        <v>-516</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>34476</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>34992</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>37839</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>45655</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>45207</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>49558</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -815,7 +815,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-57618</v>
+        <v>159131</v>
       </c>
     </row>
     <row r="5">
@@ -835,27 +835,27 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-264</v>
+        <v>2218</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>4866</v>
+        <v>-11567</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-5130</v>
+        <v>13785</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,26 +863,26 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-145118</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-158903</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-153773</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-150816</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-173113</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-186612</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -892,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>21234</v>
+      <c r="S5" s="14" t="n">
+        <v>420</v>
       </c>
     </row>
     <row r="6">
@@ -904,65 +904,65 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>8361</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
+        <v>-96</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="14" t="n">
-        <v>2238</v>
+      <c r="E6" s="11" t="n">
+        <v>889</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-985</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-13225</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-12240</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>-18363</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-11121</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>-18</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>6123</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>-12240</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>-18363</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>-11121</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>-18</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>3566</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>62825</v>
+      <c r="S6" s="14" t="n">
+        <v>68359</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>10651</v>
+        <v>-9586</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>10651</v>
+        <v>-9586</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-10504</v>
+        <v>15381</v>
       </c>
     </row>
     <row r="8">
@@ -1067,7 +1067,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-2847</v>
+      <c r="S8" s="11" t="n">
+        <v>-516</v>
       </c>
     </row>
     <row r="9">
@@ -1089,27 +1089,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>518457</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+        <v>-27905</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>620146</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="E9" s="11" t="n">
+        <v>81644</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-101689</v>
+      <c r="G9" s="11" t="n">
+        <v>-109549</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,20 +1117,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>-33433</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>76116</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>177805</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>-57674</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>24116</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>39874</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1138,7 +1138,7 @@
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1147,7 +1147,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-10</v>
+        <v>555</v>
       </c>
     </row>
     <row r="10">
@@ -1158,27 +1158,27 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>-30</v>
+        <v>555</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-20</v>
+        <v>0</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-10</v>
+        <v>555</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,26 +1186,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>5815</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>5260</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>5270</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4240</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4495</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4345</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1215,8 +1215,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>1254</v>
+      <c r="S10" s="11" t="n">
+        <v>915</v>
       </c>
     </row>
     <row r="11">
@@ -1225,67 +1225,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>27039</v>
+      <c r="C11" s="14" t="n">
+        <v>58213</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>90633</v>
+        <v>-7333</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>65546</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-163045</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-228591</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-164997</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-128530</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-184525</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-63594</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-228591</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-164997</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-128530</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-184525</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-176285</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-42059</v>
+      <c r="S11" s="11" t="n">
+        <v>-54</v>
       </c>
     </row>
     <row r="12">
@@ -1296,27 +1296,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>268920</v>
+        <v>-46319</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>103628</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>-89769</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>165292</v>
+      <c r="G12" s="14" t="n">
+        <v>43450</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,26 +1324,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>190664</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>147214</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-18078</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>181963</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>155914</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>132067</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1353,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-8318</v>
+      <c r="S12" s="11" t="n">
+        <v>-6048</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>814386</v>
+        <v>-15456</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>814387</v>
+        <v>-15458</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1400,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-2873</v>
+      <c r="S13" s="14" t="n">
+        <v>-1171</v>
       </c>
     </row>
     <row r="14">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-5130</v>
+        <v>13785</v>
       </c>
     </row>
     <row r="15">
@@ -1479,29 +1479,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>314918</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>441482</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>372536</v>
+      <c r="E15" s="14" t="n">
+        <v>282351</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-57618</v>
+        <v>159131</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-398489</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-557620</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-500002</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-561032</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-687620</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-470209</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-63594</v>
+        <v>65546</v>
       </c>
     </row>
     <row r="16">
@@ -1548,29 +1548,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>1254</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="C16" s="11" t="n">
+        <v>915</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1254</v>
+      <c r="G16" s="11" t="n">
+        <v>915</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,26 +1578,26 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>50694</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>49779</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>48525</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>51905</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>52700</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>52405</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1607,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-24556</v>
+      <c r="S16" s="14" t="n">
+        <v>-73545</v>
       </c>
     </row>
     <row r="17">
@@ -1617,29 +1617,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>32510</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>19209</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>57066</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>92754</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-24556</v>
+      <c r="G17" s="14" t="n">
+        <v>-73545</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,26 +1647,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>387627</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>461172</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>485728</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>433395</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>453770</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>440725</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>8537</v>
+      <c r="S17" s="14" t="n">
+        <v>3089</v>
       </c>
     </row>
     <row r="18">
@@ -1686,29 +1686,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>156640</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>50608</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>75719</v>
+      <c r="E18" s="14" t="n">
+        <v>137110</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>80921</v>
+        <v>-86502</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,26 +1716,26 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>-39833</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>46669</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-34252</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>75732</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>181150</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-22921</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1745,8 +1745,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-22267</v>
+      <c r="S18" s="11" t="n">
+        <v>-2081</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>505322</v>
+        <v>512214</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>505321</v>
+        <v>512215</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>21282</v>
+        <v>-1135</v>
       </c>
     </row>
     <row r="20">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="Q20" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>6123</v>
+        <v>-985</v>
       </c>
     </row>
     <row r="21">
@@ -1873,27 +1873,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>25105</v>
+        <v>-2371</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>3871</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>-2791</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>21234</v>
+      <c r="G21" s="14" t="n">
+        <v>420</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,26 +1901,26 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2902343</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2901923</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2880689</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2850398</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2847521</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2855594</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>165292</v>
+      <c r="S21" s="14" t="n">
+        <v>43450</v>
       </c>
     </row>
     <row r="22">
@@ -1940,29 +1940,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>2866</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>21612</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>44925</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>21666</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-42059</v>
+      <c r="G22" s="11" t="n">
+        <v>-54</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,20 +1970,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-3961705</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3961651</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3919592</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3922923</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3939708</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3931438</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>80921</v>
+        <v>-86502</v>
       </c>
     </row>
     <row r="23">
@@ -2009,29 +2009,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>16435</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>11480</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>7898</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="11" t="n">
+        <v>8391</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>8537</v>
+      <c r="G23" s="14" t="n">
+        <v>3089</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,20 +2039,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>639164</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>636075</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>627538</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>643226</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>644463</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>622289</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2060,7 +2060,7 @@
       </c>
       <c r="Q23" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>12288</v>
+        <v>-3455</v>
       </c>
     </row>
     <row r="24">
@@ -2078,29 +2078,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>22490</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>9312</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>10202</v>
+      <c r="E24" s="11" t="n">
+        <v>12767</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>12288</v>
+        <v>-3455</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,26 +2108,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>420198</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>423653</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>411365</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>429299</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>447724</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>453555</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-32240</v>
+      <c r="S24" s="11" t="n">
+        <v>-60230</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>66896</v>
+        <v>40033</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>66896</v>
+        <v>40033</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,7 +2174,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2184,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-7905</v>
+      <c r="S25" s="14" t="n">
+        <v>-13075</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2245,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>135343</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="n">
+        <v>118436</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>72518</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="E27" s="11" t="n">
+        <v>50077</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>62825</v>
+      <c r="G27" s="14" t="n">
+        <v>68359</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>881410</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>813051</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>750226</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>637041</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>563611</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>528528</v>
       </c>
     </row>
     <row r="28">
@@ -2296,29 +2296,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>8318</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>6548</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-8318</v>
+      <c r="G28" s="11" t="n">
+        <v>-6048</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-237569</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-231521</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-223203</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-218001</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-180983</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-164398</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,29 +2355,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>18605</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>18064</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>40872</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>20145</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-22267</v>
+      <c r="G29" s="11" t="n">
+        <v>-2081</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-112310</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-110229</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-87962</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-80823</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-73941</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-65238</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 05-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 06-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,29 +2414,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>56720</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>26288</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>88960</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>86518</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>-32240</v>
+      <c r="G30" s="11" t="n">
+        <v>-60230</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-531531</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-471301</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-439061</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-338217</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-308687</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-298892</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24669.2</v>
+        <v>24641</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24677.6</v>
+        <v>24677.05</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>210668</v>
+        <v>163288</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>210668</v>
+        <v>163288</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24497.95</v>
+        <v>24604.15</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24624.65</v>
+        <v>24636</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24881.83333333334</v>
+        <v>24746.88333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24612.35833333334</v>
+        <v>24637.53333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2593,29 +2593,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>40004</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="n">
+        <v>49196</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>50508</v>
+      <c r="E33" s="14" t="n">
+        <v>33815</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-10504</v>
+        <v>15381</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-256298</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-271679</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-261175</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-219439</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-245403</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-262416</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24779.71666666667</v>
+        <v>24711.96666666666</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24600.06666666667</v>
+        <v>24639.06666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2660,29 +2660,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="n">
+        <v>118</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>2893</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>1289</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-2873</v>
+      <c r="G34" s="14" t="n">
+        <v>-1171</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>25575</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>26746</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>29619</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>30096</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>31346</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>30626</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24702.18333333334</v>
+        <v>24673.98333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24587.775</v>
+        <v>24640.6</v>
       </c>
     </row>
     <row r="35">
@@ -2727,29 +2727,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>36721</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>16484</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>15439</v>
+      <c r="E35" s="14" t="n">
+        <v>17619</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>21282</v>
+        <v>-1135</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>127441</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>128576</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>107294</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>97917</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>93348</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>85982</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24600.06666666667</v>
+        <v>24639.06666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2788,29 +2788,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>40663</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>19926</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>48568</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
+      <c r="E36" s="14" t="n">
+        <v>33001</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n">
-        <v>-7905</v>
+      <c r="G36" s="14" t="n">
+        <v>-13075</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>103282</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>116357</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>124262</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>91426</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>120709</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>145808</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24522.53333333334</v>
+        <v>24601.08333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>117408</v>
+        <v>85724</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>117408</v>
+        <v>85724</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24420.41666666667</v>
+        <v>24566.16666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24342.88333333334</v>
+        <v>24528.18333333333</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.06</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.19</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.93</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.76</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.16</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,625    PCR(OI) 0.72    Max Pain 24,550</t>
+          <t>Spot 24,636    PCR(OI) 0.92    Max Pain 24,600</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,16 +3010,16 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24600</v>
+        <v>24700</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>121838</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>23183</v>
+        <v>128178</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>14201</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>3169999</v>
+        <v>2358979</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3032,13 +3032,13 @@
         <v>25000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>135553</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>39890</v>
+        <v>135650</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>97</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1460738</v>
+        <v>1234182</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3051,13 +3051,13 @@
         <v>26000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>132731</v>
+        <v>129341</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>49532</v>
+        <v>-3390</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>423346</v>
+        <v>231389</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3105,20 +3105,20 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>24200</v>
+        <v>24600</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>81815</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>34061</v>
+        <v>131438</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>53936</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>1156619</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>3100342</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3127,17 +3127,17 @@
         <v>24000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>113539</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>31977</v>
+        <v>144432</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>30893</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1370223</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>626197</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3146,13 +3146,13 @@
         <v>23500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>87860</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>19410</v>
+        <v>101423</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>13563</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>503851</v>
+        <v>399588</v>
       </c>
       <c r="T52" s="30" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 05-Aug-2026    1 DAY AGO = 04-Aug-2026    2 DAYS AGO = 03-Aug-2026    3 DAYS AGO = 31-Jul-2026    4 DAYS AGO = 30-Jul-2026    (generated 05-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 06-Aug-2026    1 DAY AGO = 05-Aug-2026    2 DAYS AGO = 04-Aug-2026    3 DAYS AGO = 03-Aug-2026    4 DAYS AGO = 31-Jul-2026    (generated 06-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-07
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -189,14 +189,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -677,7 +677,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-12284</v>
+        <v>6519</v>
       </c>
     </row>
     <row r="3">
@@ -697,65 +697,65 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-11192</v>
+        <v>6148</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1092</v>
+        <v>-371</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>6519</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="n">
+        <v>130386</v>
+      </c>
+      <c r="K3" s="12" t="n">
+        <v>123867</v>
+      </c>
+      <c r="L3" s="12" t="n">
+        <v>136151</v>
+      </c>
+      <c r="M3" s="12" t="n">
+        <v>134297</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>116282</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>-12284</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>123867</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>136151</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>134297</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>116282</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>127924</v>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>-109549</v>
+      <c r="S3" s="14" t="n">
+        <v>-927</v>
       </c>
     </row>
     <row r="4">
@@ -764,29 +764,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="11" t="n">
-        <v>-516</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="C4" s="14" t="n">
+        <v>-143</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-516</v>
+      <c r="G4" s="14" t="n">
+        <v>-143</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>34333</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>34476</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>34992</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>37839</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>45655</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>45207</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -815,7 +815,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>159131</v>
+        <v>-168262</v>
       </c>
     </row>
     <row r="5">
@@ -835,65 +835,65 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>2218</v>
+        <v>-1526</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-11567</v>
+        <v>3414</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-4940</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-150058</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-145118</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-158903</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-153773</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-150816</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>13785</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-145118</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-158903</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-153773</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-150816</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-173113</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>420</v>
+      <c r="S5" s="11" t="n">
+        <v>12567</v>
       </c>
     </row>
     <row r="6">
@@ -902,29 +902,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>-96</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C6" s="14" t="n">
+        <v>-568</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>889</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>868</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>-985</v>
+      <c r="G6" s="14" t="n">
+        <v>-1436</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,26 +932,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-14661</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-13225</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-12240</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-18363</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-11121</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-18</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -961,8 +961,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>68359</v>
+      <c r="S6" s="11" t="n">
+        <v>98783</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-9586</v>
+        <v>3911</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-9586</v>
+        <v>3911</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>15381</v>
+        <v>-18769</v>
       </c>
     </row>
     <row r="8">
@@ -1067,7 +1067,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
+      <c r="Q8" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-516</v>
+      <c r="S8" s="14" t="n">
+        <v>-143</v>
       </c>
     </row>
     <row r="9">
@@ -1089,27 +1089,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-27905</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+        <v>529447</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>81644</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="E9" s="14" t="n">
+        <v>530374</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-109549</v>
+      <c r="G9" s="14" t="n">
+        <v>-927</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,26 +1117,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>-34360</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>-33433</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>76116</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>177805</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>-57674</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>24116</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>555</v>
+      <c r="S9" s="11" t="n">
+        <v>1163</v>
       </c>
     </row>
     <row r="10">
@@ -1156,29 +1156,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>555</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="n">
+        <v>1175</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="E10" s="14" t="n">
+        <v>12</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>555</v>
+      <c r="G10" s="11" t="n">
+        <v>1163</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,26 +1186,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>6978</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>5815</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>5260</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>5270</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4240</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4495</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1215,8 +1215,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>915</v>
+      <c r="S10" s="14" t="n">
+        <v>1470</v>
       </c>
     </row>
     <row r="11">
@@ -1225,29 +1225,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>58213</v>
+      <c r="C11" s="11" t="n">
+        <v>81880</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>-7333</v>
+        <v>131866</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>65546</v>
+        <v>-49986</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,26 +1255,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-213031</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-163045</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-228591</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-164997</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-128530</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-184525</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1284,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-54</v>
+      <c r="S11" s="14" t="n">
+        <v>-6892</v>
       </c>
     </row>
     <row r="12">
@@ -1296,27 +1296,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-46319</v>
+        <v>255116</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>-89769</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>205367</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>43450</v>
+      <c r="G12" s="11" t="n">
+        <v>49749</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,26 +1324,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>240413</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>190664</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>147214</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>-18078</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>181963</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>155914</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1353,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-6048</v>
+      <c r="S12" s="14" t="n">
+        <v>-24229</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-15456</v>
+        <v>867618</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-15458</v>
+        <v>867619</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1400,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-1171</v>
+      <c r="S13" s="11" t="n">
+        <v>-597</v>
       </c>
     </row>
     <row r="14">
@@ -1461,7 +1461,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>13785</v>
+        <v>-4940</v>
       </c>
     </row>
     <row r="15">
@@ -1479,29 +1479,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>441482</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="C15" s="14" t="n">
+        <v>17154</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>282351</v>
+      <c r="E15" s="11" t="n">
+        <v>185416</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>159131</v>
+        <v>-168262</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-566751</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-398489</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-557620</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-500002</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-561032</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-687620</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>65546</v>
+        <v>-49986</v>
       </c>
     </row>
     <row r="16">
@@ -1548,29 +1548,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>915</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="n">
+        <v>1470</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>915</v>
+      <c r="G16" s="14" t="n">
+        <v>1470</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,20 +1578,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>52164</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50694</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>49779</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>48525</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>51905</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>52700</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-73545</v>
+        <v>26785</v>
       </c>
     </row>
     <row r="17">
@@ -1617,67 +1617,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>19209</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C17" s="14" t="n">
+        <v>30658</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>92754</v>
+      <c r="E17" s="11" t="n">
+        <v>3873</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>26785</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>414412</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>387627</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>461172</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>485728</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>433395</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-73545</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>387627</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>461172</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>485728</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>433395</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>453770</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>3089</v>
+        <v>-5630</v>
       </c>
     </row>
     <row r="18">
@@ -1686,67 +1686,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>50608</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="n">
+        <v>159615</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>137110</v>
+      <c r="E18" s="11" t="n">
+        <v>19608</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>140007</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>100174</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-39833</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>46669</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>-34252</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>75732</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-86502</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-39833</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>46669</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>-34252</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>75732</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>181150</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-2081</v>
+      <c r="S18" s="14" t="n">
+        <v>-22745</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>512214</v>
+        <v>208897</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>512215</v>
+        <v>208897</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-1135</v>
+        <v>4887</v>
       </c>
     </row>
     <row r="20">
@@ -1851,7 +1851,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>-985</v>
+      <c r="S20" s="14" t="n">
+        <v>-1436</v>
       </c>
     </row>
     <row r="21">
@@ -1873,27 +1873,27 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-2371</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>8542</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>-2791</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="E21" s="11" t="n">
+        <v>-4025</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>420</v>
+      <c r="G21" s="11" t="n">
+        <v>12567</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,26 +1901,26 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2914910</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2902343</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2901923</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2880689</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2850398</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2847521</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
+      <c r="Q21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>43450</v>
+      <c r="S21" s="11" t="n">
+        <v>49749</v>
       </c>
     </row>
     <row r="22">
@@ -1940,29 +1940,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>21612</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>10801</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>21666</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>17693</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-54</v>
+      <c r="G22" s="14" t="n">
+        <v>-6892</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,20 +1970,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-3968597</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3961705</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3961651</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3919592</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3922923</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3939708</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>-86502</v>
+        <v>140007</v>
       </c>
     </row>
     <row r="23">
@@ -2011,27 +2011,27 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>11480</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+        <v>-1952</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>8391</v>
+      <c r="E23" s="14" t="n">
+        <v>3678</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>3089</v>
+        <v>-5630</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,26 +2039,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>633534</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>639164</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>636075</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>627538</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>643226</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>644463</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-3455</v>
+      <c r="S23" s="14" t="n">
+        <v>-45</v>
       </c>
     </row>
     <row r="24">
@@ -2078,29 +2078,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>9312</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>2014</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>12767</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>2059</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-3455</v>
+      <c r="G24" s="14" t="n">
+        <v>-45</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,26 +2108,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>420153</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>420198</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>423653</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>411365</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>429299</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>447724</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>-60230</v>
+      <c r="S24" s="14" t="n">
+        <v>-51809</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>40033</v>
+        <v>19405</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>40033</v>
+        <v>19405</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>-13075</v>
+        <v>14479</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2245,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>118436</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>184452</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>50077</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>85669</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>68359</v>
+      <c r="G27" s="11" t="n">
+        <v>98783</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>980193</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>881410</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>813051</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>750226</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>637041</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>563611</v>
       </c>
     </row>
     <row r="28">
@@ -2296,29 +2296,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n">
-        <v>500</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="C28" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>6548</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>24229</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-6048</v>
+      <c r="G28" s="14" t="n">
+        <v>-24229</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-261798</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-237569</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-231521</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-223203</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-218001</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-180983</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,29 +2355,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>18064</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>5396</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>20145</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>28141</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>-2081</v>
+      <c r="G29" s="14" t="n">
+        <v>-22745</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-135055</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-112310</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-110229</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-87962</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-80823</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-73941</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 06-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 07-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,29 +2414,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>26288</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>32604</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>86518</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>84413</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>-60230</v>
+      <c r="G30" s="14" t="n">
+        <v>-51809</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-583340</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-531531</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-471301</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-439061</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-338217</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-308687</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24641</v>
+        <v>24538.9</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24677.05</v>
+        <v>24630.4</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>163288</v>
+        <v>222452</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>163288</v>
+        <v>222452</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24604.15</v>
+        <v>24522.75</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24636</v>
+        <v>24570.65</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24746.88333333333</v>
+        <v>24734.10000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24637.53333333333</v>
+        <v>24572.625</v>
       </c>
     </row>
     <row r="33">
@@ -2593,29 +2593,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>49196</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>27596</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>33815</v>
+      <c r="E33" s="11" t="n">
+        <v>46365</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>15381</v>
+        <v>-18769</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-275067</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-256298</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-271679</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-261175</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-219439</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-245403</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24711.96666666666</v>
+        <v>24682.25</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24639.06666666667</v>
+        <v>24574.6</v>
       </c>
     </row>
     <row r="34">
@@ -2662,27 +2662,27 @@
       </c>
       <c r="B34" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>118</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+        <v>-36</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>1289</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>561</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="14" t="n">
-        <v>-1171</v>
+      <c r="G34" s="11" t="n">
+        <v>-597</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>24978</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>25575</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>26746</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>29619</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>30096</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>31346</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24673.98333333333</v>
+        <v>24626.45</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24640.6</v>
+        <v>24576.575</v>
       </c>
     </row>
     <row r="35">
@@ -2727,29 +2727,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>16484</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>16780</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>17619</v>
+      <c r="E35" s="11" t="n">
+        <v>11893</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-1135</v>
+        <v>4887</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>132328</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>127441</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>128576</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>107294</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>97917</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>93348</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24639.06666666667</v>
+        <v>24574.6</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2788,29 +2788,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>19926</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>39041</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>33001</v>
+      <c r="E36" s="11" t="n">
+        <v>24562</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>-13075</v>
+        <v>14479</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>117761</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>103282</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>116357</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>124262</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>91426</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>120709</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24601.08333333333</v>
+        <v>24518.8</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>85724</v>
+        <v>83381</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>85724</v>
+        <v>83381</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24566.16666666667</v>
+        <v>24466.95</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24528.18333333333</v>
+        <v>24411.15</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2936,16 +2936,16 @@
         <v>12.16</v>
       </c>
       <c r="K40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="L40" s="24" t="n">
         <v>12.06</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.19</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.93</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.76</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,636    PCR(OI) 0.92    Max Pain 24,600</t>
+          <t>Spot 24,571    PCR(OI) 0.73    Max Pain 24,600</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,16 +3010,16 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24700</v>
+        <v>24600</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>128178</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>14201</v>
+        <v>184330</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>99208</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2358979</v>
+        <v>4743018</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,16 +3029,16 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>25000</v>
+        <v>24700</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>135650</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>97</v>
+        <v>154059</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>25881</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1234182</v>
+        <v>2749988</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3048,25 +3048,25 @@
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>26000</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>129341</v>
+        <v>174429</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-3390</v>
+        <v>38779</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>231389</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1630908</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,17 +3104,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>24600</v>
+      <c r="P50" s="31" t="n">
+        <v>24500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>131438</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>53936</v>
+        <v>112685</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>23072</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>3100342</v>
+        <v>4313484</v>
       </c>
       <c r="T50" s="28" t="inlineStr">
         <is>
@@ -3123,38 +3123,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
+      <c r="P51" s="31" t="n">
+        <v>24200</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>100008</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>12271</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>1243456</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>144432</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>30893</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>626197</v>
-      </c>
-      <c r="T51" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>23500</v>
-      </c>
       <c r="Q52" s="12" t="n">
-        <v>101423</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>13563</v>
+        <v>159069</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>14637</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>399588</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
+        <v>1029411</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 06-Aug-2026    1 DAY AGO = 05-Aug-2026    2 DAYS AGO = 04-Aug-2026    3 DAYS AGO = 03-Aug-2026    4 DAYS AGO = 31-Jul-2026    (generated 06-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 07-Aug-2026    1 DAY AGO = 06-Aug-2026    2 DAYS AGO = 05-Aug-2026    3 DAYS AGO = 04-Aug-2026    4 DAYS AGO = 03-Aug-2026    (generated 07-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-10
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,22 +128,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,7 +186,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -194,9 +194,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -677,7 +674,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +683,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>6519</v>
+        <v>-34</v>
       </c>
     </row>
     <row r="3">
@@ -695,67 +692,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n">
-        <v>6148</v>
+      <c r="C3" s="13" t="n">
+        <v>1828</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-371</v>
+        <v>1862</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="n">
+        <v>-34</v>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="n">
+        <v>130352</v>
+      </c>
+      <c r="K3" s="14" t="n">
+        <v>130386</v>
+      </c>
+      <c r="L3" s="14" t="n">
+        <v>123867</v>
+      </c>
+      <c r="M3" s="14" t="n">
+        <v>136151</v>
+      </c>
+      <c r="N3" s="14" t="n">
+        <v>134297</v>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G3" s="11" t="n">
-        <v>6519</v>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J3" s="12" t="n">
-        <v>130386</v>
-      </c>
-      <c r="K3" s="12" t="n">
-        <v>123867</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>136151</v>
-      </c>
-      <c r="M3" s="12" t="n">
-        <v>134297</v>
-      </c>
-      <c r="N3" s="12" t="n">
-        <v>116282</v>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R3" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-927</v>
+      <c r="S3" s="13" t="n">
+        <v>13700</v>
       </c>
     </row>
     <row r="4">
@@ -764,50 +761,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-143</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="n">
+        <v>260</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="E4" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>-143</v>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="n">
+        <v>260</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>34593</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>34333</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>34476</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>34992</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>37839</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>45655</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -815,7 +812,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -824,7 +821,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-168262</v>
+        <v>13894</v>
       </c>
     </row>
     <row r="5">
@@ -833,56 +830,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>-1526</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="11" t="n">
+        <v>-573</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>3414</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="11" t="n">
+        <v>1532</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-4940</v>
+      <c r="G5" s="11" t="n">
+        <v>-2105</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-152163</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-150058</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-145118</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-158903</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-153773</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-150816</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
+      <c r="Q5" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -892,8 +889,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>12567</v>
+      <c r="S5" s="13" t="n">
+        <v>10313</v>
       </c>
     </row>
     <row r="6">
@@ -902,56 +899,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>-568</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
         <v>868</v>
       </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-1436</v>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>-1011</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="13" t="n">
+        <v>1879</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>-12782</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>-14661</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>-13225</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>-12240</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>-18363</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-11121</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="9" t="inlineStr">
+      <c r="Q6" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -961,8 +958,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>98783</v>
+      <c r="S6" s="13" t="n">
+        <v>49531</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +970,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>3911</v>
+        <v>2383</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>3911</v>
+        <v>2383</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1000,7 +997,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,7 +1006,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-18769</v>
+        <v>23821</v>
       </c>
     </row>
     <row r="8">
@@ -1067,9 +1064,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1077,8 +1074,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-143</v>
+      <c r="S8" s="13" t="n">
+        <v>260</v>
       </c>
     </row>
     <row r="9">
@@ -1087,56 +1084,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
-        <v>529447</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="C9" s="13" t="n">
+        <v>309525</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>530374</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>-927</v>
+      <c r="E9" s="11" t="n">
+        <v>295825</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>13700</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
+        <v>-20660</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>-34360</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>-33433</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="14" t="n">
         <v>76116</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>177805</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>-57674</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1146,8 +1143,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>1163</v>
+      <c r="S9" s="13" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -1156,58 +1153,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>1175</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="C10" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>-32</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>1163</v>
+      <c r="G10" s="13" t="n">
+        <v>32</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>7010</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>6978</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>5815</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>5260</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>5270</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4240</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1215,8 +1212,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>1470</v>
+      <c r="S10" s="13" t="n">
+        <v>-1517</v>
       </c>
     </row>
     <row r="11">
@@ -1227,65 +1224,65 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>81880</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>131866</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>-12482</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>-25577</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>13095</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>-199936</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>-213031</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>-163045</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>-228591</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>-164997</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-49986</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-213031</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-163045</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-228591</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-164997</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-128530</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-6892</v>
+      <c r="S11" s="11" t="n">
+        <v>-5873</v>
       </c>
     </row>
     <row r="12">
@@ -1294,56 +1291,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>255116</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="C12" s="13" t="n">
+        <v>63843</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="14" t="n">
-        <v>205367</v>
+      <c r="E12" s="11" t="n">
+        <v>90670</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>49749</v>
+        <v>-26827</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>213586</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>240413</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>190664</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>147214</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>-18078</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>181963</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1353,8 +1350,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-24229</v>
+      <c r="S12" s="11" t="n">
+        <v>-23087</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1362,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>867618</v>
+        <v>360886</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>867619</v>
+        <v>360886</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,7 +1387,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1400,8 +1397,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-597</v>
+      <c r="S13" s="13" t="n">
+        <v>-1279</v>
       </c>
     </row>
     <row r="14">
@@ -1459,7 +1456,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1469,8 +1466,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-4940</v>
+      <c r="S14" s="11" t="n">
+        <v>-2105</v>
       </c>
     </row>
     <row r="15">
@@ -1479,58 +1476,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>17154</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>508652</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>185416</v>
+      <c r="E15" s="13" t="n">
+        <v>494758</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-168262</v>
+        <v>13894</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-552857</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-566751</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-398489</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-557620</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-500002</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-561032</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1538,8 +1535,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-49986</v>
+      <c r="S15" s="13" t="n">
+        <v>13095</v>
       </c>
     </row>
     <row r="16">
@@ -1548,67 +1545,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>1470</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>-1517</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>-1517</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="n">
+        <v>50647</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <v>52164</v>
+      </c>
+      <c r="L16" s="14" t="n">
+        <v>50694</v>
+      </c>
+      <c r="M16" s="14" t="n">
+        <v>49779</v>
+      </c>
+      <c r="N16" s="14" t="n">
+        <v>48525</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1470</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>52164</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>50694</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>49779</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>48525</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>51905</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>26785</v>
+      <c r="S16" s="11" t="n">
+        <v>15380</v>
       </c>
     </row>
     <row r="17">
@@ -1617,56 +1614,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>30658</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>64855</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>3873</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="E17" s="13" t="n">
+        <v>49475</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>26785</v>
+      <c r="G17" s="11" t="n">
+        <v>15380</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
+        <v>429792</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>414412</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>387627</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="14" t="n">
         <v>461172</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>485728</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>433395</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1676,8 +1673,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-5630</v>
+      <c r="S17" s="11" t="n">
+        <v>-6584</v>
       </c>
     </row>
     <row r="18">
@@ -1686,56 +1683,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>159615</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>193531</v>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>19608</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
-        <v>140007</v>
+      <c r="E18" s="13" t="n">
+        <v>221288</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>-27757</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
+        <v>72417</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <v>100174</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>-39833</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="14" t="n">
         <v>46669</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>-34252</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>75732</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="13" t="inlineStr">
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1745,8 +1742,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-22745</v>
+      <c r="S18" s="11" t="n">
+        <v>-9019</v>
       </c>
     </row>
     <row r="19">
@@ -1757,11 +1754,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>208897</v>
+        <v>765521</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>208897</v>
+        <v>765521</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1782,7 +1779,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1792,8 +1789,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>4887</v>
+      <c r="S19" s="11" t="n">
+        <v>4174</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1848,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1858,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-1436</v>
+      <c r="S20" s="13" t="n">
+        <v>1879</v>
       </c>
     </row>
     <row r="21">
@@ -1871,50 +1868,50 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="11" t="n">
-        <v>8542</v>
+      <c r="C21" s="13" t="n">
+        <v>16073</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-4025</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
+        <v>5760</v>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>12567</v>
+      <c r="G21" s="13" t="n">
+        <v>10313</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>2925223</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>2914910</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>2902343</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>2901923</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>2880689</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2850398</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1922,7 +1919,7 @@
       </c>
       <c r="Q21" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1931,7 +1928,7 @@
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>49749</v>
+        <v>-26827</v>
       </c>
     </row>
     <row r="22">
@@ -1940,58 +1937,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>10801</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="13" t="n">
+        <v>4916</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>17693</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>10789</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-6892</v>
+      <c r="G22" s="11" t="n">
+        <v>-5873</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-3974470</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-3968597</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-3961705</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-3961651</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-3919592</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3922923</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -1999,8 +1996,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>140007</v>
+      <c r="S22" s="13" t="n">
+        <v>-27757</v>
       </c>
     </row>
     <row r="23">
@@ -2009,58 +2006,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>-1952</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="11" t="n">
+        <v>-2668</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>3678</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="E23" s="11" t="n">
+        <v>3916</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-5630</v>
+      <c r="G23" s="11" t="n">
+        <v>-6584</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>626950</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>633534</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>639164</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>636075</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>627538</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>643226</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2068,8 +2065,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-45</v>
+      <c r="S23" s="13" t="n">
+        <v>2144</v>
       </c>
     </row>
     <row r="24">
@@ -2078,67 +2075,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>2014</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="13" t="n">
+        <v>8880</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>2059</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>6736</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>2144</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>422297</v>
+      </c>
+      <c r="K24" s="14" t="n">
+        <v>420153</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>420198</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>423653</v>
+      </c>
+      <c r="N24" s="14" t="n">
+        <v>411365</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-45</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>420153</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>420198</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>423653</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>411365</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>429299</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-51809</v>
+      <c r="S24" s="11" t="n">
+        <v>-17425</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2146,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>19405</v>
+        <v>27201</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>19405</v>
+        <v>27201</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,9 +2171,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2184,8 +2181,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>14479</v>
+      <c r="S25" s="13" t="n">
+        <v>-26716</v>
       </c>
     </row>
     <row r="26">
@@ -2245,49 +2242,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>184452</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="13" t="n">
+        <v>102099</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>85669</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="E27" s="11" t="n">
+        <v>52568</v>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>98783</v>
+      <c r="G27" s="13" t="n">
+        <v>49531</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>1029724</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>980193</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>881410</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>813051</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>750226</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>637041</v>
       </c>
     </row>
     <row r="28">
@@ -2296,49 +2293,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+      <c r="C28" s="13" t="n">
+        <v>105</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>24229</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="11" t="n">
+        <v>23192</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-24229</v>
+      <c r="G28" s="11" t="n">
+        <v>-23087</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-284885</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-261798</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-237569</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-231521</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-223203</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-218001</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,53 +2352,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>5396</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="13" t="n">
+        <v>13033</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>28141</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
+      <c r="E29" s="11" t="n">
+        <v>22052</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="14" t="n">
-        <v>-22745</v>
+      <c r="G29" s="11" t="n">
+        <v>-9019</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-144074</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-135055</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-112310</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-110229</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-87962</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-80823</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 07-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 10-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,57 +2411,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>32604</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="13" t="n">
+        <v>27931</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>84413</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>45356</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>-51809</v>
+      <c r="G30" s="11" t="n">
+        <v>-17425</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-600765</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-583340</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-531531</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-471301</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-439061</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-338217</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24538.9</v>
+        <v>24581.25</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2469,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24630.4</v>
+        <v>24620.95</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2480,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>222452</v>
+        <v>143168</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>222452</v>
+        <v>143168</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2506,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24522.75</v>
+        <v>24511.1</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2514,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24570.65</v>
+        <v>24583.8</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2573,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24734.10000000001</v>
+        <v>24742.65000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2581,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24572.625</v>
+        <v>24577.875</v>
       </c>
     </row>
     <row r="33">
@@ -2593,57 +2590,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>27596</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="n">
+        <v>59763</v>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>46365</v>
+      <c r="E33" s="13" t="n">
+        <v>35942</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-18769</v>
+        <v>23821</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-251246</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-275067</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-256298</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-271679</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-261175</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-219439</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24682.25</v>
+        <v>24681.8</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2648,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24574.6</v>
+        <v>24571.95</v>
       </c>
     </row>
     <row r="34">
@@ -2660,57 +2657,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>-36</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="13" t="n">
+        <v>-8</v>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>561</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="13" t="n">
+        <v>1271</v>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>-597</v>
+      <c r="G34" s="13" t="n">
+        <v>-1279</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>23699</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>24978</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>25575</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>26746</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>29619</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>30096</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24626.45</v>
+        <v>24632.8</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2715,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24576.575</v>
+        <v>24566.025</v>
       </c>
     </row>
     <row r="35">
@@ -2727,57 +2724,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>16780</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>18027</v>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>11893</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="E35" s="13" t="n">
+        <v>13853</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>4887</v>
+      <c r="G35" s="11" t="n">
+        <v>4174</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>136502</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>132328</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>127441</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>128576</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>107294</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>97917</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24574.6</v>
+        <v>24571.95</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2788,57 +2785,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>39041</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>10849</v>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>24562</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>14479</v>
+      <c r="E36" s="13" t="n">
+        <v>37565</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>-26716</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>91045</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>117761</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>103282</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>116357</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>124262</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>91426</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24518.8</v>
+        <v>24522.95</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2848,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>83381</v>
+        <v>88631</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>83381</v>
+        <v>88631</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2874,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24466.95</v>
+        <v>24462.1</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2886,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24411.15</v>
+        <v>24413.1</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2930,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
-        <v>12.16</v>
+        <v>12.25</v>
       </c>
       <c r="K40" s="24" t="n">
         <v>12.16</v>
       </c>
       <c r="L40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="M40" s="24" t="n">
         <v>12.06</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.19</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.93</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2959,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,571    PCR(OI) 0.73    Max Pain 24,600</t>
+          <t>Spot 24,584    PCR(OI) 0.85    Max Pain 24,600</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3012,14 +3009,14 @@
       <c r="P45" s="27" t="n">
         <v>24600</v>
       </c>
-      <c r="Q45" s="12" t="n">
-        <v>184330</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>99208</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>4743018</v>
+      <c r="Q45" s="14" t="n">
+        <v>225356</v>
+      </c>
+      <c r="R45" s="13" t="n">
+        <v>41026</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>8379660</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,20 +3026,20 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24700</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>154059</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>25881</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>2749988</v>
+        <v>24900</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>181031</v>
+      </c>
+      <c r="R46" s="13" t="n">
+        <v>63475</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>2420775</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3050,18 +3047,18 @@
       <c r="P47" s="27" t="n">
         <v>25000</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>174429</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>38779</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>1630908</v>
+      <c r="Q47" s="14" t="n">
+        <v>198347</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>23918</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>2199878</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3105,16 +3102,16 @@
     </row>
     <row r="50">
       <c r="P50" s="31" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>112685</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>23072</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>4313484</v>
+        <v>24600</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>168278</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>50569</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>8133717</v>
       </c>
       <c r="T50" s="28" t="inlineStr">
         <is>
@@ -3124,20 +3121,20 @@
     </row>
     <row r="51">
       <c r="P51" s="31" t="n">
-        <v>24200</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>100008</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>12271</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1243456</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>24500</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>172617</v>
+      </c>
+      <c r="R51" s="13" t="n">
+        <v>59932</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>6130778</v>
+      </c>
+      <c r="T51" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3145,25 +3142,25 @@
       <c r="P52" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q52" s="12" t="n">
-        <v>159069</v>
+      <c r="Q52" s="14" t="n">
+        <v>155499</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>14637</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>1029411</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
+        <v>-3570</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>1624104</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="33" t="inlineStr">
-        <is>
-          <t>TODAY = 07-Aug-2026    1 DAY AGO = 06-Aug-2026    2 DAYS AGO = 05-Aug-2026    3 DAYS AGO = 04-Aug-2026    4 DAYS AGO = 03-Aug-2026    (generated 07-Aug-2026 20:30 IST)</t>
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>TODAY = 10-Aug-2026    1 DAY AGO = 07-Aug-2026    2 DAYS AGO = 06-Aug-2026    3 DAYS AGO = 05-Aug-2026    4 DAYS AGO = 04-Aug-2026    (generated 10-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-11
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -128,22 +128,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,10 +183,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -194,6 +194,9 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -674,7 +677,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -683,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-34</v>
+        <v>5322</v>
       </c>
     </row>
     <row r="3">
@@ -692,56 +695,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C3" s="13" t="n">
-        <v>1828</v>
+      <c r="C3" s="11" t="n">
+        <v>4933</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>1862</v>
+        <v>-389</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-34</v>
+        <v>5322</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>135674</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>130352</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>130386</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>123867</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>136151</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>134297</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -751,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>13700</v>
+      <c r="S3" s="11" t="n">
+        <v>209393</v>
       </c>
     </row>
     <row r="4">
@@ -761,67 +764,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="13" t="n">
-        <v>260</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-2976</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
+      <c r="E4" s="14" t="n">
+        <v>32</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-3008</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>31585</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>34593</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>34333</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>34476</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>34992</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="13" t="n">
-        <v>260</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="14" t="n">
-        <v>34593</v>
-      </c>
-      <c r="K4" s="14" t="n">
-        <v>34333</v>
-      </c>
-      <c r="L4" s="14" t="n">
-        <v>34476</v>
-      </c>
-      <c r="M4" s="14" t="n">
-        <v>34992</v>
-      </c>
-      <c r="N4" s="14" t="n">
-        <v>37839</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>13894</v>
+      <c r="S4" s="14" t="n">
+        <v>29587</v>
       </c>
     </row>
     <row r="5">
@@ -830,56 +833,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
-        <v>-573</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="C5" s="14" t="n">
+        <v>-1287</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n">
-        <v>1532</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>2681</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="11" t="n">
-        <v>-2105</v>
+      <c r="G5" s="14" t="n">
+        <v>-3968</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-156131</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-152163</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-150058</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-145118</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-158903</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-153773</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="12" t="inlineStr">
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -889,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="13" t="n">
-        <v>10313</v>
+      <c r="S5" s="11" t="n">
+        <v>22435</v>
       </c>
     </row>
     <row r="6">
@@ -899,56 +902,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="13" t="n">
-        <v>868</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="C6" s="11" t="n">
+        <v>813</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
-        <v>-1011</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="n">
+        <v>-841</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>1879</v>
+      <c r="G6" s="11" t="n">
+        <v>1654</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>-11128</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-12782</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>-14661</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>-13225</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>-12240</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>-18363</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="12" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -958,8 +961,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="13" t="n">
-        <v>49531</v>
+      <c r="S6" s="11" t="n">
+        <v>98832</v>
       </c>
     </row>
     <row r="7">
@@ -970,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>2383</v>
+        <v>1483</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>2383</v>
+        <v>1483</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -997,7 +1000,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1006,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>23821</v>
+        <v>-28823</v>
       </c>
     </row>
     <row r="8">
@@ -1064,9 +1067,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1074,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="13" t="n">
-        <v>260</v>
+      <c r="S8" s="14" t="n">
+        <v>-3008</v>
       </c>
     </row>
     <row r="9">
@@ -1084,58 +1087,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>309525</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-1192064</v>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>295825</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+        <v>-1401457</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
-        <v>13700</v>
+      <c r="G9" s="11" t="n">
+        <v>209393</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>188733</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>-20660</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>-34360</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>-33433</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>76116</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>177805</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1143,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>32</v>
+      <c r="S9" s="14" t="n">
+        <v>-20</v>
       </c>
     </row>
     <row r="10">
@@ -1153,67 +1156,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-50</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>-32</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>-30</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-20</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>6990</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>7010</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>6978</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>5815</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>5260</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="14" t="n">
-        <v>7010</v>
-      </c>
-      <c r="K10" s="14" t="n">
-        <v>6978</v>
-      </c>
-      <c r="L10" s="14" t="n">
-        <v>5815</v>
-      </c>
-      <c r="M10" s="14" t="n">
-        <v>5260</v>
-      </c>
-      <c r="N10" s="14" t="n">
-        <v>5270</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>-1517</v>
+      <c r="S10" s="14" t="n">
+        <v>553</v>
       </c>
     </row>
     <row r="11">
@@ -1222,56 +1225,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>-12482</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="C11" s="14" t="n">
+        <v>-156547</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E11" s="13" t="n">
-        <v>-25577</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="E11" s="11" t="n">
+        <v>-158904</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>13095</v>
+      <c r="G11" s="11" t="n">
+        <v>2357</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-197579</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-199936</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-213031</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-163045</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-228591</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-164997</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1281,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>-5873</v>
+      <c r="S11" s="14" t="n">
+        <v>-18467</v>
       </c>
     </row>
     <row r="12">
@@ -1291,56 +1294,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="n">
-        <v>63843</v>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-520696</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="11" t="n">
-        <v>90670</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>-308965</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>-26827</v>
+      <c r="G12" s="14" t="n">
+        <v>-211731</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>1855</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>213586</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>240413</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>190664</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>147214</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-18078</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1350,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-23087</v>
+      <c r="S12" s="14" t="n">
+        <v>-8102</v>
       </c>
     </row>
     <row r="13">
@@ -1362,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>360886</v>
+        <v>-1869357</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>360886</v>
+        <v>-1869356</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1387,7 +1390,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="Q13" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1397,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="13" t="n">
-        <v>-1279</v>
+      <c r="S13" s="11" t="n">
+        <v>-1580</v>
       </c>
     </row>
     <row r="14">
@@ -1456,7 +1459,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1466,8 +1469,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>-2105</v>
+      <c r="S14" s="14" t="n">
+        <v>-3968</v>
       </c>
     </row>
     <row r="15">
@@ -1478,54 +1481,54 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>508652</v>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="n">
-        <v>494758</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>-1244851</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1274438</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>13894</v>
+      <c r="G15" s="14" t="n">
+        <v>29587</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-523270</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-552857</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-566751</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-398489</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-557620</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-500002</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1535,8 +1538,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>13095</v>
+      <c r="S15" s="11" t="n">
+        <v>2357</v>
       </c>
     </row>
     <row r="16">
@@ -1545,56 +1548,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>-1517</v>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>553</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>-1517</v>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>553</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>51200</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50647</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>52164</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>50694</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>49779</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>48525</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1604,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>15380</v>
+      <c r="S16" s="14" t="n">
+        <v>55352</v>
       </c>
     </row>
     <row r="17">
@@ -1616,54 +1619,54 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>64855</v>
-      </c>
-      <c r="D17" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="n">
-        <v>49475</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+        <v>-105613</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-160965</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>15380</v>
+      <c r="G17" s="14" t="n">
+        <v>55352</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>485144</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>429792</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>414412</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>387627</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>461172</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>485728</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1673,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>-6584</v>
+      <c r="S17" s="14" t="n">
+        <v>-10436</v>
       </c>
     </row>
     <row r="18">
@@ -1685,54 +1688,54 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>193531</v>
-      </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="13" t="n">
-        <v>221288</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+        <v>-476050</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-390559</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>-27757</v>
+      <c r="G18" s="11" t="n">
+        <v>-85491</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>-13074</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>72417</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>100174</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>-39833</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>46669</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>-34252</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="9" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1742,8 +1745,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>-9019</v>
+      <c r="S18" s="14" t="n">
+        <v>-14904</v>
       </c>
     </row>
     <row r="19">
@@ -1754,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>765521</v>
+        <v>-1825961</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>765521</v>
+        <v>-1825962</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1779,7 +1782,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1789,8 +1792,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>4174</v>
+      <c r="S19" s="14" t="n">
+        <v>6369</v>
       </c>
     </row>
     <row r="20">
@@ -1848,7 +1851,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="Q20" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1858,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>1879</v>
+      <c r="S20" s="11" t="n">
+        <v>1654</v>
       </c>
     </row>
     <row r="21">
@@ -1868,56 +1871,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C21" s="13" t="n">
-        <v>16073</v>
+      <c r="C21" s="11" t="n">
+        <v>20232</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>5760</v>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
+        <v>-2203</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="13" t="n">
-        <v>10313</v>
+      <c r="G21" s="11" t="n">
+        <v>22435</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>2947658</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2925223</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>2914910</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>2902343</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>2901923</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>2880689</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1927,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>-26827</v>
+      <c r="S21" s="14" t="n">
+        <v>-211731</v>
       </c>
     </row>
     <row r="22">
@@ -1937,56 +1940,56 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="13" t="n">
-        <v>4916</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>5183</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>10789</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>23650</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>-5873</v>
+      <c r="G22" s="14" t="n">
+        <v>-18467</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-3992937</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3974470</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3968597</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3961705</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3961651</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-3919592</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1996,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>-27757</v>
+      <c r="S22" s="11" t="n">
+        <v>-85491</v>
       </c>
     </row>
     <row r="23">
@@ -2006,56 +2009,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>-2668</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>-6512</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>3916</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>3924</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-6584</v>
+      <c r="G23" s="14" t="n">
+        <v>-10436</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>616514</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>626950</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>633534</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>639164</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>636075</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>627538</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2065,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>2144</v>
+      <c r="S23" s="11" t="n">
+        <v>6468</v>
       </c>
     </row>
     <row r="24">
@@ -2075,56 +2078,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C24" s="13" t="n">
-        <v>8880</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>15080</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>6736</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>8612</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>2144</v>
+      <c r="G24" s="11" t="n">
+        <v>6468</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>428765</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>422297</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>420153</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>420198</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>423653</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>411365</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2134,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>-17425</v>
+      <c r="S24" s="14" t="n">
+        <v>-75826</v>
       </c>
     </row>
     <row r="25">
@@ -2146,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>27201</v>
+        <v>33983</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>27201</v>
+        <v>33983</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2171,9 +2174,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2181,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>-26716</v>
+      <c r="S25" s="14" t="n">
+        <v>24034</v>
       </c>
     </row>
     <row r="26">
@@ -2242,49 +2245,49 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C27" s="13" t="n">
-        <v>102099</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>146082</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>52568</v>
-      </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>47250</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G27" s="13" t="n">
-        <v>49531</v>
+      <c r="G27" s="11" t="n">
+        <v>98832</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>1128556</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1029724</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>980193</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>881410</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>813051</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>750226</v>
       </c>
     </row>
     <row r="28">
@@ -2293,49 +2296,49 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="13" t="n">
-        <v>105</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>-5</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>23192</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>8097</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-23087</v>
+      <c r="G28" s="14" t="n">
+        <v>-8102</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-292987</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-284885</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-261798</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-237569</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-231521</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-223203</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2352,53 +2355,53 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C29" s="13" t="n">
-        <v>13033</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>3447</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>22052</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>18351</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n">
-        <v>-9019</v>
+      <c r="G29" s="14" t="n">
+        <v>-14904</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-158978</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-144074</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-135055</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-112310</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-110229</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-87962</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 10-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 11-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2411,57 +2414,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="13" t="n">
-        <v>27931</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>4148</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>45356</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>79974</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>-17425</v>
+      <c r="G30" s="14" t="n">
+        <v>-75826</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-676591</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-600765</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-583340</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-531531</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-471301</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-439061</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24581.25</v>
+        <v>24575.1</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2469,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24620.95</v>
+        <v>24576.85</v>
       </c>
     </row>
     <row r="31">
@@ -2480,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>143168</v>
+        <v>153672</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>143168</v>
+        <v>153672</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2506,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24511.1</v>
+        <v>24429.25</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2514,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24583.8</v>
+        <v>24471.7</v>
       </c>
     </row>
     <row r="32">
@@ -2573,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24742.65000000001</v>
+        <v>24703.55</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2581,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24577.875</v>
+        <v>24482.15000000001</v>
       </c>
     </row>
     <row r="33">
@@ -2590,57 +2593,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>59763</v>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>2406</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E33" s="13" t="n">
-        <v>35942</v>
+      <c r="E33" s="11" t="n">
+        <v>31229</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>23821</v>
+        <v>-28823</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-280069</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-251246</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-275067</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-256298</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-271679</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-261175</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24681.8</v>
+        <v>24640.2</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2648,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24571.95</v>
+        <v>24492.6</v>
       </c>
     </row>
     <row r="34">
@@ -2657,57 +2660,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="13" t="n">
-        <v>-8</v>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="n">
+        <v>18</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="13" t="n">
-        <v>1271</v>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="n">
+        <v>1598</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G34" s="13" t="n">
-        <v>-1279</v>
+      <c r="G34" s="11" t="n">
+        <v>-1580</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>22119</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>23699</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>24978</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>25575</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>26746</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>29619</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24632.8</v>
+        <v>24555.95</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2715,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24566.025</v>
+        <v>24503.05</v>
       </c>
     </row>
     <row r="35">
@@ -2724,57 +2727,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>18027</v>
-      </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>10737</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E35" s="13" t="n">
-        <v>13853</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="E35" s="11" t="n">
+        <v>4368</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n">
-        <v>4174</v>
+      <c r="G35" s="14" t="n">
+        <v>6369</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>142871</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>136502</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>132328</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>127441</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>128576</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>107294</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24571.95</v>
+        <v>24492.6</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2785,57 +2788,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>10849</v>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>31200</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="13" t="n">
-        <v>37565</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="13" t="n">
-        <v>-26716</v>
+      <c r="E36" s="11" t="n">
+        <v>7166</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>24034</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>115079</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>91045</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>117761</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>103282</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>116357</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>124262</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24522.95</v>
+        <v>24408.35000000001</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2848,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>88631</v>
+        <v>44361</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>88631</v>
+        <v>44361</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2874,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24462.1</v>
+        <v>24345</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2886,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24413.1</v>
+        <v>24260.75000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2930,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.86</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>12.25</v>
-      </c>
-      <c r="K40" s="24" t="n">
-        <v>12.16</v>
       </c>
       <c r="L40" s="24" t="n">
         <v>12.16</v>
       </c>
       <c r="M40" s="24" t="n">
+        <v>12.16</v>
+      </c>
+      <c r="N40" s="24" t="n">
         <v>12.06</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.19</v>
       </c>
     </row>
     <row r="41">
@@ -2959,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,584    PCR(OI) 0.85    Max Pain 24,600</t>
+          <t>Spot 24,472    PCR(OI) 0.75    Max Pain 24,450</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3007,58 +3010,58 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24600</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>225356</v>
-      </c>
-      <c r="R45" s="13" t="n">
-        <v>41026</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>8379660</v>
+        <v>24450</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>174635</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>163717</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>13651210</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24900</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>181031</v>
-      </c>
-      <c r="R46" s="13" t="n">
-        <v>63475</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>2420775</v>
+        <v>24500</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>440632</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>379056</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>22606020</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>25000</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>198347</v>
-      </c>
-      <c r="R47" s="13" t="n">
-        <v>23918</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>2199878</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>24600</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>191343</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>-34013</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>12362212</v>
+      </c>
+      <c r="T47" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3102,18 +3105,18 @@
     </row>
     <row r="50">
       <c r="P50" s="31" t="n">
-        <v>24600</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>168278</v>
-      </c>
-      <c r="R50" s="13" t="n">
-        <v>50569</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>8133717</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+        <v>24450</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>369037</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>287536</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>21704008</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3121,18 +3124,18 @@
     </row>
     <row r="51">
       <c r="P51" s="31" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>172617</v>
-      </c>
-      <c r="R51" s="13" t="n">
-        <v>59932</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>6130778</v>
-      </c>
-      <c r="T51" s="28" t="inlineStr">
+        <v>24400</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>216809</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>95625</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>18659281</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3142,25 +3145,25 @@
       <c r="P52" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>155499</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>-3570</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>1624104</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+      <c r="Q52" s="12" t="n">
+        <v>142898</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-12601</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>1606048</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="32" t="inlineStr">
-        <is>
-          <t>TODAY = 10-Aug-2026    1 DAY AGO = 07-Aug-2026    2 DAYS AGO = 06-Aug-2026    3 DAYS AGO = 05-Aug-2026    4 DAYS AGO = 04-Aug-2026    (generated 10-Aug-2026 20:30 IST)</t>
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>TODAY = 11-Aug-2026    1 DAY AGO = 10-Aug-2026    2 DAYS AGO = 07-Aug-2026    3 DAYS AGO = 06-Aug-2026    4 DAYS AGO = 05-Aug-2026    (generated 11-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-12
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -183,10 +183,13 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -194,9 +197,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>5322</v>
+        <v>9225</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>4933</v>
+        <v>5911</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-389</v>
+        <v>-3314</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>5322</v>
+        <v>9225</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,28 +725,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>144899</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>135674</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>130352</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>130386</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>123867</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>136151</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>209393</v>
+      <c r="S3" s="14" t="n">
+        <v>-40945</v>
       </c>
     </row>
     <row r="4">
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>-2976</v>
+        <v>-1308</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>32</v>
+        <v>232</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>-3008</v>
+        <v>-1540</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,28 +794,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>30045</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>31585</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>34593</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>34333</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>34476</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>34992</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -823,8 +823,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>29587</v>
+      <c r="S4" s="11" t="n">
+        <v>-50872</v>
       </c>
     </row>
     <row r="5">
@@ -833,13 +833,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>-1287</v>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>3291</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>2681</v>
+        <v>12329</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-3968</v>
+        <v>-9038</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-165169</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-156131</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-152163</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-150058</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-145118</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-158903</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>22435</v>
+        <v>29993</v>
       </c>
     </row>
     <row r="6">
@@ -908,15 +908,15 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>813</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-841</v>
+        <v>1959</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>606</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1654</v>
+        <v>1353</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-9775</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-11128</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-12782</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-14661</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-13225</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-12240</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>98832</v>
+        <v>83003</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1483</v>
+        <v>9853</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1483</v>
+        <v>9853</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-28823</v>
+        <v>-17912</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>-3008</v>
+        <v>-1540</v>
       </c>
     </row>
     <row r="9">
@@ -1087,67 +1087,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-1192064</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-1401457</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>517608</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>558553</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-40945</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>147788</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>188733</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>-20660</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>-34360</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>-33433</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>209393</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>188733</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>-20660</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>-34360</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>-33433</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>76116</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-20</v>
+      <c r="S9" s="11" t="n">
+        <v>280</v>
       </c>
     </row>
     <row r="10">
@@ -1156,67 +1156,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>-50</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-30</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>380</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>280</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>6990</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>7010</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>6978</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>5815</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-20</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>6990</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>7010</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>6978</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>5815</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>5260</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>553</v>
+      <c r="S10" s="11" t="n">
+        <v>-225</v>
       </c>
     </row>
     <row r="11">
@@ -1225,29 +1225,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-156547</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-158904</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="n">
-        <v>2357</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>42351</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>75711</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-33360</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,20 +1255,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-230939</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-197579</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-199936</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-213031</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-163045</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-228591</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-18467</v>
+        <v>-48637</v>
       </c>
     </row>
     <row r="12">
@@ -1294,67 +1294,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-520696</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-308965</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>238870</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>164843</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>74027</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>75882</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>1855</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>213586</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>240413</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>190664</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-211731</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>1855</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>213586</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>240413</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>190664</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>147214</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-8102</v>
+        <v>-9914</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1869357</v>
+        <v>799209</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1869356</v>
+        <v>799207</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,9 +1390,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q13" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1400,8 +1400,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-1580</v>
+      <c r="S13" s="14" t="n">
+        <v>796</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-3968</v>
+        <v>-9038</v>
       </c>
     </row>
     <row r="15">
@@ -1479,29 +1479,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>-1244851</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1274438</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>29587</v>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>352876</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>403748</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-50872</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,28 +1509,28 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-574142</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-523270</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-552857</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-566751</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-398489</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-557620</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1538,8 +1538,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>2357</v>
+      <c r="S15" s="14" t="n">
+        <v>-33360</v>
       </c>
     </row>
     <row r="16">
@@ -1548,13 +1548,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>553</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-225</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1564,51 +1564,51 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-225</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>50975</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>51200</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>50647</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>52164</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>50694</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>553</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>51200</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>50647</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>52164</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>50694</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>49779</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>55352</v>
+        <v>14593</v>
       </c>
     </row>
     <row r="17">
@@ -1617,21 +1617,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>-105613</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-160965</v>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>62939</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>48346</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>55352</v>
+        <v>14593</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,28 +1647,28 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>499737</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>485144</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>429792</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>414412</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>387627</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>461172</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-10436</v>
+      <c r="S17" s="11" t="n">
+        <v>7748</v>
       </c>
     </row>
     <row r="18">
@@ -1686,67 +1686,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>-476050</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-390559</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>108198</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>71694</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>36504</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>23430</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-13074</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>72417</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>100174</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-39833</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-85491</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-13074</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>72417</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>100174</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>-39833</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>46669</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-14904</v>
+        <v>-18254</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-1825961</v>
+        <v>523788</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-1825962</v>
+        <v>523788</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>6369</v>
+        <v>13765</v>
       </c>
     </row>
     <row r="20">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>1654</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="21">
@@ -1877,15 +1877,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>20232</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>-2203</v>
+        <v>38171</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>8178</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>22435</v>
+        <v>29993</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2977651</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2947658</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2925223</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2914910</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2902343</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2901923</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-211731</v>
+      <c r="S21" s="11" t="n">
+        <v>74027</v>
       </c>
     </row>
     <row r="22">
@@ -1940,13 +1940,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>5183</v>
+      <c r="B22" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>-813</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>23650</v>
+        <v>47824</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-18467</v>
+        <v>-48637</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,28 +1970,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4041574</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-3992937</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3974470</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3968597</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3961705</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3961651</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -1999,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-85491</v>
+      <c r="S22" s="14" t="n">
+        <v>36504</v>
       </c>
     </row>
     <row r="23">
@@ -2009,13 +2009,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>-6512</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>10765</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>3924</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-10436</v>
+        <v>3017</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>7748</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,20 +2039,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>624262</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>616514</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>626950</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>633534</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>639164</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>636075</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>6468</v>
+        <v>10896</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>15080</v>
+        <v>33601</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>8612</v>
+        <v>22705</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>6468</v>
+        <v>10896</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,20 +2108,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>439661</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>428765</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>422297</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>420153</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>420198</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>423653</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-75826</v>
+        <v>-54835</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>33983</v>
+        <v>81724</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>33983</v>
+        <v>81724</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>24034</v>
+        <v>3351</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>146082</v>
+        <v>125484</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>47250</v>
+        <v>42481</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>98832</v>
+        <v>83003</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1211559</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1128556</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1029724</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>980193</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>881410</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>813051</v>
       </c>
     </row>
     <row r="28">
@@ -2296,13 +2296,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>-5</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>278</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>8097</v>
+        <v>10192</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-8102</v>
+        <v>-9914</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-302901</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-292987</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-284885</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-261798</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-237569</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-231521</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>3447</v>
+        <v>8035</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>18351</v>
+        <v>26289</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-14904</v>
+        <v>-18254</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-177232</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-158978</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-144074</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-135055</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-112310</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-110229</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 11-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 12-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>4148</v>
+        <v>21383</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>79974</v>
+        <v>76218</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-75826</v>
+        <v>-54835</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-731426</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-676591</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-600765</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-583340</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-531531</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-471301</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24575.1</v>
+        <v>24472.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24576.85</v>
+        <v>24473.3</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>153672</v>
+        <v>155180</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>153672</v>
+        <v>155180</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24429.25</v>
+        <v>24265.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24471.7</v>
+        <v>24435.95</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24703.55</v>
+        <v>24724.86666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24482.15000000001</v>
+        <v>24413.84166666667</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>2406</v>
+        <v>13030</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>31229</v>
+        <v>30942</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-28823</v>
+        <v>-17912</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-297981</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-280069</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-251246</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-275067</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-256298</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-271679</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24640.2</v>
+        <v>24599.08333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24492.6</v>
+        <v>24391.73333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>18</v>
+        <v>1066</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,15 +2674,15 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1598</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G34" s="11" t="n">
-        <v>-1580</v>
+        <v>270</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>796</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>22915</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>22119</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>23699</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>24978</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>25575</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>26746</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24555.95</v>
+        <v>24517.51666666667</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24503.05</v>
+        <v>24369.625</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>10737</v>
+        <v>20835</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>4368</v>
+        <v>7070</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>6369</v>
+        <v>13765</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>156636</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>142871</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>136502</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>132328</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>127441</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>128576</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24492.6</v>
+        <v>24391.73333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>31200</v>
+        <v>31732</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>7166</v>
+        <v>28381</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>24034</v>
+        <v>3351</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>118430</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>115079</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>91045</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>117761</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>103282</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>116357</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24408.35000000001</v>
+        <v>24310.16666666667</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>44361</v>
+        <v>66663</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>44361</v>
+        <v>66663</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24345</v>
+        <v>24184.38333333334</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24260.75000000001</v>
+        <v>24102.81666666667</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,25 +2933,25 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.86</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>12.25</v>
-      </c>
-      <c r="L40" s="24" t="n">
-        <v>12.16</v>
       </c>
       <c r="M40" s="24" t="n">
         <v>12.16</v>
       </c>
       <c r="N40" s="24" t="n">
-        <v>12.06</v>
+        <v>12.16</v>
       </c>
     </row>
     <row r="41">
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 11-Aug-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 18-Aug-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,472    PCR(OI) 0.75    Max Pain 24,450</t>
+          <t>Spot 24,436    PCR(OI) 0.75    Max Pain 24,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,63 +3010,63 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24450</v>
+        <v>24500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>174635</v>
+        <v>137534</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>163717</v>
+        <v>58499</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>13651210</v>
+        <v>1988153</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24500</v>
+        <v>25000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>440632</v>
+        <v>140576</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>379056</v>
+        <v>40458</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>22606020</v>
+        <v>824244</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>24600</v>
+        <v>25500</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>191343</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>-34013</v>
+        <v>113116</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>32904</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>12362212</v>
-      </c>
-      <c r="T47" s="28" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>411472</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,57 +3104,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="31" t="n">
-        <v>24450</v>
+      <c r="P50" s="32" t="n">
+        <v>24300</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>369037</v>
+        <v>86799</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>287536</v>
+        <v>44694</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>21704008</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+        <v>2351426</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="31" t="n">
-        <v>24400</v>
+      <c r="P51" s="32" t="n">
+        <v>24000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>216809</v>
+        <v>118354</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>95625</v>
+        <v>28326</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>18659281</v>
+        <v>1229884</v>
       </c>
       <c r="T51" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="31" t="n">
-        <v>24000</v>
+      <c r="P52" s="32" t="n">
+        <v>23500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>142898</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-12601</v>
+        <v>82681</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>15836</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1606048</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
+        <v>421567</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 11-Aug-2026    1 DAY AGO = 10-Aug-2026    2 DAYS AGO = 07-Aug-2026    3 DAYS AGO = 06-Aug-2026    4 DAYS AGO = 05-Aug-2026    (generated 11-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 12-Aug-2026    1 DAY AGO = 11-Aug-2026    2 DAYS AGO = 10-Aug-2026    3 DAYS AGO = 07-Aug-2026    4 DAYS AGO = 06-Aug-2026    (generated 12-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-13
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -187,9 +187,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -686,7 +683,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>9225</v>
+        <v>4487</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +698,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5911</v>
+        <v>3989</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +706,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-3314</v>
+        <v>-498</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +714,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>9225</v>
+        <v>4487</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,28 +722,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>149386</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>144899</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>135674</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>130352</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>130386</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>123867</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +751,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-40945</v>
+      <c r="S3" s="11" t="n">
+        <v>46584</v>
       </c>
     </row>
     <row r="4">
@@ -764,13 +761,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-1308</v>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>4</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -778,15 +775,15 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>232</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G4" s="14" t="n">
-        <v>-1540</v>
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>4</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,28 +791,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>30049</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>30045</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>31585</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>34593</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>34333</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>34476</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -823,8 +820,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-50872</v>
+      <c r="S4" s="14" t="n">
+        <v>88580</v>
       </c>
     </row>
     <row r="5">
@@ -833,13 +830,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>3291</v>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>-73</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +844,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>12329</v>
+        <v>3460</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +852,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-9038</v>
+        <v>-3533</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +860,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-168702</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-165169</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-156131</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-152163</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-150058</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-145118</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +890,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>29993</v>
+        <v>19565</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +905,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1959</v>
+        <v>516</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -916,53 +913,53 @@
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>606</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>1474</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-958</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-10733</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-9775</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>-11128</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-12782</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>-14661</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>1353</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>-9775</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>-11128</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>-12782</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>-14661</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>-13225</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>83003</v>
+        <v>38284</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +970,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>9853</v>
+        <v>4436</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>9853</v>
+        <v>4436</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1006,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-17912</v>
+        <v>-14502</v>
       </c>
     </row>
     <row r="8">
@@ -1067,9 +1064,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1077,8 +1074,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-1540</v>
+      <c r="S8" s="11" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1093,7 +1090,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>517608</v>
+        <v>387638</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1101,15 +1098,15 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>558553</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="n">
-        <v>-40945</v>
+        <v>341054</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>46584</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,20 +1114,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>194372</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>147788</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>188733</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>-20660</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>-34360</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>-33433</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1147,7 +1144,7 @@
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>280</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -1162,15 +1159,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>380</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>100</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-20</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1178,7 +1175,7 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>280</v>
+        <v>20</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,20 +1183,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>7290</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>7270</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>6990</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>7010</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>6978</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>5815</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1216,7 +1213,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-225</v>
+        <v>-224</v>
       </c>
     </row>
     <row r="11">
@@ -1231,7 +1228,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>42351</v>
+        <v>17569</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1239,7 +1236,7 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>75711</v>
+        <v>75471</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1247,7 +1244,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-33360</v>
+        <v>-57902</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,20 +1252,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-288841</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-230939</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-197579</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-199936</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-213031</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-163045</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1285,7 +1282,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-48637</v>
+        <v>-28765</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1297,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>238870</v>
+        <v>134767</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1308,7 +1305,7 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>164843</v>
+        <v>123469</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1316,7 +1313,7 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>74027</v>
+        <v>11298</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,20 +1321,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>87180</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>75882</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>1855</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>213586</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>240413</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>190664</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1354,7 +1351,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-9914</v>
+        <v>-17260</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1362,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>799209</v>
+        <v>539974</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>799207</v>
+        <v>539974</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,9 +1387,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1400,8 +1397,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>796</v>
+      <c r="S13" s="11" t="n">
+        <v>-1229</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1467,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-9038</v>
+        <v>-3533</v>
       </c>
     </row>
     <row r="15">
@@ -1485,7 +1482,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>352876</v>
+        <v>382471</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1493,53 +1490,53 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>403748</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>293891</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>88580</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-485562</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-574142</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-523270</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-552857</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-566751</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>-50872</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-574142</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-523270</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-552857</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-566751</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-398489</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-33360</v>
+        <v>-57902</v>
       </c>
     </row>
     <row r="16">
@@ -1554,7 +1551,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-225</v>
+        <v>-224</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1570,7 +1567,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>-225</v>
+        <v>-224</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,28 +1575,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>50751</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50975</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>51200</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>50647</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>52164</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50694</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1607,8 +1604,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>14593</v>
+      <c r="S16" s="11" t="n">
+        <v>-25621</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1620,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>62939</v>
+        <v>32240</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1631,53 +1628,53 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>48346</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>57861</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-25621</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>474116</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>499737</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>485144</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>429792</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>414412</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>14593</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>499737</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>485144</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>429792</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>414412</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>387627</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>7748</v>
+        <v>4169</v>
       </c>
     </row>
     <row r="18">
@@ -1692,7 +1689,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>108198</v>
+        <v>89411</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1700,15 +1697,15 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>71694</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
-        <v>36504</v>
+        <v>152146</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-62735</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1713,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>-39305</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>23430</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-13074</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>72417</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>100174</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-39833</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1743,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-18254</v>
+        <v>-15603</v>
       </c>
     </row>
     <row r="19">
@@ -1757,11 +1754,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>523788</v>
+        <v>503898</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>523788</v>
+        <v>503898</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1793,7 +1790,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>13765</v>
+        <v>10577</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1848,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1858,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>1353</v>
+      <c r="S20" s="14" t="n">
+        <v>-958</v>
       </c>
     </row>
     <row r="21">
@@ -1877,15 +1874,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>38171</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>8178</v>
+        <v>19081</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>-484</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1890,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>29993</v>
+        <v>19565</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1898,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>2997216</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2977651</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2947658</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2925223</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2914910</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2902343</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1931,7 +1928,7 @@
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>74027</v>
+        <v>11298</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +1943,7 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>-813</v>
+        <v>-3472</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,7 +1951,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>47824</v>
+        <v>25293</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1962,7 +1959,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-48637</v>
+        <v>-28765</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,28 +1967,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4070339</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4041574</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-3992937</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3974470</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3968597</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3961705</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -1999,8 +1996,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>36504</v>
+      <c r="S22" s="11" t="n">
+        <v>-62735</v>
       </c>
     </row>
     <row r="23">
@@ -2015,7 +2012,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>10765</v>
+        <v>8296</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,7 +2020,7 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>3017</v>
+        <v>4127</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2031,7 +2028,7 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>7748</v>
+        <v>4169</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,20 +2036,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>628431</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>624262</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>616514</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>626950</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>633534</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>639164</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2069,7 +2066,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>10896</v>
+        <v>5031</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2081,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>33601</v>
+        <v>12112</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,7 +2089,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>22705</v>
+        <v>7081</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,7 +2097,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>10896</v>
+        <v>5031</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,20 +2105,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>444692</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>439661</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>428765</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>422297</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>420153</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>420198</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2135,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-54835</v>
+        <v>-5421</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2146,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>81724</v>
+        <v>36017</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>81724</v>
+        <v>36017</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2182,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>3351</v>
+        <v>5154</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2248,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>125484</v>
+        <v>94198</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2256,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>42481</v>
+        <v>55914</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2264,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>83003</v>
+        <v>38284</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2272,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1249843</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1211559</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1128556</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1029724</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>980193</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>881410</v>
       </c>
     </row>
     <row r="28">
@@ -2302,7 +2299,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,7 +2307,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>10192</v>
+        <v>17260</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2318,7 +2315,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-9914</v>
+        <v>-17260</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2323,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-320161</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-302901</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-292987</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-284885</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-261798</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-237569</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2358,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>8035</v>
+        <v>3824</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2366,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>26289</v>
+        <v>19427</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2374,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-18254</v>
+        <v>-15603</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2382,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-192835</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-177232</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-158978</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-144074</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-135055</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-112310</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 12-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 13-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2417,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>21383</v>
+        <v>23352</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2425,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>76218</v>
+        <v>28773</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2433,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-54835</v>
+        <v>-5421</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2441,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-736847</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-731426</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-676591</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-600765</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-583340</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-531531</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24472.45</v>
+        <v>24431.6</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2469,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24473.3</v>
+        <v>24431.6</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2480,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>155180</v>
+        <v>121374</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>155180</v>
+        <v>121374</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2506,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24265.95</v>
+        <v>24311.4</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2514,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24435.95</v>
+        <v>24395.85</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2573,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24724.86666666666</v>
+        <v>24568.03333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2581,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24413.84166666667</v>
+        <v>24387.73333333334</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2596,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>13030</v>
+        <v>2747</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2604,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>30942</v>
+        <v>17249</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2612,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-17912</v>
+        <v>-14502</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2620,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-312483</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-297981</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-280069</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-251246</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-275067</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-256298</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24599.08333333333</v>
+        <v>24499.81666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2648,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24391.73333333333</v>
+        <v>24379.61666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2663,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>1066</v>
+        <v>67</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,15 +2671,15 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>270</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="n">
-        <v>796</v>
+        <v>1296</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>-1229</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2687,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>21686</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>22915</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>22119</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>23699</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>24978</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>25575</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24517.51666666667</v>
+        <v>24447.83333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2715,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24369.625</v>
+        <v>24371.5</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2730,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>20835</v>
+        <v>19791</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2738,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>7070</v>
+        <v>9214</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2746,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>13765</v>
+        <v>10577</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2754,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>167213</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>156636</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>142871</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>136502</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>132328</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>127441</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24391.73333333333</v>
+        <v>24379.61666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2791,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>31732</v>
+        <v>10934</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2802,7 +2799,7 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>28381</v>
+        <v>5780</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2807,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>3351</v>
+        <v>5154</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2815,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>123584</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>118430</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>115079</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>91045</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>117761</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>103282</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24310.16666666667</v>
+        <v>24327.63333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2848,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>66663</v>
+        <v>33539</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>66663</v>
+        <v>33539</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2874,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24184.38333333334</v>
+        <v>24259.41666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2886,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24102.81666666667</v>
+        <v>24207.43333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,16 +2930,16 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.42</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.69</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.86</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>12.25</v>
-      </c>
-      <c r="M40" s="24" t="n">
-        <v>12.16</v>
       </c>
       <c r="N40" s="24" t="n">
         <v>12.16</v>
@@ -2962,7 +2959,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,436    PCR(OI) 0.75    Max Pain 24,400</t>
+          <t>Spot 24,396    PCR(OI) 0.78    Max Pain 24,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3013,13 +3010,13 @@
         <v>24500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>137534</v>
+        <v>161034</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>58499</v>
+        <v>23500</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>1988153</v>
+        <v>1726155</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,16 +3026,16 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>25000</v>
+        <v>24800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>140576</v>
+        <v>165741</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>40458</v>
+        <v>80203</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>824244</v>
+        <v>905114</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
@@ -3048,25 +3045,25 @@
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>25500</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>113116</v>
+        <v>202109</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>32904</v>
+        <v>61533</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>411472</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>999768</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,66 +3101,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
+      <c r="P50" s="31" t="n">
+        <v>24400</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>99860</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>25252</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>2485445</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="31" t="n">
         <v>24300</v>
       </c>
-      <c r="Q50" s="12" t="n">
-        <v>86799</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>44694</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>2351426</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+      <c r="Q51" s="12" t="n">
+        <v>119848</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>33049</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>2216367</v>
+      </c>
+      <c r="T51" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="P51" s="32" t="n">
+    <row r="52">
+      <c r="P52" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>118354</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>28326</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1229884</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
+      <c r="Q52" s="12" t="n">
+        <v>148176</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>29822</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>1001486</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>82681</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>15836</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>421567</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
     <row r="54">
-      <c r="A54" s="33" t="inlineStr">
-        <is>
-          <t>TODAY = 12-Aug-2026    1 DAY AGO = 11-Aug-2026    2 DAYS AGO = 10-Aug-2026    3 DAYS AGO = 07-Aug-2026    4 DAYS AGO = 06-Aug-2026    (generated 12-Aug-2026 20:30 IST)</t>
+      <c r="A54" s="32" t="inlineStr">
+        <is>
+          <t>TODAY = 13-Aug-2026    1 DAY AGO = 12-Aug-2026    2 DAYS AGO = 11-Aug-2026    3 DAYS AGO = 10-Aug-2026    4 DAYS AGO = 07-Aug-2026    (generated 13-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-14
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -108,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -183,10 +183,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -194,6 +194,9 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -683,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>4487</v>
+        <v>6296</v>
       </c>
     </row>
     <row r="3">
@@ -698,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>3989</v>
+        <v>5060</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -706,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-498</v>
+        <v>-1236</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -714,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>4487</v>
+        <v>6296</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -722,28 +725,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>155682</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>149386</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>144899</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>135674</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>130352</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>130386</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -751,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>46584</v>
+      <c r="S3" s="14" t="n">
+        <v>-61793</v>
       </c>
     </row>
     <row r="4">
@@ -767,7 +770,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>4</v>
+        <v>741</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -783,7 +786,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>4</v>
+        <v>741</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -791,28 +794,28 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>30790</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>30049</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>30045</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>31585</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>34593</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>34333</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -820,8 +823,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>88580</v>
+      <c r="S4" s="11" t="n">
+        <v>-122130</v>
       </c>
     </row>
     <row r="5">
@@ -836,7 +839,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-73</v>
+        <v>-1950</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -844,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>3460</v>
+        <v>6046</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -852,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-3533</v>
+        <v>-7996</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -860,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-176698</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-168702</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-165169</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-156131</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-152163</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-150058</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -890,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>19565</v>
+        <v>15935</v>
       </c>
     </row>
     <row r="6">
@@ -899,29 +902,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>516</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>1474</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-958</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>-105</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-1064</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>959</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -929,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-9774</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-10733</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-9775</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-11128</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-12782</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-14661</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -959,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>38284</v>
+        <v>42097</v>
       </c>
     </row>
     <row r="7">
@@ -970,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>4436</v>
+        <v>3746</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>4436</v>
+        <v>3746</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1006,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-14502</v>
+        <v>-11503</v>
       </c>
     </row>
     <row r="8">
@@ -1075,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>4</v>
+        <v>741</v>
       </c>
     </row>
     <row r="9">
@@ -1090,7 +1093,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>387638</v>
+        <v>126078</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1098,15 +1101,15 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>341054</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>46584</v>
+        <v>187871</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-61793</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1114,28 +1117,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>132579</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>194372</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>147788</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>188733</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>-20660</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>-34360</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1143,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>20</v>
+      <c r="S9" s="14" t="n">
+        <v>-40</v>
       </c>
     </row>
     <row r="10">
@@ -1153,50 +1156,50 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
         <v>-20</v>
       </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
         <v>20</v>
       </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-40</v>
+      </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>7250</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>7290</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>7270</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>6990</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>7010</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>6978</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1213,7 +1216,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-224</v>
+        <v>-148</v>
       </c>
     </row>
     <row r="11">
@@ -1228,7 +1231,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>17569</v>
+        <v>60106</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1236,53 +1239,53 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>75471</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>47910</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>12196</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-276645</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-288841</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-230939</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-197579</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-199936</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-57902</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-288841</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-230939</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-197579</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-199936</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-213031</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-28765</v>
+        <v>-2681</v>
       </c>
     </row>
     <row r="12">
@@ -1297,7 +1300,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>134767</v>
+        <v>77648</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1305,7 +1308,7 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>123469</v>
+        <v>28011</v>
       </c>
       <c r="F12" s="9" t="inlineStr">
         <is>
@@ -1313,7 +1316,7 @@
         </is>
       </c>
       <c r="G12" s="11" t="n">
-        <v>11298</v>
+        <v>49637</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1321,20 +1324,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>136817</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>87180</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>75882</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>1855</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>213586</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>240413</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1351,7 +1354,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-17260</v>
+        <v>-31105</v>
       </c>
     </row>
     <row r="13">
@@ -1362,11 +1365,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>539974</v>
+        <v>263812</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>539974</v>
+        <v>263812</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1398,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1229</v>
+        <v>-604</v>
       </c>
     </row>
     <row r="14">
@@ -1467,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-3533</v>
+        <v>-7996</v>
       </c>
     </row>
     <row r="15">
@@ -1482,7 +1485,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>382471</v>
+        <v>204203</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1490,53 +1493,53 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>293891</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+        <v>326333</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-122130</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-607692</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-485562</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-574142</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-523270</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-552857</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>88580</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-485562</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-574142</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-523270</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-552857</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-566751</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-57902</v>
+      <c r="S15" s="11" t="n">
+        <v>12196</v>
       </c>
     </row>
     <row r="16">
@@ -1551,7 +1554,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-224</v>
+        <v>-148</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1567,7 +1570,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>-224</v>
+        <v>-148</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1575,28 +1578,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>50603</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50751</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>50975</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>51200</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>50647</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>52164</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1604,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-25621</v>
+      <c r="S16" s="14" t="n">
+        <v>23060</v>
       </c>
     </row>
     <row r="17">
@@ -1620,7 +1623,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>32240</v>
+        <v>79748</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1628,53 +1631,53 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>57861</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+        <v>56688</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>23060</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>497176</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>474116</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>499737</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>485144</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>429792</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-25621</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>474116</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>499737</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>485144</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>429792</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>414412</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>4169</v>
+      <c r="S17" s="14" t="n">
+        <v>-4162</v>
       </c>
     </row>
     <row r="18">
@@ -1689,7 +1692,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>89411</v>
+        <v>175253</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1697,53 +1700,53 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>152146</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>76034</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>99219</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>59914</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>-39305</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>23430</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>-13074</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>72417</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-62735</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>-39305</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>23430</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>-13074</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>72417</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>100174</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-15603</v>
+        <v>-6207</v>
       </c>
     </row>
     <row r="19">
@@ -1754,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>503898</v>
+        <v>459056</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>503898</v>
+        <v>459055</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1790,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>10577</v>
+        <v>77</v>
       </c>
     </row>
     <row r="20">
@@ -1848,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1858,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-958</v>
+      <c r="S20" s="11" t="n">
+        <v>959</v>
       </c>
     </row>
     <row r="21">
@@ -1874,7 +1877,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>19081</v>
+        <v>12132</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1882,7 +1885,7 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-484</v>
+        <v>-3803</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1890,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>19565</v>
+        <v>15935</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1898,20 +1901,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3013151</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>2997216</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2977651</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2947658</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2925223</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2914910</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1928,7 +1931,7 @@
         </is>
       </c>
       <c r="S21" s="11" t="n">
-        <v>11298</v>
+        <v>49637</v>
       </c>
     </row>
     <row r="22">
@@ -1943,7 +1946,7 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>-3472</v>
+        <v>-350</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1951,7 +1954,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>25293</v>
+        <v>2331</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1959,7 +1962,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-28765</v>
+        <v>-2681</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1967,28 +1970,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4073020</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4070339</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4041574</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-3992937</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3974470</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3968597</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -1996,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-62735</v>
+      <c r="S22" s="14" t="n">
+        <v>99219</v>
       </c>
     </row>
     <row r="23">
@@ -2012,7 +2015,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>8296</v>
+        <v>6772</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2020,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>4127</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>4169</v>
+        <v>10934</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>-4162</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2036,28 +2039,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>624269</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>628431</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>624262</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>616514</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>626950</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>633534</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2065,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>5031</v>
+      <c r="S23" s="14" t="n">
+        <v>-9092</v>
       </c>
     </row>
     <row r="24">
@@ -2081,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>12112</v>
+        <v>6616</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2089,15 +2092,15 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>7081</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>5031</v>
+        <v>15708</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-9092</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2105,20 +2108,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>435600</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>444692</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>439661</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>428765</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>422297</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>420153</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2135,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-5421</v>
+        <v>-4785</v>
       </c>
     </row>
     <row r="25">
@@ -2146,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>36017</v>
+        <v>25170</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>36017</v>
+        <v>25170</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2182,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>5154</v>
+        <v>12030</v>
       </c>
     </row>
     <row r="26">
@@ -2248,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>94198</v>
+        <v>80495</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2256,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>55914</v>
+        <v>38398</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2264,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>38284</v>
+        <v>42097</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2272,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1291940</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1249843</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1211559</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1128556</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1029724</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>980193</v>
       </c>
     </row>
     <row r="28">
@@ -2307,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>17260</v>
+        <v>31105</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2315,7 +2318,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-17260</v>
+        <v>-31105</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2323,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-351266</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-320161</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-302901</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-292987</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-284885</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-261798</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2358,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>3824</v>
+        <v>9647</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2366,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>19427</v>
+        <v>15854</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2374,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-15603</v>
+        <v>-6207</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2382,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-199042</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-192835</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-177232</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-158978</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-144074</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-135055</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 13-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 14-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2417,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>23352</v>
+        <v>30661</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2425,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>28773</v>
+        <v>35446</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2433,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-5421</v>
+        <v>-4785</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2441,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-741632</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-736847</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-731426</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-676591</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-600765</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-583340</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24431.6</v>
+        <v>24361.9</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2469,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24431.6</v>
+        <v>24405.2</v>
       </c>
     </row>
     <row r="31">
@@ -2480,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>121374</v>
+        <v>120803</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>121374</v>
+        <v>120803</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2506,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24311.4</v>
+        <v>24296.8</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2514,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24395.85</v>
+        <v>24366</v>
       </c>
     </row>
     <row r="32">
@@ -2573,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24568.03333333333</v>
+        <v>24523.6</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2581,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24387.73333333334</v>
+        <v>24361</v>
       </c>
     </row>
     <row r="33">
@@ -2590,13 +2593,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>2747</v>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="n">
+        <v>-5226</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2604,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>17249</v>
+        <v>6277</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2612,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-14502</v>
+        <v>-11503</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2620,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-323986</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-312483</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-297981</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-280069</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-251246</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-275067</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24499.81666666667</v>
+        <v>24464.4</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2648,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24379.61666666667</v>
+        <v>24356</v>
       </c>
     </row>
     <row r="34">
@@ -2663,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2671,7 +2674,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1296</v>
+        <v>629</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2679,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1229</v>
+        <v>-604</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2687,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>21082</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>21686</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>22915</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>22119</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>23699</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>24978</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24447.83333333334</v>
+        <v>24415.2</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2715,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24371.5</v>
+        <v>24351</v>
       </c>
     </row>
     <row r="35">
@@ -2730,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>19791</v>
+        <v>10909</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2738,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>9214</v>
+        <v>10832</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2746,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>10577</v>
+        <v>77</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2754,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>167290</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>167213</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>156636</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>142871</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>136502</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>132328</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24379.61666666667</v>
+        <v>24356</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2791,15 +2794,15 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>10934</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="11" t="n">
-        <v>5780</v>
+        <v>9455</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>-2575</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2807,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>5154</v>
+        <v>12030</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2815,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>135614</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>123584</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>118430</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>115079</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>91045</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>117761</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24327.63333333334</v>
+        <v>24306.8</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2848,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>33539</v>
+        <v>15163</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>33539</v>
+        <v>15163</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2874,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24259.41666666667</v>
+        <v>24247.6</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2886,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24207.43333333334</v>
+        <v>24198.4</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2930,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.31</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.42</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.69</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.86</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>12.25</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.16</v>
       </c>
     </row>
     <row r="41">
@@ -2959,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,396    PCR(OI) 0.78    Max Pain 24,400</t>
+          <t>Spot 24,366    PCR(OI) 0.88    Max Pain 24,400</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,17 +3013,17 @@
         <v>24500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>161034</v>
+        <v>173266</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>23500</v>
+        <v>12232</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>1726155</v>
+        <v>3054132</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3029,17 +3032,17 @@
         <v>24800</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>165741</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>80203</v>
+        <v>159340</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>-6401</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>905114</v>
+        <v>1140822</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3048,17 +3051,17 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>202109</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>61533</v>
+        <v>178164</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>-23945</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>999768</v>
+        <v>1643293</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3102,18 +3105,18 @@
     </row>
     <row r="50">
       <c r="P50" s="31" t="n">
-        <v>24400</v>
+        <v>24300</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>99860</v>
+        <v>156999</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>25252</v>
+        <v>37151</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>2485445</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+        <v>5567965</v>
+      </c>
+      <c r="T50" s="32" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3121,20 +3124,20 @@
     </row>
     <row r="51">
       <c r="P51" s="31" t="n">
-        <v>24300</v>
+        <v>24200</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>119848</v>
+        <v>111423</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>33049</v>
+        <v>14790</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>2216367</v>
+        <v>2285806</v>
       </c>
       <c r="T51" s="28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3143,24 +3146,24 @@
         <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>148176</v>
+        <v>175496</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>29822</v>
+        <v>27320</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1001486</v>
+        <v>1372477</v>
       </c>
       <c r="T52" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="32" t="inlineStr">
-        <is>
-          <t>TODAY = 13-Aug-2026    1 DAY AGO = 12-Aug-2026    2 DAYS AGO = 11-Aug-2026    3 DAYS AGO = 10-Aug-2026    4 DAYS AGO = 07-Aug-2026    (generated 13-Aug-2026 20:30 IST)</t>
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>TODAY = 14-Aug-2026    1 DAY AGO = 13-Aug-2026    2 DAYS AGO = 12-Aug-2026    3 DAYS AGO = 11-Aug-2026    4 DAYS AGO = 10-Aug-2026    (generated 14-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-17
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -183,6 +183,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -194,9 +197,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>6296</v>
+        <v>4909</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5060</v>
+        <v>4015</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-1236</v>
+        <v>-894</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>6296</v>
+        <v>4909</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,20 +725,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>160591</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>155682</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>149386</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>144899</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>135674</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>130352</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="S3" s="14" t="n">
-        <v>-61793</v>
+        <v>-36978</v>
       </c>
     </row>
     <row r="4">
@@ -764,21 +764,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>741</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="14" t="n">
-        <v>0</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-15</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>-264</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>741</v>
+        <v>249</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>31039</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>30790</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>30049</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>30045</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>31585</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>34593</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-122130</v>
+        <v>-53074</v>
       </c>
     </row>
     <row r="5">
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="C5" s="14" t="n">
-        <v>-1950</v>
+        <v>-238</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>6046</v>
+        <v>4651</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-7996</v>
+        <v>-4889</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-181587</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-176698</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-168702</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-165169</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-156131</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-152163</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>15935</v>
+        <v>18461</v>
       </c>
     </row>
     <row r="6">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>-105</v>
+        <v>-2227</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -916,53 +916,53 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-1064</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>-1958</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-269</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-10043</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-9774</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>-10733</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-9775</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>-11128</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>959</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>-9774</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>-10733</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>-9775</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>-11128</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>-12782</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>42097</v>
+        <v>19264</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>3746</v>
+        <v>1535</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>3746</v>
+        <v>1535</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-11503</v>
+        <v>-13383</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>741</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9">
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>126078</v>
+        <v>297432</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>187871</v>
+        <v>334410</v>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="G9" s="14" t="n">
-        <v>-61793</v>
+        <v>-36978</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,28 +1117,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>95601</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>132579</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>194372</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>147788</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>188733</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>-20660</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-40</v>
+      <c r="S9" s="11" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="10">
@@ -1156,67 +1156,67 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>-20</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-50</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>60</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>7310</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>7250</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>7290</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>6990</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-40</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>7250</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>7290</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>7270</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>6990</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>7010</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-148</v>
+        <v>-4295</v>
       </c>
     </row>
     <row r="11">
@@ -1231,7 +1231,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>60106</v>
+        <v>68647</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1239,7 +1239,7 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>47910</v>
+        <v>20527</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>12196</v>
+        <v>48120</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,20 +1255,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-228525</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-276645</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-288841</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-230939</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-197579</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-199936</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-2681</v>
+        <v>-22285</v>
       </c>
     </row>
     <row r="12">
@@ -1300,7 +1300,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>77648</v>
+        <v>12517</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1308,53 +1308,53 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>28011</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>23720</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-11203</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>125614</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>136817</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>87180</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>75882</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>1855</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>49637</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>136817</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>87180</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>75882</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>1855</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>213586</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-31105</v>
+      <c r="S12" s="11" t="n">
+        <v>1896</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>263812</v>
+        <v>378606</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>263812</v>
+        <v>378607</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-604</v>
+        <v>-408</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-7996</v>
+        <v>-4889</v>
       </c>
     </row>
     <row r="15">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>204203</v>
+        <v>280447</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1493,7 +1493,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>326333</v>
+        <v>333521</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-122130</v>
+        <v>-53074</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-660766</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-607692</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-485562</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-574142</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-523270</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-552857</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>12196</v>
+        <v>48120</v>
       </c>
     </row>
     <row r="16">
@@ -1554,7 +1554,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-148</v>
+        <v>-4295</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>-148</v>
+        <v>-4295</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,20 +1578,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>46308</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>50603</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>50751</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>50975</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>51200</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50647</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>23060</v>
+        <v>5279</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>79748</v>
+        <v>44831</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>56688</v>
+        <v>39552</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>23060</v>
+        <v>5279</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,28 +1647,28 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>502455</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>497176</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>474116</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>499737</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>485144</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>429792</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q17" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-4162</v>
+      <c r="S17" s="11" t="n">
+        <v>3707</v>
       </c>
     </row>
     <row r="18">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>175253</v>
+        <v>117934</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>76034</v>
+        <v>65846</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>99219</v>
+        <v>52088</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1716,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>112002</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>59914</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>-39305</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>23430</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>-13074</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>72417</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-6207</v>
+        <v>-8639</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>459056</v>
+        <v>438917</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>459055</v>
+        <v>438919</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>77</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>959</v>
+      <c r="S20" s="14" t="n">
+        <v>-269</v>
       </c>
     </row>
     <row r="21">
@@ -1877,15 +1877,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>12132</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>-3803</v>
+        <v>18877</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>416</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>15935</v>
+        <v>18461</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3031612</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3013151</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>2997216</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2977651</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2947658</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2925223</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>49637</v>
+      <c r="S21" s="14" t="n">
+        <v>-11203</v>
       </c>
     </row>
     <row r="22">
@@ -1940,13 +1940,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C22" s="14" t="n">
-        <v>-350</v>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="n">
+        <v>4952</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>2331</v>
+        <v>27237</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-2681</v>
+        <v>-22285</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,20 +1970,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4095305</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4073020</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4070339</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4041574</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-3992937</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-3974470</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>99219</v>
+        <v>52088</v>
       </c>
     </row>
     <row r="23">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>6772</v>
+        <v>12437</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>10934</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-4162</v>
+        <v>8730</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>3707</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,28 +2039,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>627976</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>624269</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>628431</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>624262</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>616514</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>626950</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-9092</v>
+      <c r="S23" s="11" t="n">
+        <v>117</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>6616</v>
+        <v>17361</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,53 +2092,53 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>15708</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+        <v>17244</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>117</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>435717</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>435600</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>444692</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>439661</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>428765</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-9092</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>435600</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>444692</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>439661</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>428765</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>422297</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-4785</v>
+        <v>-12521</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>25170</v>
+        <v>53627</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>25170</v>
+        <v>53627</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>12030</v>
+        <v>13649</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>80495</v>
+        <v>35536</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>38398</v>
+        <v>16272</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>42097</v>
+        <v>19264</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1311204</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1291940</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1249843</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1211559</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1128556</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1029724</v>
       </c>
     </row>
     <row r="28">
@@ -2302,7 +2302,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
+        <v>4967</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,15 +2310,15 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>31105</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>-31105</v>
+        <v>3071</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>1896</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-349370</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-351266</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-320161</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-302901</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-292987</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-284885</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>9647</v>
+        <v>4869</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>15854</v>
+        <v>13508</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-6207</v>
+        <v>-8639</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-207681</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-199042</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-192835</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-177232</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-158978</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-144074</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 14-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 17-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>30661</v>
+        <v>4779</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>35446</v>
+        <v>17300</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-4785</v>
+        <v>-12521</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-754153</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-741632</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-736847</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-731426</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-676591</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-600765</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24361.9</v>
+        <v>24343.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24405.2</v>
+        <v>24360.1</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>120803</v>
+        <v>50151</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>120803</v>
+        <v>50151</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24296.8</v>
+        <v>24226.95</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24366</v>
+        <v>24287.65</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24523.6</v>
+        <v>24489.33333333334</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24361</v>
+        <v>24289.60833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-5226</v>
+        <v>-4777</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>6277</v>
+        <v>8606</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-11503</v>
+        <v>-13383</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-337369</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-323986</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-312483</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-297981</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-280069</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-251246</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24464.4</v>
+        <v>24424.71666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24356</v>
+        <v>24291.56666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>25</v>
+        <v>240</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-604</v>
+        <v>-408</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>20674</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>21082</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>21686</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>22915</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>22119</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>23699</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24415.2</v>
+        <v>24356.18333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24351</v>
+        <v>24293.525</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>10909</v>
+        <v>10950</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>10832</v>
+        <v>10808</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>77</v>
+        <v>142</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>167432</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>167290</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>167213</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>156636</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>142871</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>136502</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24356</v>
+        <v>24291.56666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>9455</v>
+        <v>8784</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>-2575</v>
+        <v>-4865</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>12030</v>
+        <v>13649</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>149263</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>135614</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>123584</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>118430</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>115079</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>91045</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24306.8</v>
+        <v>24223.03333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>15163</v>
+        <v>15197</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>15163</v>
+        <v>15197</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24247.6</v>
+        <v>24158.41666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24198.4</v>
+        <v>24089.88333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.33</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.31</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.42</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.69</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.86</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>12.25</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,366    PCR(OI) 0.88    Max Pain 24,400</t>
+          <t>Spot 24,288    PCR(OI) 0.92    Max Pain 24,350</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,63 +3010,63 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24500</v>
+        <v>24400</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>173266</v>
+        <v>160961</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>12232</v>
+        <v>36272</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>3054132</v>
+        <v>7294726</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24800</v>
+        <v>24500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>159340</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>-6401</v>
+        <v>192643</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>19377</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1140822</v>
+        <v>4712193</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>25000</v>
+        <v>24600</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>178164</v>
-      </c>
-      <c r="R47" s="14" t="n">
-        <v>-23945</v>
+        <v>158598</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>19456</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>1643293</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
+        <v>2977797</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,57 +3104,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="31" t="n">
+      <c r="P50" s="32" t="n">
         <v>24300</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>156999</v>
+        <v>207546</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>37151</v>
+        <v>50547</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>5567965</v>
-      </c>
-      <c r="T50" s="32" t="inlineStr">
+        <v>10482795</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="31" t="n">
+      <c r="P51" s="32" t="n">
         <v>24200</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>111423</v>
+        <v>160040</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>14790</v>
+        <v>48617</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>2285806</v>
-      </c>
-      <c r="T51" s="28" t="inlineStr">
+        <v>5894407</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="31" t="n">
+      <c r="P52" s="32" t="n">
         <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>175496</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>27320</v>
+        <v>174870</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-626</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>1372477</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>2727692</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 14-Aug-2026    1 DAY AGO = 13-Aug-2026    2 DAYS AGO = 12-Aug-2026    3 DAYS AGO = 11-Aug-2026    4 DAYS AGO = 10-Aug-2026    (generated 14-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 17-Aug-2026    1 DAY AGO = 14-Aug-2026    2 DAYS AGO = 13-Aug-2026    3 DAYS AGO = 12-Aug-2026    4 DAYS AGO = 11-Aug-2026    (generated 17-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-18
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -186,17 +186,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>4909</v>
+        <v>13205</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>4015</v>
+        <v>10925</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-894</v>
+        <v>-2280</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>4909</v>
+        <v>13205</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,28 +725,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>173796</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>160591</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>155682</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>149386</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>144899</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>135674</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-36978</v>
+      <c r="S3" s="11" t="n">
+        <v>200037</v>
       </c>
     </row>
     <row r="4">
@@ -764,21 +764,21 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-15</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>-264</v>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>59</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="n">
+        <v>25</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>249</v>
+        <v>34</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>31073</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>31039</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>30790</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>30049</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>30045</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>31585</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-53074</v>
+        <v>-36634</v>
       </c>
     </row>
     <row r="5">
@@ -833,13 +833,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>-238</v>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>203</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>4651</v>
+        <v>12774</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-4889</v>
+        <v>-12571</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-194158</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-181587</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-176698</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-168702</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-165169</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-156131</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>18461</v>
+        <v>31505</v>
       </c>
     </row>
     <row r="6">
@@ -902,21 +902,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>-2227</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-1958</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1470</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>2138</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
@@ -924,7 +924,7 @@
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-269</v>
+        <v>-668</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>-10711</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-10043</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-9774</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-10733</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-9775</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-11128</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>19264</v>
+        <v>36310</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1535</v>
+        <v>12657</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1535</v>
+        <v>12657</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-13383</v>
+        <v>-28121</v>
       </c>
     </row>
     <row r="8">
@@ -1078,7 +1078,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>249</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9">
@@ -1087,67 +1087,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>297432</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>334410</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-852692</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-1052729</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>200037</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>295638</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>95601</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>132579</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>194372</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>147788</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-36978</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>95601</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>132579</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>194372</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>147788</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>188733</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>60</v>
+      <c r="S9" s="14" t="n">
+        <v>-40</v>
       </c>
     </row>
     <row r="10">
@@ -1156,13 +1156,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>10</v>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="14" t="n">
+        <v>-50</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1170,53 +1170,53 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>-50</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+        <v>-10</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-40</v>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>7310</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>7250</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>7290</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="P10" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>60</v>
-      </c>
-      <c r="I10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J10" s="12" t="n">
-        <v>7310</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>7250</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>7290</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>7270</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>6990</v>
-      </c>
-      <c r="P10" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R10" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-4295</v>
+      <c r="S10" s="14" t="n">
+        <v>900</v>
       </c>
     </row>
     <row r="11">
@@ -1225,67 +1225,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>68647</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>20527</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-152954</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-149818</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-3136</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-231661</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-228525</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-276645</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-288841</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-230939</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>48120</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-228525</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-276645</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-288841</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-230939</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-197579</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-22285</v>
+      <c r="S11" s="11" t="n">
+        <v>1473</v>
       </c>
     </row>
     <row r="12">
@@ -1294,21 +1294,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>12517</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>23720</v>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-380469</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-183609</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-11203</v>
+        <v>-196860</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,28 +1324,28 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-71246</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>125614</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>136817</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>87180</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>75882</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>1855</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1353,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>1896</v>
+      <c r="S12" s="14" t="n">
+        <v>-11135</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>378606</v>
+        <v>-1386165</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>378607</v>
+        <v>-1386166</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-408</v>
+        <v>-70</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-4889</v>
+        <v>-12571</v>
       </c>
     </row>
     <row r="15">
@@ -1479,21 +1479,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n">
-        <v>280447</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>333521</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-1157817</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1121183</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-53074</v>
+        <v>-36634</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,28 +1509,28 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-697400</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-660766</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-607692</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-485562</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-574142</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-523270</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1538,8 +1538,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>48120</v>
+      <c r="S15" s="14" t="n">
+        <v>-3136</v>
       </c>
     </row>
     <row r="16">
@@ -1548,13 +1548,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>-4295</v>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>1000</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1562,15 +1562,15 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>-4295</v>
+        <v>100</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>900</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,20 +1578,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>47208</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>46308</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>50603</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>50751</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>50975</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>51200</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>5279</v>
+        <v>108625</v>
       </c>
     </row>
     <row r="17">
@@ -1617,21 +1617,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>44831</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>39552</v>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-73661</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-182286</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>5279</v>
+        <v>108625</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,28 +1647,28 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>611080</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>502455</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>497176</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>474116</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>499737</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>485144</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>3707</v>
+      <c r="S17" s="14" t="n">
+        <v>-22613</v>
       </c>
     </row>
     <row r="18">
@@ -1686,29 +1686,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>117934</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>65846</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="14" t="n">
-        <v>52088</v>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>-430280</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-357391</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-72889</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1716,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>39113</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>112002</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>59914</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>-39305</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>23430</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-13074</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-8639</v>
+        <v>-15390</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>438917</v>
+        <v>-1660758</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>438919</v>
+        <v>-1660760</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-2</v>
+        <v>2</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>142</v>
+        <v>922</v>
       </c>
     </row>
     <row r="20">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-269</v>
+        <v>-668</v>
       </c>
     </row>
     <row r="21">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>18877</v>
+        <v>37484</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>416</v>
+        <v>5979</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>18461</v>
+        <v>31505</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1901,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3063117</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3031612</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3013151</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>2997216</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2977651</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2947658</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>-11203</v>
+        <v>-196860</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>4952</v>
+        <v>4665</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,53 +1954,53 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>27237</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+        <v>3192</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>1473</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-4093832</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-4095305</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-4073020</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-4070339</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-4041574</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-22285</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-4095305</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-4073020</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-4070339</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-4041574</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-3992937</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>52088</v>
+      <c r="S22" s="11" t="n">
+        <v>-72889</v>
       </c>
     </row>
     <row r="23">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>12437</v>
+        <v>7294</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,15 +2023,15 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>8730</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>3707</v>
+        <v>29907</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>-22613</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,28 +2039,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>605363</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>627976</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>624269</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>628431</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>624262</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>616514</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>117</v>
+      <c r="S23" s="14" t="n">
+        <v>-10365</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>17361</v>
+        <v>28146</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,15 +2092,15 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>17244</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>117</v>
+        <v>38511</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-10365</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,20 +2108,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>425352</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>435717</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>435600</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>444692</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>439661</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>428765</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-12521</v>
+        <v>-9785</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>53627</v>
+        <v>77589</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>53627</v>
+        <v>77589</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>13649</v>
+        <v>27269</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>35536</v>
+        <v>41907</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>16272</v>
+        <v>5597</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>19264</v>
+        <v>36310</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1347514</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1311204</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1291940</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1249843</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1211559</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1128556</v>
       </c>
     </row>
     <row r="28">
@@ -2296,13 +2296,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="n">
-        <v>4967</v>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="n">
+        <v>-5</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,15 +2310,15 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>3071</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="11" t="n">
-        <v>1896</v>
+        <v>11130</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="14" t="n">
+        <v>-11135</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-360505</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-349370</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-351266</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-320161</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-302901</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-292987</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,13 +2355,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C29" s="11" t="n">
-        <v>4869</v>
+      <c r="B29" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="n">
+        <v>-7992</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>13508</v>
+        <v>7398</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-8639</v>
+        <v>-15390</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-223071</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-207681</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-199042</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-192835</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-177232</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-158978</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 17-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 18-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>4779</v>
+        <v>2415</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>17300</v>
+        <v>12200</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-12521</v>
+        <v>-9785</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-763938</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-754153</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-741632</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-736847</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-731426</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-676591</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24343.45</v>
+        <v>24223.85</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24360.1</v>
+        <v>24269.65</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>50151</v>
+        <v>36325</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>50151</v>
+        <v>36325</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24226.95</v>
+        <v>24154.9</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24287.65</v>
+        <v>24154.9</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24489.33333333334</v>
+        <v>24346.15000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24289.60833333334</v>
+        <v>24174.02500000001</v>
       </c>
     </row>
     <row r="33">
@@ -2599,7 +2599,7 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-4777</v>
+        <v>-16196</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>8606</v>
+        <v>11925</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-13383</v>
+        <v>-28121</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-365490</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-337369</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-323986</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-312483</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-297981</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-280069</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24424.71666666667</v>
+        <v>24307.90000000001</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24291.56666666667</v>
+        <v>24193.15000000001</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>240</v>
+        <v>1281</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>648</v>
+        <v>1351</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-408</v>
+        <v>-70</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>20604</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20674</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>21082</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>21686</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>22915</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>22119</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24356.18333333334</v>
+        <v>24231.40000000001</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24293.525</v>
+        <v>24212.275</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>10950</v>
+        <v>3193</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>10808</v>
+        <v>2271</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>142</v>
+        <v>922</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>168354</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>167432</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>167290</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>167213</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>156636</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>142871</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24291.56666666667</v>
+        <v>24193.15000000001</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>8784</v>
+        <v>19373</v>
       </c>
       <c r="D36" s="13" t="inlineStr">
         <is>
@@ -2802,7 +2802,7 @@
         </is>
       </c>
       <c r="E36" s="14" t="n">
-        <v>-4865</v>
+        <v>-7896</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>13649</v>
+        <v>27269</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>176532</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>149263</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>135614</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>123584</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>118430</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>115079</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24223.03333333334</v>
+        <v>24116.65000000001</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>15197</v>
+        <v>7651</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>15197</v>
+        <v>7651</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24158.41666666667</v>
+        <v>24078.40000000001</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24089.88333333334</v>
+        <v>24001.90000000001</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.33</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.31</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.42</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.69</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.86</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,288    PCR(OI) 0.92    Max Pain 24,350</t>
+          <t>Spot 24,155    PCR(OI) 0.63    Max Pain 24,200</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,16 +3010,16 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24400</v>
+        <v>24200</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>160961</v>
+        <v>457286</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>36272</v>
+        <v>430614</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>7294726</v>
+        <v>27670744</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,44 +3029,44 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24500</v>
+        <v>24250</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>192643</v>
+        <v>325355</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>19377</v>
+        <v>296827</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>4712193</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>29709972</v>
+      </c>
+      <c r="T46" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>24600</v>
+        <v>24300</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>158598</v>
+        <v>274204</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>19456</v>
+        <v>178268</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>2977797</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>20096526</v>
+      </c>
+      <c r="T47" s="28" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="29" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,17 +3104,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>24300</v>
+      <c r="P50" s="30" t="n">
+        <v>24150</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>207546</v>
+        <v>329853</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>50547</v>
+        <v>234228</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>10482795</v>
+        <v>28686858</v>
       </c>
       <c r="T50" s="28" t="inlineStr">
         <is>
@@ -3123,38 +3123,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>24200</v>
+      <c r="P51" s="30" t="n">
+        <v>24100</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>160040</v>
+        <v>231465</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>48617</v>
+        <v>121878</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>5894407</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
+        <v>16406269</v>
+      </c>
+      <c r="T51" s="31" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
+      <c r="P52" s="30" t="n">
         <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>174870</v>
+        <v>152925</v>
       </c>
       <c r="R52" s="14" t="n">
-        <v>-626</v>
+        <v>-21945</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>2727692</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
+        <v>4994715</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 17-Aug-2026    1 DAY AGO = 14-Aug-2026    2 DAYS AGO = 13-Aug-2026    3 DAYS AGO = 12-Aug-2026    4 DAYS AGO = 11-Aug-2026    (generated 17-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 18-Aug-2026    1 DAY AGO = 17-Aug-2026    2 DAYS AGO = 14-Aug-2026    3 DAYS AGO = 13-Aug-2026    4 DAYS AGO = 12-Aug-2026    (generated 18-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-19
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -183,7 +183,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -192,10 +195,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>13205</v>
+        <v>11612</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>10925</v>
+        <v>11361</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-2280</v>
+        <v>-251</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>13205</v>
+        <v>11612</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,28 +725,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>185408</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>173796</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>160591</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>155682</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>149386</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>144899</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>200037</v>
+      <c r="S3" s="14" t="n">
+        <v>-22677</v>
       </c>
     </row>
     <row r="4">
@@ -764,13 +764,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>59</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-3454</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -778,15 +778,15 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>34</v>
+        <v>50</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-3504</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>27569</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>31073</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>31039</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>30790</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>30049</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>30045</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-36634</v>
+        <v>-15419</v>
       </c>
     </row>
     <row r="5">
@@ -833,13 +833,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>203</v>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>-632</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>12774</v>
+        <v>15017</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-12571</v>
+        <v>-15649</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-209807</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-194158</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-181587</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-176698</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-168702</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-165169</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>31505</v>
+        <v>8572</v>
       </c>
     </row>
     <row r="6">
@@ -908,61 +908,61 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1470</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>2138</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
+        <v>2502</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-5039</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>7541</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>-3170</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>-10711</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>-10043</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-9774</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>-10733</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="14" t="n">
-        <v>-668</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>-10711</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>-10043</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>-9774</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>-10733</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>-9775</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>36310</v>
+      <c r="S6" s="14" t="n">
+        <v>-20236</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>12657</v>
+        <v>9777</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>12657</v>
+        <v>9777</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-28121</v>
+        <v>-11732</v>
       </c>
     </row>
     <row r="8">
@@ -1067,9 +1067,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>34</v>
+      <c r="S8" s="14" t="n">
+        <v>-3504</v>
       </c>
     </row>
     <row r="9">
@@ -1087,67 +1087,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-852692</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-1052729</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>682063</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>704740</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-22677</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>272961</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>295638</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>95601</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>132579</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>194372</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>200037</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>295638</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>95601</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>132579</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>194372</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>147788</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-40</v>
+      <c r="S9" s="11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1156,29 +1156,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C10" s="14" t="n">
-        <v>-50</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-10</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>-40</v>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1189,25 +1189,25 @@
         <v>7270</v>
       </c>
       <c r="K10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="L10" s="12" t="n">
         <v>7310</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>7250</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>7290</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7270</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1215,8 +1215,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>900</v>
+      <c r="S10" s="11" t="n">
+        <v>-3104</v>
       </c>
     </row>
     <row r="11">
@@ -1225,21 +1225,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-152954</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-149818</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>98716</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>180641</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-3136</v>
+        <v>-81925</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,28 +1255,28 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-313586</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-231661</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-228525</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-276645</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-288841</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-230939</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1284,8 +1284,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>1473</v>
+      <c r="S11" s="14" t="n">
+        <v>-10898</v>
       </c>
     </row>
     <row r="12">
@@ -1294,67 +1294,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-380469</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-183609</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>281627</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>177026</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>104601</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>33355</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-71246</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>125614</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>136817</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>87180</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-196860</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-71246</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>125614</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>136817</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>87180</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>75882</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-11135</v>
+        <v>-3331</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1386165</v>
+        <v>1062406</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1386166</v>
+        <v>1062407</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-70</v>
+        <v>-122</v>
       </c>
     </row>
     <row r="14">
@@ -1470,7 +1470,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-12571</v>
+        <v>-15649</v>
       </c>
     </row>
     <row r="15">
@@ -1479,21 +1479,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>-1157817</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1121183</v>
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>326449</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>341868</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1501,7 +1501,7 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-36634</v>
+        <v>-15419</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-712819</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-697400</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-660766</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-607692</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-485562</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-574142</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-3136</v>
+        <v>-81925</v>
       </c>
     </row>
     <row r="16">
@@ -1548,13 +1548,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>1000</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-3104</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1562,15 +1562,15 @@
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="n">
-        <v>900</v>
+        <v>0</v>
+      </c>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-3104</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,28 +1578,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>44104</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>47208</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>46308</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>50603</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>50751</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50975</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1607,8 +1607,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>108625</v>
+      <c r="S16" s="11" t="n">
+        <v>-39456</v>
       </c>
     </row>
     <row r="17">
@@ -1617,67 +1617,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>-73661</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-182286</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>79831</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>119287</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-39456</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>571624</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>611080</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>502455</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>497176</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>474116</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>108625</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>611080</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>502455</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>497176</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>474116</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>499737</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-22613</v>
+      <c r="S17" s="11" t="n">
+        <v>11774</v>
       </c>
     </row>
     <row r="18">
@@ -1686,67 +1686,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>-430280</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-357391</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>128922</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>70945</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>57977</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>97090</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>39113</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>112002</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>59914</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>-39305</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-72889</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>39113</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>112002</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>59914</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>-39305</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>23430</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-15390</v>
+        <v>-15474</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-1660758</v>
+        <v>532098</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-1660760</v>
+        <v>532100</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>922</v>
+        <v>457</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-668</v>
+      <c r="S20" s="11" t="n">
+        <v>7541</v>
       </c>
     </row>
     <row r="21">
@@ -1877,7 +1877,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>37484</v>
+        <v>22808</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1885,7 +1885,7 @@
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>5979</v>
+        <v>14236</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>31505</v>
+        <v>8572</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,28 +1901,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3071689</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3063117</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3031612</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3013151</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>2997216</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>2977651</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1930,8 +1930,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-196860</v>
+      <c r="S21" s="11" t="n">
+        <v>104601</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>4665</v>
+        <v>6362</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1954,53 +1954,53 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>3192</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>17260</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>-10898</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-4104730</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-4093832</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-4095305</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-4073020</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-4070339</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>1473</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-4093832</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-4095305</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-4073020</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-4070339</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-4041574</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-72889</v>
+      <c r="S22" s="14" t="n">
+        <v>57977</v>
       </c>
     </row>
     <row r="23">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>7294</v>
+        <v>25981</v>
       </c>
       <c r="D23" s="13" t="inlineStr">
         <is>
@@ -2023,53 +2023,53 @@
         </is>
       </c>
       <c r="E23" s="14" t="n">
-        <v>29907</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+        <v>14207</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>11774</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>617137</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>605363</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>627976</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>624269</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>628431</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>-22613</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>605363</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>627976</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>624269</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>628431</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>624262</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="14" t="n">
-        <v>-10365</v>
+        <v>-9448</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>28146</v>
+        <v>35964</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>38511</v>
+        <v>45412</v>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-10365</v>
+        <v>-9448</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,28 +2108,28 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>415904</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>425352</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>435717</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>435600</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>444692</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>439661</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-9785</v>
+      <c r="S24" s="11" t="n">
+        <v>39041</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>77589</v>
+        <v>91115</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>77589</v>
+        <v>91115</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>27269</v>
+        <v>11397</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2245,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="n">
-        <v>41907</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>5597</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="n">
-        <v>36310</v>
+      <c r="B27" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C27" s="14" t="n">
+        <v>-45087</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n">
+        <v>-24851</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G27" s="14" t="n">
+        <v>-20236</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1327278</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1347514</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1311204</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1291940</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1249843</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1211559</v>
       </c>
     </row>
     <row r="28">
@@ -2296,13 +2296,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>-5</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2310,7 +2310,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>11130</v>
+        <v>3331</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2318,7 +2318,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-11135</v>
+        <v>-3331</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-363836</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-360505</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-349370</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-351266</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-320161</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-302901</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="14" t="n">
-        <v>-7992</v>
+        <v>-13362</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>7398</v>
+        <v>2112</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-15390</v>
+        <v>-15474</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-238545</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-223071</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-207681</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-199042</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-192835</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-177232</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 18-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 19-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,23 +2420,23 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>2415</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>12200</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>-9785</v>
+        <v>14855</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="n">
+        <v>-24186</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>39041</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-724897</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-763938</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-754153</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-741632</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-736847</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-731426</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24223.85</v>
+        <v>24152.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24269.65</v>
+        <v>24172.85</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>36325</v>
+        <v>-43594</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>36325</v>
+        <v>-43594</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24154.9</v>
+        <v>24025.65</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24154.9</v>
+        <v>24078.3</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24346.15000000001</v>
+        <v>24306.08333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24174.02500000001</v>
+        <v>24085.28333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2599,15 +2599,15 @@
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-16196</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E33" s="11" t="n">
-        <v>11925</v>
+        <v>-21420</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>-9688</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-28121</v>
+        <v>-11732</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-377222</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-365490</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-337369</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-323986</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-312483</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-297981</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24307.90000000001</v>
+        <v>24239.46666666666</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24193.15000000001</v>
+        <v>24092.26666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,7 +2666,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>1281</v>
+        <v>455</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2674,7 +2674,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>1351</v>
+        <v>577</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-70</v>
+        <v>-122</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>20482</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20604</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>20674</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>21082</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>21686</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>22915</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24231.40000000001</v>
+        <v>24158.88333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24212.275</v>
+        <v>24099.25</v>
       </c>
     </row>
     <row r="35">
@@ -2727,21 +2727,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="n">
-        <v>3193</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E35" s="11" t="n">
-        <v>2271</v>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>-11060</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>-11517</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>922</v>
+        <v>457</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>168811</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>168354</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>167432</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>167290</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>167213</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>156636</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24193.15000000001</v>
+        <v>24092.26666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,15 +2794,15 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>19373</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>-7896</v>
+        <v>17992</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>6595</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
@@ -2810,7 +2810,7 @@
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>27269</v>
+        <v>11397</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>187929</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>176532</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>149263</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>135614</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>123584</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>118430</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24116.65000000001</v>
+        <v>24011.68333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>7651</v>
+        <v>-14033</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>7651</v>
+        <v>-14033</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24078.40000000001</v>
+        <v>23945.06666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24001.90000000001</v>
+        <v>23864.48333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,25 +2933,25 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.33</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.31</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.42</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.69</v>
       </c>
     </row>
     <row r="41">
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 18-Aug-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 25-Aug-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,155    PCR(OI) 0.63    Max Pain 24,200</t>
+          <t>Spot 24,078    PCR(OI) 0.70    Max Pain 24,200</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,63 +3010,63 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24200</v>
+        <v>24500</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>457286</v>
+        <v>228681</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>430614</v>
+        <v>42774</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>27670744</v>
+        <v>951238</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>24250</v>
+        <v>25000</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>325355</v>
+        <v>224540</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>296827</v>
+        <v>11042</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>29709972</v>
-      </c>
-      <c r="T46" s="28" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>791116</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>24300</v>
+        <v>25500</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>274204</v>
+        <v>180366</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>178268</v>
+        <v>35647</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>20096526</v>
-      </c>
-      <c r="T47" s="28" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>443967</v>
+      </c>
+      <c r="T47" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="29" t="inlineStr">
+      <c r="P48" s="30" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,57 +3104,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="30" t="n">
-        <v>24150</v>
+      <c r="P50" s="31" t="n">
+        <v>24000</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>329853</v>
+        <v>210294</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>234228</v>
+        <v>34745</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>28686858</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+        <v>2509725</v>
+      </c>
+      <c r="T50" s="32" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="30" t="n">
-        <v>24100</v>
+      <c r="P51" s="31" t="n">
+        <v>23500</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>231465</v>
+        <v>129792</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>121878</v>
+        <v>26812</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>16406269</v>
-      </c>
-      <c r="T51" s="31" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>460825</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="30" t="n">
-        <v>24000</v>
+      <c r="P52" s="31" t="n">
+        <v>23000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>152925</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-21945</v>
+        <v>155396</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>19446</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>4994715</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
+        <v>345854</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 18-Aug-2026    1 DAY AGO = 17-Aug-2026    2 DAYS AGO = 14-Aug-2026    3 DAYS AGO = 13-Aug-2026    4 DAYS AGO = 12-Aug-2026    (generated 18-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 19-Aug-2026    1 DAY AGO = 18-Aug-2026    2 DAYS AGO = 17-Aug-2026    3 DAYS AGO = 14-Aug-2026    4 DAYS AGO = 13-Aug-2026    (generated 19-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-20
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -36,10 +36,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -677,7 +677,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>11612</v>
+        <v>-12103</v>
       </c>
     </row>
     <row r="3">
@@ -697,27 +697,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>11361</v>
+        <v>-7241</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-251</v>
+        <v>4862</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>11612</v>
+        <v>-12103</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,26 +725,26 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>173305</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>185408</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>173796</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>160591</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>155682</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>149386</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="13" t="inlineStr">
+      <c r="Q3" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -754,8 +754,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="14" t="n">
-        <v>-22677</v>
+      <c r="S3" s="11" t="n">
+        <v>-161624</v>
       </c>
     </row>
     <row r="4">
@@ -764,29 +764,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>-3454</v>
+      <c r="C4" s="11" t="n">
+        <v>-307</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>50</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+        <v>-16</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-3504</v>
+      <c r="G4" s="11" t="n">
+        <v>-291</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,20 +794,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>27278</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>27569</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>31073</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>31039</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>30790</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>30049</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -815,7 +815,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -824,7 +824,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-15419</v>
+        <v>22157</v>
       </c>
     </row>
     <row r="5">
@@ -833,29 +833,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>-632</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="11" t="n">
+        <v>-535</v>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>15017</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="11" t="n">
+        <v>1771</v>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-15649</v>
+      <c r="G5" s="11" t="n">
+        <v>-2306</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,20 +863,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-212113</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-209807</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-194158</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-181587</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-176698</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-168702</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -884,7 +884,7 @@
       </c>
       <c r="Q5" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -893,7 +893,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>8572</v>
+        <v>-11954</v>
       </c>
     </row>
     <row r="6">
@@ -902,29 +902,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="11" t="n">
-        <v>2502</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="C6" s="14" t="n">
+        <v>11546</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>-5039</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>-3154</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>7541</v>
+      <c r="G6" s="14" t="n">
+        <v>14700</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,26 +932,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>11530</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>-3170</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-10711</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-10043</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-9774</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-10733</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -961,8 +961,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>-20236</v>
+      <c r="S6" s="11" t="n">
+        <v>-152920</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>9777</v>
+        <v>3463</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>9777</v>
+        <v>3463</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-11732</v>
+        <v>50112</v>
       </c>
     </row>
     <row r="8">
@@ -1067,7 +1067,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-3504</v>
+      <c r="S8" s="11" t="n">
+        <v>-291</v>
       </c>
     </row>
     <row r="9">
@@ -1089,27 +1089,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>682063</v>
+        <v>-354938</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>704740</v>
-      </c>
-      <c r="F9" s="13" t="inlineStr">
+        <v>-193314</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="14" t="n">
-        <v>-22677</v>
+      <c r="G9" s="11" t="n">
+        <v>-161624</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,26 +1117,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>111337</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>272961</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>295638</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>95601</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>132579</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>194372</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>0</v>
+      <c r="S9" s="14" t="n">
+        <v>871</v>
       </c>
     </row>
     <row r="10">
@@ -1156,29 +1156,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="C10" s="14" t="n">
+        <v>881</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>0</v>
+      <c r="G10" s="14" t="n">
+        <v>871</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,20 +1186,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
-        <v>7270</v>
+        <v>8141</v>
       </c>
       <c r="K10" s="12" t="n">
         <v>7270</v>
       </c>
       <c r="L10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="M10" s="12" t="n">
         <v>7310</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>7250</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7290</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1207,7 +1207,7 @@
       </c>
       <c r="Q10" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>-3104</v>
+        <v>150</v>
       </c>
     </row>
     <row r="11">
@@ -1225,67 +1225,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
-        <v>98716</v>
+      <c r="C11" s="14" t="n">
+        <v>3255</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>180641</v>
+        <v>-76538</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>79793</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-233793</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-313586</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-231661</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-228525</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-276645</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-81925</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-313586</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-231661</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-228525</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-276645</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-288841</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-10898</v>
+      <c r="S11" s="11" t="n">
+        <v>-11632</v>
       </c>
     </row>
     <row r="12">
@@ -1296,27 +1296,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>281627</v>
+        <v>-60262</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>177026</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
+        <v>-141222</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>104601</v>
+      <c r="G12" s="14" t="n">
+        <v>80960</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,20 +1324,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>114315</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>33355</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-71246</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>125614</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>136817</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>87180</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1345,7 +1345,7 @@
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1354,7 +1354,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-3331</v>
+        <v>5405</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1365,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1062406</v>
+        <v>-411064</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1062407</v>
+        <v>-411064</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="Q13" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-122</v>
+        <v>257</v>
       </c>
     </row>
     <row r="14">
@@ -1459,7 +1459,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1469,8 +1469,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-15649</v>
+      <c r="S14" s="11" t="n">
+        <v>-2306</v>
       </c>
     </row>
     <row r="15">
@@ -1479,29 +1479,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>326449</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
+      <c r="C15" s="11" t="n">
+        <v>551714</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
-        <v>341868</v>
+      <c r="E15" s="14" t="n">
+        <v>529557</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-15419</v>
+        <v>22157</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,20 +1509,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-690662</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-712819</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-697400</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-660766</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-607692</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-485562</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1530,7 +1530,7 @@
       </c>
       <c r="Q15" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1539,7 +1539,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-81925</v>
+        <v>79793</v>
       </c>
     </row>
     <row r="16">
@@ -1550,65 +1550,65 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>-3104</v>
+        <v>50</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E16" s="11" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>150</v>
+      </c>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="n">
+        <v>44254</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>44104</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>47208</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>46308</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>50603</v>
+      </c>
+      <c r="P16" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>-3104</v>
-      </c>
-      <c r="I16" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J16" s="12" t="n">
-        <v>44104</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>47208</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>46308</v>
-      </c>
-      <c r="M16" s="12" t="n">
-        <v>50603</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>50751</v>
-      </c>
-      <c r="P16" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R16" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-39456</v>
+      <c r="S16" s="14" t="n">
+        <v>-92708</v>
       </c>
     </row>
     <row r="17">
@@ -1617,29 +1617,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>79831</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
+      <c r="C17" s="11" t="n">
+        <v>43384</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
-        <v>119287</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="E17" s="14" t="n">
+        <v>136092</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-39456</v>
+      <c r="G17" s="14" t="n">
+        <v>-92708</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,26 +1647,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>478916</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>571624</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>611080</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>502455</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>497176</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>474116</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="9" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1676,8 +1676,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>11774</v>
+      <c r="S17" s="14" t="n">
+        <v>49161</v>
       </c>
     </row>
     <row r="18">
@@ -1686,29 +1686,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>128922</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C18" s="11" t="n">
+        <v>300905</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n">
-        <v>70945</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="E18" s="14" t="n">
+        <v>230503</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>57977</v>
+      <c r="G18" s="11" t="n">
+        <v>70402</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1716,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>167492</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>97090</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>39113</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>112002</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>59914</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>-39305</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-15474</v>
+        <v>1698</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>532098</v>
+        <v>896053</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>532100</v>
+        <v>896052</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1784,7 +1784,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>457</v>
+        <v>-2411</v>
       </c>
     </row>
     <row r="20">
@@ -1851,7 +1851,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>7541</v>
+      <c r="S20" s="14" t="n">
+        <v>14700</v>
       </c>
     </row>
     <row r="21">
@@ -1873,65 +1873,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>22808</v>
+        <v>-32867</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>14236</v>
+        <v>-20913</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-11954</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3059735</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3071689</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3063117</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3031612</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3013151</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>8572</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3071689</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3063117</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3031612</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3013151</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>2997216</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>104601</v>
+      <c r="S21" s="14" t="n">
+        <v>80960</v>
       </c>
     </row>
     <row r="22">
@@ -1940,29 +1940,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="9" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="11" t="n">
-        <v>6362</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="C22" s="14" t="n">
+        <v>6014</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>17260</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="11" t="n">
+        <v>17646</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-10898</v>
+      <c r="G22" s="11" t="n">
+        <v>-11632</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,26 +1970,26 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4116362</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4104730</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4093832</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4095305</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4073020</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4070339</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1999,8 +1999,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>57977</v>
+      <c r="S22" s="11" t="n">
+        <v>70402</v>
       </c>
     </row>
     <row r="23">
@@ -2009,29 +2009,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>25981</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>49739</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>14207</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="E23" s="11" t="n">
+        <v>578</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>11774</v>
+      <c r="G23" s="14" t="n">
+        <v>49161</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,26 +2039,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>666298</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>617137</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>605363</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>627976</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>624269</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>628431</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
+      <c r="Q23" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2068,8 +2068,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-9448</v>
+      <c r="S23" s="11" t="n">
+        <v>-25575</v>
       </c>
     </row>
     <row r="24">
@@ -2080,27 +2080,27 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>35964</v>
+        <v>-84852</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>45412</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+        <v>-59277</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-9448</v>
+      <c r="G24" s="11" t="n">
+        <v>-25575</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,26 +2108,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>390329</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>415904</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>425352</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>435717</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>435600</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>444692</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2137,8 +2137,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>39041</v>
+      <c r="S24" s="14" t="n">
+        <v>145817</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>91115</v>
+        <v>-61966</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>91115</v>
+        <v>-61966</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2176,7 +2176,7 @@
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="S25" s="14" t="n">
-        <v>11397</v>
+        <v>-47958</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2245,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>-45087</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>-185555</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>-24851</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>-32635</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>-20236</v>
+      <c r="G27" s="11" t="n">
+        <v>-152920</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1174358</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1327278</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1347514</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1311204</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1291940</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1249843</v>
       </c>
     </row>
     <row r="28">
@@ -2296,29 +2296,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n">
-        <v>0</v>
+      <c r="C28" s="14" t="n">
+        <v>25</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>3331</v>
+        <v>-5380</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-3331</v>
+        <v>5405</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-358431</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-363836</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-360505</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-349370</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-351266</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-320161</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,29 +2355,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>-13362</v>
+      <c r="C29" s="11" t="n">
+        <v>-19248</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>2112</v>
+        <v>-20946</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-15474</v>
+        <v>1698</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-236847</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-238545</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-223071</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-207681</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-199042</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-192835</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 19-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 20-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,29 +2414,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>14855</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>57859</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>-24186</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>-87958</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>39041</v>
+      <c r="G30" s="14" t="n">
+        <v>145817</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-579080</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-724897</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-763938</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-754153</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-741632</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-736847</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24152.05</v>
+        <v>24225.45</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24172.85</v>
+        <v>24265.15</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-43594</v>
+        <v>-146919</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-43594</v>
+        <v>-146919</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24025.65</v>
+        <v>24184.55</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24078.3</v>
+        <v>24231.85</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24306.08333333333</v>
+        <v>24350.41666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24085.28333333333</v>
+        <v>24229.51666666666</v>
       </c>
     </row>
     <row r="33">
@@ -2595,27 +2595,27 @@
       </c>
       <c r="B33" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C33" s="11" t="n">
-        <v>-21420</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+        <v>11312</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>-9688</v>
+      <c r="E33" s="11" t="n">
+        <v>-38800</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-11732</v>
+        <v>50112</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-327110</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-377222</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-365490</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-337369</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-323986</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-312483</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24239.46666666666</v>
+        <v>24307.78333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24092.26666666667</v>
+        <v>24227.18333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2660,29 +2660,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>455</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="11" t="n">
+        <v>436</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>577</v>
+      <c r="E34" s="14" t="n">
+        <v>179</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-122</v>
+        <v>257</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>20739</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20482</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>20604</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>20674</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>21082</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>21686</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24158.88333333333</v>
+        <v>24269.81666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24099.25</v>
+        <v>24224.85</v>
       </c>
     </row>
     <row r="35">
@@ -2727,29 +2727,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>-11060</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>-16084</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>-11517</v>
+      <c r="E35" s="11" t="n">
+        <v>-13673</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>457</v>
+        <v>-2411</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>166400</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>168811</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>168354</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>167432</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>167290</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>167213</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24092.26666666667</v>
+        <v>24227.18333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2790,27 +2790,27 @@
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>17992</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+        <v>-18902</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>6595</v>
+      <c r="E36" s="14" t="n">
+        <v>29056</v>
       </c>
       <c r="F36" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>11397</v>
+        <v>-47958</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>139971</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>187929</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>176532</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>149263</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>135614</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>123584</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24011.68333333333</v>
+        <v>24189.21666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-14033</v>
+        <v>-23238</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-14033</v>
+        <v>-23238</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23945.06666666667</v>
+        <v>24146.58333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23864.48333333334</v>
+        <v>24108.61666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>10.76</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.32</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.33</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.31</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.42</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,078    PCR(OI) 0.70    Max Pain 24,200</t>
+          <t>Spot 24,232    PCR(OI) 1.10    Max Pain 24,250</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3010,16 +3010,16 @@
     </row>
     <row r="45">
       <c r="P45" s="27" t="n">
-        <v>24500</v>
+        <v>24300</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>228681</v>
+        <v>150552</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>42774</v>
+        <v>-28055</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>951238</v>
+        <v>1907612</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
@@ -3029,35 +3029,35 @@
     </row>
     <row r="46">
       <c r="P46" s="27" t="n">
-        <v>25000</v>
+        <v>24500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>224540</v>
+        <v>192533</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>11042</v>
+        <v>-36148</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>791116</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1340280</v>
+      </c>
+      <c r="T46" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="P47" s="27" t="n">
-        <v>25500</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>180366</v>
+        <v>183448</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>35647</v>
+        <v>-41092</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>443967</v>
+        <v>986702</v>
       </c>
       <c r="T47" s="29" t="inlineStr">
         <is>
@@ -3105,16 +3105,16 @@
     </row>
     <row r="50">
       <c r="P50" s="31" t="n">
-        <v>24000</v>
+        <v>24200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>210294</v>
-      </c>
-      <c r="R50" s="11" t="n">
-        <v>34745</v>
+        <v>204446</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>106433</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>2509725</v>
+        <v>3030619</v>
       </c>
       <c r="T50" s="32" t="inlineStr">
         <is>
@@ -3124,20 +3124,20 @@
     </row>
     <row r="51">
       <c r="P51" s="31" t="n">
-        <v>23500</v>
+        <v>24000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>129792</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>26812</v>
+        <v>251506</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>41212</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>460825</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>1144062</v>
+      </c>
+      <c r="T51" s="28" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3146,13 +3146,13 @@
         <v>23000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>155396</v>
+        <v>154798</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>19446</v>
+        <v>-598</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>345854</v>
+        <v>547607</v>
       </c>
       <c r="T52" s="29" t="inlineStr">
         <is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 19-Aug-2026    1 DAY AGO = 18-Aug-2026    2 DAYS AGO = 17-Aug-2026    3 DAYS AGO = 14-Aug-2026    4 DAYS AGO = 13-Aug-2026    (generated 19-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 20-Aug-2026    1 DAY AGO = 19-Aug-2026    2 DAYS AGO = 18-Aug-2026    3 DAYS AGO = 17-Aug-2026    4 DAYS AGO = 14-Aug-2026    (generated 20-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-21
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -183,6 +183,9 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -194,9 +197,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-12103</v>
+        <v>-2289</v>
       </c>
     </row>
     <row r="3">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-7241</v>
+        <v>-1979</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>4862</v>
+        <v>310</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-12103</v>
+        <v>-2289</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,20 +725,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>171016</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>173305</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>185408</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>173796</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>160591</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>155682</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-161624</v>
+        <v>-46473</v>
       </c>
     </row>
     <row r="4">
@@ -764,13 +764,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>-307</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>793</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -778,53 +778,53 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>-16</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+        <v>-44</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>837</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>28115</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>27278</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>27569</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>31073</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>31039</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-291</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>27278</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>27569</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>31073</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>31039</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>30790</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>22157</v>
+      <c r="S4" s="14" t="n">
+        <v>-6874</v>
       </c>
     </row>
     <row r="5">
@@ -833,29 +833,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>-535</v>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>1771</v>
-      </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>-2306</v>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>1725</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>-533</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>2258</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -863,28 +863,28 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-209855</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-212113</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-209807</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-194158</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-181587</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-176698</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -892,8 +892,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>-11954</v>
+      <c r="S5" s="14" t="n">
+        <v>16452</v>
       </c>
     </row>
     <row r="6">
@@ -908,23 +908,23 @@
         </is>
       </c>
       <c r="C6" s="14" t="n">
-        <v>11546</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>-3154</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>14700</v>
+        <v>716</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>1522</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>-806</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -932,20 +932,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>10724</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>11530</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>-3170</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>-10711</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-10043</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-9774</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-152920</v>
+        <v>-76605</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +973,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>3463</v>
+        <v>1255</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>3463</v>
+        <v>1255</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>50112</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="8">
@@ -1067,9 +1067,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1077,8 +1077,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>-291</v>
+      <c r="S8" s="14" t="n">
+        <v>837</v>
       </c>
     </row>
     <row r="9">
@@ -1087,21 +1087,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>-354938</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>-193314</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>203886</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>250359</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>-161624</v>
+        <v>-46473</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1117,28 +1117,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>64864</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>111337</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>272961</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>295638</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>95601</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>132579</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1146,8 +1146,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>871</v>
+      <c r="S9" s="11" t="n">
+        <v>-50</v>
       </c>
     </row>
     <row r="10">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="C10" s="14" t="n">
-        <v>881</v>
+        <v>0</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
@@ -1170,15 +1170,15 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="14" t="n">
-        <v>871</v>
+        <v>50</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>-50</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,20 +1186,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>8091</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>8141</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>7270</v>
       </c>
       <c r="L10" s="12" t="n">
         <v>7270</v>
       </c>
       <c r="M10" s="12" t="n">
+        <v>7270</v>
+      </c>
+      <c r="N10" s="12" t="n">
         <v>7310</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7250</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1216,7 +1216,7 @@
         </is>
       </c>
       <c r="S10" s="11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1231,15 +1231,15 @@
         </is>
       </c>
       <c r="C11" s="14" t="n">
-        <v>3255</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>-76538</v>
+        <v>50940</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>35260</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1247,7 +1247,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>79793</v>
+        <v>15680</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,20 +1255,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-218113</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-233793</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-313586</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-231661</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-228525</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-276645</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1285,7 +1285,7 @@
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>-11632</v>
+        <v>-2617</v>
       </c>
     </row>
     <row r="12">
@@ -1294,21 +1294,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>-60262</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>-141222</v>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>145739</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>114896</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
@@ -1316,7 +1316,7 @@
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>80960</v>
+        <v>30843</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,28 +1324,28 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>145158</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>114315</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>33355</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>-71246</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>125614</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>136817</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q12" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1353,8 +1353,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>5405</v>
+      <c r="S12" s="11" t="n">
+        <v>-2534</v>
       </c>
     </row>
     <row r="13">
@@ -1365,11 +1365,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-411064</v>
+        <v>400565</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-411064</v>
+        <v>400565</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1401,7 +1401,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>257</v>
+        <v>1298</v>
       </c>
     </row>
     <row r="14">
@@ -1459,9 +1459,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q14" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1469,8 +1469,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="11" t="n">
-        <v>-2306</v>
+      <c r="S14" s="14" t="n">
+        <v>2258</v>
       </c>
     </row>
     <row r="15">
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>551714</v>
+        <v>277151</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1493,53 +1493,53 @@
         </is>
       </c>
       <c r="E15" s="14" t="n">
-        <v>529557</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+        <v>284025</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>-6874</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-697536</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-690662</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-712819</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-697400</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-660766</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>22157</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-690662</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-712819</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-697400</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-660766</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-607692</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>79793</v>
+        <v>15680</v>
       </c>
     </row>
     <row r="16">
@@ -1554,15 +1554,15 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="n">
-        <v>-100</v>
+        <v>0</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>0</v>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         </is>
       </c>
       <c r="G16" s="11" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1581,17 +1581,17 @@
         <v>44254</v>
       </c>
       <c r="K16" s="12" t="n">
+        <v>44254</v>
+      </c>
+      <c r="L16" s="12" t="n">
         <v>44104</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>47208</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>46308</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>50603</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1608,7 +1608,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-92708</v>
+        <v>-10969</v>
       </c>
     </row>
     <row r="17">
@@ -1623,7 +1623,7 @@
         </is>
       </c>
       <c r="C17" s="11" t="n">
-        <v>43384</v>
+        <v>37997</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1631,7 +1631,7 @@
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>136092</v>
+        <v>48966</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
@@ -1639,7 +1639,7 @@
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-92708</v>
+        <v>-10969</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,20 +1647,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>467947</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>478916</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>571624</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>611080</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>502455</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>497176</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1677,7 +1677,7 @@
         </is>
       </c>
       <c r="S17" s="14" t="n">
-        <v>49161</v>
+        <v>15461</v>
       </c>
     </row>
     <row r="18">
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>300905</v>
+        <v>127834</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>230503</v>
+        <v>109991</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>70402</v>
+        <v>17843</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1716,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>185335</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>167492</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>97090</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>39113</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>112002</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>59914</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1746,7 +1746,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>1698</v>
+        <v>2278</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1757,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>896053</v>
+        <v>442982</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>896052</v>
+        <v>442982</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>-2411</v>
+        <v>-6385</v>
       </c>
     </row>
     <row r="20">
@@ -1851,9 +1851,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1861,8 +1861,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>14700</v>
+      <c r="S20" s="11" t="n">
+        <v>-806</v>
       </c>
     </row>
     <row r="21">
@@ -1871,29 +1871,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>-32867</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>-20913</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>-11954</v>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>21032</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>4580</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>16452</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1901,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3076187</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3059735</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3071689</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3063117</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3031612</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3013151</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>80960</v>
+        <v>30843</v>
       </c>
     </row>
     <row r="22">
@@ -1946,7 +1946,7 @@
         </is>
       </c>
       <c r="C22" s="14" t="n">
-        <v>6014</v>
+        <v>15572</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="E22" s="11" t="n">
-        <v>17646</v>
+        <v>18189</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-11632</v>
+        <v>-2617</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,20 +1970,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4118979</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4116362</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4104730</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4093832</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4095305</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4073020</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2000,7 +2000,7 @@
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>70402</v>
+        <v>17843</v>
       </c>
     </row>
     <row r="23">
@@ -2015,7 +2015,7 @@
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>49739</v>
+        <v>24783</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>578</v>
+        <v>9322</v>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
@@ -2031,7 +2031,7 @@
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>49161</v>
+        <v>15461</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,20 +2039,20 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>681759</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>666298</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>617137</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>605363</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>627976</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>624269</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>-25575</v>
+        <v>-29296</v>
       </c>
     </row>
     <row r="24">
@@ -2084,7 +2084,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-84852</v>
+        <v>-33630</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>-59277</v>
+        <v>-4334</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>-25575</v>
+        <v>-29296</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,20 +2108,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>361033</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>390329</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>415904</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>425352</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>435717</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>435600</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2138,7 +2138,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>145817</v>
+        <v>76861</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2149,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-61966</v>
+        <v>27757</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-61966</v>
+        <v>27757</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2174,9 +2174,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2184,8 +2184,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>-47958</v>
+      <c r="S25" s="11" t="n">
+        <v>2529</v>
       </c>
     </row>
     <row r="26">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-185555</v>
+        <v>-113043</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>-32635</v>
+        <v>-36438</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-152920</v>
+        <v>-76605</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2275,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>1097753</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1174358</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1327278</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1347514</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1311204</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1291940</v>
       </c>
     </row>
     <row r="28">
@@ -2296,29 +2296,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C28" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>-5380</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>5405</v>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n">
+        <v>-20</v>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n">
+        <v>2514</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n">
+        <v>-2534</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2326,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-360965</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-358431</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-363836</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-360505</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-349370</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-351266</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,7 +2361,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>-19248</v>
+        <v>-5939</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2369,7 +2369,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>-20946</v>
+        <v>-8217</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2377,7 +2377,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>1698</v>
+        <v>2278</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2385,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-234569</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-236847</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-238545</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-223071</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-207681</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-199042</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 20-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 21-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,13 +2414,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C30" s="14" t="n">
-        <v>57859</v>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n">
+        <v>-22635</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>-87958</v>
+        <v>-99496</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2436,7 +2436,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>145817</v>
+        <v>76861</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2444,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-502219</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-579080</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-724897</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-763938</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-754153</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-741632</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24225.45</v>
+        <v>24284.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2472,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24265.15</v>
+        <v>24284.05</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-146919</v>
+        <v>-141637</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-146919</v>
+        <v>-141637</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2509,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24184.55</v>
+        <v>24206.8</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2517,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24231.85</v>
+        <v>24252</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2576,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24350.41666666666</v>
+        <v>24365.68333333334</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24229.51666666666</v>
+        <v>24249.80833333334</v>
       </c>
     </row>
     <row r="33">
@@ -2593,13 +2593,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="11" t="n">
-        <v>11312</v>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="n">
+        <v>-10569</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-38800</v>
+        <v>-13127</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2615,7 +2615,7 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>50112</v>
+        <v>2558</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2623,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-324552</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-327110</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-377222</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-365490</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-337369</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-323986</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24307.78333333333</v>
+        <v>24324.86666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24227.18333333333</v>
+        <v>24247.61666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,15 +2666,15 @@
         </is>
       </c>
       <c r="C34" s="11" t="n">
-        <v>436</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E34" s="14" t="n">
-        <v>179</v>
+        <v>293</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="n">
+        <v>-1005</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2682,7 +2682,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>257</v>
+        <v>1298</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2690,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>22037</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>20739</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>20482</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>20604</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>20674</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>21082</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24269.81666666666</v>
+        <v>24288.43333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2718,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24224.85</v>
+        <v>24245.425</v>
       </c>
     </row>
     <row r="35">
@@ -2733,7 +2733,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>-16084</v>
+        <v>-7070</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2741,7 +2741,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>-13673</v>
+        <v>-685</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2749,7 +2749,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>-2411</v>
+        <v>-6385</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2757,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>160015</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>166400</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>168811</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>168354</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>167432</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>167290</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24227.18333333333</v>
+        <v>24247.61666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2794,23 +2794,23 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>-18902</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E36" s="14" t="n">
-        <v>29056</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>-47958</v>
+        <v>-9805</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="n">
+        <v>-12334</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>2529</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2818,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>142500</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>139971</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>187929</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>176532</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>149263</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>135614</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24189.21666666666</v>
+        <v>24211.18333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2851,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-23238</v>
+        <v>-27151</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-23238</v>
+        <v>-27151</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2877,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24146.58333333333</v>
+        <v>24170.36666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24108.61666666666</v>
+        <v>24133.93333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,19 +2933,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>10.76</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.32</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.33</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.31</v>
       </c>
     </row>
     <row r="41">
@@ -2962,7 +2962,7 @@
     <row r="42">
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,232    PCR(OI) 1.10    Max Pain 24,250</t>
+          <t>Spot 24,252    PCR(OI) 1.08    Max Pain 24,250</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3013,17 +3013,17 @@
         <v>24300</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>150552</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>-28055</v>
+        <v>207228</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>56676</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>1907612</v>
+        <v>4041618</v>
       </c>
       <c r="T45" s="28" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3032,15 +3032,15 @@
         <v>24500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>192533</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>-36148</v>
+        <v>200444</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>7911</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1340280</v>
-      </c>
-      <c r="T46" s="28" t="inlineStr">
+        <v>1663955</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3051,22 +3051,22 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>183448</v>
+        <v>180772</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-41092</v>
+        <v>-2676</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>986702</v>
-      </c>
-      <c r="T47" s="29" t="inlineStr">
+        <v>519167</v>
+      </c>
+      <c r="T47" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="P48" s="30" t="inlineStr">
+      <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3104,57 +3104,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="31" t="n">
+      <c r="P50" s="32" t="n">
         <v>24200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>204446</v>
+        <v>231507</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>106433</v>
+        <v>27061</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>3030619</v>
-      </c>
-      <c r="T50" s="32" t="inlineStr">
+        <v>4481468</v>
+      </c>
+      <c r="T50" s="28" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="31" t="n">
+      <c r="P51" s="32" t="n">
         <v>24000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>251506</v>
+        <v>272916</v>
       </c>
       <c r="R51" s="14" t="n">
-        <v>41212</v>
+        <v>21410</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1144062</v>
-      </c>
-      <c r="T51" s="28" t="inlineStr">
+        <v>1612499</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="31" t="n">
+      <c r="P52" s="32" t="n">
         <v>23000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>154798</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>-598</v>
+        <v>177746</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>22948</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>547607</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
+        <v>432352</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3163,7 +3163,7 @@
     <row r="54">
       <c r="A54" s="33" t="inlineStr">
         <is>
-          <t>TODAY = 20-Aug-2026    1 DAY AGO = 19-Aug-2026    2 DAYS AGO = 18-Aug-2026    3 DAYS AGO = 17-Aug-2026    4 DAYS AGO = 14-Aug-2026    (generated 20-Aug-2026 20:30 IST)</t>
+          <t>TODAY = 21-Aug-2026    1 DAY AGO = 20-Aug-2026    2 DAYS AGO = 19-Aug-2026    3 DAYS AGO = 18-Aug-2026    4 DAYS AGO = 17-Aug-2026    (generated 21-Aug-2026 20:30 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-24
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -16,9 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="#,##,##0;-#,##,##0;0"/>
-    <numFmt numFmtId="165" formatCode="#,##,##0.00"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="#,##,##0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -36,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -108,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -153,25 +154,28 @@
     <xf numFmtId="164" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,13 +190,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -677,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -686,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-2289</v>
+        <v>10140</v>
       </c>
     </row>
     <row r="3">
@@ -697,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-1979</v>
+        <v>8017</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>310</v>
+        <v>-2123</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-2289</v>
+        <v>10140</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -725,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>181156</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>171016</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>173305</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>185408</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>173796</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>160591</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -746,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -755,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-46473</v>
+        <v>162148</v>
       </c>
     </row>
     <row r="4">
@@ -766,27 +770,27 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C4" s="14" t="n">
-        <v>793</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>-3122</v>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>-44</v>
+      <c r="E4" s="11" t="n">
+        <v>-27</v>
       </c>
       <c r="F4" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G4" s="14" t="n">
-        <v>837</v>
+        <v>-3095</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -794,26 +798,26 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>25020</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>28115</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>27278</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>27569</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>31073</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>31039</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="13" t="inlineStr">
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -823,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>-6874</v>
+      <c r="S4" s="11" t="n">
+        <v>-146453</v>
       </c>
     </row>
     <row r="5">
@@ -833,67 +837,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>1725</v>
+      <c r="C5" s="11" t="n">
+        <v>1019</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-533</v>
+        <v>10547</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>-9528</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-219383</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-209855</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-212113</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-209807</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-194158</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>2258</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-209855</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-212113</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-209807</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-194158</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-181587</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>16452</v>
+      <c r="S5" s="11" t="n">
+        <v>3988</v>
       </c>
     </row>
     <row r="6">
@@ -902,67 +906,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C6" s="14" t="n">
-        <v>716</v>
+      <c r="C6" s="11" t="n">
+        <v>1700</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1522</v>
+        <v>-783</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>2483</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>13207</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>10724</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>11530</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>-3170</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>-10711</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>-806</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>10724</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>11530</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>-3170</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>-10711</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>-10043</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="11" t="n">
-        <v>-76605</v>
+      <c r="S6" s="14" t="n">
+        <v>-102843</v>
       </c>
     </row>
     <row r="7">
@@ -973,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>1255</v>
+        <v>7614</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>1255</v>
+        <v>7614</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -998,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1008,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>2558</v>
+      <c r="S7" s="14" t="n">
+        <v>4097</v>
       </c>
     </row>
     <row r="8">
@@ -1069,7 +1073,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1078,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="14" t="n">
-        <v>837</v>
+        <v>-3095</v>
       </c>
     </row>
     <row r="9">
@@ -1087,67 +1091,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C9" s="14" t="n">
-        <v>203886</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="C9" s="11" t="n">
+        <v>948571</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
-        <v>250359</v>
+      <c r="E9" s="14" t="n">
+        <v>786423</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>162148</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="n">
+        <v>227012</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>64864</v>
+      </c>
+      <c r="L9" s="12" t="n">
+        <v>111337</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>272961</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>295638</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-46473</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>64864</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>111337</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>272961</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>295638</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>95601</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>-50</v>
+      <c r="S9" s="14" t="n">
+        <v>-82</v>
       </c>
     </row>
     <row r="10">
@@ -1156,29 +1160,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C10" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="C10" s="11" t="n">
+        <v>25</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>50</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="14" t="n">
+        <v>107</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-50</v>
+      <c r="G10" s="14" t="n">
+        <v>-82</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1186,26 +1190,26 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>8009</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>8091</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>8141</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>7270</v>
       </c>
       <c r="M10" s="12" t="n">
         <v>7270</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>7310</v>
+        <v>7270</v>
       </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1215,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>0</v>
+      <c r="S10" s="14" t="n">
+        <v>19298</v>
       </c>
     </row>
     <row r="11">
@@ -1225,29 +1229,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
-        <v>50940</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="C11" s="11" t="n">
+        <v>229305</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
-        <v>35260</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="E11" s="14" t="n">
+        <v>210872</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>15680</v>
+      <c r="G11" s="11" t="n">
+        <v>18433</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1255,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-199680</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-218113</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-233793</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-313586</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-231661</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-228525</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1276,7 +1280,7 @@
       </c>
       <c r="Q11" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1285,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="11" t="n">
-        <v>-2617</v>
+        <v>3144</v>
       </c>
     </row>
     <row r="12">
@@ -1294,29 +1298,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C12" s="14" t="n">
-        <v>145739</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="C12" s="11" t="n">
+        <v>184291</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>114896</v>
+      <c r="E12" s="14" t="n">
+        <v>364789</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>30843</v>
+        <v>-180498</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1324,26 +1328,26 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-35340</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>145158</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>114315</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>33355</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>-71246</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>125614</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="9" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1353,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="11" t="n">
-        <v>-2534</v>
+      <c r="S12" s="14" t="n">
+        <v>-6407</v>
       </c>
     </row>
     <row r="13">
@@ -1365,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>400565</v>
+        <v>1362192</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>400565</v>
+        <v>1362191</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1390,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1400,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>1298</v>
+      <c r="S13" s="14" t="n">
+        <v>4114</v>
       </c>
     </row>
     <row r="14">
@@ -1461,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1470,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>2258</v>
+        <v>-9528</v>
       </c>
     </row>
     <row r="15">
@@ -1481,27 +1485,27 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>277151</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
+        <v>-115225</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
-        <v>284025</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="E15" s="11" t="n">
+        <v>31228</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="14" t="n">
-        <v>-6874</v>
+      <c r="G15" s="11" t="n">
+        <v>-146453</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1509,26 +1513,26 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-843989</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-697536</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-690662</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-712819</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-697400</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-660766</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
+      <c r="Q15" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1538,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>15680</v>
+      <c r="S15" s="11" t="n">
+        <v>18433</v>
       </c>
     </row>
     <row r="16">
@@ -1548,29 +1552,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="C16" s="14" t="n">
+        <v>19318</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="E16" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="11" t="n">
-        <v>0</v>
+      <c r="G16" s="14" t="n">
+        <v>19298</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1578,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
-        <v>44254</v>
+        <v>63552</v>
       </c>
       <c r="K16" s="12" t="n">
         <v>44254</v>
       </c>
       <c r="L16" s="12" t="n">
+        <v>44254</v>
+      </c>
+      <c r="M16" s="12" t="n">
         <v>44104</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>47208</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>46308</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1599,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1608,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>-10969</v>
+        <v>114011</v>
       </c>
     </row>
     <row r="17">
@@ -1617,29 +1621,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n">
-        <v>37997</v>
+      <c r="C17" s="14" t="n">
+        <v>58690</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
-        <v>48966</v>
+        <v>-55321</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>-10969</v>
+        <v>114011</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1647,26 +1651,26 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>581958</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>467947</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>478916</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>571624</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>611080</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>502455</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="13" t="inlineStr">
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1676,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>15461</v>
+      <c r="S17" s="11" t="n">
+        <v>2057</v>
       </c>
     </row>
     <row r="18">
@@ -1688,27 +1692,27 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C18" s="11" t="n">
-        <v>127834</v>
+        <v>-96847</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E18" s="14" t="n">
-        <v>109991</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>-109992</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>17843</v>
+      <c r="G18" s="14" t="n">
+        <v>13145</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1716,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>198480</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>185335</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>167492</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>97090</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>39113</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>112002</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1737,7 +1741,7 @@
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R18" s="10" t="inlineStr">
@@ -1746,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>2278</v>
+        <v>-3008</v>
       </c>
     </row>
     <row r="19">
@@ -1757,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>442982</v>
+        <v>-134064</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>442982</v>
+        <v>-134065</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1782,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1792,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>-6385</v>
+      <c r="S19" s="11" t="n">
+        <v>-7716</v>
       </c>
     </row>
     <row r="20">
@@ -1853,7 +1857,7 @@
       </c>
       <c r="Q20" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1862,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>-806</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="21">
@@ -1873,27 +1877,27 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C21" s="14" t="n">
-        <v>21032</v>
+        <v>-9976</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>4580</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+        <v>-13964</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>16452</v>
+      <c r="G21" s="11" t="n">
+        <v>3988</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1901,20 +1905,20 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3080175</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3076187</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3059735</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3071689</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3063117</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3031612</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1922,7 +1926,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1931,7 +1935,7 @@
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>30843</v>
+        <v>-180498</v>
       </c>
     </row>
     <row r="22">
@@ -1940,29 +1944,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C22" s="14" t="n">
-        <v>15572</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
+      <c r="C22" s="11" t="n">
+        <v>15210</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="11" t="n">
-        <v>18189</v>
+      <c r="E22" s="14" t="n">
+        <v>12066</v>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G22" s="11" t="n">
-        <v>-2617</v>
+        <v>3144</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1970,26 +1974,26 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4115835</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4118979</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4116362</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4104730</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4093832</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4095305</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1999,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>17843</v>
+      <c r="S22" s="14" t="n">
+        <v>13145</v>
       </c>
     </row>
     <row r="23">
@@ -2011,27 +2015,27 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C23" s="14" t="n">
-        <v>24783</v>
+        <v>-26682</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>9322</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
+        <v>-28739</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>15461</v>
+      <c r="G23" s="11" t="n">
+        <v>2057</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2039,26 +2043,26 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>683816</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>681759</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>666298</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>617137</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>605363</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>627976</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2068,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>-29296</v>
+      <c r="S23" s="14" t="n">
+        <v>-9189</v>
       </c>
     </row>
     <row r="24">
@@ -2078,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="11" t="n">
-        <v>-33630</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="C24" s="14" t="n">
+        <v>-30748</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>-4334</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
+      <c r="E24" s="11" t="n">
+        <v>-21559</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="11" t="n">
-        <v>-29296</v>
+      <c r="G24" s="14" t="n">
+        <v>-9189</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2108,26 +2112,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>351844</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>361033</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>390329</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>415904</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>425352</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>435717</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
+      <c r="Q24" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2137,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>76861</v>
+      <c r="S24" s="11" t="n">
+        <v>112258</v>
       </c>
     </row>
     <row r="25">
@@ -2149,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>27757</v>
+        <v>-52196</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>27757</v>
+        <v>-52196</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2176,7 +2180,7 @@
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2185,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>2529</v>
+        <v>-495</v>
       </c>
     </row>
     <row r="26">
@@ -2245,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n">
-        <v>-113043</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+      <c r="C27" s="14" t="n">
+        <v>-176909</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>-36438</v>
-      </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="E27" s="11" t="n">
+        <v>-74066</v>
+      </c>
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="11" t="n">
-        <v>-76605</v>
+      <c r="G27" s="14" t="n">
+        <v>-102843</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2275,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>994910</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>1097753</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1174358</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1327278</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1347514</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1311204</v>
       </c>
     </row>
     <row r="28">
@@ -2298,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-20</v>
-      </c>
-      <c r="D28" s="9" t="inlineStr">
+        <v>3264</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n">
-        <v>2514</v>
-      </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>9671</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n">
-        <v>-2534</v>
+      <c r="G28" s="14" t="n">
+        <v>-6407</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2326,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-367372</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-360965</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-358431</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-363836</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-360505</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-349370</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2355,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n">
-        <v>-5939</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="C29" s="14" t="n">
+        <v>-20759</v>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>-8217</v>
+      <c r="E29" s="11" t="n">
+        <v>-17751</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>2278</v>
+        <v>-3008</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2385,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-237577</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-234569</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-236847</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-238545</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-223071</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-207681</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 21-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 24-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2414,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n">
-        <v>-22635</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+      <c r="C30" s="14" t="n">
+        <v>-2713</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>-99496</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
+      <c r="E30" s="11" t="n">
+        <v>-114971</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="14" t="n">
-        <v>76861</v>
+      <c r="G30" s="11" t="n">
+        <v>112258</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2444,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-389961</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-502219</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-579080</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-724897</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-763938</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-754153</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24284.05</v>
+        <v>24285.05</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2472,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24284.05</v>
+        <v>24313</v>
       </c>
     </row>
     <row r="31">
@@ -2483,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-141637</v>
+        <v>-197117</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-141637</v>
+        <v>-197117</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2509,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24206.8</v>
+        <v>24144.3</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2517,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24252</v>
+        <v>24219.05</v>
       </c>
     </row>
     <row r="32">
@@ -2576,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24365.68333333334</v>
+        <v>24475.3</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2584,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24249.80833333334</v>
+        <v>24222.25</v>
       </c>
     </row>
     <row r="33">
@@ -2593,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>-10569</v>
-      </c>
-      <c r="D33" s="9" t="inlineStr">
+      <c r="C33" s="11" t="n">
+        <v>-43530</v>
+      </c>
+      <c r="D33" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="11" t="n">
-        <v>-13127</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="E33" s="14" t="n">
+        <v>-47627</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="11" t="n">
-        <v>2558</v>
+      <c r="G33" s="14" t="n">
+        <v>4097</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2623,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-320455</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-324552</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-327110</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-377222</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-365490</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-337369</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24324.86666666667</v>
+        <v>24394.15</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2651,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24247.61666666667</v>
+        <v>24225.45</v>
       </c>
     </row>
     <row r="34">
@@ -2660,29 +2664,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="11" t="n">
-        <v>293</v>
-      </c>
-      <c r="D34" s="9" t="inlineStr">
+      <c r="C34" s="14" t="n">
+        <v>656</v>
+      </c>
+      <c r="D34" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E34" s="11" t="n">
-        <v>-1005</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="E34" s="14" t="n">
+        <v>-3458</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G34" s="11" t="n">
-        <v>1298</v>
+      <c r="G34" s="14" t="n">
+        <v>4114</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2690,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>26151</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>22037</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>20739</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>20482</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>20604</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>20674</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24288.43333333334</v>
+        <v>24306.6</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2718,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24245.425</v>
+        <v>24228.65</v>
       </c>
     </row>
     <row r="35">
@@ -2727,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>-7070</v>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="11" t="n">
+        <v>-25541</v>
+      </c>
+      <c r="D35" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n">
-        <v>-685</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+      <c r="E35" s="14" t="n">
+        <v>-17825</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>-6385</v>
+      <c r="G35" s="11" t="n">
+        <v>-7716</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2757,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>152299</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>160015</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>166400</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>168811</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>168354</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>167432</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24247.61666666667</v>
+        <v>24225.45</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2788,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>-9805</v>
-      </c>
-      <c r="D36" s="9" t="inlineStr">
+      <c r="C36" s="11" t="n">
+        <v>-22084</v>
+      </c>
+      <c r="D36" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E36" s="11" t="n">
-        <v>-12334</v>
+      <c r="E36" s="14" t="n">
+        <v>-21589</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>2529</v>
+        <v>-495</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2818,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>142005</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>142500</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>139971</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>187929</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>176532</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>149263</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24211.18333333334</v>
+        <v>24137.9</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2851,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-27151</v>
+        <v>-90499</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-27151</v>
+        <v>-90499</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2877,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24170.36666666667</v>
+        <v>24056.75</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2889,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>24133.93333333334</v>
+        <v>23969.2</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2933,22 +2937,52 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.53</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.2</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>10.76</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.32</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.39</v>
       </c>
-      <c r="N40" s="24" t="n">
-        <v>11.33</v>
-      </c>
     </row>
     <row r="41">
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>Nifty Daily SRT</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>TODAY</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>1 DAY AGO</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>2 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr">
+        <is>
+          <t>3 DAYS AGO</t>
+        </is>
+      </c>
+      <c r="N41" s="3" t="inlineStr">
+        <is>
+          <t>4 DAYS AGO</t>
+        </is>
+      </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
           <t>Nifty Option-Chain S/R   -   Weekly expiry 25-Aug-2026</t>
@@ -2960,9 +2994,29 @@
       <c r="T41" s="2" t="n"/>
     </row>
     <row r="42">
+      <c r="I42" s="7" t="inlineStr">
+        <is>
+          <t>SRT</t>
+        </is>
+      </c>
+      <c r="J42" s="25" t="n">
+        <v>1.009644797702047</v>
+      </c>
+      <c r="K42" s="25" t="n">
+        <v>1.01059871674965</v>
+      </c>
+      <c r="L42" s="25" t="n">
+        <v>1.00922747639189</v>
+      </c>
+      <c r="M42" s="25" t="n">
+        <v>1.002329484832365</v>
+      </c>
+      <c r="N42" s="25" t="n">
+        <v>1.004976874300015</v>
+      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,252    PCR(OI) 1.08    Max Pain 24,250</t>
+          <t>Spot 24,219    PCR(OI) 0.69    Max Pain 24,200</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -2971,7 +3025,27 @@
       <c r="T42" s="6" t="n"/>
     </row>
     <row r="43">
-      <c r="P43" s="25" t="inlineStr">
+      <c r="I43" s="7" t="inlineStr">
+        <is>
+          <t>124-day SMA</t>
+        </is>
+      </c>
+      <c r="J43" s="18" t="n">
+        <v>23987.6935483871</v>
+      </c>
+      <c r="K43" s="18" t="n">
+        <v>23997.65564516129</v>
+      </c>
+      <c r="L43" s="18" t="n">
+        <v>24010.29556451613</v>
+      </c>
+      <c r="M43" s="18" t="n">
+        <v>24022.34032258065</v>
+      </c>
+      <c r="N43" s="18" t="n">
+        <v>24035.27943548387</v>
+      </c>
+      <c r="P43" s="26" t="inlineStr">
         <is>
           <t>RESISTANCE   -   Call OI walls (higher = stronger cap)</t>
         </is>
@@ -2982,82 +3056,172 @@
       <c r="T43" s="6" t="n"/>
     </row>
     <row r="44">
-      <c r="P44" s="26" t="inlineStr">
+      <c r="I44" s="7" t="inlineStr">
+        <is>
+          <t>Nifty Close</t>
+        </is>
+      </c>
+      <c r="J44" s="18" t="n">
+        <v>24219.05</v>
+      </c>
+      <c r="K44" s="18" t="n">
+        <v>24252</v>
+      </c>
+      <c r="L44" s="18" t="n">
+        <v>24231.85</v>
+      </c>
+      <c r="M44" s="18" t="n">
+        <v>24078.3</v>
+      </c>
+      <c r="N44" s="18" t="n">
+        <v>24154.9</v>
+      </c>
+      <c r="P44" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="Q44" s="26" t="inlineStr">
+      <c r="Q44" s="27" t="inlineStr">
         <is>
           <t>Call OI</t>
         </is>
       </c>
-      <c r="R44" s="26" t="inlineStr">
+      <c r="R44" s="27" t="inlineStr">
         <is>
           <t>Chg OI</t>
         </is>
       </c>
-      <c r="S44" s="26" t="inlineStr">
+      <c r="S44" s="27" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="T44" s="26" t="inlineStr">
+      <c r="T44" s="27" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="P45" s="27" t="n">
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>Nifty Weekly SRT</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>THIS WEEK</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>1 WEEK AGO</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>2 WEEKS AGO</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr">
+        <is>
+          <t>3 WEEKS AGO</t>
+        </is>
+      </c>
+      <c r="N45" s="3" t="inlineStr">
+        <is>
+          <t>4 WEEKS AGO</t>
+        </is>
+      </c>
+      <c r="P45" s="28" t="n">
+        <v>24200</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>254530</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>118418</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>5973736</v>
+      </c>
+      <c r="T45" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="I46" s="7" t="inlineStr">
+        <is>
+          <t>SRT</t>
+        </is>
+      </c>
+      <c r="J46" s="25" t="n">
+        <v>0.9951481114124615</v>
+      </c>
+      <c r="K46" s="25" t="n">
+        <v>0.9970635633790684</v>
+      </c>
+      <c r="L46" s="25" t="n">
+        <v>1.002328084679025</v>
+      </c>
+      <c r="M46" s="25" t="n">
+        <v>1.011430829957649</v>
+      </c>
+      <c r="N46" s="25" t="n">
+        <v>1.004556069227693</v>
+      </c>
+      <c r="P46" s="28" t="n">
         <v>24300</v>
       </c>
-      <c r="Q45" s="12" t="n">
-        <v>207228</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>56676</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>4041618</v>
-      </c>
-      <c r="T45" s="28" t="inlineStr">
+      <c r="Q46" s="12" t="n">
+        <v>332664</v>
+      </c>
+      <c r="R46" s="11" t="n">
+        <v>125436</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>6936175</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="P46" s="27" t="n">
+    <row r="47">
+      <c r="I47" s="7" t="inlineStr">
+        <is>
+          <t>124-week SMA</t>
+        </is>
+      </c>
+      <c r="J47" s="18" t="n">
+        <v>24337.1310483871</v>
+      </c>
+      <c r="K47" s="18" t="n">
+        <v>24323.42419354839</v>
+      </c>
+      <c r="L47" s="18" t="n">
+        <v>24309.40564516129</v>
+      </c>
+      <c r="M47" s="18" t="n">
+        <v>24292.96129032258</v>
+      </c>
+      <c r="N47" s="18" t="n">
+        <v>24273.01048387097</v>
+      </c>
+      <c r="P47" s="28" t="n">
         <v>24500</v>
       </c>
-      <c r="Q46" s="12" t="n">
-        <v>200444</v>
-      </c>
-      <c r="R46" s="14" t="n">
-        <v>7911</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>1663955</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="P47" s="27" t="n">
-        <v>25000</v>
-      </c>
       <c r="Q47" s="12" t="n">
-        <v>180772</v>
+        <v>250577</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-2676</v>
+        <v>50133</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>519167</v>
+        <v>2595532</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3066,6 +3230,26 @@
       </c>
     </row>
     <row r="48">
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>Weekly Close</t>
+        </is>
+      </c>
+      <c r="J48" s="18" t="n">
+        <v>24219.05</v>
+      </c>
+      <c r="K48" s="18" t="n">
+        <v>24252</v>
+      </c>
+      <c r="L48" s="18" t="n">
+        <v>24366</v>
+      </c>
+      <c r="M48" s="18" t="n">
+        <v>24570.65</v>
+      </c>
+      <c r="N48" s="18" t="n">
+        <v>24383.6</v>
+      </c>
       <c r="P48" s="31" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
@@ -3077,93 +3261,123 @@
       <c r="T48" s="6" t="n"/>
     </row>
     <row r="49">
-      <c r="P49" s="26" t="inlineStr">
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>Week ending</t>
+        </is>
+      </c>
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>24-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
+        <is>
+          <t>21-Aug-2026</t>
+        </is>
+      </c>
+      <c r="L49" s="32" t="inlineStr">
+        <is>
+          <t>14-Aug-2026</t>
+        </is>
+      </c>
+      <c r="M49" s="32" t="inlineStr">
+        <is>
+          <t>07-Aug-2026</t>
+        </is>
+      </c>
+      <c r="N49" s="32" t="inlineStr">
+        <is>
+          <t>31-Jul-2026</t>
+        </is>
+      </c>
+      <c r="P49" s="27" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="Q49" s="26" t="inlineStr">
+      <c r="Q49" s="27" t="inlineStr">
         <is>
           <t>Put OI</t>
         </is>
       </c>
-      <c r="R49" s="26" t="inlineStr">
+      <c r="R49" s="27" t="inlineStr">
         <is>
           <t>Chg OI</t>
         </is>
       </c>
-      <c r="S49" s="26" t="inlineStr">
+      <c r="S49" s="27" t="inlineStr">
         <is>
           <t>Volume</t>
         </is>
       </c>
-      <c r="T49" s="26" t="inlineStr">
+      <c r="T49" s="27" t="inlineStr">
         <is>
           <t>Strength</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
+      <c r="P50" s="33" t="n">
         <v>24200</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>231507</v>
+        <v>188745</v>
       </c>
       <c r="R50" s="14" t="n">
-        <v>27061</v>
+        <v>-42762</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>4481468</v>
-      </c>
-      <c r="T50" s="28" t="inlineStr">
+        <v>8307507</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
+      <c r="P51" s="33" t="n">
+        <v>24100</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>140659</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>13990</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>4705240</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="33" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="12" t="n">
-        <v>272916</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>21410</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>1612499</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
+      <c r="Q52" s="12" t="n">
+        <v>250314</v>
+      </c>
+      <c r="R52" s="14" t="n">
+        <v>-22602</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>3797281</v>
+      </c>
+      <c r="T52" s="32" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>23000</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>177746</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>22948</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>432352</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-    </row>
     <row r="54">
-      <c r="A54" s="33" t="inlineStr">
-        <is>
-          <t>TODAY = 21-Aug-2026    1 DAY AGO = 20-Aug-2026    2 DAYS AGO = 19-Aug-2026    3 DAYS AGO = 18-Aug-2026    4 DAYS AGO = 17-Aug-2026    (generated 21-Aug-2026 20:30 IST)</t>
+      <c r="A54" s="34" t="inlineStr">
+        <is>
+          <t>TODAY = 24-Aug-2026    1 DAY AGO = 21-Aug-2026    2 DAYS AGO = 20-Aug-2026    3 DAYS AGO = 19-Aug-2026    4 DAYS AGO = 18-Aug-2026    (generated 24-Aug-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-25
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
       <b val="1"/>
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>10140</v>
+        <v>-23520</v>
       </c>
     </row>
     <row r="3">
@@ -701,27 +701,27 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>8017</v>
+        <v>-18323</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-2123</v>
+        <v>5197</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>10140</v>
+        <v>-23520</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>157636</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>181156</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>171016</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>173305</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>185408</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>173796</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>162148</v>
+        <v>-132319</v>
       </c>
     </row>
     <row r="4">
@@ -768,29 +768,29 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C4" s="14" t="n">
-        <v>-3122</v>
+      <c r="C4" s="11" t="n">
+        <v>-7678</v>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>-27</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-3095</v>
+      <c r="G4" s="11" t="n">
+        <v>-7678</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="12" t="n">
+        <v>17342</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>25020</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="12" t="n">
         <v>28115</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="12" t="n">
         <v>27278</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="12" t="n">
         <v>27569</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>31073</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -819,7 +819,7 @@
       </c>
       <c r="Q4" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-146453</v>
+        <v>239967</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>1019</v>
+        <v>-3222</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>10547</v>
+        <v>-38378</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>35156</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="n">
+        <v>-184227</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>-219383</v>
+      </c>
+      <c r="L5" s="12" t="n">
+        <v>-209855</v>
+      </c>
+      <c r="M5" s="12" t="n">
+        <v>-212113</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>-209807</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-9528</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-219383</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-209855</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-212113</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-209807</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-194158</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>3988</v>
+        <v>-31020</v>
       </c>
     </row>
     <row r="6">
@@ -908,27 +908,27 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1700</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
+        <v>-19471</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
-        <v>-783</v>
+      <c r="E6" s="14" t="n">
+        <v>-15513</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>2483</v>
+        <v>-3958</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,26 +936,26 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>9249</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>13207</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>10724</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>11530</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>-3170</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-10711</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q6" s="13" t="inlineStr">
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -965,8 +965,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S6" s="14" t="n">
-        <v>-102843</v>
+      <c r="S6" s="11" t="n">
+        <v>-671773</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>7614</v>
+        <v>-48694</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>7614</v>
+        <v>-48694</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,7 +1002,7 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
+      <c r="Q7" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>4097</v>
+      <c r="S7" s="11" t="n">
+        <v>67629</v>
       </c>
     </row>
     <row r="8">
@@ -1071,7 +1071,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
+      <c r="Q8" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-3095</v>
+      <c r="S8" s="11" t="n">
+        <v>-7678</v>
       </c>
     </row>
     <row r="9">
@@ -1093,27 +1093,27 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>948571</v>
+        <v>-2456438</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>786423</v>
+        <v>-2324119</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>162148</v>
+        <v>-132319</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,26 +1121,26 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>94693</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>227012</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>64864</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>111337</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>272961</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>295638</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="13" t="inlineStr">
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="14" t="n">
-        <v>-82</v>
+      <c r="S9" s="11" t="n">
+        <v>-4074</v>
       </c>
     </row>
     <row r="10">
@@ -1162,27 +1162,27 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>25</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+        <v>-4045</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
-        <v>107</v>
-      </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="E10" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="14" t="n">
-        <v>-82</v>
+      <c r="G10" s="11" t="n">
+        <v>-4074</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,16 +1190,16 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>3935</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>8009</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>8091</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>8141</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>7270</v>
       </c>
       <c r="N10" s="12" t="n">
         <v>7270</v>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="14" t="n">
-        <v>19298</v>
+        <v>-33089</v>
       </c>
     </row>
     <row r="11">
@@ -1231,27 +1231,27 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>229305</v>
+        <v>-502261</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>210872</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+        <v>-503511</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>18433</v>
+      <c r="G11" s="14" t="n">
+        <v>1250</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,26 +1259,26 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-198430</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-199680</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-218113</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-233793</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-313586</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-231661</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>3144</v>
+      <c r="S11" s="14" t="n">
+        <v>15529</v>
       </c>
     </row>
     <row r="12">
@@ -1300,27 +1300,27 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>184291</v>
+        <v>-752450</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>364789</v>
+        <v>-887591</v>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
-        <v>-180498</v>
+        <v>135141</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>99801</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>-35340</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>145158</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>114315</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>33355</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-71246</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-6407</v>
+        <v>261828</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1362192</v>
+        <v>-3715194</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1362191</v>
+        <v>-3715192</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1396,7 +1396,7 @@
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="14" t="n">
-        <v>4114</v>
+        <v>-2876</v>
       </c>
     </row>
     <row r="14">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-9528</v>
+        <v>35156</v>
       </c>
     </row>
     <row r="15">
@@ -1483,29 +1483,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C15" s="11" t="n">
-        <v>-115225</v>
+      <c r="C15" s="14" t="n">
+        <v>-1276661</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>31228</v>
+        <v>-1516628</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-146453</v>
+        <v>239967</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,26 +1513,26 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-604022</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-843989</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-697536</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-690662</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-712819</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-697400</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>18433</v>
+      <c r="S15" s="14" t="n">
+        <v>1250</v>
       </c>
     </row>
     <row r="16">
@@ -1554,27 +1554,27 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>19318</v>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
+        <v>-33069</v>
+      </c>
+      <c r="D16" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="14" t="n">
         <v>20</v>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>19298</v>
+        <v>-33089</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>30463</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>63552</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>44254</v>
       </c>
       <c r="L16" s="12" t="n">
         <v>44254</v>
       </c>
       <c r="M16" s="12" t="n">
+        <v>44254</v>
+      </c>
+      <c r="N16" s="12" t="n">
         <v>44104</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>47208</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1603,7 +1603,7 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="14" t="n">
-        <v>114011</v>
+        <v>-32522</v>
       </c>
     </row>
     <row r="17">
@@ -1623,27 +1623,27 @@
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>58690</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+        <v>-346909</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
-        <v>-55321</v>
+      <c r="E17" s="11" t="n">
+        <v>-314387</v>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>114011</v>
+        <v>-32522</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>549436</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>581958</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>467947</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>478916</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>571624</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>611080</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1672,7 +1672,7 @@
       </c>
       <c r="Q17" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R17" s="10" t="inlineStr">
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>2057</v>
+        <v>-83198</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n">
-        <v>-96847</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="C18" s="14" t="n">
+        <v>-561657</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
-        <v>-109992</v>
+      <c r="E18" s="11" t="n">
+        <v>-387301</v>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>-174356</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>24124</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>198480</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>185335</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>167492</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>97090</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>13145</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>198480</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>185335</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>167492</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>97090</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>39113</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-3008</v>
+        <v>171520</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-134064</v>
+        <v>-2218296</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-134065</v>
+        <v>-2218296</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>-7716</v>
+      <c r="S19" s="14" t="n">
+        <v>-88873</v>
       </c>
     </row>
     <row r="20">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="Q20" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>2483</v>
+        <v>-3958</v>
       </c>
     </row>
     <row r="21">
@@ -1875,67 +1875,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
-        <v>-9976</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
+      <c r="C21" s="11" t="n">
+        <v>-100117</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E21" s="11" t="n">
-        <v>-13964</v>
+      <c r="E21" s="14" t="n">
+        <v>-69097</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>-31020</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3049155</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3080175</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3076187</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3059735</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3071689</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>3988</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3080175</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3076187</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3059735</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3071689</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3063117</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S21" s="14" t="n">
-        <v>-180498</v>
+        <v>135141</v>
       </c>
     </row>
     <row r="22">
@@ -1946,27 +1946,27 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>15210</v>
+        <v>-119251</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>12066</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
+        <v>-134780</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>3144</v>
+      <c r="G22" s="14" t="n">
+        <v>15529</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4100306</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4115835</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4118979</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4116362</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4104730</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4093832</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2004,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="14" t="n">
-        <v>13145</v>
+        <v>-174356</v>
       </c>
     </row>
     <row r="23">
@@ -2013,67 +2013,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="14" t="n">
-        <v>-26682</v>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
+      <c r="C23" s="11" t="n">
+        <v>-193808</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E23" s="11" t="n">
-        <v>-28739</v>
+      <c r="E23" s="14" t="n">
+        <v>-110610</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>-83198</v>
+      </c>
+      <c r="I23" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J23" s="12" t="n">
+        <v>600618</v>
+      </c>
+      <c r="K23" s="12" t="n">
+        <v>683816</v>
+      </c>
+      <c r="L23" s="12" t="n">
+        <v>681759</v>
+      </c>
+      <c r="M23" s="12" t="n">
+        <v>666298</v>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>617137</v>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>2057</v>
-      </c>
-      <c r="I23" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J23" s="12" t="n">
-        <v>683816</v>
-      </c>
-      <c r="K23" s="12" t="n">
-        <v>681759</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>666298</v>
-      </c>
-      <c r="M23" s="12" t="n">
-        <v>617137</v>
-      </c>
-      <c r="N23" s="12" t="n">
-        <v>605363</v>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R23" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S23" s="14" t="n">
-        <v>-9189</v>
+        <v>98689</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C24" s="14" t="n">
-        <v>-30748</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
+      <c r="C24" s="11" t="n">
+        <v>-95900</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E24" s="11" t="n">
-        <v>-21559</v>
+      <c r="E24" s="14" t="n">
+        <v>-194589</v>
       </c>
       <c r="F24" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>-9189</v>
+        <v>98689</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,26 +2112,26 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>450533</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>351844</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>361033</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>390329</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>415904</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>425352</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>112258</v>
+      <c r="S24" s="14" t="n">
+        <v>238425</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-52196</v>
+        <v>-509076</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-52196</v>
+        <v>-509076</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="Q25" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2189,7 +2189,7 @@
         </is>
       </c>
       <c r="S25" s="11" t="n">
-        <v>-495</v>
+        <v>24120</v>
       </c>
     </row>
     <row r="26">
@@ -2249,29 +2249,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B27" s="13" t="inlineStr">
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C27" s="14" t="n">
-        <v>-176909</v>
-      </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="C27" s="11" t="n">
+        <v>-1384505</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n">
-        <v>-74066</v>
-      </c>
-      <c r="F27" s="13" t="inlineStr">
+      <c r="E27" s="14" t="n">
+        <v>-712732</v>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G27" s="14" t="n">
-        <v>-102843</v>
+      <c r="G27" s="11" t="n">
+        <v>-671773</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>323137</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>994910</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>1097753</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>1174358</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>1327278</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1347514</v>
       </c>
     </row>
     <row r="28">
@@ -2302,27 +2302,27 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>3264</v>
+        <v>-4842</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
-          <t>Added Shorts</t>
+          <t>Closed Shorts</t>
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>9671</v>
+        <v>-266670</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-6407</v>
+        <v>261828</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-105544</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-367372</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-360965</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-358431</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-363836</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-360505</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2359,29 +2359,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B29" s="13" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n">
-        <v>-20759</v>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="C29" s="11" t="n">
+        <v>-118210</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n">
-        <v>-17751</v>
+      <c r="E29" s="14" t="n">
+        <v>-289730</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-3008</v>
+        <v>171520</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-66057</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-237577</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-234569</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-236847</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-238545</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-223071</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 24-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 25-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2418,29 +2418,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C30" s="14" t="n">
-        <v>-2713</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
+      <c r="C30" s="11" t="n">
+        <v>-627601</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n">
-        <v>-114971</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>-866026</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n">
-        <v>112258</v>
+      <c r="G30" s="14" t="n">
+        <v>238425</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-151536</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-389961</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-502219</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-579080</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-724897</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-763938</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24285.05</v>
+        <v>24175.75</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24313</v>
+        <v>24334.55</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-197117</v>
+        <v>-2135158</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-197117</v>
+        <v>-2135158</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24144.3</v>
+        <v>24115.45</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24219.05</v>
+        <v>24334.55</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24475.3</v>
+        <v>24626.68333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24222.25</v>
+        <v>24298.03333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2597,29 +2597,29 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C33" s="11" t="n">
-        <v>-43530</v>
-      </c>
-      <c r="D33" s="13" t="inlineStr">
+      <c r="C33" s="14" t="n">
+        <v>-437818</v>
+      </c>
+      <c r="D33" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E33" s="14" t="n">
-        <v>-47627</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
+      <c r="E33" s="11" t="n">
+        <v>-505447</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G33" s="14" t="n">
-        <v>4097</v>
+      <c r="G33" s="11" t="n">
+        <v>67629</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-252826</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-320455</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-324552</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-327110</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-377222</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-365490</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24394.15</v>
+        <v>24480.61666666666</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24225.45</v>
+        <v>24261.51666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2666,27 +2666,27 @@
       </c>
       <c r="B34" s="13" t="inlineStr">
         <is>
-          <t>Added Longs</t>
+          <t>Closed Longs</t>
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>656</v>
-      </c>
-      <c r="D34" s="13" t="inlineStr">
+        <v>-15126</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E34" s="14" t="n">
-        <v>-3458</v>
+      <c r="E34" s="11" t="n">
+        <v>-12250</v>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>4114</v>
+        <v>-2876</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>23275</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>26151</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>22037</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>20739</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>20482</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>20604</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24306.6</v>
+        <v>24407.58333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24228.65</v>
+        <v>24225</v>
       </c>
     </row>
     <row r="35">
@@ -2731,29 +2731,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C35" s="11" t="n">
-        <v>-25541</v>
-      </c>
-      <c r="D35" s="13" t="inlineStr">
+      <c r="C35" s="14" t="n">
+        <v>-234239</v>
+      </c>
+      <c r="D35" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E35" s="14" t="n">
-        <v>-17825</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="E35" s="11" t="n">
+        <v>-145366</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G35" s="11" t="n">
-        <v>-7716</v>
+      <c r="G35" s="14" t="n">
+        <v>-88873</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>63426</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>152299</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>160015</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>166400</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>168811</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>168354</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24225.45</v>
+        <v>24261.51666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,29 +2792,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="9" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C36" s="11" t="n">
-        <v>-22084</v>
-      </c>
-      <c r="D36" s="13" t="inlineStr">
+      <c r="C36" s="14" t="n">
+        <v>-525209</v>
+      </c>
+      <c r="D36" s="9" t="inlineStr">
         <is>
           <t>Closed Shorts</t>
         </is>
       </c>
-      <c r="E36" s="14" t="n">
-        <v>-21589</v>
+      <c r="E36" s="11" t="n">
+        <v>-549329</v>
       </c>
       <c r="F36" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G36" s="11" t="n">
-        <v>-495</v>
+        <v>24120</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>166125</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>142005</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>142500</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>139971</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>187929</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>176532</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24137.9</v>
+        <v>24188.48333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-90499</v>
+        <v>-1212392</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-90499</v>
+        <v>-1212392</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24056.75</v>
+        <v>24042.41666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23969.2</v>
+        <v>23969.38333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.08</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.53</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.2</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>10.76</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.32</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.39</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.014881725047644</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.009644797702047</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.01059871674965</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.00922747639189</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.002329484832365</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.004976874300015</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,219    PCR(OI) 0.69    Max Pain 24,200</t>
+          <t>Spot 24,335    PCR(OI) 1.09    Max Pain 24,300</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23977.72016129032</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23987.6935483871</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23997.65564516129</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>24010.29556451613</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>24022.34032258065</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>24035.27943548387</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24334.55</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24219.05</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24252</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24231.85</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24078.3</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24154.9</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24200</v>
+        <v>24350</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>254530</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>118418</v>
+        <v>234835</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>86531</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>5973736</v>
+        <v>11962826</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9951481114124615</v>
+        <v>0.9998556787336708</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9970635633790684</v>
@@ -3173,20 +3173,20 @@
         <v>1.004556069227693</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24300</v>
+        <v>24500</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>332664</v>
+        <v>140165</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>125436</v>
+        <v>-110412</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>6936175</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>2859356</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24337.1310483871</v>
+        <v>24338.0625</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24323.42419354839</v>
@@ -3212,16 +3212,16 @@
         <v>24273.01048387097</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>250577</v>
+        <v>156032</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>50133</v>
+        <v>-36209</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>2595532</v>
+        <v>1433911</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24219.05</v>
+        <v>24334.55</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24252</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>24-Aug-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>25-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>31-Jul-2026</t>
         </is>
@@ -3318,57 +3318,57 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
+      <c r="P50" s="32" t="n">
+        <v>24300</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>272100</v>
+      </c>
+      <c r="R50" s="14" t="n">
+        <v>176748</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>6104115</v>
+      </c>
+      <c r="T50" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="32" t="n">
         <v>24200</v>
       </c>
-      <c r="Q50" s="12" t="n">
-        <v>188745</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>-42762</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>8307507</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
+      <c r="Q51" s="12" t="n">
+        <v>234674</v>
+      </c>
+      <c r="R51" s="14" t="n">
+        <v>45929</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>21625843</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>24100</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>140659</v>
-      </c>
-      <c r="R51" s="11" t="n">
-        <v>13990</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>4705240</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
+      <c r="P52" s="32" t="n">
         <v>24000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>250314</v>
-      </c>
-      <c r="R52" s="14" t="n">
-        <v>-22602</v>
+        <v>191212</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>-59102</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>3797281</v>
-      </c>
-      <c r="T52" s="32" t="inlineStr">
+        <v>8016808</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 24-Aug-2026    1 DAY AGO = 21-Aug-2026    2 DAYS AGO = 20-Aug-2026    3 DAYS AGO = 19-Aug-2026    4 DAYS AGO = 18-Aug-2026    (generated 24-Aug-2026 20:31 IST)</t>
+          <t>TODAY = 25-Aug-2026    1 DAY AGO = 24-Aug-2026    2 DAYS AGO = 21-Aug-2026    3 DAYS AGO = 20-Aug-2026    4 DAYS AGO = 19-Aug-2026    (generated 25-Aug-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-26
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -37,10 +37,10 @@
       <b val="1"/>
     </font>
     <font>
-      <color rgb="00C00000"/>
+      <color rgb="000B7A34"/>
     </font>
     <font>
-      <color rgb="000B7A34"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <b val="1"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,7 +187,7 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -196,11 +196,11 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -681,7 +681,7 @@
       </c>
       <c r="Q2" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R2" s="10" t="inlineStr">
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>-23520</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="3">
@@ -701,48 +701,48 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>-18323</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
+        <v>5233</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E3" s="11" t="n">
-        <v>5197</v>
+      <c r="E3" s="13" t="n">
+        <v>2586</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>-23520</v>
+        <v>2647</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>160283</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>157636</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>181156</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>171016</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>173305</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>185408</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -750,7 +750,7 @@
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>-132319</v>
+        <v>96378</v>
       </c>
     </row>
     <row r="4">
@@ -770,65 +770,65 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>-7678</v>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
+        <v>247</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="11" t="n">
+      <c r="E4" s="13" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>247</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="14" t="n">
+        <v>17589</v>
+      </c>
+      <c r="K4" s="14" t="n">
+        <v>17342</v>
+      </c>
+      <c r="L4" s="14" t="n">
+        <v>25020</v>
+      </c>
+      <c r="M4" s="14" t="n">
+        <v>28115</v>
+      </c>
+      <c r="N4" s="14" t="n">
+        <v>27278</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>-7678</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>17342</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>25020</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>28115</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>27278</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>27569</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>239967</v>
+        <v>-58982</v>
       </c>
     </row>
     <row r="5">
@@ -839,65 +839,65 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>-3222</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E5" s="14" t="n">
-        <v>-38378</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+        <v>1794</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>3627</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>-1833</v>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J5" s="14" t="n">
+        <v>-186060</v>
+      </c>
+      <c r="K5" s="14" t="n">
+        <v>-184227</v>
+      </c>
+      <c r="L5" s="14" t="n">
+        <v>-219383</v>
+      </c>
+      <c r="M5" s="14" t="n">
+        <v>-209855</v>
+      </c>
+      <c r="N5" s="14" t="n">
+        <v>-212113</v>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q5" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>35156</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J5" s="12" t="n">
-        <v>-184227</v>
-      </c>
-      <c r="K5" s="12" t="n">
-        <v>-219383</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>-209855</v>
-      </c>
-      <c r="M5" s="12" t="n">
-        <v>-212113</v>
-      </c>
-      <c r="N5" s="12" t="n">
-        <v>-209807</v>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R5" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>-31020</v>
+        <v>65876</v>
       </c>
     </row>
     <row r="6">
@@ -908,48 +908,48 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>-19471</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>-15513</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>5600</v>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>6661</v>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>-3958</v>
+      <c r="G6" s="13" t="n">
+        <v>-1061</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>8188</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>9249</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>13207</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>10724</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>11530</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>-3170</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -957,7 +957,7 @@
       </c>
       <c r="Q6" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R6" s="10" t="inlineStr">
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>-671773</v>
+        <v>104057</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>-48694</v>
+        <v>12874</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>-48694</v>
+        <v>12874</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="Q7" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>67629</v>
+        <v>-52012</v>
       </c>
     </row>
     <row r="8">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="Q8" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>-7678</v>
+        <v>247</v>
       </c>
     </row>
     <row r="9">
@@ -1093,65 +1093,65 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>-2456438</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>-2324119</v>
+        <v>838639</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>742261</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>96378</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>191071</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>94693</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>227012</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>64864</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>111337</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>-132319</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>94693</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>227012</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>64864</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>111337</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>272961</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>-4074</v>
+      <c r="S9" s="13" t="n">
+        <v>-30</v>
       </c>
     </row>
     <row r="10">
@@ -1162,56 +1162,56 @@
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>-4045</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
-        <v>29</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="E10" s="13" t="n">
+        <v>30</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G10" s="11" t="n">
-        <v>-4074</v>
+      <c r="G10" s="13" t="n">
+        <v>-30</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>3905</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>3935</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>8009</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>8091</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>8141</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>7270</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q10" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>-33089</v>
+      <c r="S10" s="13" t="n">
+        <v>1516</v>
       </c>
     </row>
     <row r="11">
@@ -1231,56 +1231,56 @@
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>-502261</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>-503511</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="n">
-        <v>1250</v>
+        <v>100627</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>138082</v>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="13" t="n">
+        <v>-37455</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
+        <v>-235885</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-198430</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>-199680</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="14" t="n">
         <v>-218113</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>-233793</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-313586</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>15529</v>
+      <c r="S11" s="13" t="n">
+        <v>-24026</v>
       </c>
     </row>
     <row r="12">
@@ -1300,56 +1300,56 @@
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>-752450</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>-887591</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="n">
-        <v>135141</v>
+        <v>206254</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>265147</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>-58893</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
+        <v>40908</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>99801</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>-35340</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="14" t="n">
         <v>145158</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>114315</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>33355</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q12" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R12" s="10" t="inlineStr">
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>261828</v>
+      <c r="S12" s="13" t="n">
+        <v>-44922</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-3715194</v>
+        <v>1145520</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-3715192</v>
+        <v>1145520</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1394,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q13" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>-2876</v>
+      <c r="S13" s="13" t="n">
+        <v>6167</v>
       </c>
     </row>
     <row r="14">
@@ -1463,9 +1463,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q14" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R14" s="10" t="inlineStr">
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>35156</v>
+      <c r="S14" s="13" t="n">
+        <v>-1833</v>
       </c>
     </row>
     <row r="15">
@@ -1483,58 +1483,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="14" t="n">
-        <v>-1276661</v>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>317100</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>-1516628</v>
+        <v>376082</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>239967</v>
+        <v>-58982</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-663004</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-604022</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-843989</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-697536</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-690662</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-712819</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>1250</v>
+      <c r="S15" s="13" t="n">
+        <v>-37455</v>
       </c>
     </row>
     <row r="16">
@@ -1552,58 +1552,58 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>-33069</v>
-      </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="n">
+        <v>1516</v>
+      </c>
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="n">
-        <v>-33089</v>
+      <c r="E16" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="13" t="n">
+        <v>1516</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>31979</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>30463</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>63552</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>44254</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>44254</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>44104</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>-32522</v>
+      <c r="S16" s="13" t="n">
+        <v>6315</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="14" t="n">
-        <v>-346909</v>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>47822</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>-314387</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>41507</v>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="n">
+        <v>6315</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>555751</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>549436</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>581958</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>467947</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>478916</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>-32522</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>549436</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>581958</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>467947</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>478916</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>571624</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>-83198</v>
+      <c r="S17" s="13" t="n">
+        <v>-32855</v>
       </c>
     </row>
     <row r="18">
@@ -1690,67 +1690,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="14" t="n">
-        <v>-561657</v>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>88455</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>-387301</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>37305</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>51150</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>75274</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>24124</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>198480</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>185335</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>167492</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>-174356</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>24124</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>198480</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>185335</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>167492</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>97090</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>171520</v>
+      <c r="S18" s="13" t="n">
+        <v>-13067</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-2218296</v>
+        <v>454893</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-2218296</v>
+        <v>454894</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>-88873</v>
+      <c r="S19" s="11" t="n">
+        <v>-2331</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
+      <c r="Q20" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>-3958</v>
+      <c r="S20" s="13" t="n">
+        <v>-1061</v>
       </c>
     </row>
     <row r="21">
@@ -1877,65 +1877,65 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>-100117</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="n">
-        <v>-69097</v>
+        <v>77290</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="n">
+        <v>11414</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>65876</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="n">
+        <v>3115031</v>
+      </c>
+      <c r="K21" s="14" t="n">
+        <v>3049155</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>3080175</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>3076187</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>3059735</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n">
-        <v>-31020</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3049155</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3080175</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3076187</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3059735</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3071689</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>135141</v>
+      <c r="S21" s="13" t="n">
+        <v>-58893</v>
       </c>
     </row>
     <row r="22">
@@ -1946,65 +1946,65 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>-119251</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="n">
-        <v>-134780</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+        <v>9721</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="n">
+        <v>33747</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="13" t="n">
+        <v>-24026</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="14" t="n">
+        <v>-4124332</v>
+      </c>
+      <c r="K22" s="14" t="n">
+        <v>-4100306</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>-4115835</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>-4118979</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>-4116362</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>15529</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="12" t="n">
-        <v>-4100306</v>
-      </c>
-      <c r="K22" s="12" t="n">
-        <v>-4115835</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>-4118979</v>
-      </c>
-      <c r="M22" s="12" t="n">
-        <v>-4116362</v>
-      </c>
-      <c r="N22" s="12" t="n">
-        <v>-4104730</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>-174356</v>
+      <c r="S22" s="13" t="n">
+        <v>51150</v>
       </c>
     </row>
     <row r="23">
@@ -2013,58 +2013,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="11" t="n">
-        <v>-193808</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>-110610</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="C23" s="13" t="n">
+        <v>-9473</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="n">
+        <v>23382</v>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>-83198</v>
+      <c r="G23" s="13" t="n">
+        <v>-32855</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>567763</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>600618</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>683816</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>681759</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>666298</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>617137</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>98689</v>
+      <c r="S23" s="13" t="n">
+        <v>-8995</v>
       </c>
     </row>
     <row r="24">
@@ -2084,56 +2084,56 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>-95900</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="14" t="n">
-        <v>-194589</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="n">
-        <v>98689</v>
+        <v>24633</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="n">
+        <v>33628</v>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="n">
+        <v>-8995</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>441538</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>450533</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>351844</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>361033</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>390329</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>415904</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>238425</v>
+      <c r="S24" s="13" t="n">
+        <v>-46068</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-509076</v>
+        <v>102171</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-509076</v>
+        <v>102171</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
+      <c r="Q25" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>24120</v>
+      <c r="S25" s="13" t="n">
+        <v>48176</v>
       </c>
     </row>
     <row r="26">
@@ -2251,47 +2251,47 @@
       </c>
       <c r="B27" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>-1384505</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E27" s="14" t="n">
-        <v>-712732</v>
+        <v>247618</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>143561</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Sold Net</t>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>-671773</v>
+        <v>104057</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>427194</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>323137</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>994910</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>1097753</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>1174358</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1327278</v>
       </c>
     </row>
     <row r="28">
@@ -2302,47 +2302,47 @@
       </c>
       <c r="B28" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>-4842</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E28" s="14" t="n">
-        <v>-266670</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G28" s="14" t="n">
-        <v>261828</v>
+        <v>100</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="n">
+        <v>45022</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G28" s="13" t="n">
+        <v>-44922</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-150466</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-105544</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-367372</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-360965</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-358431</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-363836</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2361,51 +2361,51 @@
       </c>
       <c r="B29" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>-118210</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="n">
-        <v>-289730</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>171520</v>
+        <v>17934</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>31001</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>-13067</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-79124</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-66057</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-237577</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-234569</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-236847</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-238545</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 25-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 26-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2420,55 +2420,55 @@
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>Closed Longs</t>
+          <t>Added Longs</t>
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>-627601</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E30" s="14" t="n">
-        <v>-866026</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>238425</v>
+        <v>111730</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="n">
+        <v>157798</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>-46068</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-197604</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-151536</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-389961</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-502219</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-579080</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-724897</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24175.75</v>
+        <v>24341.95</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24334.55</v>
+        <v>24378.6</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>-2135158</v>
+        <v>377382</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>-2135158</v>
+        <v>377382</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24115.45</v>
+        <v>24207.75</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24334.55</v>
+        <v>24207.75</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24626.68333333333</v>
+        <v>24492.5</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24298.03333333333</v>
+        <v>24236.225</v>
       </c>
     </row>
     <row r="33">
@@ -2597,57 +2597,57 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C33" s="14" t="n">
-        <v>-437818</v>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>88420</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>-505447</v>
+        <v>140432</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
-          <t>Bought Net</t>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>67629</v>
+        <v>-52012</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-304838</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-252826</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-320455</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-324552</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-327110</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-377222</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24480.61666666666</v>
+        <v>24435.55</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24261.51666666667</v>
+        <v>24264.7</v>
       </c>
     </row>
     <row r="34">
@@ -2664,57 +2664,57 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C34" s="14" t="n">
-        <v>-15126</v>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>9406</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>-12250</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="n">
-        <v>-2876</v>
+        <v>3239</v>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>6167</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>29442</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>23275</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>26151</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>22037</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>20739</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>20482</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24407.58333333333</v>
+        <v>24321.65</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24225</v>
+        <v>24293.175</v>
       </c>
     </row>
     <row r="35">
@@ -2731,57 +2731,57 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C35" s="14" t="n">
-        <v>-234239</v>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>23885</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>-145366</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+        <v>26216</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>-88873</v>
+      <c r="G35" s="11" t="n">
+        <v>-2331</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>61095</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>63426</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>152299</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>160015</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>166400</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>168811</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24261.51666666667</v>
+        <v>24264.7</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,57 +2792,57 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C36" s="14" t="n">
-        <v>-525209</v>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="n">
+        <v>130824</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
-          <t>Closed Shorts</t>
+          <t>Added Shorts</t>
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>-549329</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
+        <v>82648</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G36" s="11" t="n">
-        <v>24120</v>
+      <c r="G36" s="13" t="n">
+        <v>48176</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>214301</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>166125</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>142005</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>142500</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>139971</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>187929</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24188.48333333333</v>
+        <v>24150.8</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>-1212392</v>
+        <v>252535</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>-1212392</v>
+        <v>252535</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24042.41666666667</v>
+        <v>24093.85</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23969.38333333334</v>
+        <v>23979.95</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.08</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.53</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.2</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>10.76</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.32</v>
       </c>
     </row>
     <row r="41">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 25-Aug-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 01-Sep-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.010104864602446</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.014881725047644</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.009644797702047</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.01059871674965</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.00922747639189</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.002329484832365</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,335    PCR(OI) 1.09    Max Pain 24,300</t>
+          <t>Spot 24,208    PCR(OI) 0.73    Max Pain 24,300</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23965.5810483871</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23977.72016129032</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23987.6935483871</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23997.65564516129</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>24010.29556451613</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>24022.34032258065</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24207.75</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24334.55</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24219.05</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24252</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24231.85</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24078.3</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3134,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24350</v>
-      </c>
-      <c r="Q45" s="12" t="n">
-        <v>234835</v>
-      </c>
-      <c r="R45" s="14" t="n">
-        <v>86531</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>11962826</v>
+        <v>24300</v>
+      </c>
+      <c r="Q45" s="14" t="n">
+        <v>136089</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>77964</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>2248121</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9998556787336708</v>
+        <v>0.9946875248681325</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9970635633790684</v>
@@ -3175,18 +3175,18 @@
       <c r="P46" s="28" t="n">
         <v>24500</v>
       </c>
-      <c r="Q46" s="12" t="n">
-        <v>140165</v>
+      <c r="Q46" s="14" t="n">
+        <v>159876</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>-110412</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>2859356</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>75784</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>1922348</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24338.0625</v>
+        <v>24337.03991935484</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24323.42419354839</v>
@@ -3214,14 +3214,14 @@
       <c r="P47" s="28" t="n">
         <v>25000</v>
       </c>
-      <c r="Q47" s="12" t="n">
-        <v>156032</v>
+      <c r="Q47" s="14" t="n">
+        <v>136952</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>-36209</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>1433911</v>
+        <v>56437</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>665814</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24334.55</v>
+        <v>24207.75</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24252</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>25-Aug-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="32" t="inlineStr">
+        <is>
+          <t>26-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="32" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="32" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="32" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="32" t="inlineStr">
         <is>
           <t>31-Jul-2026</t>
         </is>
@@ -3318,66 +3318,66 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>24300</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>272100</v>
-      </c>
-      <c r="R50" s="14" t="n">
-        <v>176748</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>6104115</v>
-      </c>
-      <c r="T50" s="30" t="inlineStr">
+      <c r="P50" s="33" t="n">
+        <v>24200</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>95353</v>
+      </c>
+      <c r="R50" s="13" t="n">
+        <v>-17347</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>1848955</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="P51" s="33" t="n">
+        <v>24000</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>86691</v>
+      </c>
+      <c r="R51" s="11" t="n">
+        <v>23294</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>1034495</v>
+      </c>
+      <c r="T51" s="32" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="P52" s="33" t="n">
+        <v>23500</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>82753</v>
+      </c>
+      <c r="R52" s="11" t="n">
+        <v>20901</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>509256</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
         <is>
           <t>Low</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>24200</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>234674</v>
-      </c>
-      <c r="R51" s="14" t="n">
-        <v>45929</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>21625843</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>191212</v>
-      </c>
-      <c r="R52" s="11" t="n">
-        <v>-59102</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>8016808</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 25-Aug-2026    1 DAY AGO = 24-Aug-2026    2 DAYS AGO = 21-Aug-2026    3 DAYS AGO = 20-Aug-2026    4 DAYS AGO = 19-Aug-2026    (generated 25-Aug-2026 20:31 IST)</t>
+          <t>TODAY = 26-Aug-2026    1 DAY AGO = 25-Aug-2026    2 DAYS AGO = 24-Aug-2026    3 DAYS AGO = 21-Aug-2026    4 DAYS AGO = 20-Aug-2026    (generated 26-Aug-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-27
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -190,17 +190,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>2647</v>
+        <v>13875</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>5233</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>2586</v>
+        <v>12631</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>-1244</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,28 +721,28 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>2647</v>
+        <v>13875</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>174158</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>160283</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>157636</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>181156</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>171016</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>173305</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>96378</v>
+        <v>98082</v>
       </c>
     </row>
     <row r="4">
@@ -774,14 +774,14 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>247</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+        <v>1924</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -790,28 +790,28 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>247</v>
+        <v>1924</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>19513</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>17589</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>17342</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>25020</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>28115</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>27278</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="11" t="n">
-        <v>-58982</v>
+        <v>-97979</v>
       </c>
     </row>
     <row r="5">
@@ -837,50 +837,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>1794</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>-1461</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>3627</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>10271</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-1833</v>
+      <c r="G5" s="14" t="n">
+        <v>-11732</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-197792</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-186060</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-184227</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-219383</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-209855</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-212113</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>65876</v>
+        <v>39137</v>
       </c>
     </row>
     <row r="6">
@@ -912,44 +912,44 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>5600</v>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
+        <v>2119</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E6" s="13" t="n">
-        <v>6661</v>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="E6" s="14" t="n">
+        <v>6186</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
-        <v>-1061</v>
+      <c r="G6" s="14" t="n">
+        <v>-4067</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>4121</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>8188</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>9249</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>13207</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>10724</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>11530</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>104057</v>
+        <v>112129</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>12874</v>
+        <v>15213</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>12874</v>
+        <v>15213</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1013,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-52012</v>
+        <v>-51363</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>247</v>
+        <v>1924</v>
       </c>
     </row>
     <row r="9">
@@ -1097,15 +1097,15 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>838639</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
+        <v>835724</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="13" t="n">
-        <v>742261</v>
+      <c r="E9" s="14" t="n">
+        <v>737642</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1113,36 +1113,36 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>96378</v>
+        <v>98082</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>289153</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>191071</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>94693</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>227012</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>64864</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>111337</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1150,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>-30</v>
+      <c r="S9" s="11" t="n">
+        <v>420</v>
       </c>
     </row>
     <row r="10">
@@ -1166,50 +1166,50 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
+        <v>475</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E10" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>-30</v>
+      <c r="E10" s="14" t="n">
+        <v>55</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>420</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>4325</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>3905</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>3935</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>8009</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>8091</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>8141</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
+      <c r="Q10" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>1516</v>
+      <c r="S10" s="14" t="n">
+        <v>1535</v>
       </c>
     </row>
     <row r="11">
@@ -1235,50 +1235,50 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>100627</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
+        <v>68158</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E11" s="13" t="n">
-        <v>138082</v>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="E11" s="14" t="n">
+        <v>98129</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>-37455</v>
+      <c r="G11" s="14" t="n">
+        <v>-29971</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J11" s="14" t="n">
+      <c r="J11" s="12" t="n">
+        <v>-265856</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-235885</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="12" t="n">
         <v>-198430</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="12" t="n">
         <v>-199680</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="12" t="n">
         <v>-218113</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-233793</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="12" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1288,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-24026</v>
+      <c r="S11" s="14" t="n">
+        <v>-12040</v>
       </c>
     </row>
     <row r="12">
@@ -1304,50 +1304,50 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>206254</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
+        <v>192558</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E12" s="13" t="n">
-        <v>265147</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="E12" s="14" t="n">
+        <v>261088</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>-58893</v>
+      <c r="G12" s="14" t="n">
+        <v>-68530</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>-27622</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>40908</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>99801</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>-35340</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>145158</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>114315</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1357,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-44922</v>
+      <c r="S12" s="14" t="n">
+        <v>-22512</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1145520</v>
+        <v>1096915</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1145520</v>
+        <v>1096914</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="13" t="n">
-        <v>6167</v>
+      <c r="S13" s="14" t="n">
+        <v>552</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-1833</v>
+      <c r="S14" s="14" t="n">
+        <v>-11732</v>
       </c>
     </row>
     <row r="15">
@@ -1483,13 +1483,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="13" t="n">
-        <v>317100</v>
+      <c r="C15" s="14" t="n">
+        <v>152392</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>376082</v>
+        <v>250371</v>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
@@ -1505,34 +1505,34 @@
         </is>
       </c>
       <c r="G15" s="11" t="n">
-        <v>-58982</v>
+        <v>-97979</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-760983</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-663004</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-604022</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-843989</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-697536</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-690662</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="12" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="13" t="n">
-        <v>-37455</v>
+      <c r="S15" s="14" t="n">
+        <v>-29971</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="13" t="n">
-        <v>1516</v>
+      <c r="C16" s="14" t="n">
+        <v>1535</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,40 +1568,40 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
-        <v>1516</v>
+      <c r="G16" s="14" t="n">
+        <v>1535</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>33514</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>31979</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>30463</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>63552</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>44254</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>44254</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="12" t="inlineStr">
+      <c r="Q16" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="13" t="n">
-        <v>6315</v>
+      <c r="S16" s="14" t="n">
+        <v>70609</v>
       </c>
     </row>
     <row r="17">
@@ -1621,13 +1621,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="13" t="n">
-        <v>47822</v>
+      <c r="C17" s="14" t="n">
+        <v>109678</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,42 +1635,42 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>41507</v>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
+        <v>39069</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
-        <v>6315</v>
+      <c r="G17" s="14" t="n">
+        <v>70609</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J17" s="14" t="n">
+      <c r="J17" s="12" t="n">
+        <v>626360</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>555751</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="12" t="n">
         <v>549436</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="12" t="n">
         <v>581958</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="12" t="n">
         <v>467947</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>478916</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q17" s="12" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1680,8 +1680,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="13" t="n">
-        <v>-32855</v>
+      <c r="S17" s="14" t="n">
+        <v>-26393</v>
       </c>
     </row>
     <row r="18">
@@ -1690,13 +1690,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="13" t="n">
-        <v>88455</v>
+      <c r="C18" s="14" t="n">
+        <v>135654</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,42 +1704,42 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>37305</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
+        <v>109819</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
-        <v>51150</v>
+      <c r="G18" s="14" t="n">
+        <v>25835</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>101109</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>75274</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>24124</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>198480</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>185335</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>167492</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1749,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-13067</v>
+      <c r="S18" s="14" t="n">
+        <v>-24015</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>454893</v>
+        <v>399259</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>454894</v>
+        <v>399259</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q19" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="11" t="n">
-        <v>-2331</v>
+      <c r="S19" s="14" t="n">
+        <v>13759</v>
       </c>
     </row>
     <row r="20">
@@ -1855,7 +1855,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="12" t="inlineStr">
+      <c r="Q20" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="13" t="n">
-        <v>-1061</v>
+      <c r="S20" s="14" t="n">
+        <v>-4067</v>
       </c>
     </row>
     <row r="21">
@@ -1881,15 +1881,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>77290</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
+        <v>46539</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="13" t="n">
-        <v>11414</v>
+      <c r="E21" s="14" t="n">
+        <v>7402</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,34 +1897,34 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>65876</v>
+        <v>39137</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>3154168</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3115031</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>3049155</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>3080175</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>3076187</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3059735</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>-58893</v>
+      <c r="S21" s="14" t="n">
+        <v>-68530</v>
       </c>
     </row>
     <row r="22">
@@ -1950,50 +1950,50 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>9721</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
+        <v>8251</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="13" t="n">
-        <v>33747</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+      <c r="E22" s="14" t="n">
+        <v>20291</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>-24026</v>
+      <c r="G22" s="14" t="n">
+        <v>-12040</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="14" t="n">
+      <c r="J22" s="12" t="n">
+        <v>-4136372</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4124332</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4100306</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4115835</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4118979</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4116362</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="12" t="inlineStr">
+      <c r="Q22" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>51150</v>
+      <c r="S22" s="14" t="n">
+        <v>25835</v>
       </c>
     </row>
     <row r="23">
@@ -2013,56 +2013,56 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C23" s="13" t="n">
-        <v>-9473</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="C23" s="14" t="n">
+        <v>-4816</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>23382</v>
-      </c>
-      <c r="F23" s="12" t="inlineStr">
+      <c r="E23" s="14" t="n">
+        <v>21577</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G23" s="13" t="n">
-        <v>-32855</v>
+      <c r="G23" s="14" t="n">
+        <v>-26393</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>541370</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>567763</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>600618</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>683816</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>681759</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>666298</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="12" t="inlineStr">
+      <c r="Q23" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="13" t="n">
-        <v>-8995</v>
+      <c r="S23" s="14" t="n">
+        <v>-704</v>
       </c>
     </row>
     <row r="24">
@@ -2088,50 +2088,50 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>24633</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
+        <v>12283</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="13" t="n">
-        <v>33628</v>
-      </c>
-      <c r="F24" s="12" t="inlineStr">
+      <c r="E24" s="14" t="n">
+        <v>12987</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="13" t="n">
-        <v>-8995</v>
+      <c r="G24" s="14" t="n">
+        <v>-704</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>440834</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>441538</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>450533</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>351844</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>361033</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>390329</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-46068</v>
+      <c r="S24" s="14" t="n">
+        <v>-65602</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>102171</v>
+        <v>62257</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>102171</v>
+        <v>62257</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2178,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>48176</v>
+      <c r="S25" s="14" t="n">
+        <v>37052</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>247618</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>221364</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>143561</v>
+      <c r="E27" s="14" t="n">
+        <v>109235</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>104057</v>
+        <v>112129</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>539323</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>427194</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>323137</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>994910</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>1097753</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>1174358</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>100</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+        <v>150</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>45022</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>22662</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-44922</v>
+      <c r="G28" s="14" t="n">
+        <v>-22512</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-172978</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-150466</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-105544</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-367372</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-360965</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-358431</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>17934</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+        <v>6974</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>31001</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>30989</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>-13067</v>
+      <c r="G29" s="14" t="n">
+        <v>-24015</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-103139</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-79124</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-66057</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-237577</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-234569</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-236847</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 26-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 27-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>111730</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+        <v>54113</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>157798</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>119715</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n">
-        <v>-46068</v>
+      <c r="G30" s="14" t="n">
+        <v>-65602</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-263206</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-197604</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-151536</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-389961</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-502219</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-579080</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24341.95</v>
+        <v>24277.6</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24378.6</v>
+        <v>24297.45</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>377382</v>
+        <v>282601</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>377382</v>
+        <v>282601</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24207.75</v>
+        <v>24090.85</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24207.75</v>
+        <v>24090.85</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24492.5</v>
+        <v>24435.18333333333</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24236.225</v>
+        <v>24125.28333333333</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="13" t="n">
-        <v>88420</v>
+      <c r="C33" s="14" t="n">
+        <v>72664</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,7 +2611,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>140432</v>
+        <v>124027</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,35 +2619,35 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-52012</v>
+        <v>-51363</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-356201</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-304838</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-252826</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-320455</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-324552</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-327110</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24435.55</v>
+        <v>24366.31666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24264.7</v>
+        <v>24159.71666666666</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="13" t="n">
-        <v>9406</v>
+      <c r="C34" s="14" t="n">
+        <v>1300</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>3239</v>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
+        <v>748</v>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G34" s="13" t="n">
-        <v>6167</v>
+      <c r="G34" s="14" t="n">
+        <v>552</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>29994</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>29442</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>23275</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>26151</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>22037</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>20739</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24321.65</v>
+        <v>24228.58333333333</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24293.175</v>
+        <v>24194.15</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>23885</v>
+      <c r="C35" s="14" t="n">
+        <v>25628</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>26216</v>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G35" s="11" t="n">
-        <v>-2331</v>
+        <v>11869</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G35" s="14" t="n">
+        <v>13759</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>74854</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>61095</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>63426</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>152299</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>160015</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>166400</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24264.7</v>
+        <v>24159.71666666666</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>130824</v>
+      <c r="C36" s="14" t="n">
+        <v>93409</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2806,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>82648</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
+        <v>56357</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G36" s="13" t="n">
-        <v>48176</v>
+      <c r="G36" s="14" t="n">
+        <v>37052</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>251353</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>214301</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>166125</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>142005</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>142500</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>139971</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24150.8</v>
+        <v>24021.98333333333</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>252535</v>
+        <v>193001</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>252535</v>
+        <v>193001</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24093.85</v>
+        <v>23953.11666666666</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23979.95</v>
+        <v>23815.38333333332</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.07</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>10.57</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.08</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.53</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.2</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>10.76</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.005678413660525</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.010104864602446</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.014881725047644</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.009644797702047</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.01059871674965</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.00922747639189</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,208    PCR(OI) 0.73    Max Pain 24,300</t>
+          <t>Spot 24,091    PCR(OI) 0.59    Max Pain 24,200</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23954.82459677419</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23965.5810483871</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23977.72016129032</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23987.6935483871</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23997.65564516129</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>24010.29556451613</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24090.85</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24207.75</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24334.55</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24219.05</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24252</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24231.85</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3136,14 +3136,14 @@
       <c r="P45" s="28" t="n">
         <v>24300</v>
       </c>
-      <c r="Q45" s="14" t="n">
-        <v>136089</v>
+      <c r="Q45" s="12" t="n">
+        <v>203330</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>77964</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>2248121</v>
+        <v>67241</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>2217212</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9946875248681325</v>
+        <v>0.989922493502906</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9970635633790684</v>
@@ -3173,20 +3173,20 @@
         <v>1.004556069227693</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>159876</v>
+        <v>24400</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>188213</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>75784</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>1922348</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>54409</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>1402679</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24337.03991935484</v>
+        <v>24336.09717741935</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24323.42419354839</v>
@@ -3212,20 +3212,20 @@
         <v>24273.01048387097</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>25000</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>136952</v>
+        <v>24500</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>192893</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>56437</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>665814</v>
+        <v>33017</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>1311554</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24207.75</v>
+        <v>24090.85</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24252</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="32" t="inlineStr">
-        <is>
-          <t>26-Aug-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="32" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>27-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="32" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="32" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="32" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>31-Jul-2026</t>
         </is>
@@ -3318,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="33" t="n">
-        <v>24200</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>95353</v>
-      </c>
-      <c r="R50" s="13" t="n">
-        <v>-17347</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>1848955</v>
+      <c r="P50" s="32" t="n">
+        <v>24000</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>109318</v>
+      </c>
+      <c r="R50" s="11" t="n">
+        <v>22627</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>1698841</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3337,38 +3337,38 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="33" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q51" s="14" t="n">
-        <v>86691</v>
+      <c r="P51" s="32" t="n">
+        <v>23800</v>
+      </c>
+      <c r="Q51" s="12" t="n">
+        <v>97609</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>23294</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>1034495</v>
-      </c>
-      <c r="T51" s="32" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>27506</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>706345</v>
+      </c>
+      <c r="T51" s="33" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="33" t="n">
+      <c r="P52" s="32" t="n">
         <v>23500</v>
       </c>
-      <c r="Q52" s="14" t="n">
-        <v>82753</v>
+      <c r="Q52" s="12" t="n">
+        <v>107092</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>20901</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>509256</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
+        <v>24339</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>467606</v>
+      </c>
+      <c r="T52" s="33" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 26-Aug-2026    1 DAY AGO = 25-Aug-2026    2 DAYS AGO = 24-Aug-2026    3 DAYS AGO = 21-Aug-2026    4 DAYS AGO = 20-Aug-2026    (generated 26-Aug-2026 20:31 IST)</t>
+          <t>TODAY = 27-Aug-2026    1 DAY AGO = 26-Aug-2026    2 DAYS AGO = 25-Aug-2026    3 DAYS AGO = 24-Aug-2026    4 DAYS AGO = 21-Aug-2026    (generated 27-Aug-2026 20:42 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-28
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,10 +187,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -199,7 +199,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>13875</v>
+        <v>2801</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +705,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>12631</v>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>-1244</v>
+        <v>3851</v>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="n">
+        <v>1050</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,36 +721,36 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>13875</v>
+        <v>2801</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
+        <v>176959</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>174158</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>160283</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="14" t="n">
         <v>157636</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>181156</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>171016</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>98082</v>
+      <c r="S3" s="13" t="n">
+        <v>-197956</v>
       </c>
     </row>
     <row r="4">
@@ -774,15 +774,15 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>1924</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
+        <v>4100</v>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
-        <v>0</v>
+      <c r="E4" s="13" t="n">
+        <v>3400</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,36 +790,36 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>1924</v>
+        <v>700</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
+        <v>20213</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>19513</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>17589</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="M4" s="14" t="n">
         <v>17342</v>
       </c>
-      <c r="M4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>25020</v>
       </c>
-      <c r="N4" s="12" t="n">
-        <v>28115</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q4" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +827,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-97979</v>
+      <c r="S4" s="13" t="n">
+        <v>35917</v>
       </c>
     </row>
     <row r="5">
@@ -837,50 +837,50 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="12" t="inlineStr">
         <is>
           <t>Closed Longs</t>
         </is>
       </c>
-      <c r="C5" s="14" t="n">
-        <v>-1461</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="C5" s="13" t="n">
+        <v>-33</v>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
-        <v>10271</v>
-      </c>
-      <c r="F5" s="13" t="inlineStr">
+      <c r="E5" s="13" t="n">
+        <v>4808</v>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="14" t="n">
-        <v>-11732</v>
+      <c r="G5" s="13" t="n">
+        <v>-4841</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
+        <v>-202633</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-197792</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>-186060</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="14" t="n">
         <v>-184227</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>-219383</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-209855</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>39137</v>
+        <v>6850</v>
       </c>
     </row>
     <row r="6">
@@ -912,44 +912,44 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>2119</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>6186</v>
-      </c>
-      <c r="F6" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G6" s="14" t="n">
-        <v>-4067</v>
+        <v>1127</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-213</v>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>1340</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
+        <v>5461</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>4121</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>8188</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="14" t="n">
         <v>9249</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>13207</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>10724</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>112129</v>
+        <v>32488</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>15213</v>
+        <v>9045</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>15213</v>
+        <v>9045</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-51363</v>
+      <c r="S7" s="13" t="n">
+        <v>15131</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>1924</v>
+        <v>700</v>
       </c>
     </row>
     <row r="9">
@@ -1091,67 +1091,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>835724</v>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>-44242</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
-        <v>737642</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="E9" s="13" t="n">
+        <v>153714</v>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="13" t="n">
+        <v>-197956</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>91197</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>289153</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>191071</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>94693</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>227012</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G9" s="11" t="n">
-        <v>98082</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="12" t="n">
-        <v>289153</v>
-      </c>
-      <c r="K9" s="12" t="n">
-        <v>191071</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>94693</v>
-      </c>
-      <c r="M9" s="12" t="n">
-        <v>227012</v>
-      </c>
-      <c r="N9" s="12" t="n">
-        <v>64864</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S9" s="11" t="n">
-        <v>420</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10">
@@ -1166,15 +1166,15 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>475</v>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="n">
-        <v>55</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-25</v>
       </c>
       <c r="F10" s="9" t="inlineStr">
         <is>
@@ -1182,34 +1182,34 @@
         </is>
       </c>
       <c r="G10" s="11" t="n">
-        <v>420</v>
+        <v>25</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
+        <v>4350</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>4325</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>3905</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="14" t="n">
         <v>3935</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>8009</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>8091</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
+      <c r="Q10" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>1535</v>
+      <c r="S10" s="13" t="n">
+        <v>975</v>
       </c>
     </row>
     <row r="11">
@@ -1235,61 +1235,61 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>68158</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>98129</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>34995</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-841</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>35836</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="14" t="n">
+        <v>-230020</v>
+      </c>
+      <c r="K11" s="14" t="n">
+        <v>-265856</v>
+      </c>
+      <c r="L11" s="14" t="n">
+        <v>-235885</v>
+      </c>
+      <c r="M11" s="14" t="n">
+        <v>-198430</v>
+      </c>
+      <c r="N11" s="14" t="n">
+        <v>-199680</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-29971</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-265856</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-235885</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-198430</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-199680</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-218113</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="14" t="n">
-        <v>-12040</v>
+      <c r="S11" s="13" t="n">
+        <v>-27612</v>
       </c>
     </row>
     <row r="12">
@@ -1304,61 +1304,61 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>192558</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>261088</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>103687</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-58408</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>162095</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="14" t="n">
+        <v>134473</v>
+      </c>
+      <c r="K12" s="14" t="n">
+        <v>-27622</v>
+      </c>
+      <c r="L12" s="14" t="n">
+        <v>40908</v>
+      </c>
+      <c r="M12" s="14" t="n">
+        <v>99801</v>
+      </c>
+      <c r="N12" s="14" t="n">
+        <v>-35340</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-68530</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-27622</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>40908</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>99801</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>-35340</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>145158</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="14" t="n">
-        <v>-22512</v>
+      <c r="S12" s="13" t="n">
+        <v>-33971</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1096915</v>
+        <v>94440</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1096914</v>
+        <v>94440</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1394,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="14" t="n">
-        <v>552</v>
+      <c r="S13" s="11" t="n">
+        <v>-765</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1463,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="13" t="inlineStr">
+      <c r="Q14" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1473,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="14" t="n">
-        <v>-11732</v>
+      <c r="S14" s="13" t="n">
+        <v>-4841</v>
       </c>
     </row>
     <row r="15">
@@ -1483,13 +1483,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
-        <v>152392</v>
+      <c r="C15" s="13" t="n">
+        <v>433413</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,44 +1497,44 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>250371</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>-97979</v>
+        <v>397496</v>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="13" t="n">
+        <v>35917</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
+        <v>-725066</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-760983</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>-663004</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="14" t="n">
         <v>-604022</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>-843989</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-697536</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-29971</v>
+      <c r="S15" s="11" t="n">
+        <v>35836</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C16" s="14" t="n">
-        <v>1535</v>
+      <c r="C16" s="13" t="n">
+        <v>975</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,42 +1568,42 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="F16" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G16" s="14" t="n">
-        <v>1535</v>
+      <c r="G16" s="13" t="n">
+        <v>975</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
+        <v>34489</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>33514</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>31979</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="14" t="n">
         <v>30463</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>63552</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>44254</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>70609</v>
+      <c r="S16" s="11" t="n">
+        <v>-32000</v>
       </c>
     </row>
     <row r="17">
@@ -1621,13 +1621,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
-        <v>109678</v>
+      <c r="C17" s="13" t="n">
+        <v>41958</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,53 +1635,53 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>39069</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>73958</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-32000</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>594360</v>
+      </c>
+      <c r="K17" s="14" t="n">
+        <v>626360</v>
+      </c>
+      <c r="L17" s="14" t="n">
+        <v>555751</v>
+      </c>
+      <c r="M17" s="14" t="n">
+        <v>549436</v>
+      </c>
+      <c r="N17" s="14" t="n">
+        <v>581958</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>70609</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>626360</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>555751</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>549436</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>581958</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>467947</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-26393</v>
+      <c r="S17" s="11" t="n">
+        <v>7856</v>
       </c>
     </row>
     <row r="18">
@@ -1690,13 +1690,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C18" s="14" t="n">
-        <v>135654</v>
+      <c r="C18" s="13" t="n">
+        <v>131680</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,53 +1704,53 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>109819</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>136572</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-4892</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>96217</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>101109</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>75274</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>24124</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>198480</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>25835</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>101109</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>75274</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>24124</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>198480</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>185335</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-24015</v>
+      <c r="S18" s="11" t="n">
+        <v>96</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>399259</v>
+        <v>608026</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>399259</v>
+        <v>608026</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,7 +1786,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
+      <c r="Q19" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>13759</v>
+      <c r="S19" s="13" t="n">
+        <v>1696</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q20" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="14" t="n">
-        <v>-4067</v>
+      <c r="S20" s="11" t="n">
+        <v>1340</v>
       </c>
     </row>
     <row r="21">
@@ -1881,15 +1881,15 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>46539</v>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
+        <v>10390</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
-        <v>7402</v>
+      <c r="E21" s="13" t="n">
+        <v>3540</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,36 +1897,36 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>39137</v>
+        <v>6850</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
+        <v>3161018</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3154168</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>3115031</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="14" t="n">
         <v>3049155</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>3080175</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3076187</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-68530</v>
+      <c r="S21" s="11" t="n">
+        <v>162095</v>
       </c>
     </row>
     <row r="22">
@@ -1950,52 +1950,52 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>8251</v>
-      </c>
-      <c r="D22" s="13" t="inlineStr">
+        <v>6135</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
-        <v>20291</v>
-      </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="E22" s="13" t="n">
+        <v>33747</v>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="14" t="n">
-        <v>-12040</v>
+      <c r="G22" s="13" t="n">
+        <v>-27612</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
+        <v>-4163984</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4136372</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4124332</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4100306</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4115835</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4118979</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>25835</v>
+      <c r="S22" s="11" t="n">
+        <v>-4892</v>
       </c>
     </row>
     <row r="23">
@@ -2013,58 +2013,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>-4816</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>12839</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
-        <v>21577</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-26393</v>
+      <c r="E23" s="13" t="n">
+        <v>4983</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>7856</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
+        <v>549226</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>541370</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>567763</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="14" t="n">
         <v>600618</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>683816</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>681759</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-704</v>
+      <c r="S23" s="11" t="n">
+        <v>12906</v>
       </c>
     </row>
     <row r="24">
@@ -2088,52 +2088,52 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>12283</v>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
+        <v>14992</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
-        <v>12987</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G24" s="14" t="n">
-        <v>-704</v>
+      <c r="E24" s="13" t="n">
+        <v>2086</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>12906</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
+        <v>453740</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>440834</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>441538</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="14" t="n">
         <v>450533</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>351844</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>361033</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="14" t="n">
-        <v>-65602</v>
+      <c r="S24" s="11" t="n">
+        <v>1387</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>62257</v>
+        <v>44356</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>62257</v>
+        <v>44356</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>37052</v>
+      <c r="S25" s="11" t="n">
+        <v>-16062</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2255,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>221364</v>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
+        <v>109815</v>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
-        <v>109235</v>
+      <c r="E27" s="13" t="n">
+        <v>77327</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2271,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>112129</v>
+        <v>32488</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
+        <v>571811</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>539323</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>427194</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="14" t="n">
         <v>323137</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>994910</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>1097753</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2306,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>150</v>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
-        <v>22662</v>
-      </c>
-      <c r="F28" s="13" t="inlineStr">
+      <c r="E28" s="13" t="n">
+        <v>33971</v>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="14" t="n">
-        <v>-22512</v>
+      <c r="G28" s="13" t="n">
+        <v>-33971</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
+        <v>-206949</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-172978</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>-150466</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="14" t="n">
         <v>-105544</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>-367372</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-360965</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2365,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>6974</v>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+        <v>13660</v>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
-        <v>30989</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>-24015</v>
+      <c r="E29" s="13" t="n">
+        <v>13564</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>96</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
+        <v>-103043</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-103139</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>-79124</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="14" t="n">
         <v>-66057</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>-237577</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-234569</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 27-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 28-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2424,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>54113</v>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
+        <v>71915</v>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="14" t="n">
-        <v>119715</v>
-      </c>
-      <c r="F30" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G30" s="14" t="n">
-        <v>-65602</v>
+      <c r="E30" s="13" t="n">
+        <v>70528</v>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n">
+        <v>1387</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="12" t="n">
+      <c r="J30" s="14" t="n">
+        <v>-261819</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-263206</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <v>-197604</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="14" t="n">
         <v>-151536</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="14" t="n">
         <v>-389961</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-502219</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24277.6</v>
+        <v>24122.6</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24297.45</v>
+        <v>24188.3</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>282601</v>
+        <v>195390</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>282601</v>
+        <v>195390</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24090.85</v>
+        <v>24076.85</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24090.85</v>
+        <v>24175.65</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24435.18333333333</v>
+        <v>24328.46666666666</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24125.28333333333</v>
+        <v>24161.29166666666</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2597,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="14" t="n">
-        <v>72664</v>
+      <c r="C33" s="13" t="n">
+        <v>46059</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,43 +2611,43 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>124027</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-51363</v>
+        <v>30928</v>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="n">
+        <v>15131</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="12" t="n">
+      <c r="J33" s="14" t="n">
+        <v>-341070</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-356201</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="14" t="n">
         <v>-304838</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="14" t="n">
         <v>-252826</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="14" t="n">
         <v>-320455</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-324552</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24366.31666666667</v>
+        <v>24258.38333333333</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24159.71666666666</v>
+        <v>24146.93333333333</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2664,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="13" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="14" t="n">
-        <v>1300</v>
+      <c r="C34" s="13" t="n">
+        <v>0</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,43 +2678,43 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>748</v>
-      </c>
-      <c r="F34" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="14" t="n">
-        <v>552</v>
+        <v>765</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>-765</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="12" t="n">
+      <c r="J34" s="14" t="n">
+        <v>29229</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>29994</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="14" t="n">
         <v>29442</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="14" t="n">
         <v>23275</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="14" t="n">
         <v>26151</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>22037</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24228.58333333333</v>
+        <v>24217.01666666666</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24194.15</v>
+        <v>24132.575</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2731,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="13" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="14" t="n">
-        <v>25628</v>
+      <c r="C35" s="13" t="n">
+        <v>15411</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2745,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>11869</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
+        <v>13715</v>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="14" t="n">
-        <v>13759</v>
+      <c r="G35" s="13" t="n">
+        <v>1696</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="12" t="n">
+      <c r="J35" s="14" t="n">
+        <v>76550</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>74854</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="14" t="n">
         <v>61095</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="14" t="n">
         <v>63426</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="14" t="n">
         <v>152299</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>160015</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24159.71666666666</v>
+        <v>24146.93333333333</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2792,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="14" t="n">
-        <v>93409</v>
+      <c r="C36" s="13" t="n">
+        <v>30663</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2806,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>56357</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>37052</v>
+        <v>46725</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-16062</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="12" t="n">
+      <c r="J36" s="14" t="n">
+        <v>235291</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>251353</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="14" t="n">
         <v>214301</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="14" t="n">
         <v>166125</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="14" t="n">
         <v>142005</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>142500</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24021.98333333333</v>
+        <v>24105.56666666666</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>193001</v>
+        <v>92133</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>193001</v>
+        <v>92133</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23953.11666666666</v>
+        <v>24035.48333333333</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23815.38333333332</v>
+        <v>23994.11666666666</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.07</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>10.57</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.08</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.53</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.2</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.009662619345433</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.005678413660525</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.010104864602446</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.014881725047644</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.009644797702047</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.01059871674965</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,091    PCR(OI) 0.59    Max Pain 24,200</t>
+          <t>Spot 24,176    PCR(OI) 0.78    Max Pain 24,200</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23944.28548387097</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23954.82459677419</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23965.5810483871</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23977.72016129032</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23987.6935483871</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23997.65564516129</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24175.65</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24090.85</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24207.75</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24334.55</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24219.05</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24252</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3136,18 +3136,18 @@
       <c r="P45" s="28" t="n">
         <v>24300</v>
       </c>
-      <c r="Q45" s="12" t="n">
-        <v>203330</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>67241</v>
-      </c>
-      <c r="S45" s="12" t="n">
-        <v>2217212</v>
+      <c r="Q45" s="14" t="n">
+        <v>201210</v>
+      </c>
+      <c r="R45" s="13" t="n">
+        <v>-2120</v>
+      </c>
+      <c r="S45" s="14" t="n">
+        <v>3905932</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.989922493502906</v>
+        <v>0.9933791141865997</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9970635633790684</v>
@@ -3173,20 +3173,20 @@
         <v>1.004556069227693</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24400</v>
-      </c>
-      <c r="Q46" s="12" t="n">
-        <v>188213</v>
+        <v>24500</v>
+      </c>
+      <c r="Q46" s="14" t="n">
+        <v>197870</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>54409</v>
-      </c>
-      <c r="S46" s="12" t="n">
-        <v>1402679</v>
+        <v>4977</v>
+      </c>
+      <c r="S46" s="14" t="n">
+        <v>2225944</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24336.09717741935</v>
+        <v>24336.7810483871</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24323.42419354839</v>
@@ -3212,20 +3212,20 @@
         <v>24273.01048387097</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q47" s="12" t="n">
-        <v>192893</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>33017</v>
-      </c>
-      <c r="S47" s="12" t="n">
-        <v>1311554</v>
+        <v>25000</v>
+      </c>
+      <c r="Q47" s="14" t="n">
+        <v>161658</v>
+      </c>
+      <c r="R47" s="13" t="n">
+        <v>-12667</v>
+      </c>
+      <c r="S47" s="14" t="n">
+        <v>883680</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24090.85</v>
+        <v>24175.65</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24252</v>
@@ -3266,27 +3266,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="30" t="inlineStr">
-        <is>
-          <t>27-Aug-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="30" t="inlineStr">
+      <c r="J49" s="29" t="inlineStr">
+        <is>
+          <t>28-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="30" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="30" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="30" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>31-Jul-2026</t>
         </is>
@@ -3319,65 +3319,65 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>24000</v>
-      </c>
-      <c r="Q50" s="12" t="n">
-        <v>109318</v>
+        <v>24200</v>
+      </c>
+      <c r="Q50" s="14" t="n">
+        <v>122754</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>22627</v>
-      </c>
-      <c r="S50" s="12" t="n">
-        <v>1698841</v>
+        <v>21576</v>
+      </c>
+      <c r="S50" s="14" t="n">
+        <v>4914187</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>23800</v>
-      </c>
-      <c r="Q51" s="12" t="n">
-        <v>97609</v>
+        <v>24100</v>
+      </c>
+      <c r="Q51" s="14" t="n">
+        <v>152558</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>27506</v>
-      </c>
-      <c r="S51" s="12" t="n">
-        <v>706345</v>
+        <v>68375</v>
+      </c>
+      <c r="S51" s="14" t="n">
+        <v>7597655</v>
       </c>
       <c r="T51" s="33" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>23500</v>
-      </c>
-      <c r="Q52" s="12" t="n">
-        <v>107092</v>
+        <v>24000</v>
+      </c>
+      <c r="Q52" s="14" t="n">
+        <v>157877</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>24339</v>
-      </c>
-      <c r="S52" s="12" t="n">
-        <v>467606</v>
-      </c>
-      <c r="T52" s="33" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>48559</v>
+      </c>
+      <c r="S52" s="14" t="n">
+        <v>4451756</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 27-Aug-2026    1 DAY AGO = 26-Aug-2026    2 DAYS AGO = 25-Aug-2026    3 DAYS AGO = 24-Aug-2026    4 DAYS AGO = 21-Aug-2026    (generated 27-Aug-2026 20:42 IST)</t>
+          <t>TODAY = 28-Aug-2026    1 DAY AGO = 27-Aug-2026    2 DAYS AGO = 26-Aug-2026    3 DAYS AGO = 25-Aug-2026    4 DAYS AGO = 24-Aug-2026    (generated 28-Aug-2026 20:34 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-08-31
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>2801</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>3851</v>
+        <v>3044</v>
       </c>
       <c r="D3" s="12" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="13" t="n">
-        <v>1050</v>
+        <v>1784</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>2801</v>
+        <v>1260</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="14" t="n">
+        <v>178219</v>
+      </c>
+      <c r="K3" s="14" t="n">
         <v>176959</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="14" t="n">
         <v>174158</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="14" t="n">
         <v>160283</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="14" t="n">
         <v>157636</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>181156</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q3" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="13" t="n">
-        <v>-197956</v>
+      <c r="S3" s="11" t="n">
+        <v>104485</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>4100</v>
+        <v>75</v>
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
@@ -782,7 +782,7 @@
         </is>
       </c>
       <c r="E4" s="13" t="n">
-        <v>3400</v>
+        <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>700</v>
+        <v>75</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
@@ -798,20 +798,20 @@
         </is>
       </c>
       <c r="J4" s="14" t="n">
+        <v>20288</v>
+      </c>
+      <c r="K4" s="14" t="n">
         <v>20213</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="14" t="n">
         <v>19513</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="14" t="n">
         <v>17589</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="14" t="n">
         <v>17342</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>25020</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -828,7 +828,7 @@
         </is>
       </c>
       <c r="S4" s="13" t="n">
-        <v>35917</v>
+        <v>39020</v>
       </c>
     </row>
     <row r="5">
@@ -837,13 +837,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>-33</v>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="n">
+        <v>38</v>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>4808</v>
+        <v>6720</v>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="13" t="n">
-        <v>-4841</v>
+        <v>-6682</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="14" t="n">
+        <v>-209315</v>
+      </c>
+      <c r="K5" s="14" t="n">
         <v>-202633</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="14" t="n">
         <v>-197792</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="14" t="n">
         <v>-186060</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="14" t="n">
         <v>-184227</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-219383</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>6850</v>
+        <v>31605</v>
       </c>
     </row>
     <row r="6">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1127</v>
+        <v>3177</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-213</v>
+        <v>-2170</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>1340</v>
+        <v>5347</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="14" t="n">
+        <v>10808</v>
+      </c>
+      <c r="K6" s="14" t="n">
         <v>5461</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="14" t="n">
         <v>4121</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="14" t="n">
         <v>8188</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="14" t="n">
         <v>9249</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>13207</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>32488</v>
+        <v>137004</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>9045</v>
+        <v>6334</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>9045</v>
+        <v>6334</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="13" t="n">
-        <v>15131</v>
+      <c r="S7" s="11" t="n">
+        <v>-20348</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>700</v>
+        <v>75</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="n">
-        <v>-44242</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>449744</v>
       </c>
       <c r="D9" s="12" t="inlineStr">
         <is>
@@ -1105,53 +1105,53 @@
         </is>
       </c>
       <c r="E9" s="13" t="n">
-        <v>153714</v>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
+        <v>345259</v>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="n">
+        <v>104485</v>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>195682</v>
+      </c>
+      <c r="K9" s="14" t="n">
+        <v>91197</v>
+      </c>
+      <c r="L9" s="14" t="n">
+        <v>289153</v>
+      </c>
+      <c r="M9" s="14" t="n">
+        <v>191071</v>
+      </c>
+      <c r="N9" s="14" t="n">
+        <v>94693</v>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q9" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
-        <v>-197956</v>
-      </c>
-      <c r="I9" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J9" s="14" t="n">
-        <v>91197</v>
-      </c>
-      <c r="K9" s="14" t="n">
-        <v>289153</v>
-      </c>
-      <c r="L9" s="14" t="n">
-        <v>191071</v>
-      </c>
-      <c r="M9" s="14" t="n">
-        <v>94693</v>
-      </c>
-      <c r="N9" s="14" t="n">
-        <v>227012</v>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R9" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>25</v>
+      <c r="S9" s="13" t="n">
+        <v>-40</v>
       </c>
     </row>
     <row r="10">
@@ -1168,21 +1168,21 @@
       <c r="C10" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-25</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>25</v>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>40</v>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="13" t="n">
+        <v>-40</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,28 +1190,28 @@
         </is>
       </c>
       <c r="J10" s="14" t="n">
+        <v>4310</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>4350</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="14" t="n">
         <v>4325</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="14" t="n">
         <v>3905</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="14" t="n">
         <v>3935</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>8009</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="13" t="n">
-        <v>975</v>
+      <c r="S10" s="11" t="n">
+        <v>-2705</v>
       </c>
     </row>
     <row r="11">
@@ -1235,15 +1235,15 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>34995</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-841</v>
+        <v>109975</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>105417</v>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="11" t="n">
-        <v>35836</v>
+        <v>4558</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="14" t="n">
+        <v>-225462</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>-230020</v>
       </c>
-      <c r="K11" s="14" t="n">
+      <c r="L11" s="14" t="n">
         <v>-265856</v>
       </c>
-      <c r="L11" s="14" t="n">
+      <c r="M11" s="14" t="n">
         <v>-235885</v>
       </c>
-      <c r="M11" s="14" t="n">
+      <c r="N11" s="14" t="n">
         <v>-198430</v>
       </c>
-      <c r="N11" s="14" t="n">
-        <v>-199680</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="13" t="n">
-        <v>-27612</v>
+        <v>-56855</v>
       </c>
     </row>
     <row r="12">
@@ -1304,23 +1304,23 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>103687</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-58408</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>162095</v>
+        <v>65630</v>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n">
+        <v>174632</v>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="n">
+        <v>-109002</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="14" t="n">
+        <v>25471</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <v>134473</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="14" t="n">
         <v>-27622</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="14" t="n">
         <v>40908</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="14" t="n">
         <v>99801</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>-35340</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="13" t="n">
-        <v>-33971</v>
+        <v>-26033</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>94440</v>
+        <v>625349</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>94440</v>
+        <v>625348</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1394,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q13" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1404,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="11" t="n">
-        <v>-765</v>
+      <c r="S13" s="13" t="n">
+        <v>282</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="13" t="n">
-        <v>-4841</v>
+        <v>-6682</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="13" t="n">
-        <v>433413</v>
+        <v>441033</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>397496</v>
+        <v>402013</v>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
@@ -1505,7 +1505,7 @@
         </is>
       </c>
       <c r="G15" s="13" t="n">
-        <v>35917</v>
+        <v>39020</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="14" t="n">
+        <v>-686046</v>
+      </c>
+      <c r="K15" s="14" t="n">
         <v>-725066</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="14" t="n">
         <v>-760983</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="14" t="n">
         <v>-663004</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="14" t="n">
         <v>-604022</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-843989</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="11" t="n">
-        <v>35836</v>
+        <v>4558</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="13" t="n">
-        <v>975</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-2705</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,13 +1568,13 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="13" t="n">
-        <v>975</v>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-2705</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,20 +1582,20 @@
         </is>
       </c>
       <c r="J16" s="14" t="n">
+        <v>31784</v>
+      </c>
+      <c r="K16" s="14" t="n">
         <v>34489</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="14" t="n">
         <v>33514</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="14" t="n">
         <v>31979</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="14" t="n">
         <v>30463</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>63552</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1612,7 +1612,7 @@
         </is>
       </c>
       <c r="S16" s="11" t="n">
-        <v>-32000</v>
+        <v>-42953</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="13" t="n">
-        <v>41958</v>
+        <v>56808</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>73958</v>
+        <v>99761</v>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="G17" s="11" t="n">
-        <v>-32000</v>
+        <v>-42953</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="14" t="n">
+        <v>551407</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <v>594360</v>
       </c>
-      <c r="K17" s="14" t="n">
+      <c r="L17" s="14" t="n">
         <v>626360</v>
       </c>
-      <c r="L17" s="14" t="n">
+      <c r="M17" s="14" t="n">
         <v>555751</v>
       </c>
-      <c r="M17" s="14" t="n">
+      <c r="N17" s="14" t="n">
         <v>549436</v>
       </c>
-      <c r="N17" s="14" t="n">
-        <v>581958</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>7856</v>
+        <v>14654</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="13" t="n">
-        <v>131680</v>
+        <v>155914</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,53 +1704,53 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>136572</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>149276</v>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>6638</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="14" t="n">
+        <v>102855</v>
+      </c>
+      <c r="K18" s="14" t="n">
+        <v>96217</v>
+      </c>
+      <c r="L18" s="14" t="n">
+        <v>101109</v>
+      </c>
+      <c r="M18" s="14" t="n">
+        <v>75274</v>
+      </c>
+      <c r="N18" s="14" t="n">
+        <v>24124</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="12" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-4892</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="14" t="n">
-        <v>96217</v>
-      </c>
-      <c r="K18" s="14" t="n">
-        <v>101109</v>
-      </c>
-      <c r="L18" s="14" t="n">
-        <v>75274</v>
-      </c>
-      <c r="M18" s="14" t="n">
-        <v>24124</v>
-      </c>
-      <c r="N18" s="14" t="n">
-        <v>198480</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="11" t="n">
-        <v>96</v>
+      <c r="S18" s="13" t="n">
+        <v>-36008</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>608026</v>
+        <v>651050</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>608026</v>
+        <v>651050</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="13" t="n">
-        <v>1696</v>
+        <v>15923</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>1340</v>
+        <v>5347</v>
       </c>
     </row>
     <row r="21">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>10390</v>
+        <v>33152</v>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="E21" s="13" t="n">
-        <v>3540</v>
+        <v>1547</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>6850</v>
+        <v>31605</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="14" t="n">
+        <v>3192623</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <v>3161018</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="14" t="n">
         <v>3154168</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="14" t="n">
         <v>3115031</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="14" t="n">
         <v>3049155</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3080175</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q21" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>162095</v>
+      <c r="S21" s="13" t="n">
+        <v>-109002</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>6135</v>
+        <v>8281</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>33747</v>
+        <v>65136</v>
       </c>
       <c r="F22" s="12" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="13" t="n">
-        <v>-27612</v>
+        <v>-56855</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="14" t="n">
+        <v>-4220839</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <v>-4163984</v>
       </c>
-      <c r="K22" s="14" t="n">
+      <c r="L22" s="14" t="n">
         <v>-4136372</v>
       </c>
-      <c r="L22" s="14" t="n">
+      <c r="M22" s="14" t="n">
         <v>-4124332</v>
       </c>
-      <c r="M22" s="14" t="n">
+      <c r="N22" s="14" t="n">
         <v>-4100306</v>
       </c>
-      <c r="N22" s="14" t="n">
-        <v>-4115835</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-4892</v>
+      <c r="S22" s="13" t="n">
+        <v>6638</v>
       </c>
     </row>
     <row r="23">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>12839</v>
+        <v>27049</v>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="13" t="n">
-        <v>4983</v>
+        <v>12395</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>7856</v>
+        <v>14654</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,20 +2043,20 @@
         </is>
       </c>
       <c r="J23" s="14" t="n">
+        <v>563880</v>
+      </c>
+      <c r="K23" s="14" t="n">
         <v>549226</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="14" t="n">
         <v>541370</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="14" t="n">
         <v>567763</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="14" t="n">
         <v>600618</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>683816</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2073,7 +2073,7 @@
         </is>
       </c>
       <c r="S23" s="11" t="n">
-        <v>12906</v>
+        <v>10596</v>
       </c>
     </row>
     <row r="24">
@@ -2088,7 +2088,7 @@
         </is>
       </c>
       <c r="C24" s="11" t="n">
-        <v>14992</v>
+        <v>19892</v>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="E24" s="13" t="n">
-        <v>2086</v>
+        <v>9296</v>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
@@ -2104,7 +2104,7 @@
         </is>
       </c>
       <c r="G24" s="11" t="n">
-        <v>12906</v>
+        <v>10596</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,28 +2112,28 @@
         </is>
       </c>
       <c r="J24" s="14" t="n">
+        <v>464336</v>
+      </c>
+      <c r="K24" s="14" t="n">
         <v>453740</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="14" t="n">
         <v>440834</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="14" t="n">
         <v>441538</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="14" t="n">
         <v>450533</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>351844</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q24" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R24" s="10" t="inlineStr">
@@ -2141,8 +2141,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="11" t="n">
-        <v>1387</v>
+      <c r="S24" s="13" t="n">
+        <v>-74963</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>44356</v>
+        <v>88374</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>44356</v>
+        <v>88374</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-16062</v>
+      <c r="S25" s="13" t="n">
+        <v>4143</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>109815</v>
+        <v>186028</v>
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="13" t="n">
-        <v>77327</v>
+        <v>49024</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>32488</v>
+        <v>137004</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="14" t="n">
+        <v>708815</v>
+      </c>
+      <c r="K27" s="14" t="n">
         <v>571811</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="14" t="n">
         <v>539323</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="14" t="n">
         <v>427194</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="14" t="n">
         <v>323137</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>994910</v>
       </c>
     </row>
     <row r="28">
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>33971</v>
+        <v>26033</v>
       </c>
       <c r="F28" s="12" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="13" t="n">
-        <v>-33971</v>
+        <v>-26033</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="14" t="n">
+        <v>-232982</v>
+      </c>
+      <c r="K28" s="14" t="n">
         <v>-206949</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="14" t="n">
         <v>-172978</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="14" t="n">
         <v>-150466</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="14" t="n">
         <v>-105544</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-367372</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>13660</v>
+        <v>5604</v>
       </c>
       <c r="D29" s="12" t="inlineStr">
         <is>
@@ -2373,15 +2373,15 @@
         </is>
       </c>
       <c r="E29" s="13" t="n">
-        <v>13564</v>
-      </c>
-      <c r="F29" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G29" s="11" t="n">
-        <v>96</v>
+        <v>41612</v>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="n">
+        <v>-36008</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="14" t="n">
+        <v>-139051</v>
+      </c>
+      <c r="K29" s="14" t="n">
         <v>-103043</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="14" t="n">
         <v>-103139</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="14" t="n">
         <v>-79124</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="14" t="n">
         <v>-66057</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-237577</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 28-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 31-Aug-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>71915</v>
+        <v>19809</v>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
@@ -2432,15 +2432,15 @@
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>70528</v>
-      </c>
-      <c r="F30" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="n">
-        <v>1387</v>
+        <v>94772</v>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G30" s="13" t="n">
+        <v>-74963</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="14" t="n">
+        <v>-336782</v>
+      </c>
+      <c r="K30" s="14" t="n">
         <v>-261819</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="14" t="n">
         <v>-263206</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="14" t="n">
         <v>-197604</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="14" t="n">
         <v>-151536</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-389961</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24122.6</v>
+        <v>24117.55</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24188.3</v>
+        <v>24128.7</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>195390</v>
+        <v>211441</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>195390</v>
+        <v>211441</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>24076.85</v>
+        <v>23993.6</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24175.65</v>
+        <v>24080.4</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24328.46666666666</v>
+        <v>24276.63333333334</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24161.29166666666</v>
+        <v>24073.98333333334</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="13" t="n">
-        <v>46059</v>
+        <v>16039</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>30928</v>
-      </c>
-      <c r="F33" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="n">
-        <v>15131</v>
+        <v>36387</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-20348</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="14" t="n">
+        <v>-361418</v>
+      </c>
+      <c r="K33" s="14" t="n">
         <v>-341070</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="14" t="n">
         <v>-356201</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="14" t="n">
         <v>-304838</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="14" t="n">
         <v>-252826</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-320455</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24258.38333333333</v>
+        <v>24202.66666666667</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24146.93333333333</v>
+        <v>24067.56666666667</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="13" t="n">
-        <v>0</v>
+        <v>2480</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,15 +2678,15 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>765</v>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G34" s="11" t="n">
-        <v>-765</v>
+        <v>2198</v>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="n">
+        <v>282</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="14" t="n">
+        <v>29511</v>
+      </c>
+      <c r="K34" s="14" t="n">
         <v>29229</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="14" t="n">
         <v>29994</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="14" t="n">
         <v>29442</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="14" t="n">
         <v>23275</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>26151</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24217.01666666666</v>
+        <v>24141.53333333334</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24132.575</v>
+        <v>24061.15</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="13" t="n">
-        <v>15411</v>
+        <v>27742</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>13715</v>
+        <v>11819</v>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="13" t="n">
-        <v>1696</v>
+        <v>15923</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="14" t="n">
+        <v>92473</v>
+      </c>
+      <c r="K35" s="14" t="n">
         <v>76550</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="14" t="n">
         <v>74854</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="14" t="n">
         <v>61095</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="14" t="n">
         <v>63426</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>152299</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24146.93333333333</v>
+        <v>24067.56666666667</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="13" t="n">
-        <v>30663</v>
+        <v>36820</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>46725</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-16062</v>
+        <v>32677</v>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="13" t="n">
+        <v>4143</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="14" t="n">
+        <v>239434</v>
+      </c>
+      <c r="K36" s="14" t="n">
         <v>235291</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="14" t="n">
         <v>251353</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="14" t="n">
         <v>214301</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="14" t="n">
         <v>166125</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>142005</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24105.56666666666</v>
+        <v>24006.43333333334</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>92133</v>
+        <v>83081</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>92133</v>
+        <v>83081</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>24035.48333333333</v>
+        <v>23932.46666666667</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23994.11666666666</v>
+        <v>23871.33333333334</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.19</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.07</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>10.57</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.08</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.53</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.006164539061341</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.009662619345433</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.005678413660525</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.010104864602446</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.014881725047644</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.009644797702047</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,176    PCR(OI) 0.78    Max Pain 24,200</t>
+          <t>Spot 24,080    PCR(OI) 0.81    Max Pain 24,100</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23932.86491935484</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23944.28548387097</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23954.82459677419</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23965.5810483871</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23977.72016129032</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23987.6935483871</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24080.4</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24090.85</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24207.75</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24334.55</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24219.05</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24300</v>
+        <v>24200</v>
       </c>
       <c r="Q45" s="14" t="n">
-        <v>201210</v>
-      </c>
-      <c r="R45" s="13" t="n">
-        <v>-2120</v>
+        <v>200604</v>
+      </c>
+      <c r="R45" s="11" t="n">
+        <v>60758</v>
       </c>
       <c r="S45" s="14" t="n">
-        <v>3905932</v>
+        <v>6612183</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,35 +3158,35 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
+        <v>0.9888317666598201</v>
+      </c>
+      <c r="K46" s="25" t="n">
         <v>0.9933791141865997</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="L46" s="25" t="n">
         <v>0.9970635633790684</v>
       </c>
-      <c r="L46" s="25" t="n">
+      <c r="M46" s="25" t="n">
         <v>1.002328084679025</v>
       </c>
-      <c r="M46" s="25" t="n">
+      <c r="N46" s="25" t="n">
         <v>1.011430829957649</v>
       </c>
-      <c r="N46" s="25" t="n">
-        <v>1.004556069227693</v>
-      </c>
       <c r="P46" s="28" t="n">
-        <v>24500</v>
+        <v>24300</v>
       </c>
       <c r="Q46" s="14" t="n">
-        <v>197870</v>
+        <v>228704</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>4977</v>
+        <v>27494</v>
       </c>
       <c r="S46" s="14" t="n">
-        <v>2225944</v>
-      </c>
-      <c r="T46" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>4521751</v>
+      </c>
+      <c r="T46" s="29" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3197,31 +3197,31 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
+        <v>24352.37298387097</v>
+      </c>
+      <c r="K47" s="18" t="n">
         <v>24336.7810483871</v>
       </c>
-      <c r="K47" s="18" t="n">
+      <c r="L47" s="18" t="n">
         <v>24323.42419354839</v>
       </c>
-      <c r="L47" s="18" t="n">
+      <c r="M47" s="18" t="n">
         <v>24309.40564516129</v>
       </c>
-      <c r="M47" s="18" t="n">
+      <c r="N47" s="18" t="n">
         <v>24292.96129032258</v>
       </c>
-      <c r="N47" s="18" t="n">
-        <v>24273.01048387097</v>
-      </c>
       <c r="P47" s="28" t="n">
-        <v>25000</v>
+        <v>24500</v>
       </c>
       <c r="Q47" s="14" t="n">
-        <v>161658</v>
-      </c>
-      <c r="R47" s="13" t="n">
-        <v>-12667</v>
+        <v>262486</v>
+      </c>
+      <c r="R47" s="11" t="n">
+        <v>64616</v>
       </c>
       <c r="S47" s="14" t="n">
-        <v>883680</v>
+        <v>2499631</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
@@ -3236,19 +3236,19 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
+        <v>24080.4</v>
+      </c>
+      <c r="K48" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="K48" s="18" t="n">
+      <c r="L48" s="18" t="n">
         <v>24252</v>
       </c>
-      <c r="L48" s="18" t="n">
+      <c r="M48" s="18" t="n">
         <v>24366</v>
       </c>
-      <c r="M48" s="18" t="n">
+      <c r="N48" s="18" t="n">
         <v>24570.65</v>
-      </c>
-      <c r="N48" s="18" t="n">
-        <v>24383.6</v>
       </c>
       <c r="P48" s="31" t="inlineStr">
         <is>
@@ -3268,27 +3268,27 @@
       </c>
       <c r="J49" s="29" t="inlineStr">
         <is>
+          <t>31-Aug-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="29" t="inlineStr">
+        <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="L49" s="29" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="M49" s="29" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="N49" s="29" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
-        </is>
-      </c>
-      <c r="N49" s="29" t="inlineStr">
-        <is>
-          <t>31-Jul-2026</t>
         </is>
       </c>
       <c r="P49" s="27" t="inlineStr">
@@ -3319,35 +3319,35 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>24200</v>
+        <v>24100</v>
       </c>
       <c r="Q50" s="14" t="n">
-        <v>122754</v>
+        <v>160251</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>21576</v>
+        <v>7693</v>
       </c>
       <c r="S50" s="14" t="n">
-        <v>4914187</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>8664178</v>
+      </c>
+      <c r="T50" s="33" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="32" t="n">
-        <v>24100</v>
+        <v>24000</v>
       </c>
       <c r="Q51" s="14" t="n">
-        <v>152558</v>
+        <v>262269</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>68375</v>
+        <v>104392</v>
       </c>
       <c r="S51" s="14" t="n">
-        <v>7597655</v>
+        <v>11947246</v>
       </c>
       <c r="T51" s="33" t="inlineStr">
         <is>
@@ -3357,27 +3357,27 @@
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>24000</v>
+        <v>23800</v>
       </c>
       <c r="Q52" s="14" t="n">
-        <v>157877</v>
+        <v>147168</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>48559</v>
+        <v>32920</v>
       </c>
       <c r="S52" s="14" t="n">
-        <v>4451756</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>3187671</v>
+      </c>
+      <c r="T52" s="30" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 28-Aug-2026    1 DAY AGO = 27-Aug-2026    2 DAYS AGO = 26-Aug-2026    3 DAYS AGO = 25-Aug-2026    4 DAYS AGO = 24-Aug-2026    (generated 28-Aug-2026 20:34 IST)</t>
+          <t>TODAY = 31-Aug-2026    1 DAY AGO = 28-Aug-2026    2 DAYS AGO = 27-Aug-2026    3 DAYS AGO = 26-Aug-2026    4 DAYS AGO = 25-Aug-2026    (generated 31-Aug-2026 21:27 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-01
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -138,13 +138,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -187,10 +187,10 @@
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -198,9 +198,6 @@
     </xf>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -690,7 +687,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>1260</v>
+        <v>8911</v>
       </c>
     </row>
     <row r="3">
@@ -705,15 +702,15 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>3044</v>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="n">
-        <v>1784</v>
+        <v>8720</v>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>-191</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,28 +718,28 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>1260</v>
+        <v>8911</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J3" s="14" t="n">
+      <c r="J3" s="12" t="n">
+        <v>187130</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>178219</v>
       </c>
-      <c r="K3" s="14" t="n">
+      <c r="L3" s="12" t="n">
         <v>176959</v>
       </c>
-      <c r="L3" s="14" t="n">
+      <c r="M3" s="12" t="n">
         <v>174158</v>
       </c>
-      <c r="M3" s="14" t="n">
+      <c r="N3" s="12" t="n">
         <v>160283</v>
       </c>
-      <c r="N3" s="14" t="n">
-        <v>157636</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +756,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>104485</v>
+        <v>66301</v>
       </c>
     </row>
     <row r="4">
@@ -774,14 +771,14 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>75</v>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
+        <v>189</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E4" s="13" t="n">
+      <c r="E4" s="14" t="n">
         <v>0</v>
       </c>
       <c r="F4" s="9" t="inlineStr">
@@ -790,36 +787,36 @@
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>75</v>
+        <v>189</v>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J4" s="14" t="n">
+      <c r="J4" s="12" t="n">
+        <v>20477</v>
+      </c>
+      <c r="K4" s="12" t="n">
         <v>20288</v>
       </c>
-      <c r="K4" s="14" t="n">
+      <c r="L4" s="12" t="n">
         <v>20213</v>
       </c>
-      <c r="L4" s="14" t="n">
+      <c r="M4" s="12" t="n">
         <v>19513</v>
       </c>
-      <c r="M4" s="14" t="n">
+      <c r="N4" s="12" t="n">
         <v>17589</v>
       </c>
-      <c r="N4" s="14" t="n">
-        <v>17342</v>
-      </c>
       <c r="P4" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q4" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q4" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R4" s="10" t="inlineStr">
@@ -827,8 +824,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="13" t="n">
-        <v>39020</v>
+      <c r="S4" s="11" t="n">
+        <v>-70902</v>
       </c>
     </row>
     <row r="5">
@@ -843,52 +840,52 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>38</v>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
+        <v>523</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
-        <v>6720</v>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="E5" s="14" t="n">
+        <v>13240</v>
+      </c>
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G5" s="13" t="n">
-        <v>-6682</v>
+      <c r="G5" s="14" t="n">
+        <v>-12717</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J5" s="14" t="n">
+      <c r="J5" s="12" t="n">
+        <v>-222032</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-209315</v>
       </c>
-      <c r="K5" s="14" t="n">
+      <c r="L5" s="12" t="n">
         <v>-202633</v>
       </c>
-      <c r="L5" s="14" t="n">
+      <c r="M5" s="12" t="n">
         <v>-197792</v>
       </c>
-      <c r="M5" s="14" t="n">
+      <c r="N5" s="12" t="n">
         <v>-186060</v>
       </c>
-      <c r="N5" s="14" t="n">
-        <v>-184227</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +893,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="11" t="n">
-        <v>31605</v>
+      <c r="S5" s="14" t="n">
+        <v>-7295</v>
       </c>
     </row>
     <row r="6">
@@ -906,13 +903,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>3177</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>-112</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
@@ -920,7 +917,7 @@
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>-2170</v>
+        <v>-3729</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -928,28 +925,28 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>5347</v>
+        <v>3617</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J6" s="14" t="n">
+      <c r="J6" s="12" t="n">
+        <v>14425</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>10808</v>
       </c>
-      <c r="K6" s="14" t="n">
+      <c r="L6" s="12" t="n">
         <v>5461</v>
       </c>
-      <c r="L6" s="14" t="n">
+      <c r="M6" s="12" t="n">
         <v>4121</v>
       </c>
-      <c r="M6" s="14" t="n">
+      <c r="N6" s="12" t="n">
         <v>8188</v>
       </c>
-      <c r="N6" s="14" t="n">
-        <v>9249</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +963,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>137004</v>
+        <v>115146</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +974,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>6334</v>
+        <v>9320</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>6334</v>
+        <v>9320</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1013,7 +1010,7 @@
         </is>
       </c>
       <c r="S7" s="11" t="n">
-        <v>-20348</v>
+        <v>-34699</v>
       </c>
     </row>
     <row r="8">
@@ -1082,7 +1079,7 @@
         </is>
       </c>
       <c r="S8" s="11" t="n">
-        <v>75</v>
+        <v>189</v>
       </c>
     </row>
     <row r="9">
@@ -1091,21 +1088,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>449744</v>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="n">
-        <v>345259</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-1348907</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>-1415208</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1113,36 +1110,36 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>104485</v>
+        <v>66301</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J9" s="14" t="n">
+      <c r="J9" s="12" t="n">
+        <v>261983</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>195682</v>
       </c>
-      <c r="K9" s="14" t="n">
+      <c r="L9" s="12" t="n">
         <v>91197</v>
       </c>
-      <c r="L9" s="14" t="n">
+      <c r="M9" s="12" t="n">
         <v>289153</v>
       </c>
-      <c r="M9" s="14" t="n">
+      <c r="N9" s="12" t="n">
         <v>191071</v>
       </c>
-      <c r="N9" s="14" t="n">
-        <v>94693</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q9" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1150,8 +1147,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="13" t="n">
-        <v>-40</v>
+      <c r="S9" s="11" t="n">
+        <v>525</v>
       </c>
     </row>
     <row r="10">
@@ -1166,52 +1163,52 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="13" t="n">
-        <v>40</v>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G10" s="13" t="n">
-        <v>-40</v>
+        <v>500</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>-25</v>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="n">
+        <v>525</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J10" s="14" t="n">
+      <c r="J10" s="12" t="n">
+        <v>4835</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4310</v>
       </c>
-      <c r="K10" s="14" t="n">
+      <c r="L10" s="12" t="n">
         <v>4350</v>
       </c>
-      <c r="L10" s="14" t="n">
+      <c r="M10" s="12" t="n">
         <v>4325</v>
       </c>
-      <c r="M10" s="14" t="n">
+      <c r="N10" s="12" t="n">
         <v>3905</v>
       </c>
-      <c r="N10" s="14" t="n">
-        <v>3935</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1216,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-2705</v>
+      <c r="S10" s="14" t="n">
+        <v>139</v>
       </c>
     </row>
     <row r="11">
@@ -1229,67 +1226,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="n">
-        <v>109975</v>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="n">
-        <v>105417</v>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="n">
+        <v>-242134</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-219535</v>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G11" s="14" t="n">
+        <v>-22599</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-248061</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-225462</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-230020</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-265856</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-235885</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G11" s="11" t="n">
-        <v>4558</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="14" t="n">
-        <v>-225462</v>
-      </c>
-      <c r="K11" s="14" t="n">
-        <v>-230020</v>
-      </c>
-      <c r="L11" s="14" t="n">
-        <v>-265856</v>
-      </c>
-      <c r="M11" s="14" t="n">
-        <v>-235885</v>
-      </c>
-      <c r="N11" s="14" t="n">
-        <v>-198430</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="12" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="13" t="n">
-        <v>-56855</v>
+      <c r="S11" s="11" t="n">
+        <v>24958</v>
       </c>
     </row>
     <row r="12">
@@ -1298,56 +1295,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>65630</v>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="n">
-        <v>174632</v>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n">
+        <v>-378438</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-334209</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
-        <v>-109002</v>
+      <c r="G12" s="14" t="n">
+        <v>-44229</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J12" s="14" t="n">
+      <c r="J12" s="12" t="n">
+        <v>-18758</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>25471</v>
       </c>
-      <c r="K12" s="14" t="n">
+      <c r="L12" s="12" t="n">
         <v>134473</v>
       </c>
-      <c r="L12" s="14" t="n">
+      <c r="M12" s="12" t="n">
         <v>-27622</v>
       </c>
-      <c r="M12" s="14" t="n">
+      <c r="N12" s="12" t="n">
         <v>40908</v>
       </c>
-      <c r="N12" s="14" t="n">
-        <v>99801</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q12" s="12" t="inlineStr">
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1357,8 +1354,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S12" s="13" t="n">
-        <v>-26033</v>
+      <c r="S12" s="14" t="n">
+        <v>-18538</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1366,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>625349</v>
+        <v>-1968979</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>625348</v>
+        <v>-1968977</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>1</v>
+        <v>-2</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1394,9 +1391,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q13" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q13" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R13" s="10" t="inlineStr">
@@ -1404,8 +1401,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S13" s="13" t="n">
-        <v>282</v>
+      <c r="S13" s="11" t="n">
+        <v>-571</v>
       </c>
     </row>
     <row r="14">
@@ -1463,7 +1460,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q14" s="12" t="inlineStr">
+      <c r="Q14" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1473,8 +1470,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S14" s="13" t="n">
-        <v>-6682</v>
+      <c r="S14" s="14" t="n">
+        <v>-12717</v>
       </c>
     </row>
     <row r="15">
@@ -1483,58 +1480,58 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="n">
-        <v>441033</v>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="n">
-        <v>402013</v>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="13" t="n">
-        <v>39020</v>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>-1278790</v>
+      </c>
+      <c r="D15" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>-1207888</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-70902</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J15" s="14" t="n">
+      <c r="J15" s="12" t="n">
+        <v>-756948</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-686046</v>
       </c>
-      <c r="K15" s="14" t="n">
+      <c r="L15" s="12" t="n">
         <v>-725066</v>
       </c>
-      <c r="L15" s="14" t="n">
+      <c r="M15" s="12" t="n">
         <v>-760983</v>
       </c>
-      <c r="M15" s="14" t="n">
+      <c r="N15" s="12" t="n">
         <v>-663004</v>
       </c>
-      <c r="N15" s="14" t="n">
-        <v>-604022</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1539,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="11" t="n">
-        <v>4558</v>
+      <c r="S15" s="14" t="n">
+        <v>-22599</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1549,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>-2705</v>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>139</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,42 +1565,42 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>-2705</v>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>139</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J16" s="14" t="n">
+      <c r="J16" s="12" t="n">
+        <v>31923</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>31784</v>
       </c>
-      <c r="K16" s="14" t="n">
+      <c r="L16" s="12" t="n">
         <v>34489</v>
       </c>
-      <c r="L16" s="14" t="n">
+      <c r="M16" s="12" t="n">
         <v>33514</v>
       </c>
-      <c r="M16" s="14" t="n">
+      <c r="N16" s="12" t="n">
         <v>31979</v>
       </c>
-      <c r="N16" s="14" t="n">
-        <v>30463</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1608,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-42953</v>
+      <c r="S16" s="14" t="n">
+        <v>81058</v>
       </c>
     </row>
     <row r="17">
@@ -1621,67 +1618,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="13" t="n">
-        <v>56808</v>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>99761</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>-164146</v>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>-245204</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>81058</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>632465</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>551407</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>594360</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>626360</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>555751</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G17" s="11" t="n">
-        <v>-42953</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="14" t="n">
-        <v>551407</v>
-      </c>
-      <c r="K17" s="14" t="n">
-        <v>594360</v>
-      </c>
-      <c r="L17" s="14" t="n">
-        <v>626360</v>
-      </c>
-      <c r="M17" s="14" t="n">
-        <v>555751</v>
-      </c>
-      <c r="N17" s="14" t="n">
-        <v>549436</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="11" t="n">
-        <v>14654</v>
+      <c r="S17" s="14" t="n">
+        <v>-12557</v>
       </c>
     </row>
     <row r="18">
@@ -1690,56 +1687,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="13" t="n">
-        <v>155914</v>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="n">
-        <v>149276</v>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G18" s="13" t="n">
-        <v>6638</v>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>-415860</v>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>-405564</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-10296</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J18" s="14" t="n">
+      <c r="J18" s="12" t="n">
+        <v>92559</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>102855</v>
       </c>
-      <c r="K18" s="14" t="n">
+      <c r="L18" s="12" t="n">
         <v>96217</v>
       </c>
-      <c r="L18" s="14" t="n">
+      <c r="M18" s="12" t="n">
         <v>101109</v>
       </c>
-      <c r="M18" s="14" t="n">
+      <c r="N18" s="12" t="n">
         <v>75274</v>
       </c>
-      <c r="N18" s="14" t="n">
-        <v>24124</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q18" s="12" t="inlineStr">
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1749,8 +1746,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="13" t="n">
-        <v>-36008</v>
+      <c r="S18" s="14" t="n">
+        <v>-11794</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1758,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>651050</v>
+        <v>-1858657</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>651050</v>
+        <v>-1858656</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1786,7 +1783,7 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="12" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -1796,8 +1793,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="13" t="n">
-        <v>15923</v>
+      <c r="S19" s="14" t="n">
+        <v>7881</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1863,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>5347</v>
+        <v>3617</v>
       </c>
     </row>
     <row r="21">
@@ -1875,56 +1872,56 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>33152</v>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="n">
-        <v>1547</v>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>31605</v>
+      <c r="B21" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="n">
+        <v>-10789</v>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>-3494</v>
+      </c>
+      <c r="F21" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>-7295</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J21" s="14" t="n">
+      <c r="J21" s="12" t="n">
+        <v>3185328</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3192623</v>
       </c>
-      <c r="K21" s="14" t="n">
+      <c r="L21" s="12" t="n">
         <v>3161018</v>
       </c>
-      <c r="L21" s="14" t="n">
+      <c r="M21" s="12" t="n">
         <v>3154168</v>
       </c>
-      <c r="M21" s="14" t="n">
+      <c r="N21" s="12" t="n">
         <v>3115031</v>
       </c>
-      <c r="N21" s="14" t="n">
-        <v>3049155</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="12" t="inlineStr">
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -1934,8 +1931,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="13" t="n">
-        <v>-109002</v>
+      <c r="S21" s="14" t="n">
+        <v>-44229</v>
       </c>
     </row>
     <row r="22">
@@ -1950,61 +1947,61 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>8281</v>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="13" t="n">
-        <v>65136</v>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
+        <v>5674</v>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>-19284</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n">
+        <v>24958</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J22" s="12" t="n">
+        <v>-4195881</v>
+      </c>
+      <c r="K22" s="12" t="n">
+        <v>-4220839</v>
+      </c>
+      <c r="L22" s="12" t="n">
+        <v>-4163984</v>
+      </c>
+      <c r="M22" s="12" t="n">
+        <v>-4136372</v>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>-4124332</v>
+      </c>
+      <c r="P22" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q22" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G22" s="13" t="n">
-        <v>-56855</v>
-      </c>
-      <c r="I22" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J22" s="14" t="n">
-        <v>-4220839</v>
-      </c>
-      <c r="K22" s="14" t="n">
-        <v>-4163984</v>
-      </c>
-      <c r="L22" s="14" t="n">
-        <v>-4136372</v>
-      </c>
-      <c r="M22" s="14" t="n">
-        <v>-4124332</v>
-      </c>
-      <c r="N22" s="14" t="n">
-        <v>-4100306</v>
-      </c>
-      <c r="P22" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q22" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R22" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="13" t="n">
-        <v>6638</v>
+      <c r="S22" s="11" t="n">
+        <v>-10296</v>
       </c>
     </row>
     <row r="23">
@@ -2013,58 +2010,58 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>27049</v>
-      </c>
-      <c r="D23" s="12" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>-10900</v>
+      </c>
+      <c r="D23" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E23" s="13" t="n">
-        <v>12395</v>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="n">
-        <v>14654</v>
+      <c r="E23" s="14" t="n">
+        <v>1657</v>
+      </c>
+      <c r="F23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>-12557</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J23" s="14" t="n">
+      <c r="J23" s="12" t="n">
+        <v>551323</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>563880</v>
       </c>
-      <c r="K23" s="14" t="n">
+      <c r="L23" s="12" t="n">
         <v>549226</v>
       </c>
-      <c r="L23" s="14" t="n">
+      <c r="M23" s="12" t="n">
         <v>541370</v>
       </c>
-      <c r="M23" s="14" t="n">
+      <c r="N23" s="12" t="n">
         <v>567763</v>
       </c>
-      <c r="N23" s="14" t="n">
-        <v>600618</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2069,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>10596</v>
+      <c r="S23" s="14" t="n">
+        <v>-5106</v>
       </c>
     </row>
     <row r="24">
@@ -2082,56 +2079,56 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>19892</v>
-      </c>
-      <c r="D24" s="12" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="n">
-        <v>9296</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>10596</v>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>-7767</v>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="11" t="n">
+        <v>-2661</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-5106</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J24" s="14" t="n">
+      <c r="J24" s="12" t="n">
+        <v>459230</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>464336</v>
       </c>
-      <c r="K24" s="14" t="n">
+      <c r="L24" s="12" t="n">
         <v>453740</v>
       </c>
-      <c r="L24" s="14" t="n">
+      <c r="M24" s="12" t="n">
         <v>440834</v>
       </c>
-      <c r="M24" s="14" t="n">
+      <c r="N24" s="12" t="n">
         <v>441538</v>
       </c>
-      <c r="N24" s="14" t="n">
-        <v>450533</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q24" s="12" t="inlineStr">
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
@@ -2141,8 +2138,8 @@
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S24" s="13" t="n">
-        <v>-74963</v>
+      <c r="S24" s="14" t="n">
+        <v>-84814</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2150,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>88374</v>
+        <v>-23782</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>88374</v>
+        <v>-23782</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,7 +2175,7 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="12" t="inlineStr">
+      <c r="Q25" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
@@ -2188,8 +2185,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="13" t="n">
-        <v>4143</v>
+      <c r="S25" s="14" t="n">
+        <v>27389</v>
       </c>
     </row>
     <row r="26">
@@ -2255,15 +2252,15 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>186028</v>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
+        <v>163573</v>
+      </c>
+      <c r="D27" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E27" s="13" t="n">
-        <v>49024</v>
+      <c r="E27" s="14" t="n">
+        <v>48427</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,27 +2268,27 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>137004</v>
+        <v>115146</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J27" s="14" t="n">
+      <c r="J27" s="12" t="n">
+        <v>823961</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>708815</v>
       </c>
-      <c r="K27" s="14" t="n">
+      <c r="L27" s="12" t="n">
         <v>571811</v>
       </c>
-      <c r="L27" s="14" t="n">
+      <c r="M27" s="12" t="n">
         <v>539323</v>
       </c>
-      <c r="M27" s="14" t="n">
+      <c r="N27" s="12" t="n">
         <v>427194</v>
-      </c>
-      <c r="N27" s="14" t="n">
-        <v>323137</v>
       </c>
     </row>
     <row r="28">
@@ -2306,43 +2303,43 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="12" t="inlineStr">
+        <v>90</v>
+      </c>
+      <c r="D28" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E28" s="13" t="n">
-        <v>26033</v>
-      </c>
-      <c r="F28" s="12" t="inlineStr">
+      <c r="E28" s="14" t="n">
+        <v>18628</v>
+      </c>
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G28" s="13" t="n">
-        <v>-26033</v>
+      <c r="G28" s="14" t="n">
+        <v>-18538</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J28" s="14" t="n">
+      <c r="J28" s="12" t="n">
+        <v>-251520</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-232982</v>
       </c>
-      <c r="K28" s="14" t="n">
+      <c r="L28" s="12" t="n">
         <v>-206949</v>
       </c>
-      <c r="L28" s="14" t="n">
+      <c r="M28" s="12" t="n">
         <v>-172978</v>
       </c>
-      <c r="M28" s="14" t="n">
+      <c r="N28" s="12" t="n">
         <v>-150466</v>
-      </c>
-      <c r="N28" s="14" t="n">
-        <v>-105544</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,47 +2362,47 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>5604</v>
-      </c>
-      <c r="D29" s="12" t="inlineStr">
+        <v>15691</v>
+      </c>
+      <c r="D29" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E29" s="13" t="n">
-        <v>41612</v>
-      </c>
-      <c r="F29" s="12" t="inlineStr">
+      <c r="E29" s="14" t="n">
+        <v>27485</v>
+      </c>
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G29" s="13" t="n">
-        <v>-36008</v>
+      <c r="G29" s="14" t="n">
+        <v>-11794</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J29" s="14" t="n">
+      <c r="J29" s="12" t="n">
+        <v>-150845</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-139051</v>
       </c>
-      <c r="K29" s="14" t="n">
+      <c r="L29" s="12" t="n">
         <v>-103043</v>
       </c>
-      <c r="L29" s="14" t="n">
+      <c r="M29" s="12" t="n">
         <v>-103139</v>
       </c>
-      <c r="M29" s="14" t="n">
+      <c r="N29" s="12" t="n">
         <v>-79124</v>
       </c>
-      <c r="N29" s="14" t="n">
-        <v>-66057</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 31-Aug-2026 OHLC</t>
+          <t>Next session  -  based on 01-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,51 +2421,51 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>19809</v>
-      </c>
-      <c r="D30" s="12" t="inlineStr">
+        <v>16886</v>
+      </c>
+      <c r="D30" s="13" t="inlineStr">
         <is>
           <t>Added Shorts</t>
         </is>
       </c>
-      <c r="E30" s="13" t="n">
-        <v>94772</v>
-      </c>
-      <c r="F30" s="12" t="inlineStr">
+      <c r="E30" s="14" t="n">
+        <v>101700</v>
+      </c>
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G30" s="13" t="n">
-        <v>-74963</v>
+      <c r="G30" s="14" t="n">
+        <v>-84814</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J30" s="14" t="n">
+      <c r="J30" s="12" t="n">
+        <v>-421596</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-336782</v>
       </c>
-      <c r="K30" s="14" t="n">
+      <c r="L30" s="12" t="n">
         <v>-261819</v>
       </c>
-      <c r="L30" s="14" t="n">
+      <c r="M30" s="12" t="n">
         <v>-263206</v>
       </c>
-      <c r="M30" s="14" t="n">
+      <c r="N30" s="12" t="n">
         <v>-197604</v>
       </c>
-      <c r="N30" s="14" t="n">
-        <v>-151536</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24117.55</v>
+        <v>24077.55</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2473,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24128.7</v>
+        <v>24143.15</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2484,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>211441</v>
+        <v>196240</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>211441</v>
+        <v>196240</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2510,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23993.6</v>
+        <v>23952.55</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2518,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24080.4</v>
+        <v>24055.8</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2577,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24276.63333333334</v>
+        <v>24339.05</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2585,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24073.98333333334</v>
+        <v>24053.15</v>
       </c>
     </row>
     <row r="33">
@@ -2597,13 +2594,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C33" s="13" t="n">
-        <v>16039</v>
+      <c r="C33" s="14" t="n">
+        <v>4131</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,7 +2608,7 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>36387</v>
+        <v>38830</v>
       </c>
       <c r="F33" s="9" t="inlineStr">
         <is>
@@ -2619,35 +2616,35 @@
         </is>
       </c>
       <c r="G33" s="11" t="n">
-        <v>-20348</v>
+        <v>-34699</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="J33" s="14" t="n">
+      <c r="J33" s="12" t="n">
+        <v>-396117</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-361418</v>
       </c>
-      <c r="K33" s="14" t="n">
+      <c r="L33" s="12" t="n">
         <v>-341070</v>
       </c>
-      <c r="L33" s="14" t="n">
+      <c r="M33" s="12" t="n">
         <v>-356201</v>
       </c>
-      <c r="M33" s="14" t="n">
+      <c r="N33" s="12" t="n">
         <v>-304838</v>
       </c>
-      <c r="N33" s="14" t="n">
-        <v>-252826</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24202.66666666667</v>
+        <v>24241.1</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2652,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24067.56666666667</v>
+        <v>24050.5</v>
       </c>
     </row>
     <row r="34">
@@ -2664,13 +2661,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C34" s="13" t="n">
-        <v>2480</v>
+      <c r="C34" s="14" t="n">
+        <v>39</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,43 +2675,43 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>2198</v>
-      </c>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G34" s="13" t="n">
-        <v>282</v>
+        <v>610</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="n">
+        <v>-571</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="J34" s="14" t="n">
+      <c r="J34" s="12" t="n">
+        <v>28940</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>29511</v>
       </c>
-      <c r="K34" s="14" t="n">
+      <c r="L34" s="12" t="n">
         <v>29229</v>
       </c>
-      <c r="L34" s="14" t="n">
+      <c r="M34" s="12" t="n">
         <v>29994</v>
       </c>
-      <c r="M34" s="14" t="n">
+      <c r="N34" s="12" t="n">
         <v>29442</v>
       </c>
-      <c r="N34" s="14" t="n">
-        <v>23275</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24141.53333333334</v>
+        <v>24148.45</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2719,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24061.15</v>
+        <v>24047.85</v>
       </c>
     </row>
     <row r="35">
@@ -2731,13 +2728,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C35" s="13" t="n">
-        <v>27742</v>
+      <c r="C35" s="14" t="n">
+        <v>19904</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,43 +2742,43 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>11819</v>
-      </c>
-      <c r="F35" s="12" t="inlineStr">
+        <v>12023</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G35" s="13" t="n">
-        <v>15923</v>
+      <c r="G35" s="14" t="n">
+        <v>7881</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="J35" s="14" t="n">
+      <c r="J35" s="12" t="n">
+        <v>100354</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>92473</v>
       </c>
-      <c r="K35" s="14" t="n">
+      <c r="L35" s="12" t="n">
         <v>76550</v>
       </c>
-      <c r="L35" s="14" t="n">
+      <c r="M35" s="12" t="n">
         <v>74854</v>
       </c>
-      <c r="M35" s="14" t="n">
+      <c r="N35" s="12" t="n">
         <v>61095</v>
       </c>
-      <c r="N35" s="14" t="n">
-        <v>63426</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24067.56666666667</v>
+        <v>24050.5</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2792,13 +2789,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>Added Longs</t>
         </is>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>36820</v>
+      <c r="C36" s="14" t="n">
+        <v>51689</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,43 +2803,43 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>32677</v>
-      </c>
-      <c r="F36" s="12" t="inlineStr">
+        <v>24300</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G36" s="13" t="n">
-        <v>4143</v>
+      <c r="G36" s="14" t="n">
+        <v>27389</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="J36" s="14" t="n">
+      <c r="J36" s="12" t="n">
+        <v>266823</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>239434</v>
       </c>
-      <c r="K36" s="14" t="n">
+      <c r="L36" s="12" t="n">
         <v>235291</v>
       </c>
-      <c r="L36" s="14" t="n">
+      <c r="M36" s="12" t="n">
         <v>251353</v>
       </c>
-      <c r="M36" s="14" t="n">
+      <c r="N36" s="12" t="n">
         <v>214301</v>
       </c>
-      <c r="N36" s="14" t="n">
-        <v>166125</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>24006.43333333334</v>
+        <v>23957.85</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2852,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>83081</v>
+        <v>75763</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>83081</v>
+        <v>75763</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2878,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23932.46666666667</v>
+        <v>23859.9</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2890,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23871.33333333334</v>
+        <v>23767.25</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2934,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.49</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.19</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.07</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>10.57</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.08</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +2997,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>1.005517111378178</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.006164539061341</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.009662619345433</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.005678413660525</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.010104864602446</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.014881725047644</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,080    PCR(OI) 0.81    Max Pain 24,100</t>
+          <t>Spot 24,056    PCR(OI) 0.86    Max Pain 24,050</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3028,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23923.80967741935</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23932.86491935484</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23944.28548387097</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23954.82459677419</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23965.5810483871</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23977.72016129032</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3059,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>24055.8</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24080.4</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24090.85</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24207.75</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24334.55</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3134,20 +3131,20 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24200</v>
-      </c>
-      <c r="Q45" s="14" t="n">
-        <v>200604</v>
+        <v>24050</v>
+      </c>
+      <c r="Q45" s="12" t="n">
+        <v>244781</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>60758</v>
-      </c>
-      <c r="S45" s="14" t="n">
-        <v>6612183</v>
+        <v>177666</v>
+      </c>
+      <c r="S45" s="12" t="n">
+        <v>27773147</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3158,7 +3155,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9888317666598201</v>
+        <v>0.9878296455375508</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9933791141865997</v>
@@ -3173,20 +3170,20 @@
         <v>1.011430829957649</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24300</v>
-      </c>
-      <c r="Q46" s="14" t="n">
-        <v>228704</v>
+        <v>24100</v>
+      </c>
+      <c r="Q46" s="12" t="n">
+        <v>380629</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>27494</v>
-      </c>
-      <c r="S46" s="14" t="n">
-        <v>4521751</v>
+        <v>226852</v>
+      </c>
+      <c r="S46" s="12" t="n">
+        <v>32652760</v>
       </c>
       <c r="T46" s="29" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3194,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24352.37298387097</v>
+        <v>24352.17459677419</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24336.7810483871</v>
@@ -3212,20 +3209,20 @@
         <v>24292.96129032258</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24500</v>
-      </c>
-      <c r="Q47" s="14" t="n">
-        <v>262486</v>
+        <v>24150</v>
+      </c>
+      <c r="Q47" s="12" t="n">
+        <v>201933</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>64616</v>
-      </c>
-      <c r="S47" s="14" t="n">
-        <v>2499631</v>
+        <v>95312</v>
+      </c>
+      <c r="S47" s="12" t="n">
+        <v>20805029</v>
       </c>
       <c r="T47" s="30" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3233,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24080.4</v>
+        <v>24055.8</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24175.65</v>
@@ -3266,27 +3263,27 @@
           <t>Week ending</t>
         </is>
       </c>
-      <c r="J49" s="29" t="inlineStr">
-        <is>
-          <t>31-Aug-2026</t>
-        </is>
-      </c>
-      <c r="K49" s="29" t="inlineStr">
+      <c r="J49" s="30" t="inlineStr">
+        <is>
+          <t>01-Sep-2026</t>
+        </is>
+      </c>
+      <c r="K49" s="30" t="inlineStr">
         <is>
           <t>28-Aug-2026</t>
         </is>
       </c>
-      <c r="L49" s="29" t="inlineStr">
+      <c r="L49" s="30" t="inlineStr">
         <is>
           <t>21-Aug-2026</t>
         </is>
       </c>
-      <c r="M49" s="29" t="inlineStr">
+      <c r="M49" s="30" t="inlineStr">
         <is>
           <t>14-Aug-2026</t>
         </is>
       </c>
-      <c r="N49" s="29" t="inlineStr">
+      <c r="N49" s="30" t="inlineStr">
         <is>
           <t>07-Aug-2026</t>
         </is>
@@ -3319,18 +3316,18 @@
     </row>
     <row r="50">
       <c r="P50" s="32" t="n">
-        <v>24100</v>
-      </c>
-      <c r="Q50" s="14" t="n">
-        <v>160251</v>
+        <v>24050</v>
+      </c>
+      <c r="Q50" s="12" t="n">
+        <v>371988</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>7693</v>
-      </c>
-      <c r="S50" s="14" t="n">
-        <v>8664178</v>
-      </c>
-      <c r="T50" s="33" t="inlineStr">
+        <v>240921</v>
+      </c>
+      <c r="S50" s="12" t="n">
+        <v>28783616</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3340,16 +3337,16 @@
       <c r="P51" s="32" t="n">
         <v>24000</v>
       </c>
-      <c r="Q51" s="14" t="n">
-        <v>262269</v>
+      <c r="Q51" s="12" t="n">
+        <v>361954</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>104392</v>
-      </c>
-      <c r="S51" s="14" t="n">
-        <v>11947246</v>
-      </c>
-      <c r="T51" s="33" t="inlineStr">
+        <v>115425</v>
+      </c>
+      <c r="S51" s="12" t="n">
+        <v>36941900</v>
+      </c>
+      <c r="T51" s="29" t="inlineStr">
         <is>
           <t>High</t>
         </is>
@@ -3357,27 +3354,27 @@
     </row>
     <row r="52">
       <c r="P52" s="32" t="n">
-        <v>23800</v>
-      </c>
-      <c r="Q52" s="14" t="n">
-        <v>147168</v>
+        <v>23950</v>
+      </c>
+      <c r="Q52" s="12" t="n">
+        <v>217029</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>32920</v>
-      </c>
-      <c r="S52" s="14" t="n">
-        <v>3187671</v>
-      </c>
-      <c r="T52" s="30" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>117514</v>
+      </c>
+      <c r="S52" s="12" t="n">
+        <v>26604108</v>
+      </c>
+      <c r="T52" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="34" t="inlineStr">
-        <is>
-          <t>TODAY = 31-Aug-2026    1 DAY AGO = 28-Aug-2026    2 DAYS AGO = 27-Aug-2026    3 DAYS AGO = 26-Aug-2026    4 DAYS AGO = 25-Aug-2026    (generated 31-Aug-2026 21:27 IST)</t>
+      <c r="A54" s="33" t="inlineStr">
+        <is>
+          <t>TODAY = 01-Sep-2026    1 DAY AGO = 31-Aug-2026    2 DAYS AGO = 28-Aug-2026    3 DAYS AGO = 27-Aug-2026    4 DAYS AGO = 26-Aug-2026    (generated 01-Sep-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-02
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -191,6 +191,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -687,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>8911</v>
+        <v>12940</v>
       </c>
     </row>
     <row r="3">
@@ -702,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>8720</v>
+        <v>8396</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -710,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-191</v>
+        <v>-4544</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -718,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>8911</v>
+        <v>12940</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -726,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>200070</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>187130</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>178219</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>176959</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>174158</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>160283</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -756,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>66301</v>
+        <v>11084</v>
       </c>
     </row>
     <row r="4">
@@ -765,13 +768,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>189</v>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>-1528</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -779,53 +782,53 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+        <v>5682</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-7210</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>13267</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>20477</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>20288</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>20213</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>19513</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>189</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>20477</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>20288</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>20213</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>19513</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>17589</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-70902</v>
+      <c r="S4" s="14" t="n">
+        <v>44808</v>
       </c>
     </row>
     <row r="5">
@@ -840,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>523</v>
+        <v>3819</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -848,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>13240</v>
+        <v>10950</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -856,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-12717</v>
+        <v>-7131</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -864,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-229163</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-222032</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-209315</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-202633</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-197792</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-186060</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -894,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="14" t="n">
-        <v>-7295</v>
+        <v>-11832</v>
       </c>
     </row>
     <row r="6">
@@ -903,21 +906,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>-112</v>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>-3729</v>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1807</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="n">
+        <v>406</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -925,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="11" t="n">
-        <v>3617</v>
+        <v>1401</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -933,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>15826</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>14425</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>10808</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>5461</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>4121</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>8188</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -963,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>115146</v>
+        <v>79191</v>
       </c>
     </row>
     <row r="7">
@@ -974,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>9320</v>
+        <v>12494</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>9320</v>
+        <v>12494</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -999,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1009,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-34699</v>
+      <c r="S7" s="14" t="n">
+        <v>12283</v>
       </c>
     </row>
     <row r="8">
@@ -1068,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1078,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>189</v>
+      <c r="S8" s="14" t="n">
+        <v>-7210</v>
       </c>
     </row>
     <row r="9">
@@ -1088,21 +1091,21 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="n">
-        <v>-1348907</v>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="n">
-        <v>-1415208</v>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n">
+        <v>654712</v>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>643628</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1110,7 +1113,7 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>66301</v>
+        <v>11084</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1118,28 +1121,28 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>273067</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>261983</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>195682</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>91197</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>289153</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>191071</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R9" s="10" t="inlineStr">
@@ -1147,8 +1150,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S9" s="11" t="n">
-        <v>525</v>
+      <c r="S9" s="14" t="n">
+        <v>-575</v>
       </c>
     </row>
     <row r="10">
@@ -1163,23 +1166,23 @@
         </is>
       </c>
       <c r="C10" s="11" t="n">
-        <v>500</v>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>-25</v>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>525</v>
+        <v>0</v>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="n">
+        <v>575</v>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G10" s="14" t="n">
+        <v>-575</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1187,28 +1190,28 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>4260</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4835</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4310</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4350</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4325</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>3905</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q10" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1216,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="14" t="n">
-        <v>139</v>
+      <c r="S10" s="11" t="n">
+        <v>-1915</v>
       </c>
     </row>
     <row r="11">
@@ -1226,21 +1229,21 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="n">
-        <v>-242134</v>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="n">
-        <v>-219535</v>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>57199</v>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>108391</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1248,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-22599</v>
+        <v>-51192</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1256,28 +1259,28 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-299253</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-248061</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-225462</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-230020</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-265856</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-235885</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q11" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q11" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R11" s="10" t="inlineStr">
@@ -1285,8 +1288,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S11" s="11" t="n">
-        <v>24958</v>
+      <c r="S11" s="14" t="n">
+        <v>-38604</v>
       </c>
     </row>
     <row r="12">
@@ -1295,67 +1298,67 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="n">
-        <v>-378438</v>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>-334209</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>109535</v>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="n">
+        <v>68852</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>40683</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>21925</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-18758</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>25471</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>134473</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>-27622</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-44229</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-18758</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>25471</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>134473</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>-27622</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>40908</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-18538</v>
+        <v>-40056</v>
       </c>
     </row>
     <row r="13">
@@ -1366,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>-1968979</v>
+        <v>821446</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>-1968977</v>
+        <v>821446</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1402,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-571</v>
+        <v>-393</v>
       </c>
     </row>
     <row r="14">
@@ -1471,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-12717</v>
+        <v>-7131</v>
       </c>
     </row>
     <row r="15">
@@ -1480,67 +1483,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="n">
-        <v>-1278790</v>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E15" s="14" t="n">
-        <v>-1207888</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="n">
+        <v>532741</v>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>487933</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>44808</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="n">
+        <v>-712140</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>-756948</v>
+      </c>
+      <c r="L15" s="12" t="n">
+        <v>-686046</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>-725066</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>-760983</v>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G15" s="11" t="n">
-        <v>-70902</v>
-      </c>
-      <c r="I15" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J15" s="12" t="n">
-        <v>-756948</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>-686046</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>-725066</v>
-      </c>
-      <c r="M15" s="12" t="n">
-        <v>-760983</v>
-      </c>
-      <c r="N15" s="12" t="n">
-        <v>-663004</v>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R15" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-22599</v>
+        <v>-51192</v>
       </c>
     </row>
     <row r="16">
@@ -1549,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="14" t="n">
-        <v>139</v>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>-1915</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1565,13 +1568,13 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G16" s="14" t="n">
-        <v>139</v>
+      <c r="F16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="n">
+        <v>-1915</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1579,28 +1582,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>30008</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>31923</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>31784</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>34489</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>33514</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>31979</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1608,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>81058</v>
+      <c r="S16" s="11" t="n">
+        <v>-39242</v>
       </c>
     </row>
     <row r="17">
@@ -1618,67 +1621,67 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>-164146</v>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E17" s="14" t="n">
-        <v>-245204</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>59991</v>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>99233</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-39242</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>593223</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>632465</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>551407</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>594360</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>626360</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>81058</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>632465</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>551407</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>594360</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>626360</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>555751</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S17" s="14" t="n">
-        <v>-12557</v>
+      <c r="S17" s="11" t="n">
+        <v>41679</v>
       </c>
     </row>
     <row r="18">
@@ -1687,21 +1690,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="n">
-        <v>-415860</v>
-      </c>
-      <c r="D18" s="13" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
-        <v>-405564</v>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>77306</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>80956</v>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
@@ -1709,7 +1712,7 @@
         </is>
       </c>
       <c r="G18" s="11" t="n">
-        <v>-10296</v>
+        <v>-3650</v>
       </c>
       <c r="I18" s="8" t="inlineStr">
         <is>
@@ -1717,20 +1720,20 @@
         </is>
       </c>
       <c r="J18" s="12" t="n">
+        <v>88909</v>
+      </c>
+      <c r="K18" s="12" t="n">
         <v>92559</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="L18" s="12" t="n">
         <v>102855</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="M18" s="12" t="n">
         <v>96217</v>
       </c>
-      <c r="M18" s="12" t="n">
+      <c r="N18" s="12" t="n">
         <v>101109</v>
       </c>
-      <c r="N18" s="12" t="n">
-        <v>75274</v>
-      </c>
       <c r="P18" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1747,7 +1750,7 @@
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-11794</v>
+        <v>-18313</v>
       </c>
     </row>
     <row r="19">
@@ -1758,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>-1858657</v>
+        <v>668123</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>-1858656</v>
+        <v>668122</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1794,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>7881</v>
+        <v>7849</v>
       </c>
     </row>
     <row r="20">
@@ -1863,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="11" t="n">
-        <v>3617</v>
+        <v>1401</v>
       </c>
     </row>
     <row r="21">
@@ -1878,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="14" t="n">
-        <v>-10789</v>
+        <v>-13345</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
@@ -1886,7 +1889,7 @@
         </is>
       </c>
       <c r="E21" s="11" t="n">
-        <v>-3494</v>
+        <v>-1513</v>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
@@ -1894,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="14" t="n">
-        <v>-7295</v>
+        <v>-11832</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1902,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3173496</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3185328</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3192623</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3161018</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3154168</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3115031</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1931,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-44229</v>
+      <c r="S21" s="11" t="n">
+        <v>40683</v>
       </c>
     </row>
     <row r="22">
@@ -1947,23 +1950,23 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>5674</v>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E22" s="11" t="n">
-        <v>-19284</v>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G22" s="11" t="n">
-        <v>24958</v>
+        <v>7848</v>
+      </c>
+      <c r="D22" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>46452</v>
+      </c>
+      <c r="F22" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>-38604</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1971,20 +1974,20 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4234485</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4195881</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4220839</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4163984</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4136372</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4124332</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2001,7 +2004,7 @@
         </is>
       </c>
       <c r="S22" s="11" t="n">
-        <v>-10296</v>
+        <v>-3650</v>
       </c>
     </row>
     <row r="23">
@@ -2010,29 +2013,29 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="14" t="n">
-        <v>-10900</v>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E23" s="14" t="n">
-        <v>1657</v>
-      </c>
-      <c r="F23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G23" s="14" t="n">
-        <v>-12557</v>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="n">
+        <v>16965</v>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="n">
+        <v>-24714</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n">
+        <v>41679</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2040,28 +2043,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>593002</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>551323</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>563880</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>549226</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>541370</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>567763</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2069,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-5106</v>
+      <c r="S23" s="11" t="n">
+        <v>8757</v>
       </c>
     </row>
     <row r="24">
@@ -2079,13 +2082,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>-7767</v>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>6785</v>
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
@@ -2093,53 +2096,53 @@
         </is>
       </c>
       <c r="E24" s="11" t="n">
-        <v>-2661</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+        <v>-1972</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>8757</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>467987</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>459230</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>464336</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>453740</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>440834</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-5106</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>459230</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>464336</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>453740</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>440834</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>441538</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-84814</v>
+        <v>-20822</v>
       </c>
     </row>
     <row r="25">
@@ -2150,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>-23782</v>
+        <v>18253</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>-23782</v>
+        <v>18253</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2175,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2185,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>27389</v>
+      <c r="S25" s="11" t="n">
+        <v>-19739</v>
       </c>
     </row>
     <row r="26">
@@ -2252,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>163573</v>
+        <v>138628</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2260,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>48427</v>
+        <v>59437</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2268,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>115146</v>
+        <v>79191</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2276,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>903152</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>823961</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>708815</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>571811</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>539323</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>427194</v>
       </c>
     </row>
     <row r="28">
@@ -2303,7 +2306,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2311,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>18628</v>
+        <v>40056</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2319,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-18538</v>
+        <v>-40056</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2327,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-291576</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-251520</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-232982</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-206949</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-172978</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-150466</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2362,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>15691</v>
+        <v>12952</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2370,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>27485</v>
+        <v>31265</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2378,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-11794</v>
+        <v>-18313</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2386,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-169158</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-150845</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-139051</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-103043</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-103139</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-79124</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 01-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 02-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2421,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>16886</v>
+        <v>44715</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2429,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>101700</v>
+        <v>65537</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2437,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-84814</v>
+        <v>-20822</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2445,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-442418</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-421596</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-336782</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-261819</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-263206</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-197604</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>24077.55</v>
+        <v>23858</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2473,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24143.15</v>
+        <v>23914.45</v>
       </c>
     </row>
     <row r="31">
@@ -2484,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>196240</v>
+        <v>196295</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>196240</v>
+        <v>196295</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2510,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23952.55</v>
+        <v>23786.8</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2518,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>24055.8</v>
+        <v>23914.45</v>
       </c>
     </row>
     <row r="32">
@@ -2577,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24339.05</v>
+        <v>24084.65</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2585,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>24053.15</v>
+        <v>23893.175</v>
       </c>
     </row>
     <row r="33">
@@ -2600,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>4131</v>
+        <v>39831</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2608,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>38830</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-34699</v>
+        <v>27548</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>12283</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2624,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-383834</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-396117</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-361418</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-341070</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-356201</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-304838</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24241.1</v>
+        <v>23999.55</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2652,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>24050.5</v>
+        <v>23871.9</v>
       </c>
     </row>
     <row r="34">
@@ -2667,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>39</v>
+        <v>351</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2675,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>610</v>
+        <v>744</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2683,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-571</v>
+        <v>-393</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2691,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>28547</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>28940</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>29511</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>29229</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>29994</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>29442</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>24148.45</v>
+        <v>23957</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2719,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>24047.85</v>
+        <v>23850.625</v>
       </c>
     </row>
     <row r="35">
@@ -2734,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>19904</v>
+        <v>21530</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2742,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>12023</v>
+        <v>13681</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2750,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>7881</v>
+        <v>7849</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2758,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>108203</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>100354</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>92473</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>76550</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>74854</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>61095</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>24050.5</v>
+        <v>23871.9</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2795,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>51689</v>
+        <v>27430</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2803,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>24300</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>27389</v>
+        <v>47169</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-19739</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2819,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>247084</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>266823</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>239434</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>235291</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>251353</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>214301</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23957.85</v>
+        <v>23829.34999999999</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2852,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>75763</v>
+        <v>89142</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>75763</v>
+        <v>89142</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2878,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23859.9</v>
+        <v>23744.25</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2890,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23767.25</v>
+        <v>23701.69999999999</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2934,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.59</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.49</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.19</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>10.68</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.07</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>10.57</v>
       </c>
     </row>
     <row r="41">
@@ -2982,7 +2985,7 @@
       </c>
       <c r="P41" s="3" t="inlineStr">
         <is>
-          <t>Nifty Option-Chain S/R   -   Weekly expiry 01-Sep-2026</t>
+          <t>Nifty Option-Chain S/R   -   Weekly expiry 08-Sep-2026</t>
         </is>
       </c>
       <c r="Q41" s="2" t="n"/>
@@ -2997,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9999294072299643</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>1.005517111378178</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.006164539061341</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.009662619345433</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.005678413660525</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.010104864602446</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 24,056    PCR(OI) 0.86    Max Pain 24,050</t>
+          <t>Spot 23,914    PCR(OI) 0.73    Max Pain 23,950</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3028,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23916.13830645161</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23923.80967741935</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23932.86491935484</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23944.28548387097</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23954.82459677419</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23965.5810483871</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3059,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23914.45</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>24055.8</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24080.4</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24175.65</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24090.85</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24207.75</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3131,16 +3134,16 @@
         </is>
       </c>
       <c r="P45" s="28" t="n">
-        <v>24050</v>
+        <v>24000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>244781</v>
+        <v>134710</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>177666</v>
+        <v>45881</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>27773147</v>
+        <v>2832927</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3155,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9878296455375508</v>
+        <v>0.9820712062874193</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9933791141865997</v>
@@ -3170,20 +3173,20 @@
         <v>1.011430829957649</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24100</v>
+        <v>24200</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>380629</v>
+        <v>155299</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>226852</v>
+        <v>41535</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>32652760</v>
-      </c>
-      <c r="T46" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1308169</v>
+      </c>
+      <c r="T46" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
@@ -3194,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24352.17459677419</v>
+        <v>24351.03467741935</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24336.7810483871</v>
@@ -3209,20 +3212,20 @@
         <v>24292.96129032258</v>
       </c>
       <c r="P47" s="28" t="n">
-        <v>24150</v>
+        <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>201933</v>
+        <v>140433</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>95312</v>
+        <v>55828</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>20805029</v>
-      </c>
-      <c r="T47" s="30" t="inlineStr">
-        <is>
-          <t>Medium</t>
+        <v>574623</v>
+      </c>
+      <c r="T47" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
@@ -3233,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>24055.8</v>
+        <v>23914.45</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24175.65</v>
@@ -3247,7 +3250,7 @@
       <c r="N48" s="18" t="n">
         <v>24570.65</v>
       </c>
-      <c r="P48" s="31" t="inlineStr">
+      <c r="P48" s="32" t="inlineStr">
         <is>
           <t>SUPPORT   -   Put OI walls (higher = stronger floor)</t>
         </is>
@@ -3265,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>01-Sep-2026</t>
+          <t>02-Sep-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3315,17 +3318,17 @@
       </c>
     </row>
     <row r="50">
-      <c r="P50" s="32" t="n">
-        <v>24050</v>
+      <c r="P50" s="33" t="n">
+        <v>23800</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>371988</v>
+        <v>120404</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>240921</v>
+        <v>74010</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>28783616</v>
+        <v>3647157</v>
       </c>
       <c r="T50" s="29" t="inlineStr">
         <is>
@@ -3334,47 +3337,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="P51" s="32" t="n">
-        <v>24000</v>
+      <c r="P51" s="33" t="n">
+        <v>23500</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>361954</v>
+        <v>119969</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>115425</v>
+        <v>24665</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>36941900</v>
-      </c>
-      <c r="T51" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1114845</v>
+      </c>
+      <c r="T51" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="P52" s="32" t="n">
-        <v>23950</v>
+      <c r="P52" s="33" t="n">
+        <v>23000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>217029</v>
+        <v>128121</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>117514</v>
+        <v>52537</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>26604108</v>
-      </c>
-      <c r="T52" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>567792</v>
+      </c>
+      <c r="T52" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="33" t="inlineStr">
-        <is>
-          <t>TODAY = 01-Sep-2026    1 DAY AGO = 31-Aug-2026    2 DAYS AGO = 28-Aug-2026    3 DAYS AGO = 27-Aug-2026    4 DAYS AGO = 26-Aug-2026    (generated 01-Sep-2026 20:31 IST)</t>
+      <c r="A54" s="34" t="inlineStr">
+        <is>
+          <t>TODAY = 02-Sep-2026    1 DAY AGO = 01-Sep-2026    2 DAYS AGO = 31-Aug-2026    3 DAYS AGO = 28-Aug-2026    4 DAYS AGO = 27-Aug-2026    (generated 02-Sep-2026 21:04 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-03
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>12940</v>
+        <v>5926</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>8396</v>
+        <v>1331</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-4544</v>
+        <v>-4595</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>12940</v>
+        <v>5926</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,20 +729,20 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>205996</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>200070</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>187130</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>178219</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>176959</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>174158</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="S3" s="11" t="n">
-        <v>11084</v>
+        <v>109470</v>
       </c>
     </row>
     <row r="4">
@@ -768,13 +768,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>-1528</v>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C4" s="11" t="n">
+        <v>50</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -782,53 +782,53 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>5682</v>
-      </c>
-      <c r="F4" s="13" t="inlineStr">
+        <v>30</v>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>13287</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>13267</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>20477</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>20288</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>20213</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="9" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G4" s="14" t="n">
-        <v>-7210</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>13267</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>20477</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>20288</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>20213</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>19513</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="14" t="n">
-        <v>44808</v>
+      <c r="S4" s="11" t="n">
+        <v>-89681</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>3819</v>
+        <v>4965</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>10950</v>
+        <v>10904</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-7131</v>
+        <v>-5939</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,28 +867,28 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-235102</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-229163</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-222032</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-209315</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-202633</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-197792</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q5" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q5" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R5" s="10" t="inlineStr">
@@ -896,8 +896,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S5" s="14" t="n">
-        <v>-11832</v>
+      <c r="S5" s="11" t="n">
+        <v>3077</v>
       </c>
     </row>
     <row r="6">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="C6" s="11" t="n">
-        <v>1807</v>
+        <v>1959</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
@@ -920,53 +920,53 @@
         </is>
       </c>
       <c r="E6" s="14" t="n">
-        <v>406</v>
-      </c>
-      <c r="F6" s="9" t="inlineStr">
+        <v>1966</v>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="n">
+        <v>-7</v>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="n">
+        <v>15819</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>15826</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>14425</v>
+      </c>
+      <c r="M6" s="12" t="n">
+        <v>10808</v>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>5461</v>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q6" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G6" s="11" t="n">
-        <v>1401</v>
-      </c>
-      <c r="I6" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J6" s="12" t="n">
-        <v>15826</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>14425</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>10808</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>5461</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>4121</v>
-      </c>
-      <c r="P6" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q6" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R6" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>79191</v>
+        <v>38896</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>12494</v>
+        <v>8305</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>12494</v>
+        <v>8305</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q7" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="14" t="n">
-        <v>12283</v>
+      <c r="S7" s="11" t="n">
+        <v>-12518</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q8" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="14" t="n">
-        <v>-7210</v>
+      <c r="S8" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>654712</v>
+        <v>692342</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>643628</v>
+        <v>582872</v>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
@@ -1113,7 +1113,7 @@
         </is>
       </c>
       <c r="G9" s="11" t="n">
-        <v>11084</v>
+        <v>109470</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>382537</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>273067</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>261983</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>195682</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>91197</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>289153</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-575</v>
+        <v>-150</v>
       </c>
     </row>
     <row r="10">
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>575</v>
+        <v>150</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-575</v>
+        <v>-150</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,28 +1190,28 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>4110</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4260</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4835</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4310</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4350</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4325</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q10" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R10" s="10" t="inlineStr">
@@ -1219,8 +1219,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S10" s="11" t="n">
-        <v>-1915</v>
+      <c r="S10" s="14" t="n">
+        <v>2031</v>
       </c>
     </row>
     <row r="11">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>57199</v>
+        <v>93060</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
         </is>
       </c>
       <c r="E11" s="14" t="n">
-        <v>108391</v>
+        <v>106014</v>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
@@ -1251,7 +1251,7 @@
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>-51192</v>
+        <v>-12954</v>
       </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
@@ -1259,20 +1259,20 @@
         </is>
       </c>
       <c r="J11" s="12" t="n">
+        <v>-312207</v>
+      </c>
+      <c r="K11" s="12" t="n">
         <v>-299253</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="L11" s="12" t="n">
         <v>-248061</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="M11" s="12" t="n">
         <v>-225462</v>
       </c>
-      <c r="M11" s="12" t="n">
+      <c r="N11" s="12" t="n">
         <v>-230020</v>
       </c>
-      <c r="N11" s="12" t="n">
-        <v>-265856</v>
-      </c>
       <c r="P11" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1289,7 +1289,7 @@
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-38604</v>
+        <v>-3077</v>
       </c>
     </row>
     <row r="12">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>109535</v>
+        <v>225907</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
@@ -1312,15 +1312,15 @@
         </is>
       </c>
       <c r="E12" s="14" t="n">
-        <v>68852</v>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>40683</v>
+        <v>322273</v>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>-96366</v>
       </c>
       <c r="I12" s="8" t="inlineStr">
         <is>
@@ -1328,20 +1328,20 @@
         </is>
       </c>
       <c r="J12" s="12" t="n">
+        <v>-74441</v>
+      </c>
+      <c r="K12" s="12" t="n">
         <v>21925</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="L12" s="12" t="n">
         <v>-18758</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="M12" s="12" t="n">
         <v>25471</v>
       </c>
-      <c r="M12" s="12" t="n">
+      <c r="N12" s="12" t="n">
         <v>134473</v>
       </c>
-      <c r="N12" s="12" t="n">
-        <v>-27622</v>
-      </c>
       <c r="P12" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-40056</v>
+        <v>-6997</v>
       </c>
     </row>
     <row r="13">
@@ -1369,11 +1369,11 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>821446</v>
+        <v>1011309</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>821446</v>
+        <v>1011309</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-393</v>
+        <v>-1588</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-7131</v>
+        <v>-5939</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>532741</v>
+        <v>233565</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,15 +1497,15 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>487933</v>
-      </c>
-      <c r="F15" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>44808</v>
+        <v>323246</v>
+      </c>
+      <c r="F15" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="n">
+        <v>-89681</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,20 +1513,20 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-801821</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-712140</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-756948</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-686046</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-725066</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-760983</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1543,7 +1543,7 @@
         </is>
       </c>
       <c r="S15" s="14" t="n">
-        <v>-51192</v>
+        <v>-12954</v>
       </c>
     </row>
     <row r="16">
@@ -1552,13 +1552,13 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="n">
-        <v>-1915</v>
+      <c r="B16" s="13" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C16" s="14" t="n">
+        <v>2031</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1568,13 +1568,13 @@
       <c r="E16" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="n">
-        <v>-1915</v>
+      <c r="F16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>2031</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,28 +1582,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>32039</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>30008</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>31923</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>31784</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>34489</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>33514</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="11" t="n">
-        <v>-39242</v>
+      <c r="S16" s="14" t="n">
+        <v>56826</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>59991</v>
+        <v>79978</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,15 +1635,15 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>99233</v>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="n">
-        <v>-39242</v>
+        <v>23152</v>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>56826</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
@@ -1651,20 +1651,20 @@
         </is>
       </c>
       <c r="J17" s="12" t="n">
+        <v>650049</v>
+      </c>
+      <c r="K17" s="12" t="n">
         <v>593223</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="L17" s="12" t="n">
         <v>632465</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="M17" s="12" t="n">
         <v>551407</v>
       </c>
-      <c r="M17" s="12" t="n">
+      <c r="N17" s="12" t="n">
         <v>594360</v>
       </c>
-      <c r="N17" s="12" t="n">
-        <v>626360</v>
-      </c>
       <c r="P17" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>41679</v>
+        <v>16895</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>77306</v>
+        <v>180107</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,53 +1704,53 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>80956</v>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
+        <v>149283</v>
+      </c>
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="n">
+        <v>30824</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>119733</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>88909</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>92559</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>102855</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>96217</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G18" s="11" t="n">
-        <v>-3650</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>88909</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>92559</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>102855</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>96217</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>101109</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S18" s="14" t="n">
-        <v>-18313</v>
+        <v>-5435</v>
       </c>
     </row>
     <row r="19">
@@ -1761,15 +1761,15 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>668123</v>
+        <v>495681</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>668122</v>
+        <v>495681</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I19" s="15" t="inlineStr">
         <is>
@@ -1797,7 +1797,7 @@
         </is>
       </c>
       <c r="S19" s="14" t="n">
-        <v>7849</v>
+        <v>10051</v>
       </c>
     </row>
     <row r="20">
@@ -1855,9 +1855,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q20" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q20" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R20" s="10" t="inlineStr">
@@ -1865,8 +1865,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S20" s="11" t="n">
-        <v>1401</v>
+      <c r="S20" s="14" t="n">
+        <v>-7</v>
       </c>
     </row>
     <row r="21">
@@ -1875,67 +1875,67 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="n">
-        <v>-13345</v>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E21" s="11" t="n">
-        <v>-1513</v>
-      </c>
-      <c r="F21" s="13" t="inlineStr">
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>10069</v>
+      </c>
+      <c r="D21" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>6992</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n">
+        <v>3077</v>
+      </c>
+      <c r="I21" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="J21" s="12" t="n">
+        <v>3176573</v>
+      </c>
+      <c r="K21" s="12" t="n">
+        <v>3173496</v>
+      </c>
+      <c r="L21" s="12" t="n">
+        <v>3185328</v>
+      </c>
+      <c r="M21" s="12" t="n">
+        <v>3192623</v>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>3161018</v>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q21" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G21" s="14" t="n">
-        <v>-11832</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="J21" s="12" t="n">
-        <v>3173496</v>
-      </c>
-      <c r="K21" s="12" t="n">
-        <v>3185328</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>3192623</v>
-      </c>
-      <c r="M21" s="12" t="n">
-        <v>3161018</v>
-      </c>
-      <c r="N21" s="12" t="n">
-        <v>3154168</v>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q21" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R21" s="10" t="inlineStr">
         <is>
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="11" t="n">
-        <v>40683</v>
+      <c r="S21" s="14" t="n">
+        <v>-96366</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>7848</v>
+        <v>12811</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>46452</v>
+        <v>15888</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-38604</v>
+        <v>-3077</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4237562</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4234485</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4195881</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4220839</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4163984</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4136372</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q22" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="11" t="n">
-        <v>-3650</v>
+      <c r="S22" s="14" t="n">
+        <v>30824</v>
       </c>
     </row>
     <row r="23">
@@ -2019,7 +2019,7 @@
         </is>
       </c>
       <c r="C23" s="11" t="n">
-        <v>16965</v>
+        <v>1041</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>-24714</v>
+        <v>-15854</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>41679</v>
+        <v>16895</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>609897</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>593002</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>551323</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>563880</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>549226</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>541370</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q23" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="11" t="n">
-        <v>8757</v>
+      <c r="S23" s="14" t="n">
+        <v>-16895</v>
       </c>
     </row>
     <row r="24">
@@ -2082,29 +2082,29 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="n">
-        <v>6785</v>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Closed Shorts</t>
-        </is>
-      </c>
-      <c r="E24" s="11" t="n">
-        <v>-1972</v>
-      </c>
-      <c r="F24" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G24" s="11" t="n">
-        <v>8757</v>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>-10968</v>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Added Shorts</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>5927</v>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>-16895</v>
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
@@ -2112,20 +2112,20 @@
         </is>
       </c>
       <c r="J24" s="12" t="n">
+        <v>451092</v>
+      </c>
+      <c r="K24" s="12" t="n">
         <v>467987</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="L24" s="12" t="n">
         <v>459230</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="M24" s="12" t="n">
         <v>464336</v>
       </c>
-      <c r="M24" s="12" t="n">
+      <c r="N24" s="12" t="n">
         <v>453740</v>
       </c>
-      <c r="N24" s="12" t="n">
-        <v>440834</v>
-      </c>
       <c r="P24" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
@@ -2142,7 +2142,7 @@
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-20822</v>
+        <v>-26464</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>18253</v>
+        <v>12953</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>18253</v>
+        <v>12953</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q25" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="11" t="n">
-        <v>-19739</v>
+      <c r="S25" s="14" t="n">
+        <v>4055</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>138628</v>
+        <v>72761</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>59437</v>
+        <v>33865</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>79191</v>
+        <v>38896</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>942048</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>903152</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>823961</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>708815</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>571811</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>539323</v>
       </c>
     </row>
     <row r="28">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>40056</v>
+        <v>7018</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-40056</v>
+        <v>-6997</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-298573</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-291576</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-251520</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-232982</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-206949</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-172978</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>12952</v>
+        <v>5750</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2373,7 +2373,7 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>31265</v>
+        <v>11185</v>
       </c>
       <c r="F29" s="13" t="inlineStr">
         <is>
@@ -2381,7 +2381,7 @@
         </is>
       </c>
       <c r="G29" s="14" t="n">
-        <v>-18313</v>
+        <v>-5435</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-174593</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-169158</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-150845</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-139051</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-103043</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-103139</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 02-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 03-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>44715</v>
+        <v>15192</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>65537</v>
+        <v>41656</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-20822</v>
+        <v>-26464</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-468882</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-442418</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-421596</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-336782</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-261819</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-263206</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23858</v>
+        <v>23997.95</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>23914.45</v>
+        <v>24025.4</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>196295</v>
+        <v>93724</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>196295</v>
+        <v>93724</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23786.8</v>
+        <v>23873.45</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23914.45</v>
+        <v>23873.45</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24084.65</v>
+        <v>24126.7</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23893.175</v>
+        <v>23898.775</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>39831</v>
+        <v>9645</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>27548</v>
-      </c>
-      <c r="F33" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n">
-        <v>12283</v>
+        <v>22163</v>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="n">
+        <v>-12518</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-396352</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-383834</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-396117</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-361418</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-341070</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-356201</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>23999.55</v>
+        <v>24076.05</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23871.9</v>
+        <v>23924.1</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>351</v>
+        <v>1122</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>744</v>
+        <v>2710</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-393</v>
+        <v>-1588</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>26959</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>28547</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>28940</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>29511</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>29229</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>29994</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23957</v>
+        <v>23974.75</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23850.625</v>
+        <v>23949.425</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>21530</v>
+        <v>15835</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,7 +2745,7 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>13681</v>
+        <v>5784</v>
       </c>
       <c r="F35" s="13" t="inlineStr">
         <is>
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>7849</v>
+        <v>10051</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>118254</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>108203</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>100354</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>92473</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>76550</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>74854</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23871.9</v>
+        <v>23924.1</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>27430</v>
+        <v>19051</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>47169</v>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="n">
-        <v>-19739</v>
+        <v>14996</v>
+      </c>
+      <c r="F36" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G36" s="14" t="n">
+        <v>4055</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>251139</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>247084</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>266823</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>239434</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>235291</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>251353</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23829.34999999999</v>
+        <v>23822.8</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>89142</v>
+        <v>45653</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>89142</v>
+        <v>45653</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23744.25</v>
+        <v>23772.15</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23701.69999999999</v>
+        <v>23670.85</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>11.34</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.59</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.49</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.19</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>10.68</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>11.07</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9984194572259013</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9999294072299643</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>1.005517111378178</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.006164539061341</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.009662619345433</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.005678413660525</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,914    PCR(OI) 0.73    Max Pain 23,950</t>
+          <t>Spot 23,873    PCR(OI) 0.65    Max Pain 23,950</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23911.24274193549</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23916.13830645161</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23923.80967741935</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23932.86491935484</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23944.28548387097</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23954.82459677419</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23873.45</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23914.45</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>24055.8</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24080.4</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24175.65</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24090.85</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,13 +3137,13 @@
         <v>24000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>134710</v>
+        <v>285418</v>
       </c>
       <c r="R45" s="11" t="n">
-        <v>45881</v>
+        <v>150708</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>2832927</v>
+        <v>3918502</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9820712062874193</v>
+        <v>0.9804008117537042</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9933791141865997</v>
@@ -3173,16 +3173,16 @@
         <v>1.011430829957649</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24200</v>
+        <v>24100</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>155299</v>
+        <v>187495</v>
       </c>
       <c r="R46" s="11" t="n">
-        <v>41535</v>
+        <v>65080</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>1308169</v>
+        <v>2198143</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24351.03467741935</v>
+        <v>24350.70403225806</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24336.7810483871</v>
@@ -3215,13 +3215,13 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>140433</v>
+        <v>256210</v>
       </c>
       <c r="R47" s="11" t="n">
-        <v>55828</v>
+        <v>115777</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>574623</v>
+        <v>635844</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23914.45</v>
+        <v>23873.45</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24175.65</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>02-Sep-2026</t>
+          <t>03-Sep-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3319,35 +3319,35 @@
     </row>
     <row r="50">
       <c r="P50" s="33" t="n">
-        <v>23800</v>
+        <v>23500</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>120404</v>
+        <v>161870</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>74010</v>
+        <v>41901</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>3647157</v>
-      </c>
-      <c r="T50" s="29" t="inlineStr">
-        <is>
-          <t>High</t>
+        <v>1072636</v>
+      </c>
+      <c r="T50" s="31" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="33" t="n">
-        <v>23500</v>
+        <v>23000</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>119969</v>
+        <v>164129</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>24665</v>
+        <v>36008</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>1114845</v>
+        <v>636033</v>
       </c>
       <c r="T51" s="31" t="inlineStr">
         <is>
@@ -3357,16 +3357,16 @@
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>23000</v>
+        <v>22500</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>128121</v>
+        <v>137056</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>52537</v>
+        <v>62909</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>567792</v>
+        <v>329317</v>
       </c>
       <c r="T52" s="31" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 02-Sep-2026    1 DAY AGO = 01-Sep-2026    2 DAYS AGO = 31-Aug-2026    3 DAYS AGO = 28-Aug-2026    4 DAYS AGO = 27-Aug-2026    (generated 02-Sep-2026 21:04 IST)</t>
+          <t>TODAY = 03-Sep-2026    1 DAY AGO = 02-Sep-2026    2 DAYS AGO = 01-Sep-2026    3 DAYS AGO = 31-Aug-2026    4 DAYS AGO = 28-Aug-2026    (generated 03-Sep-2026 20:31 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update participant OI report - 2026-09-04
</commit_message>
<xml_diff>
--- a/participant_oi.xlsx
+++ b/participant_oi.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="S2" s="11" t="n">
-        <v>5926</v>
+        <v>3846</v>
       </c>
     </row>
     <row r="3">
@@ -705,7 +705,7 @@
         </is>
       </c>
       <c r="C3" s="11" t="n">
-        <v>1331</v>
+        <v>82</v>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
@@ -713,7 +713,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>-4595</v>
+        <v>-3764</v>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>5926</v>
+        <v>3846</v>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
@@ -729,28 +729,28 @@
         </is>
       </c>
       <c r="J3" s="12" t="n">
+        <v>209842</v>
+      </c>
+      <c r="K3" s="12" t="n">
         <v>205996</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="L3" s="12" t="n">
         <v>200070</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="M3" s="12" t="n">
         <v>187130</v>
       </c>
-      <c r="M3" s="12" t="n">
+      <c r="N3" s="12" t="n">
         <v>178219</v>
       </c>
-      <c r="N3" s="12" t="n">
-        <v>176959</v>
-      </c>
       <c r="P3" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q3" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R3" s="10" t="inlineStr">
@@ -758,8 +758,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S3" s="11" t="n">
-        <v>109470</v>
+      <c r="S3" s="14" t="n">
+        <v>-156667</v>
       </c>
     </row>
     <row r="4">
@@ -774,7 +774,7 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>50</v>
+        <v>282</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
@@ -782,53 +782,53 @@
         </is>
       </c>
       <c r="E4" s="14" t="n">
-        <v>30</v>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
+        <v>2200</v>
+      </c>
+      <c r="F4" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="n">
+        <v>-1918</v>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>11369</v>
+      </c>
+      <c r="K4" s="12" t="n">
+        <v>13287</v>
+      </c>
+      <c r="L4" s="12" t="n">
+        <v>13267</v>
+      </c>
+      <c r="M4" s="12" t="n">
+        <v>20477</v>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>20288</v>
+      </c>
+      <c r="P4" s="8" t="inlineStr">
+        <is>
+          <t>Clients</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G4" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="J4" s="12" t="n">
-        <v>13287</v>
-      </c>
-      <c r="K4" s="12" t="n">
-        <v>13267</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>20477</v>
-      </c>
-      <c r="M4" s="12" t="n">
-        <v>20288</v>
-      </c>
-      <c r="N4" s="12" t="n">
-        <v>20213</v>
-      </c>
-      <c r="P4" s="8" t="inlineStr">
-        <is>
-          <t>Clients</t>
-        </is>
-      </c>
-      <c r="Q4" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R4" s="10" t="inlineStr">
         <is>
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S4" s="11" t="n">
-        <v>-89681</v>
+      <c r="S4" s="14" t="n">
+        <v>85563</v>
       </c>
     </row>
     <row r="5">
@@ -843,7 +843,7 @@
         </is>
       </c>
       <c r="C5" s="11" t="n">
-        <v>4965</v>
+        <v>187</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
         <is>
@@ -851,7 +851,7 @@
         </is>
       </c>
       <c r="E5" s="14" t="n">
-        <v>10904</v>
+        <v>923</v>
       </c>
       <c r="F5" s="13" t="inlineStr">
         <is>
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="G5" s="14" t="n">
-        <v>-5939</v>
+        <v>-736</v>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
@@ -867,20 +867,20 @@
         </is>
       </c>
       <c r="J5" s="12" t="n">
+        <v>-235838</v>
+      </c>
+      <c r="K5" s="12" t="n">
         <v>-235102</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="L5" s="12" t="n">
         <v>-229163</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="M5" s="12" t="n">
         <v>-222032</v>
       </c>
-      <c r="M5" s="12" t="n">
+      <c r="N5" s="12" t="n">
         <v>-209315</v>
       </c>
-      <c r="N5" s="12" t="n">
-        <v>-202633</v>
-      </c>
       <c r="P5" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="S5" s="11" t="n">
-        <v>3077</v>
+        <v>8511</v>
       </c>
     </row>
     <row r="6">
@@ -906,21 +906,21 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>1959</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="n">
-        <v>1966</v>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>-1920</v>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>-728</v>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="G6" s="14" t="n">
-        <v>-7</v>
+        <v>-1192</v>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
@@ -936,20 +936,20 @@
         </is>
       </c>
       <c r="J6" s="12" t="n">
+        <v>14627</v>
+      </c>
+      <c r="K6" s="12" t="n">
         <v>15819</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="L6" s="12" t="n">
         <v>15826</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="M6" s="12" t="n">
         <v>14425</v>
       </c>
-      <c r="M6" s="12" t="n">
+      <c r="N6" s="12" t="n">
         <v>10808</v>
       </c>
-      <c r="N6" s="12" t="n">
-        <v>5461</v>
-      </c>
       <c r="P6" s="8" t="inlineStr">
         <is>
           <t>Clients</t>
@@ -966,7 +966,7 @@
         </is>
       </c>
       <c r="S6" s="11" t="n">
-        <v>38896</v>
+        <v>34022</v>
       </c>
     </row>
     <row r="7">
@@ -977,11 +977,11 @@
       </c>
       <c r="B7" s="16" t="inlineStr"/>
       <c r="C7" s="17" t="n">
-        <v>8305</v>
+        <v>-1369</v>
       </c>
       <c r="D7" s="16" t="inlineStr"/>
       <c r="E7" s="17" t="n">
-        <v>8305</v>
+        <v>-1369</v>
       </c>
       <c r="F7" s="16" t="inlineStr"/>
       <c r="G7" s="17" t="n">
@@ -1002,9 +1002,9 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q7" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R7" s="10" t="inlineStr">
@@ -1012,8 +1012,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S7" s="11" t="n">
-        <v>-12518</v>
+      <c r="S7" s="14" t="n">
+        <v>3924</v>
       </c>
     </row>
     <row r="8">
@@ -1071,9 +1071,9 @@
           <t>DIIs</t>
         </is>
       </c>
-      <c r="Q8" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q8" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R8" s="10" t="inlineStr">
@@ -1081,8 +1081,8 @@
           <t>Index Futures</t>
         </is>
       </c>
-      <c r="S8" s="11" t="n">
-        <v>20</v>
+      <c r="S8" s="14" t="n">
+        <v>-1918</v>
       </c>
     </row>
     <row r="9">
@@ -1091,13 +1091,13 @@
           <t>Clients</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="n">
-        <v>692342</v>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>-82103</v>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
@@ -1105,15 +1105,15 @@
         </is>
       </c>
       <c r="E9" s="14" t="n">
-        <v>582872</v>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="n">
-        <v>109470</v>
+        <v>74564</v>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>-156667</v>
       </c>
       <c r="I9" s="8" t="inlineStr">
         <is>
@@ -1121,20 +1121,20 @@
         </is>
       </c>
       <c r="J9" s="12" t="n">
+        <v>225870</v>
+      </c>
+      <c r="K9" s="12" t="n">
         <v>382537</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="L9" s="12" t="n">
         <v>273067</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="M9" s="12" t="n">
         <v>261983</v>
       </c>
-      <c r="M9" s="12" t="n">
+      <c r="N9" s="12" t="n">
         <v>195682</v>
       </c>
-      <c r="N9" s="12" t="n">
-        <v>91197</v>
-      </c>
       <c r="P9" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="S9" s="14" t="n">
-        <v>-150</v>
+        <v>-215</v>
       </c>
     </row>
     <row r="10">
@@ -1174,7 +1174,7 @@
         </is>
       </c>
       <c r="E10" s="14" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="G10" s="14" t="n">
-        <v>-150</v>
+        <v>-215</v>
       </c>
       <c r="I10" s="8" t="inlineStr">
         <is>
@@ -1190,20 +1190,20 @@
         </is>
       </c>
       <c r="J10" s="12" t="n">
+        <v>3895</v>
+      </c>
+      <c r="K10" s="12" t="n">
         <v>4110</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="L10" s="12" t="n">
         <v>4260</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="M10" s="12" t="n">
         <v>4835</v>
       </c>
-      <c r="M10" s="12" t="n">
+      <c r="N10" s="12" t="n">
         <v>4310</v>
       </c>
-      <c r="N10" s="12" t="n">
-        <v>4350</v>
-      </c>
       <c r="P10" s="8" t="inlineStr">
         <is>
           <t>DIIs</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
       <c r="S10" s="14" t="n">
-        <v>2031</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11">
@@ -1235,61 +1235,61 @@
         </is>
       </c>
       <c r="C11" s="11" t="n">
-        <v>93060</v>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="n">
-        <v>106014</v>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
+        <v>6433</v>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>-2320</v>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="n">
+        <v>8753</v>
+      </c>
+      <c r="I11" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="n">
+        <v>-303454</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>-312207</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>-299253</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>-248061</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>-225462</v>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G11" s="14" t="n">
-        <v>-12954</v>
-      </c>
-      <c r="I11" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J11" s="12" t="n">
-        <v>-312207</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>-299253</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>-248061</v>
-      </c>
-      <c r="M11" s="12" t="n">
-        <v>-225462</v>
-      </c>
-      <c r="N11" s="12" t="n">
-        <v>-230020</v>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q11" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R11" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S11" s="14" t="n">
-        <v>-3077</v>
+        <v>-38077</v>
       </c>
     </row>
     <row r="12">
@@ -1304,61 +1304,61 @@
         </is>
       </c>
       <c r="C12" s="11" t="n">
-        <v>225907</v>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>Added Shorts</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="n">
-        <v>322273</v>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
+        <v>30446</v>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Closed Shorts</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>-117684</v>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="n">
+        <v>148130</v>
+      </c>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>73689</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>-74441</v>
+      </c>
+      <c r="L12" s="12" t="n">
+        <v>21925</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>-18758</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>25471</v>
+      </c>
+      <c r="P12" s="8" t="inlineStr">
+        <is>
+          <t>DIIs</t>
+        </is>
+      </c>
+      <c r="Q12" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G12" s="14" t="n">
-        <v>-96366</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J12" s="12" t="n">
-        <v>-74441</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>21925</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>-18758</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>25471</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>134473</v>
-      </c>
-      <c r="P12" s="8" t="inlineStr">
-        <is>
-          <t>DIIs</t>
-        </is>
-      </c>
-      <c r="Q12" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R12" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S12" s="14" t="n">
-        <v>-6997</v>
+        <v>-10130</v>
       </c>
     </row>
     <row r="13">
@@ -1369,15 +1369,15 @@
       </c>
       <c r="B13" s="16" t="inlineStr"/>
       <c r="C13" s="17" t="n">
-        <v>1011309</v>
+        <v>-45224</v>
       </c>
       <c r="D13" s="16" t="inlineStr"/>
       <c r="E13" s="17" t="n">
-        <v>1011309</v>
+        <v>-45225</v>
       </c>
       <c r="F13" s="16" t="inlineStr"/>
       <c r="G13" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I13" s="15" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="S13" s="11" t="n">
-        <v>-1588</v>
+        <v>-358</v>
       </c>
     </row>
     <row r="14">
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="S14" s="14" t="n">
-        <v>-5939</v>
+        <v>-736</v>
       </c>
     </row>
     <row r="15">
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="C15" s="14" t="n">
-        <v>233565</v>
+        <v>441611</v>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
@@ -1497,15 +1497,15 @@
         </is>
       </c>
       <c r="E15" s="11" t="n">
-        <v>323246</v>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="n">
-        <v>-89681</v>
+        <v>356048</v>
+      </c>
+      <c r="F15" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="n">
+        <v>85563</v>
       </c>
       <c r="I15" s="8" t="inlineStr">
         <is>
@@ -1513,28 +1513,28 @@
         </is>
       </c>
       <c r="J15" s="12" t="n">
+        <v>-716258</v>
+      </c>
+      <c r="K15" s="12" t="n">
         <v>-801821</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="L15" s="12" t="n">
         <v>-712140</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="M15" s="12" t="n">
         <v>-756948</v>
       </c>
-      <c r="M15" s="12" t="n">
+      <c r="N15" s="12" t="n">
         <v>-686046</v>
       </c>
-      <c r="N15" s="12" t="n">
-        <v>-725066</v>
-      </c>
       <c r="P15" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q15" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R15" s="10" t="inlineStr">
@@ -1542,8 +1542,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S15" s="14" t="n">
-        <v>-12954</v>
+      <c r="S15" s="11" t="n">
+        <v>8753</v>
       </c>
     </row>
     <row r="16">
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="C16" s="14" t="n">
-        <v>2031</v>
+        <v>68</v>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
@@ -1574,7 +1574,7 @@
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>2031</v>
+        <v>68</v>
       </c>
       <c r="I16" s="8" t="inlineStr">
         <is>
@@ -1582,28 +1582,28 @@
         </is>
       </c>
       <c r="J16" s="12" t="n">
+        <v>32107</v>
+      </c>
+      <c r="K16" s="12" t="n">
         <v>32039</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="L16" s="12" t="n">
         <v>30008</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="M16" s="12" t="n">
         <v>31923</v>
       </c>
-      <c r="M16" s="12" t="n">
+      <c r="N16" s="12" t="n">
         <v>31784</v>
       </c>
-      <c r="N16" s="12" t="n">
-        <v>34489</v>
-      </c>
       <c r="P16" s="8" t="inlineStr">
         <is>
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q16" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R16" s="10" t="inlineStr">
@@ -1611,8 +1611,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S16" s="14" t="n">
-        <v>56826</v>
+      <c r="S16" s="11" t="n">
+        <v>-69138</v>
       </c>
     </row>
     <row r="17">
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="C17" s="14" t="n">
-        <v>79978</v>
+        <v>18950</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
@@ -1635,53 +1635,53 @@
         </is>
       </c>
       <c r="E17" s="11" t="n">
-        <v>23152</v>
-      </c>
-      <c r="F17" s="13" t="inlineStr">
+        <v>88088</v>
+      </c>
+      <c r="F17" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="n">
+        <v>-69138</v>
+      </c>
+      <c r="I17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="n">
+        <v>580911</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>650049</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>593223</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>632465</v>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>551407</v>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q17" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G17" s="14" t="n">
-        <v>56826</v>
-      </c>
-      <c r="I17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="J17" s="12" t="n">
-        <v>650049</v>
-      </c>
-      <c r="K17" s="12" t="n">
-        <v>593223</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>632465</v>
-      </c>
-      <c r="M17" s="12" t="n">
-        <v>551407</v>
-      </c>
-      <c r="N17" s="12" t="n">
-        <v>594360</v>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q17" s="9" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
       <c r="R17" s="10" t="inlineStr">
         <is>
           <t>Stock Futures</t>
         </is>
       </c>
       <c r="S17" s="11" t="n">
-        <v>16895</v>
+        <v>20246</v>
       </c>
     </row>
     <row r="18">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>180107</v>
+        <v>113196</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
@@ -1704,53 +1704,53 @@
         </is>
       </c>
       <c r="E18" s="11" t="n">
-        <v>149283</v>
-      </c>
-      <c r="F18" s="13" t="inlineStr">
+        <v>129689</v>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="n">
+        <v>-16493</v>
+      </c>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="n">
+        <v>103240</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>119733</v>
+      </c>
+      <c r="L18" s="12" t="n">
+        <v>88909</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>92559</v>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>102855</v>
+      </c>
+      <c r="P18" s="8" t="inlineStr">
+        <is>
+          <t>FIIs</t>
+        </is>
+      </c>
+      <c r="Q18" s="9" t="inlineStr">
         <is>
           <t>Bought Net</t>
         </is>
       </c>
-      <c r="G18" s="14" t="n">
-        <v>30824</v>
-      </c>
-      <c r="I18" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J18" s="12" t="n">
-        <v>119733</v>
-      </c>
-      <c r="K18" s="12" t="n">
-        <v>88909</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>92559</v>
-      </c>
-      <c r="M18" s="12" t="n">
-        <v>102855</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>96217</v>
-      </c>
-      <c r="P18" s="8" t="inlineStr">
-        <is>
-          <t>FIIs</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R18" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
-      <c r="S18" s="14" t="n">
-        <v>-5435</v>
+      <c r="S18" s="11" t="n">
+        <v>2747</v>
       </c>
     </row>
     <row r="19">
@@ -1761,11 +1761,11 @@
       </c>
       <c r="B19" s="16" t="inlineStr"/>
       <c r="C19" s="17" t="n">
-        <v>495681</v>
+        <v>573825</v>
       </c>
       <c r="D19" s="16" t="inlineStr"/>
       <c r="E19" s="17" t="n">
-        <v>495681</v>
+        <v>573825</v>
       </c>
       <c r="F19" s="16" t="inlineStr"/>
       <c r="G19" s="17" t="n">
@@ -1786,9 +1786,9 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="Q19" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q19" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R19" s="10" t="inlineStr">
@@ -1796,8 +1796,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S19" s="14" t="n">
-        <v>10051</v>
+      <c r="S19" s="11" t="n">
+        <v>-85</v>
       </c>
     </row>
     <row r="20">
@@ -1866,7 +1866,7 @@
         </is>
       </c>
       <c r="S20" s="14" t="n">
-        <v>-7</v>
+        <v>-1192</v>
       </c>
     </row>
     <row r="21">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="C21" s="11" t="n">
-        <v>10069</v>
+        <v>10221</v>
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="E21" s="14" t="n">
-        <v>6992</v>
+        <v>1710</v>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="G21" s="11" t="n">
-        <v>3077</v>
+        <v>8511</v>
       </c>
       <c r="I21" s="8" t="inlineStr">
         <is>
@@ -1905,28 +1905,28 @@
         </is>
       </c>
       <c r="J21" s="12" t="n">
+        <v>3185084</v>
+      </c>
+      <c r="K21" s="12" t="n">
         <v>3176573</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="L21" s="12" t="n">
         <v>3173496</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="M21" s="12" t="n">
         <v>3185328</v>
       </c>
-      <c r="M21" s="12" t="n">
+      <c r="N21" s="12" t="n">
         <v>3192623</v>
       </c>
-      <c r="N21" s="12" t="n">
-        <v>3161018</v>
-      </c>
       <c r="P21" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q21" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q21" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R21" s="10" t="inlineStr">
@@ -1934,8 +1934,8 @@
           <t>Index Call</t>
         </is>
       </c>
-      <c r="S21" s="14" t="n">
-        <v>-96366</v>
+      <c r="S21" s="11" t="n">
+        <v>148130</v>
       </c>
     </row>
     <row r="22">
@@ -1950,7 +1950,7 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>12811</v>
+        <v>3508</v>
       </c>
       <c r="D22" s="13" t="inlineStr">
         <is>
@@ -1958,7 +1958,7 @@
         </is>
       </c>
       <c r="E22" s="14" t="n">
-        <v>15888</v>
+        <v>41585</v>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
@@ -1966,7 +1966,7 @@
         </is>
       </c>
       <c r="G22" s="14" t="n">
-        <v>-3077</v>
+        <v>-38077</v>
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
@@ -1974,28 +1974,28 @@
         </is>
       </c>
       <c r="J22" s="12" t="n">
+        <v>-4275639</v>
+      </c>
+      <c r="K22" s="12" t="n">
         <v>-4237562</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="L22" s="12" t="n">
         <v>-4234485</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="M22" s="12" t="n">
         <v>-4195881</v>
       </c>
-      <c r="M22" s="12" t="n">
+      <c r="N22" s="12" t="n">
         <v>-4220839</v>
       </c>
-      <c r="N22" s="12" t="n">
-        <v>-4163984</v>
-      </c>
       <c r="P22" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q22" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q22" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R22" s="10" t="inlineStr">
@@ -2003,8 +2003,8 @@
           <t>Index Put</t>
         </is>
       </c>
-      <c r="S22" s="14" t="n">
-        <v>30824</v>
+      <c r="S22" s="11" t="n">
+        <v>-16493</v>
       </c>
     </row>
     <row r="23">
@@ -2013,13 +2013,13 @@
           <t>FIIs</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>Added Longs</t>
-        </is>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>1041</v>
+      <c r="B23" s="13" t="inlineStr">
+        <is>
+          <t>Closed Longs</t>
+        </is>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>-5212</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
@@ -2027,7 +2027,7 @@
         </is>
       </c>
       <c r="E23" s="11" t="n">
-        <v>-15854</v>
+        <v>-25458</v>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="G23" s="11" t="n">
-        <v>16895</v>
+        <v>20246</v>
       </c>
       <c r="I23" s="8" t="inlineStr">
         <is>
@@ -2043,28 +2043,28 @@
         </is>
       </c>
       <c r="J23" s="12" t="n">
+        <v>630143</v>
+      </c>
+      <c r="K23" s="12" t="n">
         <v>609897</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="L23" s="12" t="n">
         <v>593002</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="M23" s="12" t="n">
         <v>551323</v>
       </c>
-      <c r="M23" s="12" t="n">
+      <c r="N23" s="12" t="n">
         <v>563880</v>
       </c>
-      <c r="N23" s="12" t="n">
-        <v>549226</v>
-      </c>
       <c r="P23" s="8" t="inlineStr">
         <is>
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q23" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
+      <c r="Q23" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
         </is>
       </c>
       <c r="R23" s="10" t="inlineStr">
@@ -2072,8 +2072,8 @@
           <t>Stock Futures</t>
         </is>
       </c>
-      <c r="S23" s="14" t="n">
-        <v>-16895</v>
+      <c r="S23" s="11" t="n">
+        <v>9320</v>
       </c>
     </row>
     <row r="24">
@@ -2082,13 +2082,13 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Closed Longs</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="n">
-        <v>-10968</v>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Added Longs</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>14708</v>
       </c>
       <c r="D24" s="13" t="inlineStr">
         <is>
@@ -2096,53 +2096,53 @@
         </is>
       </c>
       <c r="E24" s="14" t="n">
-        <v>5927</v>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
+        <v>5388</v>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>9320</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="J24" s="12" t="n">
+        <v>460412</v>
+      </c>
+      <c r="K24" s="12" t="n">
+        <v>451092</v>
+      </c>
+      <c r="L24" s="12" t="n">
+        <v>467987</v>
+      </c>
+      <c r="M24" s="12" t="n">
+        <v>459230</v>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>464336</v>
+      </c>
+      <c r="P24" s="8" t="inlineStr">
+        <is>
+          <t>Pro</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
         <is>
           <t>Sold Net</t>
         </is>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>-16895</v>
-      </c>
-      <c r="I24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="J24" s="12" t="n">
-        <v>451092</v>
-      </c>
-      <c r="K24" s="12" t="n">
-        <v>467987</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>459230</v>
-      </c>
-      <c r="M24" s="12" t="n">
-        <v>464336</v>
-      </c>
-      <c r="N24" s="12" t="n">
-        <v>453740</v>
-      </c>
-      <c r="P24" s="8" t="inlineStr">
-        <is>
-          <t>Pro</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
       <c r="R24" s="10" t="inlineStr">
         <is>
           <t>Stock Calls</t>
         </is>
       </c>
       <c r="S24" s="14" t="n">
-        <v>-26464</v>
+        <v>-26639</v>
       </c>
     </row>
     <row r="25">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B25" s="16" t="inlineStr"/>
       <c r="C25" s="17" t="n">
-        <v>12953</v>
+        <v>23225</v>
       </c>
       <c r="D25" s="16" t="inlineStr"/>
       <c r="E25" s="17" t="n">
-        <v>12953</v>
+        <v>23225</v>
       </c>
       <c r="F25" s="16" t="inlineStr"/>
       <c r="G25" s="17" t="n">
@@ -2178,9 +2178,9 @@
           <t>Pro</t>
         </is>
       </c>
-      <c r="Q25" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
+      <c r="Q25" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
         </is>
       </c>
       <c r="R25" s="10" t="inlineStr">
@@ -2188,8 +2188,8 @@
           <t>Stock Puts</t>
         </is>
       </c>
-      <c r="S25" s="14" t="n">
-        <v>4055</v>
+      <c r="S25" s="11" t="n">
+        <v>-3481</v>
       </c>
     </row>
     <row r="26">
@@ -2255,7 +2255,7 @@
         </is>
       </c>
       <c r="C27" s="11" t="n">
-        <v>72761</v>
+        <v>87376</v>
       </c>
       <c r="D27" s="13" t="inlineStr">
         <is>
@@ -2263,7 +2263,7 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>33865</v>
+        <v>53354</v>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
@@ -2271,7 +2271,7 @@
         </is>
       </c>
       <c r="G27" s="11" t="n">
-        <v>38896</v>
+        <v>34022</v>
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
@@ -2279,19 +2279,19 @@
         </is>
       </c>
       <c r="J27" s="12" t="n">
+        <v>976070</v>
+      </c>
+      <c r="K27" s="12" t="n">
         <v>942048</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="L27" s="12" t="n">
         <v>903152</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="M27" s="12" t="n">
         <v>823961</v>
       </c>
-      <c r="M27" s="12" t="n">
+      <c r="N27" s="12" t="n">
         <v>708815</v>
-      </c>
-      <c r="N27" s="12" t="n">
-        <v>571811</v>
       </c>
     </row>
     <row r="28">
@@ -2306,7 +2306,7 @@
         </is>
       </c>
       <c r="C28" s="11" t="n">
-        <v>21</v>
+        <v>218</v>
       </c>
       <c r="D28" s="13" t="inlineStr">
         <is>
@@ -2314,7 +2314,7 @@
         </is>
       </c>
       <c r="E28" s="14" t="n">
-        <v>7018</v>
+        <v>10348</v>
       </c>
       <c r="F28" s="13" t="inlineStr">
         <is>
@@ -2322,7 +2322,7 @@
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>-6997</v>
+        <v>-10130</v>
       </c>
       <c r="I28" s="8" t="inlineStr">
         <is>
@@ -2330,19 +2330,19 @@
         </is>
       </c>
       <c r="J28" s="12" t="n">
+        <v>-308703</v>
+      </c>
+      <c r="K28" s="12" t="n">
         <v>-298573</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="L28" s="12" t="n">
         <v>-291576</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="M28" s="12" t="n">
         <v>-251520</v>
       </c>
-      <c r="M28" s="12" t="n">
+      <c r="N28" s="12" t="n">
         <v>-232982</v>
-      </c>
-      <c r="N28" s="12" t="n">
-        <v>-206949</v>
       </c>
       <c r="P28" s="3" t="inlineStr">
         <is>
@@ -2365,7 +2365,7 @@
         </is>
       </c>
       <c r="C29" s="11" t="n">
-        <v>5750</v>
+        <v>13556</v>
       </c>
       <c r="D29" s="13" t="inlineStr">
         <is>
@@ -2373,15 +2373,15 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>11185</v>
-      </c>
-      <c r="F29" s="13" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n">
-        <v>-5435</v>
+        <v>10809</v>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n">
+        <v>2747</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
         </is>
       </c>
       <c r="J29" s="12" t="n">
+        <v>-171846</v>
+      </c>
+      <c r="K29" s="12" t="n">
         <v>-174593</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="L29" s="12" t="n">
         <v>-169158</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="M29" s="12" t="n">
         <v>-150845</v>
       </c>
-      <c r="M29" s="12" t="n">
+      <c r="N29" s="12" t="n">
         <v>-139051</v>
       </c>
-      <c r="N29" s="12" t="n">
-        <v>-103043</v>
-      </c>
       <c r="P29" s="5" t="inlineStr">
         <is>
-          <t>Next session  -  based on 03-Sep-2026 OHLC</t>
+          <t>Next session  -  based on 04-Sep-2026 OHLC</t>
         </is>
       </c>
       <c r="Q29" s="6" t="inlineStr"/>
@@ -2424,7 +2424,7 @@
         </is>
       </c>
       <c r="C30" s="11" t="n">
-        <v>15192</v>
+        <v>26838</v>
       </c>
       <c r="D30" s="13" t="inlineStr">
         <is>
@@ -2432,7 +2432,7 @@
         </is>
       </c>
       <c r="E30" s="14" t="n">
-        <v>41656</v>
+        <v>53477</v>
       </c>
       <c r="F30" s="13" t="inlineStr">
         <is>
@@ -2440,7 +2440,7 @@
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>-26464</v>
+        <v>-26639</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
@@ -2448,27 +2448,27 @@
         </is>
       </c>
       <c r="J30" s="12" t="n">
+        <v>-495521</v>
+      </c>
+      <c r="K30" s="12" t="n">
         <v>-468882</v>
       </c>
-      <c r="K30" s="12" t="n">
+      <c r="L30" s="12" t="n">
         <v>-442418</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="M30" s="12" t="n">
         <v>-421596</v>
       </c>
-      <c r="M30" s="12" t="n">
+      <c r="N30" s="12" t="n">
         <v>-336782</v>
       </c>
-      <c r="N30" s="12" t="n">
-        <v>-261819</v>
-      </c>
       <c r="P30" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
       <c r="Q30" s="18" t="n">
-        <v>23997.95</v>
+        <v>23910.9</v>
       </c>
       <c r="R30" s="8" t="inlineStr">
         <is>
@@ -2476,7 +2476,7 @@
         </is>
       </c>
       <c r="S30" s="18" t="n">
-        <v>24025.4</v>
+        <v>24005.75</v>
       </c>
     </row>
     <row r="31">
@@ -2487,11 +2487,11 @@
       </c>
       <c r="B31" s="16" t="inlineStr"/>
       <c r="C31" s="17" t="n">
-        <v>93724</v>
+        <v>127988</v>
       </c>
       <c r="D31" s="16" t="inlineStr"/>
       <c r="E31" s="17" t="n">
-        <v>93724</v>
+        <v>127988</v>
       </c>
       <c r="F31" s="16" t="inlineStr"/>
       <c r="G31" s="17" t="n">
@@ -2513,7 +2513,7 @@
         </is>
       </c>
       <c r="Q31" s="18" t="n">
-        <v>23873.45</v>
+        <v>23895.85</v>
       </c>
       <c r="R31" s="8" t="inlineStr">
         <is>
@@ -2521,7 +2521,7 @@
         </is>
       </c>
       <c r="S31" s="18" t="n">
-        <v>23873.45</v>
+        <v>23897.7</v>
       </c>
     </row>
     <row r="32">
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="Q32" s="20" t="n">
-        <v>24126.7</v>
+        <v>24080.25000000001</v>
       </c>
       <c r="R32" s="8" t="inlineStr">
         <is>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="S32" s="21" t="n">
-        <v>23898.775</v>
+        <v>23915.40000000001</v>
       </c>
     </row>
     <row r="33">
@@ -2603,7 +2603,7 @@
         </is>
       </c>
       <c r="C33" s="14" t="n">
-        <v>9645</v>
+        <v>34606</v>
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
@@ -2611,15 +2611,15 @@
         </is>
       </c>
       <c r="E33" s="11" t="n">
-        <v>22163</v>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
-        <is>
-          <t>Sold Net</t>
-        </is>
-      </c>
-      <c r="G33" s="11" t="n">
-        <v>-12518</v>
+        <v>30682</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Bought Net</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="n">
+        <v>3924</v>
       </c>
       <c r="I33" s="8" t="inlineStr">
         <is>
@@ -2627,27 +2627,27 @@
         </is>
       </c>
       <c r="J33" s="12" t="n">
+        <v>-392428</v>
+      </c>
+      <c r="K33" s="12" t="n">
         <v>-396352</v>
       </c>
-      <c r="K33" s="12" t="n">
+      <c r="L33" s="12" t="n">
         <v>-383834</v>
       </c>
-      <c r="L33" s="12" t="n">
+      <c r="M33" s="12" t="n">
         <v>-396117</v>
       </c>
-      <c r="M33" s="12" t="n">
+      <c r="N33" s="12" t="n">
         <v>-361418</v>
       </c>
-      <c r="N33" s="12" t="n">
-        <v>-341070</v>
-      </c>
       <c r="P33" s="19" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
       <c r="Q33" s="20" t="n">
-        <v>24076.05</v>
+        <v>24043</v>
       </c>
       <c r="R33" s="8" t="inlineStr">
         <is>
@@ -2655,7 +2655,7 @@
         </is>
       </c>
       <c r="S33" s="21" t="n">
-        <v>23924.1</v>
+        <v>23933.1</v>
       </c>
     </row>
     <row r="34">
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="C34" s="14" t="n">
-        <v>1122</v>
+        <v>700</v>
       </c>
       <c r="D34" s="9" t="inlineStr">
         <is>
@@ -2678,7 +2678,7 @@
         </is>
       </c>
       <c r="E34" s="11" t="n">
-        <v>2710</v>
+        <v>1058</v>
       </c>
       <c r="F34" s="9" t="inlineStr">
         <is>
@@ -2686,7 +2686,7 @@
         </is>
       </c>
       <c r="G34" s="11" t="n">
-        <v>-1588</v>
+        <v>-358</v>
       </c>
       <c r="I34" s="8" t="inlineStr">
         <is>
@@ -2694,27 +2694,27 @@
         </is>
       </c>
       <c r="J34" s="12" t="n">
+        <v>26601</v>
+      </c>
+      <c r="K34" s="12" t="n">
         <v>26959</v>
       </c>
-      <c r="K34" s="12" t="n">
+      <c r="L34" s="12" t="n">
         <v>28547</v>
       </c>
-      <c r="L34" s="12" t="n">
+      <c r="M34" s="12" t="n">
         <v>28940</v>
       </c>
-      <c r="M34" s="12" t="n">
+      <c r="N34" s="12" t="n">
         <v>29511</v>
       </c>
-      <c r="N34" s="12" t="n">
-        <v>29229</v>
-      </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
       <c r="Q34" s="20" t="n">
-        <v>23974.75</v>
+        <v>23970.35000000001</v>
       </c>
       <c r="R34" s="8" t="inlineStr">
         <is>
@@ -2722,7 +2722,7 @@
         </is>
       </c>
       <c r="S34" s="21" t="n">
-        <v>23949.425</v>
+        <v>23950.8</v>
       </c>
     </row>
     <row r="35">
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="C35" s="14" t="n">
-        <v>15835</v>
+        <v>11007</v>
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
@@ -2745,15 +2745,15 @@
         </is>
       </c>
       <c r="E35" s="11" t="n">
-        <v>5784</v>
-      </c>
-      <c r="F35" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G35" s="14" t="n">
-        <v>10051</v>
+        <v>11092</v>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="n">
+        <v>-85</v>
       </c>
       <c r="I35" s="8" t="inlineStr">
         <is>
@@ -2761,27 +2761,27 @@
         </is>
       </c>
       <c r="J35" s="12" t="n">
+        <v>118169</v>
+      </c>
+      <c r="K35" s="12" t="n">
         <v>118254</v>
       </c>
-      <c r="K35" s="12" t="n">
+      <c r="L35" s="12" t="n">
         <v>108203</v>
       </c>
-      <c r="L35" s="12" t="n">
+      <c r="M35" s="12" t="n">
         <v>100354</v>
       </c>
-      <c r="M35" s="12" t="n">
+      <c r="N35" s="12" t="n">
         <v>92473</v>
       </c>
-      <c r="N35" s="12" t="n">
-        <v>76550</v>
-      </c>
       <c r="P35" s="8" t="inlineStr">
         <is>
           <t>Pivot</t>
         </is>
       </c>
       <c r="Q35" s="21" t="n">
-        <v>23924.1</v>
+        <v>23933.1</v>
       </c>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="inlineStr"/>
@@ -2798,7 +2798,7 @@
         </is>
       </c>
       <c r="C36" s="14" t="n">
-        <v>19051</v>
+        <v>19733</v>
       </c>
       <c r="D36" s="9" t="inlineStr">
         <is>
@@ -2806,15 +2806,15 @@
         </is>
       </c>
       <c r="E36" s="11" t="n">
-        <v>14996</v>
-      </c>
-      <c r="F36" s="13" t="inlineStr">
-        <is>
-          <t>Bought Net</t>
-        </is>
-      </c>
-      <c r="G36" s="14" t="n">
-        <v>4055</v>
+        <v>23214</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>Sold Net</t>
+        </is>
+      </c>
+      <c r="G36" s="11" t="n">
+        <v>-3481</v>
       </c>
       <c r="I36" s="8" t="inlineStr">
         <is>
@@ -2822,27 +2822,27 @@
         </is>
       </c>
       <c r="J36" s="12" t="n">
+        <v>247658</v>
+      </c>
+      <c r="K36" s="12" t="n">
         <v>251139</v>
       </c>
-      <c r="K36" s="12" t="n">
+      <c r="L36" s="12" t="n">
         <v>247084</v>
       </c>
-      <c r="L36" s="12" t="n">
+      <c r="M36" s="12" t="n">
         <v>266823</v>
       </c>
-      <c r="M36" s="12" t="n">
+      <c r="N36" s="12" t="n">
         <v>239434</v>
       </c>
-      <c r="N36" s="12" t="n">
-        <v>235291</v>
-      </c>
       <c r="P36" s="22" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
       <c r="Q36" s="23" t="n">
-        <v>23822.8</v>
+        <v>23860.45</v>
       </c>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="inlineStr"/>
@@ -2855,11 +2855,11 @@
       </c>
       <c r="B37" s="16" t="inlineStr"/>
       <c r="C37" s="17" t="n">
-        <v>45653</v>
+        <v>66046</v>
       </c>
       <c r="D37" s="16" t="inlineStr"/>
       <c r="E37" s="17" t="n">
-        <v>45653</v>
+        <v>66046</v>
       </c>
       <c r="F37" s="16" t="inlineStr"/>
       <c r="G37" s="17" t="n">
@@ -2881,7 +2881,7 @@
         </is>
       </c>
       <c r="Q37" s="23" t="n">
-        <v>23772.15</v>
+        <v>23823.2</v>
       </c>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="inlineStr"/>
@@ -2893,7 +2893,7 @@
         </is>
       </c>
       <c r="Q38" s="23" t="n">
-        <v>23670.85</v>
+        <v>23750.55</v>
       </c>
       <c r="R38" t="inlineStr"/>
       <c r="S38" t="inlineStr"/>
@@ -2937,19 +2937,19 @@
         </is>
       </c>
       <c r="J40" s="24" t="n">
+        <v>10.68</v>
+      </c>
+      <c r="K40" s="24" t="n">
         <v>11.34</v>
       </c>
-      <c r="K40" s="24" t="n">
+      <c r="L40" s="24" t="n">
         <v>11.59</v>
       </c>
-      <c r="L40" s="24" t="n">
+      <c r="M40" s="24" t="n">
         <v>11.49</v>
       </c>
-      <c r="M40" s="24" t="n">
+      <c r="N40" s="24" t="n">
         <v>11.19</v>
-      </c>
-      <c r="N40" s="24" t="n">
-        <v>10.68</v>
       </c>
     </row>
     <row r="41">
@@ -3000,23 +3000,23 @@
         </is>
       </c>
       <c r="J42" s="25" t="n">
+        <v>0.9997263611508541</v>
+      </c>
+      <c r="K42" s="25" t="n">
         <v>0.9984194572259013</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="L42" s="25" t="n">
         <v>0.9999294072299643</v>
       </c>
-      <c r="L42" s="25" t="n">
+      <c r="M42" s="25" t="n">
         <v>1.005517111378178</v>
       </c>
-      <c r="M42" s="25" t="n">
+      <c r="N42" s="25" t="n">
         <v>1.006164539061341</v>
       </c>
-      <c r="N42" s="25" t="n">
-        <v>1.009662619345433</v>
-      </c>
       <c r="P42" s="5" t="inlineStr">
         <is>
-          <t>Spot 23,873    PCR(OI) 0.65    Max Pain 23,950</t>
+          <t>Spot 23,898    PCR(OI) 0.84    Max Pain 24,000</t>
         </is>
       </c>
       <c r="Q42" s="6" t="n"/>
@@ -3031,19 +3031,19 @@
         </is>
       </c>
       <c r="J43" s="18" t="n">
+        <v>23904.24112903226</v>
+      </c>
+      <c r="K43" s="18" t="n">
         <v>23911.24274193549</v>
       </c>
-      <c r="K43" s="18" t="n">
+      <c r="L43" s="18" t="n">
         <v>23916.13830645161</v>
       </c>
-      <c r="L43" s="18" t="n">
+      <c r="M43" s="18" t="n">
         <v>23923.80967741935</v>
       </c>
-      <c r="M43" s="18" t="n">
+      <c r="N43" s="18" t="n">
         <v>23932.86491935484</v>
-      </c>
-      <c r="N43" s="18" t="n">
-        <v>23944.28548387097</v>
       </c>
       <c r="P43" s="26" t="inlineStr">
         <is>
@@ -3062,19 +3062,19 @@
         </is>
       </c>
       <c r="J44" s="18" t="n">
+        <v>23897.7</v>
+      </c>
+      <c r="K44" s="18" t="n">
         <v>23873.45</v>
       </c>
-      <c r="K44" s="18" t="n">
+      <c r="L44" s="18" t="n">
         <v>23914.45</v>
       </c>
-      <c r="L44" s="18" t="n">
+      <c r="M44" s="18" t="n">
         <v>24055.8</v>
       </c>
-      <c r="M44" s="18" t="n">
+      <c r="N44" s="18" t="n">
         <v>24080.4</v>
-      </c>
-      <c r="N44" s="18" t="n">
-        <v>24175.65</v>
       </c>
       <c r="P44" s="27" t="inlineStr">
         <is>
@@ -3137,13 +3137,13 @@
         <v>24000</v>
       </c>
       <c r="Q45" s="12" t="n">
-        <v>285418</v>
-      </c>
-      <c r="R45" s="11" t="n">
-        <v>150708</v>
+        <v>233506</v>
+      </c>
+      <c r="R45" s="14" t="n">
+        <v>-49467</v>
       </c>
       <c r="S45" s="12" t="n">
-        <v>3918502</v>
+        <v>7532383</v>
       </c>
       <c r="T45" s="29" t="inlineStr">
         <is>
@@ -3158,7 +3158,7 @@
         </is>
       </c>
       <c r="J46" s="25" t="n">
-        <v>0.9804008117537042</v>
+        <v>0.9813887944889631</v>
       </c>
       <c r="K46" s="25" t="n">
         <v>0.9933791141865997</v>
@@ -3173,16 +3173,16 @@
         <v>1.011430829957649</v>
       </c>
       <c r="P46" s="28" t="n">
-        <v>24100</v>
+        <v>24200</v>
       </c>
       <c r="Q46" s="12" t="n">
-        <v>187495</v>
-      </c>
-      <c r="R46" s="11" t="n">
-        <v>65080</v>
+        <v>180285</v>
+      </c>
+      <c r="R46" s="14" t="n">
+        <v>-1055</v>
       </c>
       <c r="S46" s="12" t="n">
-        <v>2198143</v>
+        <v>2877335</v>
       </c>
       <c r="T46" s="30" t="inlineStr">
         <is>
@@ -3197,7 +3197,7 @@
         </is>
       </c>
       <c r="J47" s="18" t="n">
-        <v>24350.70403225806</v>
+        <v>24350.89959677419</v>
       </c>
       <c r="K47" s="18" t="n">
         <v>24336.7810483871</v>
@@ -3215,13 +3215,13 @@
         <v>25000</v>
       </c>
       <c r="Q47" s="12" t="n">
-        <v>256210</v>
-      </c>
-      <c r="R47" s="11" t="n">
-        <v>115777</v>
+        <v>218310</v>
+      </c>
+      <c r="R47" s="14" t="n">
+        <v>-38492</v>
       </c>
       <c r="S47" s="12" t="n">
-        <v>635844</v>
+        <v>752670</v>
       </c>
       <c r="T47" s="31" t="inlineStr">
         <is>
@@ -3236,7 +3236,7 @@
         </is>
       </c>
       <c r="J48" s="18" t="n">
-        <v>23873.45</v>
+        <v>23897.7</v>
       </c>
       <c r="K48" s="18" t="n">
         <v>24175.65</v>
@@ -3268,7 +3268,7 @@
       </c>
       <c r="J49" s="30" t="inlineStr">
         <is>
-          <t>03-Sep-2026</t>
+          <t>04-Sep-2026</t>
         </is>
       </c>
       <c r="K49" s="30" t="inlineStr">
@@ -3319,54 +3319,54 @@
     </row>
     <row r="50">
       <c r="P50" s="33" t="n">
-        <v>23500</v>
+        <v>23900</v>
       </c>
       <c r="Q50" s="12" t="n">
-        <v>161870</v>
+        <v>171059</v>
       </c>
       <c r="R50" s="11" t="n">
-        <v>41901</v>
+        <v>64327</v>
       </c>
       <c r="S50" s="12" t="n">
-        <v>1072636</v>
-      </c>
-      <c r="T50" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>7170241</v>
+      </c>
+      <c r="T50" s="29" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="P51" s="33" t="n">
-        <v>23000</v>
+        <v>23800</v>
       </c>
       <c r="Q51" s="12" t="n">
-        <v>164129</v>
+        <v>169564</v>
       </c>
       <c r="R51" s="11" t="n">
-        <v>36008</v>
+        <v>59469</v>
       </c>
       <c r="S51" s="12" t="n">
-        <v>636033</v>
-      </c>
-      <c r="T51" s="31" t="inlineStr">
-        <is>
-          <t>Low</t>
+        <v>3578353</v>
+      </c>
+      <c r="T51" s="30" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="P52" s="33" t="n">
-        <v>22500</v>
+        <v>23000</v>
       </c>
       <c r="Q52" s="12" t="n">
-        <v>137056</v>
+        <v>181983</v>
       </c>
       <c r="R52" s="11" t="n">
-        <v>62909</v>
+        <v>17908</v>
       </c>
       <c r="S52" s="12" t="n">
-        <v>329317</v>
+        <v>771093</v>
       </c>
       <c r="T52" s="31" t="inlineStr">
         <is>
@@ -3377,7 +3377,7 @@
     <row r="54">
       <c r="A54" s="34" t="inlineStr">
         <is>
-          <t>TODAY = 03-Sep-2026    1 DAY AGO = 02-Sep-2026    2 DAYS AGO = 01-Sep-2026    3 DAYS AGO = 31-Aug-2026    4 DAYS AGO = 28-Aug-2026    (generated 03-Sep-2026 20:31 IST)</t>
+          <t>TODAY = 04-Sep-2026    1 DAY AGO = 03-Sep-2026    2 DAYS AGO = 02-Sep-2026    3 DAYS AGO = 01-Sep-2026    4 DAYS AGO = 31-Aug-2026    (generated 04-Sep-2026 20:50 IST)</t>
         </is>
       </c>
     </row>

</xml_diff>